<commit_message>
Add subject related terms mapping and match labelling to pipeline
</commit_message>
<xml_diff>
--- a/data/reference/course_descriptions.xlsx
+++ b/data/reference/course_descriptions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,20 +429,25 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>related_terms</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>description_essex</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>description_manchester</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>description_ucas</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>combined_description</t>
         </is>
@@ -459,20 +464,25 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Accounting; Accounting and Finance; Accounting and Management; Accounting with Economics; Banking and Finance; Finance and Management</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>How can finance professionals act responsibility, but still meet business objectives? How does accounting information inform business decisions? Our BSc Accounting and Finance degree provides access to our virtual trading floor, where you make use of real-world Bloomberg Market Data Feed (B-PIPE), information and analytics to practise trading stocks and securities in the type of environment found in City finance firms. You study a wide range of topics and develop your quantitative skills, giving you the flexibility to pursue a career in finance, accounting or business management after graduation. You'll explore areas such as the preparation of financial statements and budgets, accounting standards and corporate governance, financial theory, portfolio management, options and futures markets, and risk management. BSc Accounting and Finance includes an introductory first year to familiarise you with wider business topics, such as management and marketing. In your final year, you have the opportunity to put your knowledge into practice by completing an in-depth, independent research project or dissertation. This will give you the chance to further develop vital employment skills in areas of research, time management and critical thinking. The University of Essex is one of just three UK universities to have received Q-Step Affiliate status, including for our BSc Accounting and Finance course, to support the way we develop the quantitative skills of our graduates. This means we can provide work placement bursaries to develop your skills in evaluating numerical evidence, analysing data and designing research. We also offer the opportunity to follow a specialised degree path, where you graduate with enhanced quantitative skills. These are evidenced on your degree transcript, to help give you the competitive edge in the graduate job market. BSc Accounting and Finance is taught at Essex Business School. Our finance group is one of the largest and most respected in the country and our students and staff join us from all over the world. We not only teach you how financial information underpins leadership, strategy and planning, but how financial decisions can impact society and the economy. We develop your understanding of governance and ethics, so you can take actions for the good of organisations and the wider world. Essex Business School is an Investment Management Certificate (IMC) Advantage Partner and this course is aligned to the IMC syllabus, the industry's benchmark entry-level qualification. Accredited by the Association of Chartered Certified Accountants (ACCA) for the purpose of exemptions from some professional examinations. Accredited by the Chartered Institute of Management Accountants (CIMA) for the purpose of exemption from some professional examinations through the Accredited degree accelerated route. Accredited by the Institute of Chartered Accountants in England and Wales (ICAEW) for the purpose of exemption from some professional examinations. Experience of the dual disciplines of accounting and finance means that you will be well suited to sector specific roles in chartered accountancy and management accountancy as well as more generalist roles such as management consultancy or financial management. We embed a series of core and specific skills into our undergraduate curriculum for BSc Accounting and Finance to ensure that our graduates are suited to careers in finance, accounting and management roles. All of our taught modules embed elements of our skills map which emulate the skills which are required by employers of business, accounting and finance graduates, these generally include academic and cognitive skills, research skills, technology skills, communication skills, data analysis skills and soft skills. Our students have gone on to become financial analysts, accountants, hedge fund managers and insurance trainees, with recent graduate destinations including Private Client Tax Senior Associate at PwC, Treasury Analyst at Hiscox, Junior Tax Consultant at Deloitte, Global Finance &amp; Business Analyst at J.P. Morgan and Junior Consultant - Valuation &amp; Advisory at Cushman &amp; Wakefield. Our accounting and finance graduates enjoy successful careers in their fields.</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Our BA (Economic and Social Studies), known as the BA (Econ), is a flagship interdisciplinary degree designed for students who want to understand Accounting and Finance in their full social, political and technical context. The programme’s Accounting and Finance specialisation will provide you with a rigorous education in core accounting and finance theory and practice, and quantitative methods, while equipping you with the broader perspectives needed to address today’s most complex global challenges. The BA (Econ) is the parent programme to eight distinctive specialisations: Economics, Economics and Politics, Economics and Philosophy, Economics and Sociology, Economics and Finance, Data Science and Economics, Accounting and Finance, and Finance. This structure allows students to gain a strong shared foundation in economics while benefiting from the intellectual richness of other social science disciplines. The BA (Economic and Social Studies) with specialisation in Accounting and Finance is designed for students seeking a rigorous academic foundation for careers in professional accounting and related financial roles. This pathway integrates core economics with a strong sequence of accounting and finance units, enabling you to understand how organisations measure performance, manage financial information and comply with regulatory and governance requirements. A defining feature of the Accounting and Finance pathway is its close collaboration with Alliance Manchester Business School (AMBS). Accounting and finance units are taught by AMBS academics, ensuring your learning reflects current professional standards and industry practice. Throughout the degree, you will develop expertise in financial reporting and accounting regulation, management accounting and decision-making, auditing, accountability and corporate governance, investment and financial analysis, financial markets and institutions, and applying economic reasoning to organisational and financial decisions. Subject to your optional unit choices, the degree offers exemptions from professional examinations with ICAEW, CIMA and ACCA, making it an excellent route into chartered accountancy and related professions. This pathway places accounting firmly within its wider economic, institutional and regulatory environment. You will explore how accounting information is used by investors, managers, regulators and policymakers, and how financial reporting shapes organisational behaviour and market outcomes. You will also develop an understanding of professional ethics, accountability and governance, central to modern accounting practice. Year 1 provides a strong foundation in core economics, financial and management accounting, and quantitative methods, including introductory microeconomics and macroeconomics, financial reporting, management accounting and financial decision-making, mathematics and statistics for economists, and a core social sciences unit exploring power and value. In Year 2, students develop deeper accounting and finance expertise through units including Financial Reporting and Accountability, Intermediate Management Accounting, Foundations of Finance, Financial Statement Analysis, and Investment Analysis. In Year 3, students specialise further in accounting or finance while maintaining a strong professional and analytical focus. Students take a core unit such as Financial Analysis of Corporate Performance or Empirical Finance and may pursue an accounting route focusing on financial reporting and accounting regulation, auditing, accountability and corporate governance, and advanced management accounting and performance measurement, or a finance route including corporate finance, financial markets and institutions, investment analysis and valuation, and risk management and financial decision-making. Graduates develop strong skills in financial reporting, analysis and regulation and pursue careers in audit and assurance, chartered and management accounting, professional services and consultancy, corporate finance and financial management, and public-sector accounting and regulation. The BA (Economic and Social Studies) Accounting and Finance pathway is accredited with professional accountancy bodies including the Institute of Chartered Accountants, the Association of Chartered Certified Accountants and the Chartered Institute of Management Accountants, and students may be eligible for exemptions from professional accountancy examinations depending on the course units chosen. Recent graduates have gone on to careers with organisations including Ernst and Young, KPMG, Deloitte, PricewaterhouseCoopers, Grant Thornton, BDO, American Express, Bloomberg, Bank of America, Deutsche Bank, Merrill Lynch, Morgan Stanley, Royal Bank of Canada, Santander and UBS, as well as roles in government institutions such as HM Treasury, HMRC, the National Audit Office and the Ministry of Justice.</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Where precision meets strategy, accounting and finance paves the way for a solid understanding of financial landscapes and decision-making in the business world. If you choose accounting and finance it opens doors to a strategic understanding of the financial architecture that underpins every business. You’ll gain proficiency in financial reporting, budgeting, and analysis, honing the skills needed to navigate the world of corporate finance. It can lead to many different career paths, from becoming a certified public accountant (CPA) or financial analyst, to going into roles such as financial management, investment banking, or corporate strategy. You could be at the heart of financial decision-making, contributing to the financial health of organisations and influencing business growth. Whether ensuring regulatory compliance, conducting financial audits, or crafting investment strategies, accounting and finance offers a great opportunity for those looking for a rewarding career in the financial sector. Financial markets, taxation, banking and investment, corporate finance, accounting, business policies, management accounting and business ethics are areas you could study. Ability to prepare accurate and compliant financial reports, develop expertise in identifying and managing financial risks, solid understanding of tax laws and regulations and hands-on experience with accounting software used in the industry are hard skills you’ll develop. Analytical thinking, attention to detail, time management and integrity and ethical decision-making are soft skills you’ll develop. Career options include chartered and certified accountants, finance and investment analysts and advisers, financial account managers, taxation experts, business and financial project management professionals, management consultants and business analysts, purchasing managers and directors.</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Essex: How can finance professionals act responsibility, but still meet business objectives? How does accounting information inform business decisions? Our BSc Accounting and Finance degree provides access to our virtual trading floor, where you make use of real-world Bloomberg Market Data Feed (B-PIPE), information and analytics to practise trading stocks and securities in the type of environment found in City finance firms. You study a wide range of topics and develop your quantitative skills, giving you the flexibility to pursue a career in finance, accounting or business management after graduation. You'll explore areas such as the preparation of financial statements and budgets, accounting standards and corporate governance, financial theory, portfolio management, options and futures markets, and risk management. BSc Accounting and Finance includes an introductory first year to familiarise you with wider business topics, such as management and marketing. In your final year, you have the opportunity to put your knowledge into practice by completing an in-depth, independent research project or dissertation. This will give you the chance to further develop vital employment skills in areas of research, time management and critical thinking. The University of Essex is one of just three UK universities to have received Q-Step Affiliate status, including for our BSc Accounting and Finance course, to support the way we develop the quantitative skills of our graduates. This means we can provide work placement bursaries to develop your skills in evaluating numerical evidence, analysing data and designing research. We also offer the opportunity to follow a specialised degree path, where you graduate with enhanced quantitative skills. These are evidenced on your degree transcript, to help give you the competitive edge in the graduate job market. BSc Accounting and Finance is taught at Essex Business School. Our finance group is one of the largest and most respected in the country and our students and staff join us from all over the world. We not only teach you how financial information underpins leadership, strategy and planning, but how financial decisions can impact society and the economy. We develop your understanding of governance and ethics, so you can take actions for the good of organisations and the wider world. Essex Business School is an Investment Management Certificate (IMC) Advantage Partner and this course is aligned to the IMC syllabus, the industry's benchmark entry-level qualification. Accredited by the Association of Chartered Certified Accountants (ACCA) for the purpose of exemptions from some professional examinations. Accredited by the Chartered Institute of Management Accountants (CIMA) for the purpose of exemption from some professional examinations through the Accredited degree accelerated route. Accredited by the Institute of Chartered Accountants in England and Wales (ICAEW) for the purpose of exemption from some professional examinations. Experience of the dual disciplines of accounting and finance means that you will be well suited to sector specific roles in chartered accountancy and management accountancy as well as more generalist roles such as management consultancy or financial management. We embed a series of core and specific skills into our undergraduate curriculum for BSc Accounting and Finance to ensure that our graduates are suited to careers in finance, accounting and management roles. All of our taught modules embed elements of our skills map which emulate the skills which are required by employers of business, accounting and finance graduates, these generally include academic and cognitive skills, research skills, technology skills, communication skills, data analysis skills and soft skills. Our students have gone on to become financial analysts, accountants, hedge fund managers and insurance trainees, with recent graduate destinations including Private Client Tax Senior Associate at PwC, Treasury Analyst at Hiscox, Junior Tax Consultant at Deloitte, Global Finance &amp; Business Analyst at J.P. Morgan and Junior Consultant - Valuation &amp; Advisory at Cushman &amp; Wakefield. Our accounting and finance graduates enjoy successful careers in their fields.
 Manchester: Our BA (Economic and Social Studies), known as the BA (Econ), is a flagship interdisciplinary degree designed for students who want to understand Accounting and Finance in their full social, political and technical context. The programme’s Accounting and Finance specialisation will provide you with a rigorous education in core accounting and finance theory and practice, and quantitative methods, while equipping you with the broader perspectives needed to address today’s most complex global challenges. The BA (Econ) is the parent programme to eight distinctive specialisations: Economics, Economics and Politics, Economics and Philosophy, Economics and Sociology, Economics and Finance, Data Science and Economics, Accounting and Finance, and Finance. This structure allows students to gain a strong shared foundation in economics while benefiting from the intellectual richness of other social science disciplines. The BA (Economic and Social Studies) with specialisation in Accounting and Finance is designed for students seeking a rigorous academic foundation for careers in professional accounting and related financial roles. This pathway integrates core economics with a strong sequence of accounting and finance units, enabling you to understand how organisations measure performance, manage financial information and comply with regulatory and governance requirements. A defining feature of the Accounting and Finance pathway is its close collaboration with Alliance Manchester Business School (AMBS). Accounting and finance units are taught by AMBS academics, ensuring your learning reflects current professional standards and industry practice. Throughout the degree, you will develop expertise in financial reporting and accounting regulation, management accounting and decision-making, auditing, accountability and corporate governance, investment and financial analysis, financial markets and institutions, and applying economic reasoning to organisational and financial decisions. Subject to your optional unit choices, the degree offers exemptions from professional examinations with ICAEW, CIMA and ACCA, making it an excellent route into chartered accountancy and related professions. This pathway places accounting firmly within its wider economic, institutional and regulatory environment. You will explore how accounting information is used by investors, managers, regulators and policymakers, and how financial reporting shapes organisational behaviour and market outcomes. You will also develop an understanding of professional ethics, accountability and governance, central to modern accounting practice. Year 1 provides a strong foundation in core economics, financial and management accounting, and quantitative methods, including introductory microeconomics and macroeconomics, financial reporting, management accounting and financial decision-making, mathematics and statistics for economists, and a core social sciences unit exploring power and value. In Year 2, students develop deeper accounting and finance expertise through units including Financial Reporting and Accountability, Intermediate Management Accounting, Foundations of Finance, Financial Statement Analysis, and Investment Analysis. In Year 3, students specialise further in accounting or finance while maintaining a strong professional and analytical focus. Students take a core unit such as Financial Analysis of Corporate Performance or Empirical Finance and may pursue an accounting route focusing on financial reporting and accounting regulation, auditing, accountability and corporate governance, and advanced management accounting and performance measurement, or a finance route including corporate finance, financial markets and institutions, investment analysis and valuation, and risk management and financial decision-making. Graduates develop strong skills in financial reporting, analysis and regulation and pursue careers in audit and assurance, chartered and management accounting, professional services and consultancy, corporate finance and financial management, and public-sector accounting and regulation. The BA (Economic and Social Studies) Accounting and Finance pathway is accredited with professional accountancy bodies including the Institute of Chartered Accountants, the Association of Chartered Certified Accountants and the Chartered Institute of Management Accountants, and students may be eligible for exemptions from professional accountancy examinations depending on the course units chosen. Recent graduates have gone on to careers with organisations including Ernst and Young, KPMG, Deloitte, PricewaterhouseCoopers, Grant Thornton, BDO, American Express, Bloomberg, Bank of America, Deutsche Bank, Merrill Lynch, Morgan Stanley, Royal Bank of Canada, Santander and UBS, as well as roles in government institutions such as HM Treasury, HMRC, the National Audit Office and the Ministry of Justice.
@@ -489,18 +499,19 @@
           <t>ACTUARIAL SCIENCE</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
         <is>
           <t>Actuarial science teaches you the art of turning risks into opportunities. Actuaries provide assessments of financial security systems, with a focus on their complexity, their mathematics, and their mechanisms. You benefit from an excellent starting salary, with graduates earning upwards of £30,000 on average. Our BSc (Hons) Actuarial Science course covers the syllabus of many core subjects of the Institute and Faculty of Actuaries. Depending on your choice of optional modules, and upon sufficient attainment, this can lead to exemptions from the professional exams CS1, CS2, CM1, CM2, CB1 and CB2. More generally, our course features an attractive blend of solid mathematics, an understanding of real-world financial issues, optimisation, experimental design and computing skills which provide you with core skills for entering the world of actuaries and data scientists. You study topics including mathematical finance, financial reporting, contingencies, risk management and survival analysis, mathematical, statistical and probabilistic techniques, and programming and computation in languages such as MATLAB and R. Professional actuaries in the insurance industry, including influential businesses AXA and Buck Consultants, contribute to our employability module and also host students at their offices to show typical challenges that actuaries face. As part of our School of Mathematics, Statistics and Actuarial Science, you are a member of an inclusive and approachable research community which allows you to explore topics in pure, high-level mathematics and applied mathematics. Accredited by the Institute and Faculty of Actuaries for the purpose of exemption from some professional examinations. This programme will meet the educational requirements of the Chartered Mathematician designation, awarded by the Institute of Mathematics and its Applications, when it is followed by subsequent training and experience in employment to obtain equivalent competences to those specified by the Quality Assurance Agency (QAA) for taught masters degrees. We expect our graduates of BSc (Hons) Actuarial Science to become actuaries in a range of industries. It is predicted by the US Department of Labor that the employment of actuaries is expected to grow faster than any other occupation, making it a great prospect for a graduate job. Aside from a rewarding career as an actuary, clear thinkers are required in every profession, so the successful mathematician has an extensive choice of potential careers.</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Lay the foundations of a rewarding career with mathematics at its base by undertaking an undergraduate degree at the University of Manchester. The programme offers a highly flexible structure, ensuring you obtain a strong all-round mathematical knowledge while encouraging you to focus on the areas that appeal most. You will cover core topics in the first year, developing your capacity to learn and apply mathematical ideas. In the second year you choose two from three themes: Pure Mathematics, Applied Mathematics, and Probability and Statistics, along with optional units such as Programming with Python. You will understand the significance and power of mathematics and acquire a thorough knowledge and understanding of the mathematical topics that any employer would expect of a mathematics graduate. After the first two years you can choose the areas that interest you most and may also select options from other subject areas. In your final year you can undertake a staff-supervised mathematical project. Small group teaching is a significant part of the first year and a wide range of options is available in the third year. All undergraduate students have affiliate membership of the Institute of Mathematics and its Applications. The programme enables students to obtain up to five exemptions from the Institute and Faculty of Actuaries’ professional examinations (CS1, CS2, CM1, CB1 and CB2), subject to satisfactory performance and module options. By studying mathematics at Manchester you will develop analytical, logical and problem-solving skills valued across many professions. Graduates commonly enter areas including finance, industry, computing and operational research, management, administration, statistics, teaching and postgraduate study. Many graduates pursue careers in finance at firms such as KPMG, Goldman Sachs, PricewaterhouseCoopers, Deloitte, Barclays and Deutsche Bank. The course is accredited by the Institute and Faculty of Actuaries, and studying on this degree programme enables students to obtain up to five exemptions from the Institute and Faculty of Actuaries’ professional examinations (CS1, CS2, CM1, CB1 and CB2), subject to satisfactory performance and module options.</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
         <is>
           <t>Essex: Actuarial science teaches you the art of turning risks into opportunities. Actuaries provide assessments of financial security systems, with a focus on their complexity, their mathematics, and their mechanisms. You benefit from an excellent starting salary, with graduates earning upwards of £30,000 on average. Our BSc (Hons) Actuarial Science course covers the syllabus of many core subjects of the Institute and Faculty of Actuaries. Depending on your choice of optional modules, and upon sufficient attainment, this can lead to exemptions from the professional exams CS1, CS2, CM1, CM2, CB1 and CB2. More generally, our course features an attractive blend of solid mathematics, an understanding of real-world financial issues, optimisation, experimental design and computing skills which provide you with core skills for entering the world of actuaries and data scientists. You study topics including mathematical finance, financial reporting, contingencies, risk management and survival analysis, mathematical, statistical and probabilistic techniques, and programming and computation in languages such as MATLAB and R. Professional actuaries in the insurance industry, including influential businesses AXA and Buck Consultants, contribute to our employability module and also host students at their offices to show typical challenges that actuaries face. As part of our School of Mathematics, Statistics and Actuarial Science, you are a member of an inclusive and approachable research community which allows you to explore topics in pure, high-level mathematics and applied mathematics. Accredited by the Institute and Faculty of Actuaries for the purpose of exemption from some professional examinations. This programme will meet the educational requirements of the Chartered Mathematician designation, awarded by the Institute of Mathematics and its Applications, when it is followed by subsequent training and experience in employment to obtain equivalent competences to those specified by the Quality Assurance Agency (QAA) for taught masters degrees. We expect our graduates of BSc (Hons) Actuarial Science to become actuaries in a range of industries. It is predicted by the US Department of Labor that the employment of actuaries is expected to grow faster than any other occupation, making it a great prospect for a graduate job. Aside from a rewarding career as an actuary, clear thinkers are required in every profession, so the successful mathematician has an extensive choice of potential careers.
 Manchester: Lay the foundations of a rewarding career with mathematics at its base by undertaking an undergraduate degree at the University of Manchester. The programme offers a highly flexible structure, ensuring you obtain a strong all-round mathematical knowledge while encouraging you to focus on the areas that appeal most. You will cover core topics in the first year, developing your capacity to learn and apply mathematical ideas. In the second year you choose two from three themes: Pure Mathematics, Applied Mathematics, and Probability and Statistics, along with optional units such as Programming with Python. You will understand the significance and power of mathematics and acquire a thorough knowledge and understanding of the mathematical topics that any employer would expect of a mathematics graduate. After the first two years you can choose the areas that interest you most and may also select options from other subject areas. In your final year you can undertake a staff-supervised mathematical project. Small group teaching is a significant part of the first year and a wide range of options is available in the third year. All undergraduate students have affiliate membership of the Institute of Mathematics and its Applications. The programme enables students to obtain up to five exemptions from the Institute and Faculty of Actuaries’ professional examinations (CS1, CS2, CM1, CB1 and CB2), subject to satisfactory performance and module options. By studying mathematics at Manchester you will develop analytical, logical and problem-solving skills valued across many professions. Graduates commonly enter areas including finance, industry, computing and operational research, management, administration, statistics, teaching and postgraduate study. Many graduates pursue careers in finance at firms such as KPMG, Goldman Sachs, PricewaterhouseCoopers, Deloitte, Barclays and Deutsche Bank. The course is accredited by the Institute and Faculty of Actuaries, and studying on this degree programme enables students to obtain up to five exemptions from the Institute and Faculty of Actuaries’ professional examinations (CS1, CS2, CM1, CB1 and CB2), subject to satisfactory performance and module options.</t>
@@ -516,14 +527,19 @@
           <t>AMERICAN STUDIES</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Modern Languages with Latin American Studies</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
         <is>
           <t>Our three-year American Studies degree is very attractive to those wanting to develop a deep understanding of the US, both at home and around the world. The course enables you to think in interdisciplinary ways about the United States, including its extensive forms of ‘soft’ and ‘hard’ power. This course encourages you to integrate a variety of methods and approaches, allowing you to develop critical and contextual thinking. As you progress, you will have the choice to concentrate more on one approach: you might focus on historical topics – and we employ one of the largest groups of American historians in the UK, offering classes from the beginning of European colonization to the contemporary period – or you might decide to concentrate more on American literary and cultural studies. At Manchester, we train our students to be attentive to the counter currents of US history, society and literature, and many of our course units emphasise the themes of race, capitalism, sexuality, the cultures of labour, political protest, environmental crises and questions of governance. You will learn how to analyse a wide range of texts and materials, including historical documents, literary works, social media communication, films, manuscripts, political rhetoric, marketing campaigns and popular music. Having developed these interpretive skills, you will develop an advanced grasp of theories of change and continuity in a nation that continues to exert considerable influence over international politics, culture, and economics. A degree in American Studies from the University of Manchester provides you with the skills, knowledge and confidence to embark on a successful career in the global workplace. Graduates have entered fields including teaching, law, accountancy, journalism, publishing, surveying and roles within the creative industries in the UK and internationally.</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
         <is>
           <t>Manchester: Our three-year American Studies degree is very attractive to those wanting to develop a deep understanding of the US, both at home and around the world. The course enables you to think in interdisciplinary ways about the United States, including its extensive forms of ‘soft’ and ‘hard’ power. This course encourages you to integrate a variety of methods and approaches, allowing you to develop critical and contextual thinking. As you progress, you will have the choice to concentrate more on one approach: you might focus on historical topics – and we employ one of the largest groups of American historians in the UK, offering classes from the beginning of European colonization to the contemporary period – or you might decide to concentrate more on American literary and cultural studies. At Manchester, we train our students to be attentive to the counter currents of US history, society and literature, and many of our course units emphasise the themes of race, capitalism, sexuality, the cultures of labour, political protest, environmental crises and questions of governance. You will learn how to analyse a wide range of texts and materials, including historical documents, literary works, social media communication, films, manuscripts, political rhetoric, marketing campaigns and popular music. Having developed these interpretive skills, you will develop an advanced grasp of theories of change and continuity in a nation that continues to exert considerable influence over international politics, culture, and economics. A degree in American Studies from the University of Manchester provides you with the skills, knowledge and confidence to embark on a successful career in the global workplace. Graduates have entered fields including teaching, law, accountancy, journalism, publishing, surveying and roles within the creative industries in the UK and internationally.</t>
         </is>
@@ -540,20 +556,25 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Curating with History; History; History and Economics; History and Literature; History and Sociology; Modern History; Modern History and International Relations; Modern History and Politics</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>At Essex, you will acquire a broad foundation in the history of visual culture: both by learning about canonical forms of art and architecture and by discovering what has been overlooked or marginalised, such as medical photography, tattoos or objects from political protests. You will also develop the skills you need to make exciting new connections between the forms of visual culture you study, developments in other disciplines, and broader social and political forces. To study on our course, you don't need an Art History A-Level. In fact, we believe that the best art historians are those who bring fresh eyes and new perspectives to their objects of inquiry. You will develop the skills you need to transform your excitement about art, architecture and visual culture into the ability to uncover new insights about the material you study. You will also develop a solid grounding in the history of art and other forms of visual culture, including the ideas and forces that shaped their production, distribution and reception. For students with a particular interest in pursuing careers in curating and museumship, we provide modules that explore the histories, theories and practices of museums, exhibitions and galleries, as well as practical issues such as installing and marketing artwork. The visual arts and culture industries have become an increasingly significant part of the national and international economy, and our art history graduates leave Essex with the skills to take advantage of this growing opportunity. Some of the sectors with jobs well suited for our graduates include museums and galleries, auction houses, education in schools, universities and cultural institutions, marketing and advertising, and new media. Our degree also prepares students to run their own galleries, to work as specialist arts lawyers and PR agents, and for positions in charities, fashion and publishing. Our recent graduates have gone on to work for a wide range of high-profile organisations including the National Portrait Gallery, the Victoria and Albert Museum, Sotheby's New York, Momart Ltd and John Lewis.</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>BA History of Art is a wide-ranging degree which explores art history and visual culture from the Medieval era to the present. As you progress to Years 2 and 3, tailor your studies by selecting pathways of study that align with your interests. The range of staff expertise offers you the opportunity to study a varied and exciting curriculum. We provide a wide selection of subject areas, paired with in-depth research and study. Our expertise lies in Medieval, Renaissance, Post-Renaissance, Modern, Contemporary and Global art history. Additionally, we benefit from the expertise of faculty members within the Institute of Cultural Practice. Course units cover topics such as the study of museums as institutions, collecting, practical aspects of curating and exhibition-making, and art writing. The Manchester Museum and the Whitworth Art Gallery offer access to the environment of the working museum and art gallery as well as to important works of art, and the Whitworth’s collections of paintings, prints, textiles and wallpapers are used extensively in teaching. Students also benefit from the University Library and the Special Collections Department at the John Rylands Library, which holds significant collections of rare books, manuscripts and illustrated materials relevant to Art History. A degree in Art History equips students with intellectual and practical skills for analysing visual culture and interpreting images in contemporary society. Recent graduates have pursued careers across a range of sectors, with roles including Education Officer at the De Morgan Collection, Royal Collections Exhibitions Curator, Archivist at Tate Liverpool and Art Officer at English Heritage.</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Studying the history of art is like a journey through time, giving insights into human creativity, cultural evolution, and the timeless dialogue between artists and society. The study of the history of art unveils human creativity and expression. It also promotes critical analytical skills, an understanding of cultural contexts, and a deep appreciation for visual storytelling. Studying the history of art opens up many career opportunities like art curation, museum management, art conservation, education, art and cultural consultancy. The ability to interpret visual pieces is valuable in sectors where creativity, cultural understanding, and a discerning eye are essential. Museums and society, making and meaning in architecture, reading art history, making and meaning in western art, modern British art and art and the environment are areas you could study. Comparative art analysis, visual analysis, historical knowledge and museum and gallery practices are hard skills you’ll develop. Attention to detail, creativity, flexibility, curiosity and open-mindedness are soft skills you’ll develop. Career options include artists, arts officers, producers and directors, conservators and curators, and librarians.</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Essex: At Essex, you will acquire a broad foundation in the history of visual culture: both by learning about canonical forms of art and architecture and by discovering what has been overlooked or marginalised, such as medical photography, tattoos or objects from political protests. You will also develop the skills you need to make exciting new connections between the forms of visual culture you study, developments in other disciplines, and broader social and political forces. To study on our course, you don't need an Art History A-Level. In fact, we believe that the best art historians are those who bring fresh eyes and new perspectives to their objects of inquiry. You will develop the skills you need to transform your excitement about art, architecture and visual culture into the ability to uncover new insights about the material you study. You will also develop a solid grounding in the history of art and other forms of visual culture, including the ideas and forces that shaped their production, distribution and reception. For students with a particular interest in pursuing careers in curating and museumship, we provide modules that explore the histories, theories and practices of museums, exhibitions and galleries, as well as practical issues such as installing and marketing artwork. The visual arts and culture industries have become an increasingly significant part of the national and international economy, and our art history graduates leave Essex with the skills to take advantage of this growing opportunity. Some of the sectors with jobs well suited for our graduates include museums and galleries, auction houses, education in schools, universities and cultural institutions, marketing and advertising, and new media. Our degree also prepares students to run their own galleries, to work as specialist arts lawyers and PR agents, and for positions in charities, fashion and publishing. Our recent graduates have gone on to work for a wide range of high-profile organisations including the National Portrait Gallery, the Victoria and Albert Museum, Sotheby's New York, Momart Ltd and John Lewis.
 Manchester: BA History of Art is a wide-ranging degree which explores art history and visual culture from the Medieval era to the present. As you progress to Years 2 and 3, tailor your studies by selecting pathways of study that align with your interests. The range of staff expertise offers you the opportunity to study a varied and exciting curriculum. We provide a wide selection of subject areas, paired with in-depth research and study. Our expertise lies in Medieval, Renaissance, Post-Renaissance, Modern, Contemporary and Global art history. Additionally, we benefit from the expertise of faculty members within the Institute of Cultural Practice. Course units cover topics such as the study of museums as institutions, collecting, practical aspects of curating and exhibition-making, and art writing. The Manchester Museum and the Whitworth Art Gallery offer access to the environment of the working museum and art gallery as well as to important works of art, and the Whitworth’s collections of paintings, prints, textiles and wallpapers are used extensively in teaching. Students also benefit from the University Library and the Special Collections Department at the John Rylands Library, which holds significant collections of rare books, manuscripts and illustrated materials relevant to Art History. A degree in Art History equips students with intellectual and practical skills for analysing visual culture and interpreting images in contemporary society. Recent graduates have pursued careers across a range of sectors, with roles including Education Officer at the De Morgan Collection, Royal Collections Exhibitions Curator, Archivist at Tate Liverpool and Art Officer at English Heritage.
@@ -572,16 +593,21 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>Applied Biomedical Science; Biochemistry; Biochemistry and Biotechnology; Biomedical Science</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>The BSc (Hons) Biochemistry is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll secure a strong understanding of biochemistry and biomolecules through computational approaches and bioinformatics. The BSc (Hons) Biochemistry lets you explore molecular enzymology, neurodegeneration, structural biology and bioenergetics, and you can expand your study into biomedical science, biotechnology and bioinformatics. Previous students have placed with organisations including GlaxoSmithKline (GSK), Proctor &amp; Gamble (P&amp;G), AquaTerra, AstraZeneca, Genzyme, Reckitt Benckiser, Thermo Fisher and Isogenica. You’ll graduate on the path to a career in biomedical science, biotechnology and other specialisms of biological sciences. This course is suitable for future biochemists and biochemistry researchers, those wanting to further our modern understanding of the complex cellular and molecular world, and practical learners wanting hands-on experience. In the first year you explore biochemistry, molecular cell biology, genetics and microbiology. You study areas such as enzymology, bioenergetics and macromolecular assemblies, and develop employability and transferable skills for the biosciences while tailoring your degree through a choice of applied modules. A BSc (Hons) Biochemistry degree prepares you for diverse careers including biotechnology and forensic science in biology, pharmacology and biomedical science in health, postgraduate medicine programmes, postgraduate research programmes, and primary and secondary science and biology teaching.</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Our BSc Biochemistry course will give you a grounding in a subject that forms the basis of virtually all of the biological sciences. Many exciting discoveries made in this area have contributed to our understanding of life, the solving of medical problems, and to the discovery and production of safe and effective drugs. You will learn about topics such as the structure of biomolecules and how they interact in essential processes and pathways in our cells. You will also study the actions of enzymes and how they can be inhibited by drugs, as well as genetic engineering and molecular biology. You will benefit from lectures, tutorials, practicals and research projects, including the final year project. A significant part of the final year is the project, which is assessed through a presentation and a written report. Our modern teaching laboratories are equipped for a range of biological and biomedical techniques including polymerase chain reaction (PCR), DNA sequencing, gel electrophoresis, spectrophotometry, electroencephalography (EEG), electrocardiography (ECG) and immunofluorescence microscopy. As a final year student, you have the opportunity to undertake a research project in the laboratories of bioscience researchers supported by extensive research facilities and advanced technology. Our graduates go into a wide range of sectors, with around one-third working in scientific research and development, often progressing to postgraduate study such as a PhD and careers as researchers at universities, pharmaceutical and bioscience companies and institutes. Other graduates pursue diverse careers including teaching, science communication, management, finance, marketing and the civil service.</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
         <is>
           <t>Essex: The BSc (Hons) Biochemistry is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll secure a strong understanding of biochemistry and biomolecules through computational approaches and bioinformatics. The BSc (Hons) Biochemistry lets you explore molecular enzymology, neurodegeneration, structural biology and bioenergetics, and you can expand your study into biomedical science, biotechnology and bioinformatics. Previous students have placed with organisations including GlaxoSmithKline (GSK), Proctor &amp; Gamble (P&amp;G), AquaTerra, AstraZeneca, Genzyme, Reckitt Benckiser, Thermo Fisher and Isogenica. You’ll graduate on the path to a career in biomedical science, biotechnology and other specialisms of biological sciences. This course is suitable for future biochemists and biochemistry researchers, those wanting to further our modern understanding of the complex cellular and molecular world, and practical learners wanting hands-on experience. In the first year you explore biochemistry, molecular cell biology, genetics and microbiology. You study areas such as enzymology, bioenergetics and macromolecular assemblies, and develop employability and transferable skills for the biosciences while tailoring your degree through a choice of applied modules. A BSc (Hons) Biochemistry degree prepares you for diverse careers including biotechnology and forensic science in biology, pharmacology and biomedical science in health, postgraduate medicine programmes, postgraduate research programmes, and primary and secondary science and biology teaching.
 Manchester: Our BSc Biochemistry course will give you a grounding in a subject that forms the basis of virtually all of the biological sciences. Many exciting discoveries made in this area have contributed to our understanding of life, the solving of medical problems, and to the discovery and production of safe and effective drugs. You will learn about topics such as the structure of biomolecules and how they interact in essential processes and pathways in our cells. You will also study the actions of enzymes and how they can be inhibited by drugs, as well as genetic engineering and molecular biology. You will benefit from lectures, tutorials, practicals and research projects, including the final year project. A significant part of the final year is the project, which is assessed through a presentation and a written report. Our modern teaching laboratories are equipped for a range of biological and biomedical techniques including polymerase chain reaction (PCR), DNA sequencing, gel electrophoresis, spectrophotometry, electroencephalography (EEG), electrocardiography (ECG) and immunofluorescence microscopy. As a final year student, you have the opportunity to undertake a research project in the laboratories of bioscience researchers supported by extensive research facilities and advanced technology. Our graduates go into a wide range of sectors, with around one-third working in scientific research and development, often progressing to postgraduate study such as a PhD and careers as researchers at universities, pharmaceutical and bioscience companies and institutes. Other graduates pursue diverse careers including teaching, science communication, management, finance, marketing and the civil service.</t>
@@ -597,22 +623,23 @@
           <t>BIOLOGICAL SCIENCES</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
         <is>
           <t>What is the BSc (Hons) Biological Sciences? The BSc (Hons) Biological Sciences is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll secure a broad understanding of modern biology and a strong basis to specialise from, in your undergraduate degree or beyond. The BSc (Hons) Biological Sciences lets you explore the spectrum of biology and choose what to specialise in. Your first year offers broad insights into cell and molecular biology, genetics, ecology and evolution. For your second and final years, you can deepen your knowledge across disciplines or specialise in an area of your choosing, from molecular and cell biology to ecology and conservation biology. Previous students have placed with GlaxoSmithKline (GSK), Proctor &amp; Gamble (P&amp;G), AquaTerra, AstraZeneca, Genzyme, Reckitt Benckiser, Thermo Fisher and Isogenica, some of our 40 partner labs. You’ll graduate on the path to a biologist career in a range of specialisms, such as marine biology, conservation and molecular biology. In Year One you explore molecular cell biology, genetics, ecology and microbiology. You can choose employability skills for the biosciences or professional skills for ecology and marine scientists and tailor the last two years of your degree through your choice of applied modules. A BSc (Hons) Biological Sciences degree prepares you for diverse careers in areas such as biotechnology, microbiology, genetics and forensic science; ecology, marine biology, nature conservation, water quality and soil analysis; pharmacology, biomedical science and clinical science; postgraduate research programmes; and primary and secondary science and biology teaching. Graduates from this course have progressed to roles in organisations including GlaxoSmithKline (GSK), Sainsbury Laboratory (University of Cambridge), ALS Laboratories, the NHS, Essex Wildlife Trust, Natural England and Suffolk County Council.</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Our BSc Biology course covers a diverse range of topics within the study of living organisms, allowing you to discover areas of interest early on in your degree and choose what you want to focus on. You can keep your options open and cover a wide variety of areas, or identify those that interest you and focus on particular biological topics. Interdisciplinarity is encouraged, and you have the opportunity to enrol on courses at the University College for Interdisciplinary Learning in the second and third year. Our modern teaching labs are equipped for a range of biological and biomedical techniques, including polymerase chain reaction (PCR), DNA sequencing, gel electrophoresis, spectrophotometry, dissection and histology, electroencephalography (EEG), electrocardiography (ECG) and immunofluorescence microscopy. As a final year student, you have the opportunity to undertake a project in the labs of our bioscience researchers. Our graduates go into a range of careers, with around one-third working in scientific research and development, which may require postgraduate study such as a PhD, while others pursue careers in teaching or communicating science, conservation and ecological consultancy, biotechnology and biomedical companies, as well as roles outside biological sciences including management, finance, marketing and the civil service.</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Studying biology will unravel the complexities of life, from the tiniest cells to the grandest ecosystems, to discover the science that underlies the wonders of the natural world. Biology is the study of life in all its forms, from microscopic organisms to complex ecosystems. It covers a wide range of topics, including genetics, ecology, physiology and evolution, giving an overall understanding of the natural world. Biology opens doors to diverse career paths, including roles in research, healthcare, environmental conservation and education. You could explore careers such as research scientists, environmental consultants, healthcare professionals, educators or science communicators. Ecology, anatomy and physiology, biochemistry and biotechnology, genetics, molecular biology, immunology and plant physiology are areas you could study. Hands-on experience in laboratory techniques such as pipetting, microscopy and DNA extraction, data analysis and statistical interpretation, and skills in conducting observations, collecting samples and recording data in natural environments are hard skills you’ll develop. Critical thinking, attention to detail, patience and perseverance and ethical reasoning are soft skills you’ll develop. Career options include biological scientists, natural and social science professionals, laboratory technicians, conservation professionals and environment professionals.</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Essex: What is the BSc (Hons) Biological Sciences? The BSc (Hons) Biological Sciences is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll secure a broad understanding of modern biology and a strong basis to specialise from, in your undergraduate degree or beyond. The BSc (Hons) Biological Sciences lets you explore the spectrum of biology and choose what to specialise in. Your first year offers broad insights into cell and molecular biology, genetics, ecology and evolution. For your second and final years, you can deepen your knowledge across disciplines or specialise in an area of your choosing, from molecular and cell biology to ecology and conservation biology. Previous students have placed with GlaxoSmithKline (GSK), Proctor &amp; Gamble (P&amp;G), AquaTerra, AstraZeneca, Genzyme, Reckitt Benckiser, Thermo Fisher and Isogenica, some of our 40 partner labs. You’ll graduate on the path to a biologist career in a range of specialisms, such as marine biology, conservation and molecular biology. In Year One you explore molecular cell biology, genetics, ecology and microbiology. You can choose employability skills for the biosciences or professional skills for ecology and marine scientists and tailor the last two years of your degree through your choice of applied modules. A BSc (Hons) Biological Sciences degree prepares you for diverse careers in areas such as biotechnology, microbiology, genetics and forensic science; ecology, marine biology, nature conservation, water quality and soil analysis; pharmacology, biomedical science and clinical science; postgraduate research programmes; and primary and secondary science and biology teaching. Graduates from this course have progressed to roles in organisations including GlaxoSmithKline (GSK), Sainsbury Laboratory (University of Cambridge), ALS Laboratories, the NHS, Essex Wildlife Trust, Natural England and Suffolk County Council.
 Manchester: Our BSc Biology course covers a diverse range of topics within the study of living organisms, allowing you to discover areas of interest early on in your degree and choose what you want to focus on. You can keep your options open and cover a wide variety of areas, or identify those that interest you and focus on particular biological topics. Interdisciplinarity is encouraged, and you have the opportunity to enrol on courses at the University College for Interdisciplinary Learning in the second and third year. Our modern teaching labs are equipped for a range of biological and biomedical techniques, including polymerase chain reaction (PCR), DNA sequencing, gel electrophoresis, spectrophotometry, dissection and histology, electroencephalography (EEG), electrocardiography (ECG) and immunofluorescence microscopy. As a final year student, you have the opportunity to undertake a project in the labs of our bioscience researchers. Our graduates go into a range of careers, with around one-third working in scientific research and development, which may require postgraduate study such as a PhD, while others pursue careers in teaching or communicating science, conservation and ecological consultancy, biotechnology and biomedical companies, as well as roles outside biological sciences including management, finance, marketing and the civil service.
@@ -631,16 +658,21 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>Accounting and Management; Business Administration; Business Administration and Supply Chain Management; Business Economics; Business Management; Business Management with a Modern Language; Events Management; Events Management with Hospitality; Finance and Management; Hospitality Management; Hotel Management; International Business and Entrepreneurship; Law with Business; Marketing Management; Philosophy with Business Management; Politics with Business</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>Businesses need effective managers now more than ever in a post Covid-19 world. But what makes an effective manager? And how can studying management theory create better managers for people and the planet? On this course, you learn what's involved in managing organisations in an increasingly complex world. We look at the enduring patterns in how people, groups, organisations, economies and societies function and interact. By understanding these behaviours, you can manage them effectively in times of significant change. With BSc Business Management, you gain a rich understanding of how organisations operate – what they do, how they develop strategies and why. Study areas include management, innovation and new technologies, the international business environment, organisational behaviour, operations and supply chain management, leadership, human resource management and ethical business management. The first year of your business management degree also introduces you to the core principles of accounting, finance and marketing to provide you with the essential business knowledge needed for a successful career. In your final year, you have the opportunity to put your knowledge into practice by completing an in-depth, independent research project or dissertation. This will give you the chance to further develop vital employability skills in areas of research, time management and critical thinking. This course is taught at Essex Business School. We champion responsible management and ethical business practices; you join a school not just committed to excellence in business education and social science research, but an intellectual community working to make business better. We don't just prepare you for a successful career; we'll help you shape the kind of world you want to live in. Business management skills are as highly valued as your degree by many graduate employers, therefore we embed a series of core and specific skills into our undergraduate curriculum for BSc Business Management to ensure that our graduates are suited to careers in business management and leadership roles. All of our taught modules embed elements of our skills map which emulate the skills required by employers of business graduates, including academic and cognitive skills, research skills, technology skills, communication skills, data analysis skills and soft skills. Our students have gone on to become business analysts, successful entrepreneurs, account managers and management trainees, with recent graduate destinations including CEO and Founders of WYSPR – a ‘Friendvertising' social media start-up, Business Development Manager at Footprint Digital – a digital marketing agency, Sales and Marketing Manager at Chrysodalia – a food manufacturing company, Digital Marketing Executive at Premier Labellers – a machinery manufacturer, Delivery Consultant at RED – The Global SAP Solutions Provider, and iX Business Consultant at IBM.</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
         <is>
           <t>Dive into the world of business and management, where every challenge is an opportunity, and every decision is another step forward to organisational success. Choosing business and management will give you a versatile skill set covering strategic planning, leadership and problem-solving, all essential for navigating the corporate world. This popular field opens doors into dynamic careers spanning corporate management, consulting, finance, marketing and entrepreneurship. Armed with a degree in business and management, individuals become catalysts for organisational growth, driving innovation, leading teams and shaping the strategic landscape of multiple sectors and industries on a global scale. Leadership, finance, marketing, entrepreneurship, management theory, human resources, strategy and market analysis are areas you could study. Strategic planning, market research and analysis, negotiation and conflict resolution, and entrepreneurship and innovation are hard skills you’ll develop. Communication, team collaboration, project management and networking are soft skills you’ll develop. Career options include chief executives and senior officials, financial managers and directors, purchasing managers and directors, human resource managers and directors, marketing and sales directors, advertising and public relations directors, business and related associate professionals, office managers, business and financial project management professionals and financial accounts managers.</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Essex: Businesses need effective managers now more than ever in a post Covid-19 world. But what makes an effective manager? And how can studying management theory create better managers for people and the planet? On this course, you learn what's involved in managing organisations in an increasingly complex world. We look at the enduring patterns in how people, groups, organisations, economies and societies function and interact. By understanding these behaviours, you can manage them effectively in times of significant change. With BSc Business Management, you gain a rich understanding of how organisations operate – what they do, how they develop strategies and why. Study areas include management, innovation and new technologies, the international business environment, organisational behaviour, operations and supply chain management, leadership, human resource management and ethical business management. The first year of your business management degree also introduces you to the core principles of accounting, finance and marketing to provide you with the essential business knowledge needed for a successful career. In your final year, you have the opportunity to put your knowledge into practice by completing an in-depth, independent research project or dissertation. This will give you the chance to further develop vital employability skills in areas of research, time management and critical thinking. This course is taught at Essex Business School. We champion responsible management and ethical business practices; you join a school not just committed to excellence in business education and social science research, but an intellectual community working to make business better. We don't just prepare you for a successful career; we'll help you shape the kind of world you want to live in. Business management skills are as highly valued as your degree by many graduate employers, therefore we embed a series of core and specific skills into our undergraduate curriculum for BSc Business Management to ensure that our graduates are suited to careers in business management and leadership roles. All of our taught modules embed elements of our skills map which emulate the skills required by employers of business graduates, including academic and cognitive skills, research skills, technology skills, communication skills, data analysis skills and soft skills. Our students have gone on to become business analysts, successful entrepreneurs, account managers and management trainees, with recent graduate destinations including CEO and Founders of WYSPR – a ‘Friendvertising' social media start-up, Business Development Manager at Footprint Digital – a digital marketing agency, Sales and Marketing Manager at Chrysodalia – a food manufacturing company, Digital Marketing Executive at Premier Labellers – a machinery manufacturer, Delivery Consultant at RED – The Global SAP Solutions Provider, and iX Business Consultant at IBM.
 UCAS: Dive into the world of business and management, where every challenge is an opportunity, and every decision is another step forward to organisational success. Choosing business and management will give you a versatile skill set covering strategic planning, leadership and problem-solving, all essential for navigating the corporate world. This popular field opens doors into dynamic careers spanning corporate management, consulting, finance, marketing and entrepreneurship. Armed with a degree in business and management, individuals become catalysts for organisational growth, driving innovation, leading teams and shaping the strategic landscape of multiple sectors and industries on a global scale. Leadership, finance, marketing, entrepreneurship, management theory, human resources, strategy and market analysis are areas you could study. Strategic planning, market research and analysis, negotiation and conflict resolution, and entrepreneurship and innovation are hard skills you’ll develop. Communication, team collaboration, project management and networking are soft skills you’ll develop. Career options include chief executives and senior officials, financial managers and directors, purchasing managers and directors, human resource managers and directors, marketing and sales directors, advertising and public relations directors, business and related associate professionals, office managers, business and financial project management professionals and financial accounts managers.</t>
@@ -658,20 +690,25 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>Computer Games</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>What is the BSc (Hons) Computer Science? The BSc (Hons) Computer Science is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll build a strong foundation in core computer science theory and explore its cutting-edge real-world applications, preparing you to create the technologies of tomorrow. Why this course The BSc (Hons) Computer Science gives you the theory and practical knowledge to understand – and create – computing technologies that make a real impact on the world. You’ll study a broad curriculum shaped by industry partners, gaining the most up-to-date understanding of computer science. Discover which areas you’re interested in exploring further, then specialise in assistive technologies, computer games, artificial intelligence, evolutionary computation, Big Data or robotics. By graduation, you’ll have the confidence and ability to dig deeper into how technology influences people’s lives. You’ll be ready for careers in software and systems analysis, engineering and programming. Who should apply Future software analysts and programmers, students eager to develop their own computer games, apps, online platforms and digital systems, those considering a career that benefits from a broad understanding of how computers and digital systems work, and computational thinkers with a great grasp of pattern recognition and algorithms. What you’ll learn Programming: learn to programme with multiple programming languages. Data: explore ways to work with data from data structures to Big Data. Web: understand the principles and technology behind web apps and websites. Digital systems: grasp the software and hardware underpinning digital computer systems. Your learning experience includes optional modules that allow you to tailor your degree and specialise in areas such as artificial intelligence, computer games and security. Careers and outcomes A BSc (Hons) Computer Science degree prepares you for diverse careers in IT including computer and information research, computer network architecture, database systems administration and security analysis; healthcare including health information technology, clinical data and systems administration; business and finance including financial analysis, data analysis, risk management and web development; energy including energy generation and distribution systems, data analysis and technological improvement; and computer games development and programming. Employers of graduates from this course include American Express, Red Bull Racing, JP Morgan, BT, Blizzard, Google, Formula One, IBM and Royal Bank of Scotland. Professional accreditation Accredited by BCS, the Chartered Institute for IT for the purposes of fully meeting the academic requirement for registration as a Chartered IT Professional. Accredited by BCS, the Chartered Institute for IT on behalf of the Engineering Council for the purposes of fully meeting the academic requirement for Incorporated Engineer and partially meeting the academic requirement for a Chartered Engineer. Accredited by the Institution of Engineering and Technology (IET) on behalf of the Engineering Council for the purposes of fully meeting the academic requirement for registration as an Incorporated Engineer and partially meeting the academic requirement for registration as a Chartered Engineer.</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Through the development of new applications in science, engineering, and business, Computer Science is radically changing the way in which we experience our world. This programme equips students with the skills needed to contribute to this exciting and rapidly evolving field. Computer Science is our most flexible programme, allowing you to choose course units to reflect your developing and changing interests, with a wide range of themes from across the discipline allowing you to specialise in the second and third years. You will gain not only knowledge and practical experience of the latest technologies, but also a grounding in the underlying principles of the subject. It is this combination of skills that enables graduates to keep pace with this fast-moving subject and secure rewarding careers that can be pursued almost anywhere in the world. The programme provides a broad and flexible structure that allows students to choose from a wide range of Computer Science topics while developing skills that are highly valued by industry. Graduates pursue careers in roles such as actuary, AI engineer, banker, cloud computing engineer, cyber security analyst, data analyst, games designer or developer, software engineer, and web designer or developer, working across sectors including finance, films and games, pharmaceuticals, healthcare, consumer products and public services. Employers that recruit graduates include organisations such as CERN, EA Games, IBM and Microsoft. This degree has been accredited by the British Computer Society (BCS), The Chartered Institute for IT, under licence from the Engineering Council. Accreditation confirms that the degree meets the standards set by the Engineering Council in the UK Standard for Professional Engineering Competence and provides the underpinning knowledge and skills required for registration as a Chartered IT Professional (CITP), Chartered Engineer (CEng) or Incorporated Engineer (IEng).</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Whether it’s finance, health, the creative industries or sport, the study of computer science helps build the technology that fuels future innovation. In today's technology-driven world, the demand for skilled computer scientists continues to grow across various industries. Studying computer science equips you with technical skills, from programming languages to algorithm design, opening a range of career opportunities. It opens doors to high-growth sectors such as cybersecurity, data science and machine learning, and the skills you’ll learn make you well-suited for roles in finance, healthcare, entertainment and beyond. Algorithms and data structures, database systems, mathematical principles, programming languages and software development, web and mobile apps, cyber security and artificial intelligence are areas you might study. Understanding programming languages, working with data structures, knowledge of algorithms and understanding cybersecurity principles are hard skills you’ll develop. Critical thinking, problem-solving attitude, adaptability and attention to detail are soft skills you’ll develop. Career options include programmers and software developers, web designers, software testers, IT network testers, electrical and electronics technicians, cyber security analysts and systems analysts.</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Essex: What is the BSc (Hons) Computer Science? The BSc (Hons) Computer Science is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll build a strong foundation in core computer science theory and explore its cutting-edge real-world applications, preparing you to create the technologies of tomorrow. Why this course The BSc (Hons) Computer Science gives you the theory and practical knowledge to understand – and create – computing technologies that make a real impact on the world. You’ll study a broad curriculum shaped by industry partners, gaining the most up-to-date understanding of computer science. Discover which areas you’re interested in exploring further, then specialise in assistive technologies, computer games, artificial intelligence, evolutionary computation, Big Data or robotics. By graduation, you’ll have the confidence and ability to dig deeper into how technology influences people’s lives. You’ll be ready for careers in software and systems analysis, engineering and programming. Who should apply Future software analysts and programmers, students eager to develop their own computer games, apps, online platforms and digital systems, those considering a career that benefits from a broad understanding of how computers and digital systems work, and computational thinkers with a great grasp of pattern recognition and algorithms. What you’ll learn Programming: learn to programme with multiple programming languages. Data: explore ways to work with data from data structures to Big Data. Web: understand the principles and technology behind web apps and websites. Digital systems: grasp the software and hardware underpinning digital computer systems. Your learning experience includes optional modules that allow you to tailor your degree and specialise in areas such as artificial intelligence, computer games and security. Careers and outcomes A BSc (Hons) Computer Science degree prepares you for diverse careers in IT including computer and information research, computer network architecture, database systems administration and security analysis; healthcare including health information technology, clinical data and systems administration; business and finance including financial analysis, data analysis, risk management and web development; energy including energy generation and distribution systems, data analysis and technological improvement; and computer games development and programming. Employers of graduates from this course include American Express, Red Bull Racing, JP Morgan, BT, Blizzard, Google, Formula One, IBM and Royal Bank of Scotland. Professional accreditation Accredited by BCS, the Chartered Institute for IT for the purposes of fully meeting the academic requirement for registration as a Chartered IT Professional. Accredited by BCS, the Chartered Institute for IT on behalf of the Engineering Council for the purposes of fully meeting the academic requirement for Incorporated Engineer and partially meeting the academic requirement for a Chartered Engineer. Accredited by the Institution of Engineering and Technology (IET) on behalf of the Engineering Council for the purposes of fully meeting the academic requirement for registration as an Incorporated Engineer and partially meeting the academic requirement for registration as a Chartered Engineer.
 Manchester: Through the development of new applications in science, engineering, and business, Computer Science is radically changing the way in which we experience our world. This programme equips students with the skills needed to contribute to this exciting and rapidly evolving field. Computer Science is our most flexible programme, allowing you to choose course units to reflect your developing and changing interests, with a wide range of themes from across the discipline allowing you to specialise in the second and third years. You will gain not only knowledge and practical experience of the latest technologies, but also a grounding in the underlying principles of the subject. It is this combination of skills that enables graduates to keep pace with this fast-moving subject and secure rewarding careers that can be pursued almost anywhere in the world. The programme provides a broad and flexible structure that allows students to choose from a wide range of Computer Science topics while developing skills that are highly valued by industry. Graduates pursue careers in roles such as actuary, AI engineer, banker, cloud computing engineer, cyber security analyst, data analyst, games designer or developer, software engineer, and web designer or developer, working across sectors including finance, films and games, pharmaceuticals, healthcare, consumer products and public services. Employers that recruit graduates include organisations such as CERN, EA Games, IBM and Microsoft. This degree has been accredited by the British Computer Society (BCS), The Chartered Institute for IT, under licence from the Engineering Council. Accreditation confirms that the degree meets the standards set by the Engineering Council in the UK Standard for Professional Engineering Competence and provides the underpinning knowledge and skills required for registration as a Chartered IT Professional (CITP), Chartered Engineer (CEng) or Incorporated Engineer (IEng).
@@ -690,20 +727,25 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>Drama and Creative Writing; Film and Drama</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>Theatre is a radical and influential art form. Its roots lie deep in the ancient world but its relevance to contemporary life is urgent and ongoing. Theatre enables different cultures and societies to confront the most important issues of our time; it provides a crucial space to laugh, to dream, and dare to project different worlds. Studying theatre and drama at Essex enables you to examine some of the most influential play-texts ever written, and to be ready to take part in shaping the essential performances of tomorrow. This degree is a chance to unlock and explore your creativity. You will be performing and producing work in a professional theatre context and will be developing a wide range of creative, critical and practical skills that will open the door to a future in the theatre, cultural industries or a wide range of other graduate careers. At Essex, we offer a rich combination of practical workshops, critical seminars and lectures delivered by an experienced team of playwrights, directors and actors, as well as leading academic theatre specialists. Areas of exploration in our modules include dramatic literature from Ancient Greek tragedy and Shakespeare to modern plays from around the world, contemporary playwriting and devising techniques, staging political ideas and social justice issues, gender, identity and sexual politics on stage, creating Applied Theatre in educational and community contexts, and emergent trends in interactive performance-making and audience participation. Through classroom teaching, practical experiment and professional experience, we help you craft the skillset that will be essential in your creative development. This approach reflects our core belief that engaging with both practice and theory produces a deeper understanding of how theatre works. Creativity, communication and versatility developed during the degree prepare graduates for a wide range of careers. Our students have gone on to become actors, directors and playwrights, as well as producers, live artists, dramaturgs, stage-managers and arts managers. Graduates have also pursued careers in related creative industries including journalism, television production, broadcasting, radio presenting, gaming, magazine editing, copywriting, press relations and marketing, as well as roles in business, commerce and law. Our graduates have gone on to work in roles such as Writer in Residence for the National Theatre, Artistic Director of Jermyn Street Theatre in London, Artistic Director of a touring company, Director for the Almeida Theatre in London, Manager at a regional theatre, Live Artist for Art Angel, BBC Journalist, Youth Theatre Leader and Workshop Facilitator, Outreach and Education Officer, Front of House Theatre Manager, Stage Manager and Secondary School Teacher.</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>BA Drama embraces all forms of drama across stage, screen and performance contexts. Students explore areas such as literary adaptation, performance in public spaces, performance curation, audio design, playwriting, directing and experimental film cultures. Teaching is informed by recent innovations in theatre and performance alongside historical methods and practices. The programme is embedded within a strong creative ecosystem with links to arts organisations and opportunities to engage with professional practitioners during coursework. Specialist facilities include the purpose-built Martin Harris Centre and the John Thaw Studio, a fully staffed performance, rehearsal and workshop space supporting practical production work. Studying the degree develops transferable and specialist skills including theatre analysis, performance creation, presentation and communication, creative problem solving, teamwork and leadership. Graduates pursue careers across sectors including theatre, film, television, journalism, community arts, teaching, arts administration and business, with alumni working at organisations such as BBC, ITV, Sky TV, Contact Theatre and The Lowry Arts Centre.</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Drama, as an expressive subject, offers a perspective into the human experience through the art of performance. It enhances understanding of theatrical techniques, storytelling and the collaborative process of creating compelling narratives. Graduates can use creativity, adaptability and communication skills in fields such as film and television production, advertising, public relations and event management. Acting techniques, theatre history, play analysis, directing, design and technical theatre and performance studies are areas you could study. Master acting techniques including character development, emotional expression and physical embodiment, experience in technical aspects of theatre production and analysing scripts to understand dramatic structures are hard skills you’ll develop. Communication and teamwork, adaptability and creativity, empathy and emotional intelligence are soft skills you’ll develop. Career options include actors, entertainers and presenters, dancers and choreographers, public relations professionals, authors, writers and translators, advertising accounts managers and creative directors, and events managers and organisers.</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Essex: Theatre is a radical and influential art form. Its roots lie deep in the ancient world but its relevance to contemporary life is urgent and ongoing. Theatre enables different cultures and societies to confront the most important issues of our time; it provides a crucial space to laugh, to dream, and dare to project different worlds. Studying theatre and drama at Essex enables you to examine some of the most influential play-texts ever written, and to be ready to take part in shaping the essential performances of tomorrow. This degree is a chance to unlock and explore your creativity. You will be performing and producing work in a professional theatre context and will be developing a wide range of creative, critical and practical skills that will open the door to a future in the theatre, cultural industries or a wide range of other graduate careers. At Essex, we offer a rich combination of practical workshops, critical seminars and lectures delivered by an experienced team of playwrights, directors and actors, as well as leading academic theatre specialists. Areas of exploration in our modules include dramatic literature from Ancient Greek tragedy and Shakespeare to modern plays from around the world, contemporary playwriting and devising techniques, staging political ideas and social justice issues, gender, identity and sexual politics on stage, creating Applied Theatre in educational and community contexts, and emergent trends in interactive performance-making and audience participation. Through classroom teaching, practical experiment and professional experience, we help you craft the skillset that will be essential in your creative development. This approach reflects our core belief that engaging with both practice and theory produces a deeper understanding of how theatre works. Creativity, communication and versatility developed during the degree prepare graduates for a wide range of careers. Our students have gone on to become actors, directors and playwrights, as well as producers, live artists, dramaturgs, stage-managers and arts managers. Graduates have also pursued careers in related creative industries including journalism, television production, broadcasting, radio presenting, gaming, magazine editing, copywriting, press relations and marketing, as well as roles in business, commerce and law. Our graduates have gone on to work in roles such as Writer in Residence for the National Theatre, Artistic Director of Jermyn Street Theatre in London, Artistic Director of a touring company, Director for the Almeida Theatre in London, Manager at a regional theatre, Live Artist for Art Angel, BBC Journalist, Youth Theatre Leader and Workshop Facilitator, Outreach and Education Officer, Front of House Theatre Manager, Stage Manager and Secondary School Teacher.
 Manchester: BA Drama embraces all forms of drama across stage, screen and performance contexts. Students explore areas such as literary adaptation, performance in public spaces, performance curation, audio design, playwriting, directing and experimental film cultures. Teaching is informed by recent innovations in theatre and performance alongside historical methods and practices. The programme is embedded within a strong creative ecosystem with links to arts organisations and opportunities to engage with professional practitioners during coursework. Specialist facilities include the purpose-built Martin Harris Centre and the John Thaw Studio, a fully staffed performance, rehearsal and workshop space supporting practical production work. Studying the degree develops transferable and specialist skills including theatre analysis, performance creation, presentation and communication, creative problem solving, teamwork and leadership. Graduates pursue careers across sectors including theatre, film, television, journalism, community arts, teaching, arts administration and business, with alumni working at organisations such as BBC, ITV, Sky TV, Contact Theatre and The Lowry Arts Centre.
@@ -722,20 +764,25 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>Accounting with Economics; Business Economics; Economics and Mathematics; Economics and Politics; Economics with Data Science; Financial Economics; History and Economics; Philosophy, Politics and Economics; Psychology with Economics</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>What is the BSc Economics? The BSc Economics is a three-year degree. You’ll study how economies work, how people and institutions respond to incentives, and how economic evidence is used to explain real-world outcomes. With an emphasis on analysis, data, and economic reasoning, you’ll build the confidence to interpret evidence and apply quantitative insight to complex economic questions. The BSc Economics gives you the opportunity to analyse how people, markets, and governments behave and the quantitative tools to make sense of a world defined by uncertainty, incentives, and change. If you want a degree that explores not just what is happening in the economy but why and what to do about it, this programme gives you that foundation. You’ll explore how economic decisions shape wellbeing, inequality, opportunity, and how societies function. You’ll learn how policy choices affect real lives and how economists use data to create better outcomes. You’ll study micro and macroeconomics, econometrics, behavioural economics, development, labour markets, and public policy. You’ll be taught within a department whose research informs decision-making on labour markets, behavioural change, financial regulation, and development, illustrating how economic theory connects to real policy challenges. Throughout your degree, you’ll learn to think like an economist: breaking down problems, analysing evidence, interpreting data, predicting outcomes, and communicating insights clearly and confidently. By graduation, you’ll have the foundational skills to pursue early careers in government, business, finance and other sectors that value strong analytical ability, or progress to postgraduate study. Students develop skills in microeconomics and macroeconomics to understand how markets work, how incentives influence behaviour, and how economies respond to change; mathematical and quantitative economics to analyse economic problems using mathematical tools; econometrics and data analysis to study economic relationships using statistics and data; applied economics to analyse real-world economic issues and policy questions; and research skills and evidence-based analysis to interpret economic evidence and communicate insights clearly. A BSc Economics degree prepares graduates for careers in economic analysis and data careers such as economist, economic analyst, data analyst, or policy analyst roles using quantitative methods and econometrics; roles in government, regulation and central institutions such as HM Treasury, the Bank of England, government economic units and regulatory bodies; finance, risk and economic consultancy roles in banks and consultancies; research and applied economics roles in think tanks and research institutes; and postgraduate study in economics, econometrics, finance, data science or other quantitative social science disciplines. Graduates from this course have progressed to organisations such as Bank of England, JP Morgan &amp; Chase, Goldman Sachs, HM Treasury and the Financial Conduct Authority.</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Today's turbulent economy demands high calibre, well-rounded graduates who not only specialise in economics but also understand the wider social issues and forces at play. Our BA (Economic and Social Studies), known as the BA (Econ), is a flagship interdisciplinary degree designed for students who want to understand economics in its full social, political and technical context. The programme’s Economics specialisation provides a rigorous education in core economic theory and quantitative methods while equipping students with broader perspectives to address complex global challenges. The BA (Econ) is the parent programme to eight distinctive specialisations including Economics, Economics and Politics, Economics and Philosophy, Economics and Sociology, Economics and Finance, Data Science and Economics, Accounting and Finance, and Finance, allowing students to gain a strong shared foundation in economics alongside insights from other social science disciplines. Students specialising in Economics develop technical skills expected of modern economists including economic modelling, statistical and data analysis, interpretation and policy evaluation, while also building critical thinking, ethical reasoning and real-world application skills. The programme enables students to analyse economic issues through mathematical and data-driven approaches as well as through understanding institutions, behaviour, history and social outcomes. It also examines how emerging technologies including generative AI are transforming economic decision-making, while emphasising the importance of human judgement, contextual understanding and interdisciplinary insight. Graduates are prepared to design effective policies, assess economic trade-offs critically and understand how economic decisions affect societies, communities and countries. The degree prepares students for careers in economics, public policy, finance, consultancy, data analysis and international development. Economics graduates from Manchester go on to careers across sectors including finance and banking, professional services, government and public policy, with recent graduates working at organisations such as Morgan Stanley, KPMG, the House of Lords and the Government Economic Service.</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Economics is the study of how scarce resources are allocated within societies and how individuals, businesses and governments make decisions. The subject is typically divided into microeconomics, which examines the behaviour of households, firms and industries, and macroeconomics, which focuses on the performance of the economy as a whole. Key areas of study include macroeconomics, microeconomics, probability and statistics, mathematics for economists, econometrics and programming for economic analysis. Study develops quantitative and analytical skills such as statistical modelling, economic forecasting, financial and market analysis, data interpretation and research design. Graduates may pursue careers in sectors including finance, consulting, government, policy analysis, data analytics, business strategy and international organisations.</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Essex: What is the BSc Economics? The BSc Economics is a three-year degree. You’ll study how economies work, how people and institutions respond to incentives, and how economic evidence is used to explain real-world outcomes. With an emphasis on analysis, data, and economic reasoning, you’ll build the confidence to interpret evidence and apply quantitative insight to complex economic questions. The BSc Economics gives you the opportunity to analyse how people, markets, and governments behave and the quantitative tools to make sense of a world defined by uncertainty, incentives, and change. If you want a degree that explores not just what is happening in the economy but why and what to do about it, this programme gives you that foundation. You’ll explore how economic decisions shape wellbeing, inequality, opportunity, and how societies function. You’ll learn how policy choices affect real lives and how economists use data to create better outcomes. You’ll study micro and macroeconomics, econometrics, behavioural economics, development, labour markets, and public policy. You’ll be taught within a department whose research informs decision-making on labour markets, behavioural change, financial regulation, and development, illustrating how economic theory connects to real policy challenges. Throughout your degree, you’ll learn to think like an economist: breaking down problems, analysing evidence, interpreting data, predicting outcomes, and communicating insights clearly and confidently. By graduation, you’ll have the foundational skills to pursue early careers in government, business, finance and other sectors that value strong analytical ability, or progress to postgraduate study. Students develop skills in microeconomics and macroeconomics to understand how markets work, how incentives influence behaviour, and how economies respond to change; mathematical and quantitative economics to analyse economic problems using mathematical tools; econometrics and data analysis to study economic relationships using statistics and data; applied economics to analyse real-world economic issues and policy questions; and research skills and evidence-based analysis to interpret economic evidence and communicate insights clearly. A BSc Economics degree prepares graduates for careers in economic analysis and data careers such as economist, economic analyst, data analyst, or policy analyst roles using quantitative methods and econometrics; roles in government, regulation and central institutions such as HM Treasury, the Bank of England, government economic units and regulatory bodies; finance, risk and economic consultancy roles in banks and consultancies; research and applied economics roles in think tanks and research institutes; and postgraduate study in economics, econometrics, finance, data science or other quantitative social science disciplines. Graduates from this course have progressed to organisations such as Bank of England, JP Morgan &amp; Chase, Goldman Sachs, HM Treasury and the Financial Conduct Authority.
 Manchester: Today's turbulent economy demands high calibre, well-rounded graduates who not only specialise in economics but also understand the wider social issues and forces at play. Our BA (Economic and Social Studies), known as the BA (Econ), is a flagship interdisciplinary degree designed for students who want to understand economics in its full social, political and technical context. The programme’s Economics specialisation provides a rigorous education in core economic theory and quantitative methods while equipping students with broader perspectives to address complex global challenges. The BA (Econ) is the parent programme to eight distinctive specialisations including Economics, Economics and Politics, Economics and Philosophy, Economics and Sociology, Economics and Finance, Data Science and Economics, Accounting and Finance, and Finance, allowing students to gain a strong shared foundation in economics alongside insights from other social science disciplines. Students specialising in Economics develop technical skills expected of modern economists including economic modelling, statistical and data analysis, interpretation and policy evaluation, while also building critical thinking, ethical reasoning and real-world application skills. The programme enables students to analyse economic issues through mathematical and data-driven approaches as well as through understanding institutions, behaviour, history and social outcomes. It also examines how emerging technologies including generative AI are transforming economic decision-making, while emphasising the importance of human judgement, contextual understanding and interdisciplinary insight. Graduates are prepared to design effective policies, assess economic trade-offs critically and understand how economic decisions affect societies, communities and countries. The degree prepares students for careers in economics, public policy, finance, consultancy, data analysis and international development. Economics graduates from Manchester go on to careers across sectors including finance and banking, professional services, government and public policy, with recent graduates working at organisations such as Morgan Stanley, KPMG, the House of Lords and the Government Economic Service.
@@ -754,20 +801,25 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>Business Management with a Modern Language; English Language and Literature; English Literature; Language Studies; Language Studies and Linguistics; Language Studies and Teaching English as a Foreign Language; Licence English and French Law; Linguistics; Linguistics with Data Science; Modern Languages and Linguistics; Speech and Language Therapy</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
           <t>What is the range of sounds found in human languages? Which of those sounds are used by English to construct words? How are words combined to form meaningful sentences in English, and are the same patterns of combination found in other languages? How does society and social pressure affect the way we speak? How do different varieties of English evolve? These are some of the questions you will address in the course. Language is central to all human activity, from important negotiations between nation states to doctor-patient interaction to spontaneous conversations in cafés. Through your study of language, you come to understand the nature of human social life. Foundational modules in the first and second year will teach you how to analyse linguistic sound systems, word structure, sentence structure, meaning and language use, and apply your knowledge to the analysis of English. You will then be able to make informed choices about areas of English or Linguistics you want to study in greater depth through study options such as Phonetics, English around the World, Language and the Mind, Conversation and Social Interaction, Institutional Talk, and English Language in the Media. We are 1st in UK for research impact in modern languages and linguistics (Grade Point Average, Research Excellence Framework 2021). You have an opportunity to study different kinds of linguistics from structural linguistics to applied and experimental linguistics. Studying language and linguistics allows you to develop your research and IT skills by collecting and analysing linguistic data using modern linguistic methods, and a combination of team-work and independent projects enhances your communication, problem-solving and management skills. Graduates of our department have gone on to have careers in a wide variety of fields including teaching (in the UK and abroad), journalism, branding, advertising, marketing, travel, communications, publishing, speech and occupational therapy, interpreting, translating and media. Other graduates have gone on to work for organisations including the British Council, English in Action, Royal Bank of Scotland, Macmillan Publishers, Cambridge University Press, Freshfields Bruckhaus Deringer and Decisive Media Ltd.</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Our BA English Language and English Literature joint honours course will enable you to delve into the science of language while exploring a wide range of texts dating from a variety of periods. You will be taken on a broadly chronological journey of English Literature from the Anglo-Saxon period through to the present day. In addition, you will investigate the sounds, words and grammar of the English language, discovering where English comes from, how it developed over time, how it varies across the UK and further afield, and how it is used in different situations. You will acquire the skills required for analytical language study alongside the means to apply those skills to the study of historical and present-day English. You will practise key transferable skills such as essay writing and presentation. You can broaden the scope of your studies to investigate areas such as the interaction between psychology and language (psycholinguistics), child language development, and methodological approaches used in the study of English Language and English Literature. The course provides access to specialist resources including psycholinguistics and phonetics laboratories with facilities for signal analysis, speech synthesis, laryngography and electropalatography. Studying the degree helps you develop analytical and problem-solving skills as well as transferable skills that support careers across sectors including media, marketing, speech and language therapy, lexicography and teaching. Graduates have pursued careers at organisations such as The Guardian, L’Oreal, Universal Music Group and Vodafone.</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>English Language is the study of the structure, history and use of English, including its sounds, grammar, vocabulary and variation across regions and social contexts. The subject covers areas such as linguistics, sociolinguistics, language and communication, sound and meaning, language change, digital communication, multilingualism and language revitalisation. Study develops analytical and research skills related to language description, discourse analysis, writing and communication. Graduates may pursue careers in sectors such as teaching, journalism, publishing, copywriting, public relations, digital content management, librarianship and administration, or continue to postgraduate study in linguistics or related fields.</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Essex: What is the range of sounds found in human languages? Which of those sounds are used by English to construct words? How are words combined to form meaningful sentences in English, and are the same patterns of combination found in other languages? How does society and social pressure affect the way we speak? How do different varieties of English evolve? These are some of the questions you will address in the course. Language is central to all human activity, from important negotiations between nation states to doctor-patient interaction to spontaneous conversations in cafés. Through your study of language, you come to understand the nature of human social life. Foundational modules in the first and second year will teach you how to analyse linguistic sound systems, word structure, sentence structure, meaning and language use, and apply your knowledge to the analysis of English. You will then be able to make informed choices about areas of English or Linguistics you want to study in greater depth through study options such as Phonetics, English around the World, Language and the Mind, Conversation and Social Interaction, Institutional Talk, and English Language in the Media. We are 1st in UK for research impact in modern languages and linguistics (Grade Point Average, Research Excellence Framework 2021). You have an opportunity to study different kinds of linguistics from structural linguistics to applied and experimental linguistics. Studying language and linguistics allows you to develop your research and IT skills by collecting and analysing linguistic data using modern linguistic methods, and a combination of team-work and independent projects enhances your communication, problem-solving and management skills. Graduates of our department have gone on to have careers in a wide variety of fields including teaching (in the UK and abroad), journalism, branding, advertising, marketing, travel, communications, publishing, speech and occupational therapy, interpreting, translating and media. Other graduates have gone on to work for organisations including the British Council, English in Action, Royal Bank of Scotland, Macmillan Publishers, Cambridge University Press, Freshfields Bruckhaus Deringer and Decisive Media Ltd.
 Manchester: Our BA English Language and English Literature joint honours course will enable you to delve into the science of language while exploring a wide range of texts dating from a variety of periods. You will be taken on a broadly chronological journey of English Literature from the Anglo-Saxon period through to the present day. In addition, you will investigate the sounds, words and grammar of the English language, discovering where English comes from, how it developed over time, how it varies across the UK and further afield, and how it is used in different situations. You will acquire the skills required for analytical language study alongside the means to apply those skills to the study of historical and present-day English. You will practise key transferable skills such as essay writing and presentation. You can broaden the scope of your studies to investigate areas such as the interaction between psychology and language (psycholinguistics), child language development, and methodological approaches used in the study of English Language and English Literature. The course provides access to specialist resources including psycholinguistics and phonetics laboratories with facilities for signal analysis, speech synthesis, laryngography and electropalatography. Studying the degree helps you develop analytical and problem-solving skills as well as transferable skills that support careers across sectors including media, marketing, speech and language therapy, lexicography and teaching. Graduates have pursued careers at organisations such as The Guardian, L’Oreal, Universal Music Group and Vodafone.
@@ -786,16 +838,21 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
+          <t>Economics and Politics; Global Politics; Journalism and Politics; Law with Politics; Modern History and Politics; Philosophy and Politics; Philosophy, Politics and Economics; Politics; Politics and International Relations; Politics with Business</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
           <t>Switch on the news any day of the week, or pick up just about any national newspaper, and you will be sure to come across an item on Europe. It is clear that the future of Europe is a geo-political question of profound importance for the future of the world we live in. Yet, few of us truly understand the complex phenomenon that is modern Europe. You'll examine Europe's economic, legal, and sociological context, as well as its historical origins whilst acquiring an understanding of Europe's rich cultural traditions. The artists, writers, musicians, composers and film-makers of Europe have exerted a cultural influence that even now is not eclipsed by the dominance of America on the world's stage. Based within our School of Philosophical, Historical and Interdisciplinary Studies, European studies is a subject that approaches the complex idea of Europe via a wide range of disciplines in the humanities and social sciences. We have expertise in modern languages, literature, film, history of art, history, politics and sociology. Here at Essex, our teaching and research in European studies offers maximum flexibility for you to study areas that interest you, so you can pursue a wide range of topics including European identity and the development of the EU, representations of non-Europeans in art, Europe's colonial history, religion in Europe, and EU law. The study of Europe is vital for ongoing discussion of what Europe's future ought to be; a discussion that will profoundly affect every European citizen. Through a course in European studies, you can acquire the knowledge, skills and experience to make an active contribution to one of the most important political and cultural processes of the century. This course provides excellent preparation for areas which include import/export management, banking and financial sectors, academia, airlines, information technology, management, museums, teaching, non-governmental offices, and development agencies in the UK and abroad. Our graduates have gone on to work for a wide range of organisations including the Civil Service (especially the Foreign Office), embassies around the world, the European Council on Foreign Relations, the Europe Direct Contact Centre in Brussels, the Spanish Congress of Deputies, and LEAD Europe. Other recent graduates have also undertaken traineeships with the European Commission for the Directorate-General for Education and Culture, and various internships in journalism and with NGOs.</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>The BSocSc (Hons) in Politics and International Relations is a single honours course for politics specialists. Teaching and research are structured around three core themes including Comparative Politics, International Politics and Political Theory. In Years 1 and 2 students take course units from across the three core areas alongside options from disciplines such as Economics, Sociology, History, Philosophy or Languages. By the final year students develop an advanced understanding of politics that reflects the research expertise of staff. The programme supports internationally recognised research across a range of areas and offers a variety of course units that build directly on this research expertise. Students develop solid intellectual foundations within the discipline while gaining increasing choice and diversity of subjects and approaches as they progress. The course aims to provide the opportunity to study politics in depth and breadth through a single-honours specialisation, develop intellectual independence and autonomy, support the development of skills required to undertake independent research of a high standard, and build intellectual flexibility and adaptability. Research areas explored within the programme include topics such as security, migration, war, gender, ethics, resistance and international institutions. Graduates pursue careers across sectors including consultancy, public administration, diplomacy, policy and business, with alumni working at organisations such as Google, Thomson Reuters, Deloitte, HMRC, the Royal Danish Embassy, the Ministry of Justice, Greater Manchester Chamber of Commerce, Cicero Consultancy and Essex County Council.</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr">
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
         <is>
           <t>Essex: Switch on the news any day of the week, or pick up just about any national newspaper, and you will be sure to come across an item on Europe. It is clear that the future of Europe is a geo-political question of profound importance for the future of the world we live in. Yet, few of us truly understand the complex phenomenon that is modern Europe. You'll examine Europe's economic, legal, and sociological context, as well as its historical origins whilst acquiring an understanding of Europe's rich cultural traditions. The artists, writers, musicians, composers and film-makers of Europe have exerted a cultural influence that even now is not eclipsed by the dominance of America on the world's stage. Based within our School of Philosophical, Historical and Interdisciplinary Studies, European studies is a subject that approaches the complex idea of Europe via a wide range of disciplines in the humanities and social sciences. We have expertise in modern languages, literature, film, history of art, history, politics and sociology. Here at Essex, our teaching and research in European studies offers maximum flexibility for you to study areas that interest you, so you can pursue a wide range of topics including European identity and the development of the EU, representations of non-Europeans in art, Europe's colonial history, religion in Europe, and EU law. The study of Europe is vital for ongoing discussion of what Europe's future ought to be; a discussion that will profoundly affect every European citizen. Through a course in European studies, you can acquire the knowledge, skills and experience to make an active contribution to one of the most important political and cultural processes of the century. This course provides excellent preparation for areas which include import/export management, banking and financial sectors, academia, airlines, information technology, management, museums, teaching, non-governmental offices, and development agencies in the UK and abroad. Our graduates have gone on to work for a wide range of organisations including the Civil Service (especially the Foreign Office), embassies around the world, the European Council on Foreign Relations, the Europe Direct Contact Centre in Brussels, the Spanish Congress of Deputies, and LEAD Europe. Other recent graduates have also undertaken traineeships with the European Commission for the Directorate-General for Education and Culture, and various internships in journalism and with NGOs.
 Manchester: The BSocSc (Hons) in Politics and International Relations is a single honours course for politics specialists. Teaching and research are structured around three core themes including Comparative Politics, International Politics and Political Theory. In Years 1 and 2 students take course units from across the three core areas alongside options from disciplines such as Economics, Sociology, History, Philosophy or Languages. By the final year students develop an advanced understanding of politics that reflects the research expertise of staff. The programme supports internationally recognised research across a range of areas and offers a variety of course units that build directly on this research expertise. Students develop solid intellectual foundations within the discipline while gaining increasing choice and diversity of subjects and approaches as they progress. The course aims to provide the opportunity to study politics in depth and breadth through a single-honours specialisation, develop intellectual independence and autonomy, support the development of skills required to undertake independent research of a high standard, and build intellectual flexibility and adaptability. Research areas explored within the programme include topics such as security, migration, war, gender, ethics, resistance and international institutions. Graduates pursue careers across sectors including consultancy, public administration, diplomacy, policy and business, with alumni working at organisations such as Google, Thomson Reuters, Deloitte, HMRC, the Royal Danish Embassy, the Ministry of Justice, Greater Manchester Chamber of Commerce, Cicero Consultancy and Essex County Council.</t>
@@ -813,20 +870,25 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
+          <t>Film Studies and Literature; Film and Creative Writing; Film and Drama</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
           <t>How does cinema affect us as individuals and as groups, as communities or nations? Do the moving pictures reflect our beliefs or help to change how we see the world? How powerful are visual media in shaping our interpretations of modern life? These are some of the most pressing questions cinema asks us. Our ability to read and interpret the images and stories that films deliver is crucial to how we understand contemporary life. At Essex you combine studying the history and theory of cinema with practical film production, so you don't just critically examine cinema – you create it. Your production modules enable you to develop and apply your academic knowledge and understanding of film, refining and enriching your own practical work. We give you the opportunity to explore film across a broad range of genres, time periods, and regions, from Hollywood, world and independent cinema to documentaries and television. Simultaneously, you gain hands-on experience in film production and production management, essential for careers in the film and television industry. We nurture the creative talent for tomorrow, developing filmmakers, scholars and thinkers with a dynamic worldview. You gain hands-on experience of camera work, sound recording, editing, lighting and scriptwriting, explore the formal aesthetics of film composition and structure in relation to different contexts of production and reception, discover the history and social significance of film as a global medium, understand the links between critical analysis and creative practice, and produce both group films and personal projects. By graduation you will have built up a fully rounded portfolio of work, enabling you to showcase your experience, versatility and creative potential to future employers. We offer a varied, flexible and distinctive curriculum focused on developing your abilities in film while also enabling you to take options from other courses within our Department of Literature, Film and Theatre Studies including literature, creative writing, journalism and drama. You graduate from our course with key skills in writing close analysis, critical thinking, contextual research, time management and hands-on filmmaking. The short film you will make as part of your studies serves as a calling card, showcasing your individual creative potential as part of a portfolio of practical work developed during your course. Our students are well prepared to enter careers in film production, television, journalism, publishing and teaching. Recent graduates have gone on to roles including celebrity booking for Cactus TV, editor for BBC television, subtitle writer for Sky TV, and teachers of English and Media Studies.</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>BA Drama and Film Studies enables students to benefit from teaching and research in Drama while engaging in the study of film and television. Students take courses in theatre and film history and theory alongside practical courses in theatre production and filmmaking, with opportunities to study video-making and engage with professional practitioners working in the cultural industries. Teaching reflects both contemporary innovations in theatre, performance and film studies and historical practices. The programme operates within a strong creative and cultural network with links to arts organisations and performance partners. Specialist facilities include the Martin Harris Centre and the John Thaw Studio as well as rehearsal rooms, screening rooms and sound and video-editing suites that support creative production work. Students develop skills including theatre and film analysis, creating original performance work, communication, creative problem solving, teamwork and leadership. Graduates pursue careers in theatre, film, television, journalism, arts administration and related sectors, with alumni working at organisations such as BBC, ITV, Sky TV, Tandem Theatre and The Lowry Arts Centre.</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Film studies gives an understanding of visual storytelling, film history and cultural impact. Studying film studies opens doors to career paths such as film production, directing, screenwriting and digital content creation. Creative cinematography, storytelling for the screen, production skills, analogue and digital technology, the business of Hollywood, film and photography’s role in history, principles of creativity and society of the media are areas you could study. Film analysis, scriptwriting, story structure and project planning and coordination are hard skills you’ll develop. Critical thinking, communication skills, creative expression and presentation skills are soft skills you’ll develop. Career options include arts officers, producers and directors, photographers, audio-visual and broadcasting equipment operators, TV, video and audio servicers and repairers, authors, writers and translators.</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>Essex: How does cinema affect us as individuals and as groups, as communities or nations? Do the moving pictures reflect our beliefs or help to change how we see the world? How powerful are visual media in shaping our interpretations of modern life? These are some of the most pressing questions cinema asks us. Our ability to read and interpret the images and stories that films deliver is crucial to how we understand contemporary life. At Essex you combine studying the history and theory of cinema with practical film production, so you don't just critically examine cinema – you create it. Your production modules enable you to develop and apply your academic knowledge and understanding of film, refining and enriching your own practical work. We give you the opportunity to explore film across a broad range of genres, time periods, and regions, from Hollywood, world and independent cinema to documentaries and television. Simultaneously, you gain hands-on experience in film production and production management, essential for careers in the film and television industry. We nurture the creative talent for tomorrow, developing filmmakers, scholars and thinkers with a dynamic worldview. You gain hands-on experience of camera work, sound recording, editing, lighting and scriptwriting, explore the formal aesthetics of film composition and structure in relation to different contexts of production and reception, discover the history and social significance of film as a global medium, understand the links between critical analysis and creative practice, and produce both group films and personal projects. By graduation you will have built up a fully rounded portfolio of work, enabling you to showcase your experience, versatility and creative potential to future employers. We offer a varied, flexible and distinctive curriculum focused on developing your abilities in film while also enabling you to take options from other courses within our Department of Literature, Film and Theatre Studies including literature, creative writing, journalism and drama. You graduate from our course with key skills in writing close analysis, critical thinking, contextual research, time management and hands-on filmmaking. The short film you will make as part of your studies serves as a calling card, showcasing your individual creative potential as part of a portfolio of practical work developed during your course. Our students are well prepared to enter careers in film production, television, journalism, publishing and teaching. Recent graduates have gone on to roles including celebrity booking for Cactus TV, editor for BBC television, subtitle writer for Sky TV, and teachers of English and Media Studies.
 Manchester: BA Drama and Film Studies enables students to benefit from teaching and research in Drama while engaging in the study of film and television. Students take courses in theatre and film history and theory alongside practical courses in theatre production and filmmaking, with opportunities to study video-making and engage with professional practitioners working in the cultural industries. Teaching reflects both contemporary innovations in theatre, performance and film studies and historical practices. The programme operates within a strong creative and cultural network with links to arts organisations and performance partners. Specialist facilities include the Martin Harris Centre and the John Thaw Studio as well as rehearsal rooms, screening rooms and sound and video-editing suites that support creative production work. Students develop skills including theatre and film analysis, creating original performance work, communication, creative problem solving, teamwork and leadership. Graduates pursue careers in theatre, film, television, journalism, arts administration and related sectors, with alumni working at organisations such as BBC, ITV, Sky TV, Tandem Theatre and The Lowry Arts Centre.
@@ -845,20 +907,25 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>Art History; Curating with History; History and Economics; History and Literature; History and Sociology; Modern History; Modern History and International Relations; Modern History and Politics</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
           <t>At the University of Essex we're about social conscience, wondering why, and understanding the bigger picture. We teach you to find your own critical voice and view history through the eyes of different people, telling hidden histories that might otherwise be forgotten. Our BA History allows you to explore challenging questions about the impact of political, social and cultural change on individuals, social groups and regions. From African-American slavery to Stalin's Russia—from households in Essex to witchcraft in Germany—from the history of disease to revolutions in China, we urge you to explore the past in order to better understand the present. You have the flexibility to choose from a wide range of optional modules about subjects close to home and further afield. We also provide you with opportunities to explore local history and have close ties with the Essex Record Office, one of the best county record offices in the UK. Assessed coursework generally consists of essays, concept studies, critical commentaries, research proposals and a 15,000-word dissertation. Students usually attend a two-hour seminar for each module each week, with seminar groups or workshops usually having about 15 students. In addition to the opportunity to learn about the past and come to a better understanding of the present, a course in history also provides you with important skills that will be of value after leaving university. You learn to absorb, analyse and assess a wide variety of information and viewpoints, to express your arguments in oral and written form, and to think and work both independently and in co-operation with others. You therefore graduate prepared for a wide range of careers including teaching, librarianship, museum and archive services, the Civil Service, local government, law enforcement and charity administration. Others have proceeded to work in banking, industrial and retail management, media research, electronic publishing, marketing, IT, health service administration, counselling and social work, while others have chosen to enhance their career opportunities by studying at postgraduate level. Some of our recent graduates have found employment as a warden for the Royal Collection at Windsor Castle, a planning support officer for a local council, a senior underwriting assistant at CNA Insurance Company Limited, a researcher at the House of Commons, a graduate trainee for the Royal Botanic Gardens at Kew and a library assistant for the University of Cambridge.</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Our BA History course will give you the opportunity to tailor your degree to suit your own interests while learning from one of the largest concentrations of historians in Britain. Students can choose course units covering a wide range of periods and topics including ancient, medieval, modern, economic and social history, as well as the history of science, technology and medicine. In Years 1 and 2 students may also take course units in other disciplines including languages, the humanities and the social sciences. Students have the option to specialise in a particular area of interest or continue to study a broad range of topics in their final year, choosing units covering British, European, American, African and Asian history across different periods and culminating in a dissertation. The programme provides expert training in analysis and critical reasoning while developing transferable skills in communication and presentation, argument and debate, teamwork, research and time management. Graduates pursue careers across sectors including teaching and academia, heritage and museums, the Civil Service, policy and thinktanks, creative industries, media and journalism, marketing and public relations, law and accountancy, finance and NGOs, with alumni working at organisations such as the BBC, KPMG, Deloitte, Marks and Spencer, Aviva, Accenture and Barclays.</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Gain an understanding of the economies, societies, faiths, and cultures that have shaped our world over time. Studying history will allow you to read and analyse texts and evidence, and gain an in-depth understanding of the forces that have shaped our modern world. You could combine history with other subjects like English, languages, or economics, and focus on particular periods of history you’re fascinated by. The research and critical thinking skills you gain will equip you for roles in a variety of industries such as local and central government, journalism, education, heritage, publishing, and academia. You could also go on to further study. Political communities in world history, societies and economies in world history, 19th and 20th century Britain, Europe in the making, disease and society, theory and practice of oral history, arguments and analysis, evidence and methods, Latin America: themes and problems, history and politics of the modern Middle East, contemporary US race relations and corruption in Britain and its empire are areas you could study. Exhibitions, archives, curation, marketing and cataloguing are hard skills you'll develop. Communication, management, research, customer service and planning are soft skills you'll develop. Career options include archaeologist, art gallery manager, museum curator, arts administrator, antiques dealer, heritage manager, higher education lecturer or researcher, secondary school teacher, social researcher, journalist, writer, public relations roles, publishing assistant, academic librarian and archivist.</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Essex: At the University of Essex we're about social conscience, wondering why, and understanding the bigger picture. We teach you to find your own critical voice and view history through the eyes of different people, telling hidden histories that might otherwise be forgotten. Our BA History allows you to explore challenging questions about the impact of political, social and cultural change on individuals, social groups and regions. From African-American slavery to Stalin's Russia—from households in Essex to witchcraft in Germany—from the history of disease to revolutions in China, we urge you to explore the past in order to better understand the present. You have the flexibility to choose from a wide range of optional modules about subjects close to home and further afield. We also provide you with opportunities to explore local history and have close ties with the Essex Record Office, one of the best county record offices in the UK. Assessed coursework generally consists of essays, concept studies, critical commentaries, research proposals and a 15,000-word dissertation. Students usually attend a two-hour seminar for each module each week, with seminar groups or workshops usually having about 15 students. In addition to the opportunity to learn about the past and come to a better understanding of the present, a course in history also provides you with important skills that will be of value after leaving university. You learn to absorb, analyse and assess a wide variety of information and viewpoints, to express your arguments in oral and written form, and to think and work both independently and in co-operation with others. You therefore graduate prepared for a wide range of careers including teaching, librarianship, museum and archive services, the Civil Service, local government, law enforcement and charity administration. Others have proceeded to work in banking, industrial and retail management, media research, electronic publishing, marketing, IT, health service administration, counselling and social work, while others have chosen to enhance their career opportunities by studying at postgraduate level. Some of our recent graduates have found employment as a warden for the Royal Collection at Windsor Castle, a planning support officer for a local council, a senior underwriting assistant at CNA Insurance Company Limited, a researcher at the House of Commons, a graduate trainee for the Royal Botanic Gardens at Kew and a library assistant for the University of Cambridge.
 Manchester: Our BA History course will give you the opportunity to tailor your degree to suit your own interests while learning from one of the largest concentrations of historians in Britain. Students can choose course units covering a wide range of periods and topics including ancient, medieval, modern, economic and social history, as well as the history of science, technology and medicine. In Years 1 and 2 students may also take course units in other disciplines including languages, the humanities and the social sciences. Students have the option to specialise in a particular area of interest or continue to study a broad range of topics in their final year, choosing units covering British, European, American, African and Asian history across different periods and culminating in a dissertation. The programme provides expert training in analysis and critical reasoning while developing transferable skills in communication and presentation, argument and debate, teamwork, research and time management. Graduates pursue careers across sectors including teaching and academia, heritage and museums, the Civil Service, policy and thinktanks, creative industries, media and journalism, marketing and public relations, law and accountancy, finance and NGOs, with alumni working at organisations such as the BBC, KPMG, Deloitte, Marks and Spencer, Aviva, Accenture and Barclays.
@@ -877,16 +944,21 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
+          <t>Modern Languages with Latin American Studies</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
           <t>BA Global Studies and Latin American Studies will equip you with a broad range of skills to become an active participant in a crucial time of change. You'll study some of today's most pressing issues from the migrant crisis to climate change, and you'll acquire a global perspective to face contemporary challenges. This interdisciplinary degree combines the breadth of Global Studies with deep engagement in Latin American history and culture. Latin America is one of the most fascinating and complex areas of the world, home to a rich diversity of indigenous people, as well as some of the world's fastest growing economies, greatest environmental challenges, and richest cultural traditions. Latin America is an area of study that will surprise you, challenge you and broaden your horizons. A core part of the course are modules from history and politics which explore international relations and global history, alongside Latin American Studies modules. You will study a range of topics including economic and political history of Latin America, indigenous issues in Latin America, global technologies, migration, and art and architecture in social context. Language is fundamental to our thought, our relationships and our civilisations. As part of this degree you will add a language to your portfolio through either learning Spanish from scratch or developing existing skills in Spanish and/or Brazilian Portuguese to a high level, and spending your third year at a university in a Latin American country. This course differs from BA Global Studies with Latin American Studies in that it includes a compulsory year abroad in a Latin American country and has a compulsory language component. Our graduates are well-placed to address the complex issues which confront the modern world. Our course provides you with an excellent basis for going onto a career in media, education, politics, the Civil Service, international organisations such as the UN and NATO or non-governmental organisations, and many other fields. Our Centre's recent graduates have gone on to work in a wide range of roles including an events co-ordinator for Age UK, a business provision manager for BT, an accountant in London, and an account executive for Bluesky PR.</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Our single honours BA Spanish, Portuguese and Latin American Studies course will give you a strong grounding in writing, speaking and understanding the Spanish and Portuguese languages, as well as the opportunity to learn Catalan. After Year 1, Portuguese language is not compulsory and students can choose to concentrate more on Spanish, maintain a balance between the languages or focus more on Portuguese by the final year, with the option to study Catalan. Language study enables students to explore diverse aspects of the culture, society, history, politics and literature of countries where Spanish and Portuguese are spoken while developing intercultural awareness and communication skills. A compulsory third year residence abroad allows students to live, study or work in Spanish- and Portuguese-speaking countries in Europe and Latin America, providing significant personal, linguistic and professional development. Language units are compulsory at all levels of the degree. The programme benefits from collaborations with cultural institutions such as Instituto Cervantes and links with Portuguese cultural organisations. Specialist facilities include extensive collections relating to Lusophone Africa, access to films and texts on Latin America, Portugal and Spain, and resources at the University Language Centre including interpreting suites, recording rooms and multilingual learning technologies. Graduates pursue careers across sectors including media, journalism, public relations, business services, marketing, banking and communications, with alumni working at organisations such as ASOS, Ernst &amp; Young, Procter &amp; Gamble, JD Sports, Oxfam, Greenpeace and Virgin.</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
         <is>
           <t>Essex: BA Global Studies and Latin American Studies will equip you with a broad range of skills to become an active participant in a crucial time of change. You'll study some of today's most pressing issues from the migrant crisis to climate change, and you'll acquire a global perspective to face contemporary challenges. This interdisciplinary degree combines the breadth of Global Studies with deep engagement in Latin American history and culture. Latin America is one of the most fascinating and complex areas of the world, home to a rich diversity of indigenous people, as well as some of the world's fastest growing economies, greatest environmental challenges, and richest cultural traditions. Latin America is an area of study that will surprise you, challenge you and broaden your horizons. A core part of the course are modules from history and politics which explore international relations and global history, alongside Latin American Studies modules. You will study a range of topics including economic and political history of Latin America, indigenous issues in Latin America, global technologies, migration, and art and architecture in social context. Language is fundamental to our thought, our relationships and our civilisations. As part of this degree you will add a language to your portfolio through either learning Spanish from scratch or developing existing skills in Spanish and/or Brazilian Portuguese to a high level, and spending your third year at a university in a Latin American country. This course differs from BA Global Studies with Latin American Studies in that it includes a compulsory year abroad in a Latin American country and has a compulsory language component. Our graduates are well-placed to address the complex issues which confront the modern world. Our course provides you with an excellent basis for going onto a career in media, education, politics, the Civil Service, international organisations such as the UN and NATO or non-governmental organisations, and many other fields. Our Centre's recent graduates have gone on to work in a wide range of roles including an events co-ordinator for Age UK, a business provision manager for BT, an accountant in London, and an account executive for Bluesky PR.
 Manchester: Our single honours BA Spanish, Portuguese and Latin American Studies course will give you a strong grounding in writing, speaking and understanding the Spanish and Portuguese languages, as well as the opportunity to learn Catalan. After Year 1, Portuguese language is not compulsory and students can choose to concentrate more on Spanish, maintain a balance between the languages or focus more on Portuguese by the final year, with the option to study Catalan. Language study enables students to explore diverse aspects of the culture, society, history, politics and literature of countries where Spanish and Portuguese are spoken while developing intercultural awareness and communication skills. A compulsory third year residence abroad allows students to live, study or work in Spanish- and Portuguese-speaking countries in Europe and Latin America, providing significant personal, linguistic and professional development. Language units are compulsory at all levels of the degree. The programme benefits from collaborations with cultural institutions such as Instituto Cervantes and links with Portuguese cultural organisations. Specialist facilities include extensive collections relating to Lusophone Africa, access to films and texts on Latin America, Portugal and Spain, and resources at the University Language Centre including interpreting suites, recording rooms and multilingual learning technologies. Graduates pursue careers across sectors including media, journalism, public relations, business services, marketing, banking and communications, with alumni working at organisations such as ASOS, Ernst &amp; Young, Procter &amp; Gamble, JD Sports, Oxfam, Greenpeace and Virgin.</t>
@@ -904,20 +976,25 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>Criminology with Criminal Law; Law; Law with Business; Law with Criminology; Law with Human Rights; Law with Philosophy; Law with Politics; Licence English and French Law</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t>What is LLB Law with Human Rights? The LLB Law with Human Rights is a three-year undergraduate qualifying law degree. It combines a full legal education with a dedicated focus on human rights at domestic, European, and international levels. You’ll study the core foundations of English law alongside specialist human rights modules, graduating with in-depth knowledge of how rights are protected and applied across different legal systems. The LLB Law with Human Rights combines a qualifying law degree with specialist training in UK, European, and international human rights law. It is ideal for students who want to study law through the lens of justice, rights, and social impact. The course is shaped by internationally recognised expertise in human rights. You’ll develop strong legal reasoning, research, and analytical skills while applying law to real-world human rights issues. Your studies explore how law operates as a practical tool for protecting individuals and contributing to fairer societies. Students study core legal foundations including legal method, contract, criminal law, public law, tort, land law, and equity, while also exploring UK and European human rights law and international human rights law as dedicated areas of study. The course examines how domestic law interacts with European and international legal frameworks and develops skills in case analysis, rights-based argumentation, and legal research. Students critically evaluate law within social, political, and ethical settings. An LLB Law with Human Rights prepares graduates for careers in law and policy including roles such as solicitor, barrister, paralegal or legal adviser, as well as careers within human rights organisations, charities and advocacy groups, government and public bodies, international organisations, policy research institutes and social justice organisations, and roles in compliance, governance and corporate responsibility.</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Law is at the heart of our society, informing and governing our everyday actions. The LLB Law course offers a distinctive approach to legal education that combines research-informed study with practice-led approaches. Students study the foundations of English and Welsh law and have the freedom to follow their own interests through a broad range of optional units while being challenged to analyse and critique the law and understand the social, economic, ethical and political contexts in which it operates. Career-focused learning is embedded throughout the course, including opportunities to apply legal theory in practice through clinical legal education at the Justice Hub, which offers free legal advice to members of the public and supports partnerships with the public, charitable and private sectors. Students develop a global perspective on law alongside essential skills, knowledge and experience for careers both within and beyond the legal profession. The programme includes engagement with areas such as family law, business law and criminal law, and introduces students to emerging fields such as LegalTech. Facilities supporting study include a moot court for simulated legal practice and access to specialist law library resources. The course provides preparation relevant to professional pathways including the Solicitors Qualifying Exam and academic requirements associated with training for the Bar. Graduates pursue careers across legal, business and public sector fields.</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Whether you want to argue for human rights in the international courts, or help families closer to home, studying law means you can make a difference to people’s lives. If you choose a law degree, you’ll acquire a broad set of transferable skills and a greater understanding of the world we live in. Studying law helps you better understand how we interact as humans, and how we create the frameworks of a civilised society. You’ll learn to analyse and problem solve, articulate yourself in the written and spoken word, use your initiative, bond with other people, and likely become a passionate advocate on issues you care about. You could become an advice worker, trading standards officer or even a coroner. Roles as barristers and solicitors are expected to grow by around 3.5% over the next eight years, so there are plenty of places your law career could take you. Criminal law, law of contract, public and European law, foundations of law and social justice, law of tort and land use and regulation are areas you could study. Lawsuits, business development, conveyancing, finance, concise writing and legal research skills and commercial awareness are hard skills you'll develop. Communications, listening skills and empathy, sales, critical thinking and attention to detail are soft skills you'll develop.</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>Essex: What is LLB Law with Human Rights? The LLB Law with Human Rights is a three-year undergraduate qualifying law degree. It combines a full legal education with a dedicated focus on human rights at domestic, European, and international levels. You’ll study the core foundations of English law alongside specialist human rights modules, graduating with in-depth knowledge of how rights are protected and applied across different legal systems. The LLB Law with Human Rights combines a qualifying law degree with specialist training in UK, European, and international human rights law. It is ideal for students who want to study law through the lens of justice, rights, and social impact. The course is shaped by internationally recognised expertise in human rights. You’ll develop strong legal reasoning, research, and analytical skills while applying law to real-world human rights issues. Your studies explore how law operates as a practical tool for protecting individuals and contributing to fairer societies. Students study core legal foundations including legal method, contract, criminal law, public law, tort, land law, and equity, while also exploring UK and European human rights law and international human rights law as dedicated areas of study. The course examines how domestic law interacts with European and international legal frameworks and develops skills in case analysis, rights-based argumentation, and legal research. Students critically evaluate law within social, political, and ethical settings. An LLB Law with Human Rights prepares graduates for careers in law and policy including roles such as solicitor, barrister, paralegal or legal adviser, as well as careers within human rights organisations, charities and advocacy groups, government and public bodies, international organisations, policy research institutes and social justice organisations, and roles in compliance, governance and corporate responsibility.
 Manchester: Law is at the heart of our society, informing and governing our everyday actions. The LLB Law course offers a distinctive approach to legal education that combines research-informed study with practice-led approaches. Students study the foundations of English and Welsh law and have the freedom to follow their own interests through a broad range of optional units while being challenged to analyse and critique the law and understand the social, economic, ethical and political contexts in which it operates. Career-focused learning is embedded throughout the course, including opportunities to apply legal theory in practice through clinical legal education at the Justice Hub, which offers free legal advice to members of the public and supports partnerships with the public, charitable and private sectors. Students develop a global perspective on law alongside essential skills, knowledge and experience for careers both within and beyond the legal profession. The programme includes engagement with areas such as family law, business law and criminal law, and introduces students to emerging fields such as LegalTech. Facilities supporting study include a moot court for simulated legal practice and access to specialist law library resources. The course provides preparation relevant to professional pathways including the Solicitors Qualifying Exam and academic requirements associated with training for the Bar. Graduates pursue careers across legal, business and public sector fields.
@@ -934,18 +1011,19 @@
           <t>LIBERAL ARTS</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
         <is>
           <t>Knowledge is rooted in the experiences of people across the world. It is created from memory, culture, landscape and myth. This knowledge is often split into separate ‘disciplines' such as those in the sciences, maths, history, geography, literature and art. However, true knowledge does not recognise these boundaries; the world is complex, interconnected and networked. Our course is for you if you love studying a variety of subjects, and want to maintain this breadth of knowledge at university. With the opportunity to major in Psychology, History, Literature, Art History, Philosophy, Politics, Media Studies or Sociology, you broaden your horizons by exploring the ways in which the humanities and social sciences help us to think imaginatively and critically about the worlds we live in. You take modules which cover the historical foundations of the humanities, challenge dominant worldviews, and explore innovative and subversive essays and manifestos. The flexible structure of this course allows you to choose a range of optional modules across literature, film, philosophy, history of art, history, linguistics, politics, sociology and modern languages. The types of issues and problems you might explore include how commercial and independent films interpret human relationships, how to compose your own writing inspired by the great essayists, important philosophical questions about life, death and religion, great works of art and literature, and languages. Based within our School of Philosophical, Historical and Interdisciplinary Studies, the choice is yours: you choose your modules based on your own background and interests. You engage with unusual, controversial and provocative ideas so that you can use the humanities and social sciences to become critically aware and possess the tools to change the world for the better. As a liberal arts graduate, you'll be provided with an all-round education that can lead to a broad range of knowledge, strong communication skills and the ability to think critically. A Liberal Arts course can lead to a wide variety of careers in fields such as media, journalism, publishing, local government, voluntary agencies, librarianship, finance and management. Our recent graduates have gone on to work for organisations including Euromoney, a financial publication company, a housing association and an English language school in Japan.</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>Liberal Arts is highly flexible, allowing students to create their own unique course, combining different subject areas within and beyond the School of Arts, Languages and Cultures. With an emphasis on interdisciplinary learning, students can tailor the course, aligning it to their interests and passions, whilst responding to key issues that affect the flourishing of free citizens. This course is ideal for individuals who have a wide range of interests and a passion for making a difference in the world. Our most distinctive research resource is internationally renowned The John Rylands Library, which holds one of the finest collections of rare books, manuscripts, and archives in the world. Manchester Museum, Whitworth Art Gallery, and Museum of Medicine and Health all feature throughout the course, and we also have strong links with the Museum of Science and Industry (MOSI). Studying with us helps you develop versatile, transferable and specialist skills, including independent working, time management and planning skills, collaboration, teamwork, leadership, communications skills to relate to a range of audiences, and an ability to develop research that responds to real-world challenges by engaging with organisations and institutions. Gain professional experience through a work placement year. Our undergraduate degrees are designed to make it easy to progress into postgraduate study if you choose. We offer a wide range of specialist master’s courses, with fast-tracked enrolment available for high-achieving undergraduate students. You can also take part in our Stellify programme, developing leadership and professional skills while contributing to your community through volunteering.</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
         <is>
           <t>Essex: Knowledge is rooted in the experiences of people across the world. It is created from memory, culture, landscape and myth. This knowledge is often split into separate ‘disciplines' such as those in the sciences, maths, history, geography, literature and art. However, true knowledge does not recognise these boundaries; the world is complex, interconnected and networked. Our course is for you if you love studying a variety of subjects, and want to maintain this breadth of knowledge at university. With the opportunity to major in Psychology, History, Literature, Art History, Philosophy, Politics, Media Studies or Sociology, you broaden your horizons by exploring the ways in which the humanities and social sciences help us to think imaginatively and critically about the worlds we live in. You take modules which cover the historical foundations of the humanities, challenge dominant worldviews, and explore innovative and subversive essays and manifestos. The flexible structure of this course allows you to choose a range of optional modules across literature, film, philosophy, history of art, history, linguistics, politics, sociology and modern languages. The types of issues and problems you might explore include how commercial and independent films interpret human relationships, how to compose your own writing inspired by the great essayists, important philosophical questions about life, death and religion, great works of art and literature, and languages. Based within our School of Philosophical, Historical and Interdisciplinary Studies, the choice is yours: you choose your modules based on your own background and interests. You engage with unusual, controversial and provocative ideas so that you can use the humanities and social sciences to become critically aware and possess the tools to change the world for the better. As a liberal arts graduate, you'll be provided with an all-round education that can lead to a broad range of knowledge, strong communication skills and the ability to think critically. A Liberal Arts course can lead to a wide variety of careers in fields such as media, journalism, publishing, local government, voluntary agencies, librarianship, finance and management. Our recent graduates have gone on to work for organisations including Euromoney, a financial publication company, a housing association and an English language school in Japan.
 Manchester: Liberal Arts is highly flexible, allowing students to create their own unique course, combining different subject areas within and beyond the School of Arts, Languages and Cultures. With an emphasis on interdisciplinary learning, students can tailor the course, aligning it to their interests and passions, whilst responding to key issues that affect the flourishing of free citizens. This course is ideal for individuals who have a wide range of interests and a passion for making a difference in the world. Our most distinctive research resource is internationally renowned The John Rylands Library, which holds one of the finest collections of rare books, manuscripts, and archives in the world. Manchester Museum, Whitworth Art Gallery, and Museum of Medicine and Health all feature throughout the course, and we also have strong links with the Museum of Science and Industry (MOSI). Studying with us helps you develop versatile, transferable and specialist skills, including independent working, time management and planning skills, collaboration, teamwork, leadership, communications skills to relate to a range of audiences, and an ability to develop research that responds to real-world challenges by engaging with organisations and institutions. Gain professional experience through a work placement year. Our undergraduate degrees are designed to make it easy to progress into postgraduate study if you choose. We offer a wide range of specialist master’s courses, with fast-tracked enrolment available for high-achieving undergraduate students. You can also take part in our Stellify programme, developing leadership and professional skills while contributing to your community through volunteering.</t>
@@ -963,20 +1041,25 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>Creative Producing; Creative Writing; Drama and Creative Writing; English Language and Literature; English Literature; Film Studies and Literature; Film and Creative Writing; History and Literature; Journalism and Literature</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
           <t>All writers are first of all readers and all readers are writers, for without the active participation of readers a book is never fully realised. Our BA Literature and Creative Writing offers a unique approach to the practice of reading and writing, combining more familiar British and American perspectives and readings with other influential schools of writing, from the study of tradition and myth to the innovative practice of the Workshop of Potential Literature or Oulipo in France. You deepen your knowledge of literary tradition across a variety of genres in order to develop your practical skills of understanding, expression and invention. Pursue your love of reading and explore some of the most important novels, poems, and plays from the United States, the Caribbean and Europe while developing your own writing through a variety of planned readings and writing exercises. We'll teach you to be your own editor; critically judging your own and others' work is invaluable in transforming your work from something good to something great. At the beginning of your course, you receive a highly focused introduction to the study of literature alongside intensive modules in creative writing, covering myth, innovation and tradition, prose, and poetry. A module on writing for radio allows you to go into a studio and record a radio play. You then progress to look at a range of specialist topics such as experimental writing and surrealism, myth and fairytale, translating novels for the screen, American literature, Shakespeare, and science fiction. Our course develops your abilities as a reader and writer while allowing you to take options from the other courses within our Department of Literature, Film, and Theatre Studies including filmmaking, journalism and drama. Essex has nurtured a long tradition of distinguished writers whose work has shaped literature as we know it today, from past giants such as the American poets Robert Lowell and Ted Berrigan, to contemporary writers such as mythographer and novelist Dame Marina Warner, and Booker Prize-winner Ben Okri. Many of our creative writing students have gone on to successfully publish their work, notable recent alumni including Ida Løkås, who won a major literary prize in Norway for The Beauty That Flows Past securing a book deal; Alexia Casale, whose novel Bone Dragon was published by Faber &amp; Faber and featured on The Financial Times Young Adult Books of the Year list and The Independent's Books of the Year list; Elaine Ewert, who placed second in the New Welsh Writing Awards; Patricia Borlenghi, founder of Patrician Press which has published works by a number of our alumni; and Petra Mcqueen, who has written for The Guardian and runs creative writing courses. Our graduates are also ideally prepared for careers in the media, education, publishing, advertising, and the film and theatre industries, with particular success in publishing and theatre.</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>BA English Literature with Creative Writing is a small, specialised creative writing pathway within an English Literature degree, in which you will take 33% of your credits in creative writing in your second and third years. The course covers the full range of English literature from Old English to the present day. The creative writing component of the course focuses on fiction and poetry writing. The course will introduce you to techniques of fiction and poetry writing, and develop your understanding of the craft of writing, the nature and necessity of revision, and the importance of being able to give and receive constructive feedback. The creative writing component of the degree will be taught in small group workshops. You will write your own poems and stories regularly, read relevant work from established writers, and respond to examples of contemporary poetry and fiction. There will be in-class writing exercises and an introduction to workshopping. You will become part of a thriving community of students, lecturers, and writers at The University of Manchester, based in the heart of a UNESCO City of Literature that has produced some of the world's greatest writers and has a thriving literature and arts scene, including major events like Manchester Literature Festival. Apply your subject-specific knowledge in a real-world context through a placement year in your third year of study. You can apply to spend one semester studying abroad during the second year of your degree. Exchange partners are offered in Europe, USA, Canada, Australia, New Zealand, Hong Kong, and Singapore. Manchester Literature Festival holds literary events across Manchester throughout the year, many in partnership with the University. The Centre for New Writing also hosts a regular public event series, Literature Live, which brings contemporary novelists and poets to the University to read and engage in conversation. The John Rylands Library is home to one of the world's richest and most unique collections of manuscripts, maps, works of art, and objects. The University is home to the Centre for New Writing, a major hub for new writing excellence and award-winning teaching staff. The University of Manchester Library is one of only five National Research Libraries and provides access to internationally renowned archival collections. Students also have access to cultural assets including the Whitworth Art Gallery and Manchester Museum. All courses are designed to equip students with strong critical analysis skills, the ability to articulate knowledge of concepts and theories, and the ability to work and think independently, critically and creatively. Students have access to dedicated, subject-specific careers support throughout their studies and for up to two years after graduation. Undergraduate courses are designed to provide an easy transition into postgraduate study. Students can take part in the Stellify programme alongside their degrees, developing professional and leadership skills while contributing to their communities through volunteering. Graduates have gone on to work in a variety of industries including positions with the BBC, KPMG, Deloitte, Marks and Spencer, Aviva, Accenture and Barclays.</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>We’re all natural storytellers, and studying English literature and creative writing offers a way into the human imagination and the key to creative expression. Studying English literature and creative writing engrosses you in literary masterpieces and builds essential skills that are sought after in the professional world. It encourages critical thinking, analytical skills, and effective communication, creating storytellers and perceptive interpreters of cultural differences. The comprehensive understanding of language, narrative structures, and different genres equips graduates for a variety of career paths. Whether looking at roles in publishing, journalism, content creation, marketing, or education, graduates will have the ability to craft compelling narratives and adapt to different communication styles. Beyond traditional careers, the creative and analytical skills gained prepare you for roles in digital media, advertising, and even entrepreneurship, where the power of persuasive storytelling is essential. Literature in theory, modern world literatures, creative thinking, Shakespeare, American poetry, modes of reading and contemporary fiction are areas you could study. Ability to critically analyse and interpret literary texts, close reading skills, development of characters, plot structures and dialogue, and analyse arguments and evaluate evidence are hard skills you'll develop. Creativity, critical thinking, written communication and storytelling are soft skills you'll develop. Career options include journalist, newspaper and periodical editors, authors, writers and translators, web content professionals, advertising account managers, public relations professionals, customer service managers and supervisors, human resources and industrial relations officers, business and related research professionals, and research and development managers.</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>Essex: All writers are first of all readers and all readers are writers, for without the active participation of readers a book is never fully realised. Our BA Literature and Creative Writing offers a unique approach to the practice of reading and writing, combining more familiar British and American perspectives and readings with other influential schools of writing, from the study of tradition and myth to the innovative practice of the Workshop of Potential Literature or Oulipo in France. You deepen your knowledge of literary tradition across a variety of genres in order to develop your practical skills of understanding, expression and invention. Pursue your love of reading and explore some of the most important novels, poems, and plays from the United States, the Caribbean and Europe while developing your own writing through a variety of planned readings and writing exercises. We'll teach you to be your own editor; critically judging your own and others' work is invaluable in transforming your work from something good to something great. At the beginning of your course, you receive a highly focused introduction to the study of literature alongside intensive modules in creative writing, covering myth, innovation and tradition, prose, and poetry. A module on writing for radio allows you to go into a studio and record a radio play. You then progress to look at a range of specialist topics such as experimental writing and surrealism, myth and fairytale, translating novels for the screen, American literature, Shakespeare, and science fiction. Our course develops your abilities as a reader and writer while allowing you to take options from the other courses within our Department of Literature, Film, and Theatre Studies including filmmaking, journalism and drama. Essex has nurtured a long tradition of distinguished writers whose work has shaped literature as we know it today, from past giants such as the American poets Robert Lowell and Ted Berrigan, to contemporary writers such as mythographer and novelist Dame Marina Warner, and Booker Prize-winner Ben Okri. Many of our creative writing students have gone on to successfully publish their work, notable recent alumni including Ida Løkås, who won a major literary prize in Norway for The Beauty That Flows Past securing a book deal; Alexia Casale, whose novel Bone Dragon was published by Faber &amp; Faber and featured on The Financial Times Young Adult Books of the Year list and The Independent's Books of the Year list; Elaine Ewert, who placed second in the New Welsh Writing Awards; Patricia Borlenghi, founder of Patrician Press which has published works by a number of our alumni; and Petra Mcqueen, who has written for The Guardian and runs creative writing courses. Our graduates are also ideally prepared for careers in the media, education, publishing, advertising, and the film and theatre industries, with particular success in publishing and theatre.
 Manchester: BA English Literature with Creative Writing is a small, specialised creative writing pathway within an English Literature degree, in which you will take 33% of your credits in creative writing in your second and third years. The course covers the full range of English literature from Old English to the present day. The creative writing component of the course focuses on fiction and poetry writing. The course will introduce you to techniques of fiction and poetry writing, and develop your understanding of the craft of writing, the nature and necessity of revision, and the importance of being able to give and receive constructive feedback. The creative writing component of the degree will be taught in small group workshops. You will write your own poems and stories regularly, read relevant work from established writers, and respond to examples of contemporary poetry and fiction. There will be in-class writing exercises and an introduction to workshopping. You will become part of a thriving community of students, lecturers, and writers at The University of Manchester, based in the heart of a UNESCO City of Literature that has produced some of the world's greatest writers and has a thriving literature and arts scene, including major events like Manchester Literature Festival. Apply your subject-specific knowledge in a real-world context through a placement year in your third year of study. You can apply to spend one semester studying abroad during the second year of your degree. Exchange partners are offered in Europe, USA, Canada, Australia, New Zealand, Hong Kong, and Singapore. Manchester Literature Festival holds literary events across Manchester throughout the year, many in partnership with the University. The Centre for New Writing also hosts a regular public event series, Literature Live, which brings contemporary novelists and poets to the University to read and engage in conversation. The John Rylands Library is home to one of the world's richest and most unique collections of manuscripts, maps, works of art, and objects. The University is home to the Centre for New Writing, a major hub for new writing excellence and award-winning teaching staff. The University of Manchester Library is one of only five National Research Libraries and provides access to internationally renowned archival collections. Students also have access to cultural assets including the Whitworth Art Gallery and Manchester Museum. All courses are designed to equip students with strong critical analysis skills, the ability to articulate knowledge of concepts and theories, and the ability to work and think independently, critically and creatively. Students have access to dedicated, subject-specific careers support throughout their studies and for up to two years after graduation. Undergraduate courses are designed to provide an easy transition into postgraduate study. Students can take part in the Stellify programme alongside their degrees, developing professional and leadership skills while contributing to their communities through volunteering. Graduates have gone on to work in a variety of industries including positions with the BBC, KPMG, Deloitte, Marks and Spencer, Aviva, Accenture and Barclays.
@@ -995,20 +1078,25 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
+          <t>Economics and Mathematics; Mathematics and Data Science; Mathematics with Computing; Mathematics with Physics</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
           <t>Mathematics provides the logical foundations on which all of science, engineering and technology are built. Our BSc (Hons) Mathematics course gives you the chance to study both fundamental topics and their modern applications, including pure mathematics such as geometry, algebra, analysis and number theory, applied topics such as mathematical physics, cryptography, mathematical modelling, differential equations and dynamical systems, and statistical, financial and analytical methods such as optimisation and the study of risk. As well as these mathematical topics, your degree will develop your programming skills in languages such as Python and SQL, and you will learn to solve sophisticated problems using computational toolkits such as MATLAB, Maple and R. Our School of Mathematics, Statistics and Actuarial Science recognises the stand-alone and interdisciplinary aspects of mathematics, and this degree provides an exceptional range of in-demand transferrable skills for mathematically oriented careers from business, finance and commerce to industry, research, government and education. All our mathematical sciences degrees feature an employability component in every year of study, explicitly training sought-after skills and incorporating careers day events and seminars from speakers in industry. This programme will meet the educational requirements of the Chartered Mathematician designation, awarded by the Institute of Mathematics and its Applications, when it is followed by subsequent training and experience in employment to obtain equivalent competences to those specified by the Quality Assurance Agency (QAA) for taught masters degrees. Clear thinkers are required in every profession, so the successful mathematician has an extensive choice of potential careers. Mathematics students are in demand from a wide range of employers in a host of occupations, including financial analysis, management, public administration and accountancy. Our recent graduates have gone on to work for a wide range of high-profile companies, including KPMG, British Arab Commercial Bank and Johal and Company.</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>Lay the foundations of a rewarding career with mathematics at its base by undertaking an undergraduate degree at Manchester. We offer a highly flexible degree programme, ensuring you obtain a strong all-round mathematical knowledge while encouraging you to focus on the areas that appeal most. You will cover core topics in the first year, developing your capacity to learn and apply mathematical ideas. In the second year you choose two from three themes: Pure Mathematics, Applied Mathematics, and Probability and Statistics, along with optional units such as Programming with Python. After the first two years you can choose the areas that interest you most and select options from other subject areas. In your final year you can undertake a staff-supervised mathematical project. You will develop a firm all-round mathematical knowledge and experience specialised results, methods and ideas. You can pursue whichever areas of mathematics interest you most and choose lecture courses from a widening range of options. Our flexible degree programme allows students to choose courses from other disciplines and a wide range of mathematics options. Small-group teaching in the first year supports student learning. Students may undertake a year on a work-based placement to gain professional experience. The Department of Mathematics is based in the Alan Turing Building. Facilities include computer clusters with mathematical and statistical software including Matlab and Mathematica. Studying mathematics develops skills and knowledge valued across professions including finance, industry, computing, management, statistics and teaching. Graduates have pursued careers in finance in firms such as KPMG, Goldman Sachs, PricewaterhouseCoopers, Deloitte, Barclays and Deutsche Bank. Many graduates undertake further programmes of study such as MSc degrees in Mathematics, Applied Mathematics, Finance, Business, Management and Computer Science.</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>Use logic and reason to analyse data and provide solutions in a wide range of employment sectors. As a mathematician or statistician you’ll use your problem-solving, analytical, and technical skills to help businesses in a range of sectors, from finance to government. Your interpretations could be used in anything from clinical trials, to climate predictions, to financial forecasting. You could end up in a management role, leading a team, or become self-employed as a consultant or financial adviser. You could also go on to further study, teaching or academic research, or work as a data scientist. Pure mathematics, applied mathematics, real analysis, statistics, mathematical modelling, probability and data science, differential equations, dynamics and motion, Bayesian statistics, medical statistics, stochastic modelling, scientistic computing and machine learning are areas you could study. Economics and finance, programming languages, project management, data analysis and statistics are hard skills you'll develop. Communication, management, research, planning and innovation are soft skills you'll develop. Career options include chartered accountant, bank clerk, investment analyst, insurance underwriter, actuary, financial manager, IT manager, software developers and programmers, quantity surveyor, research manager and teacher in further or higher education.</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>Essex: Mathematics provides the logical foundations on which all of science, engineering and technology are built. Our BSc (Hons) Mathematics course gives you the chance to study both fundamental topics and their modern applications, including pure mathematics such as geometry, algebra, analysis and number theory, applied topics such as mathematical physics, cryptography, mathematical modelling, differential equations and dynamical systems, and statistical, financial and analytical methods such as optimisation and the study of risk. As well as these mathematical topics, your degree will develop your programming skills in languages such as Python and SQL, and you will learn to solve sophisticated problems using computational toolkits such as MATLAB, Maple and R. Our School of Mathematics, Statistics and Actuarial Science recognises the stand-alone and interdisciplinary aspects of mathematics, and this degree provides an exceptional range of in-demand transferrable skills for mathematically oriented careers from business, finance and commerce to industry, research, government and education. All our mathematical sciences degrees feature an employability component in every year of study, explicitly training sought-after skills and incorporating careers day events and seminars from speakers in industry. This programme will meet the educational requirements of the Chartered Mathematician designation, awarded by the Institute of Mathematics and its Applications, when it is followed by subsequent training and experience in employment to obtain equivalent competences to those specified by the Quality Assurance Agency (QAA) for taught masters degrees. Clear thinkers are required in every profession, so the successful mathematician has an extensive choice of potential careers. Mathematics students are in demand from a wide range of employers in a host of occupations, including financial analysis, management, public administration and accountancy. Our recent graduates have gone on to work for a wide range of high-profile companies, including KPMG, British Arab Commercial Bank and Johal and Company.
 Manchester: Lay the foundations of a rewarding career with mathematics at its base by undertaking an undergraduate degree at Manchester. We offer a highly flexible degree programme, ensuring you obtain a strong all-round mathematical knowledge while encouraging you to focus on the areas that appeal most. You will cover core topics in the first year, developing your capacity to learn and apply mathematical ideas. In the second year you choose two from three themes: Pure Mathematics, Applied Mathematics, and Probability and Statistics, along with optional units such as Programming with Python. After the first two years you can choose the areas that interest you most and select options from other subject areas. In your final year you can undertake a staff-supervised mathematical project. You will develop a firm all-round mathematical knowledge and experience specialised results, methods and ideas. You can pursue whichever areas of mathematics interest you most and choose lecture courses from a widening range of options. Our flexible degree programme allows students to choose courses from other disciplines and a wide range of mathematics options. Small-group teaching in the first year supports student learning. Students may undertake a year on a work-based placement to gain professional experience. The Department of Mathematics is based in the Alan Turing Building. Facilities include computer clusters with mathematical and statistical software including Matlab and Mathematica. Studying mathematics develops skills and knowledge valued across professions including finance, industry, computing, management, statistics and teaching. Graduates have pursued careers in finance in firms such as KPMG, Goldman Sachs, PricewaterhouseCoopers, Deloitte, Barclays and Deutsche Bank. Many graduates undertake further programmes of study such as MSc degrees in Mathematics, Applied Mathematics, Finance, Business, Management and Computer Science.
@@ -1027,16 +1115,21 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
+          <t>Business Management with a Modern Language; Global Studies and Modern Languages; Journalism and Modern Languages; Modern History; Modern History and International Relations; Modern History and Politics; Modern Languages and Linguistics; Modern Languages with Latin American Studies; Spanish Studies and Modern Languages</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
           <t>Language is fundamental to our thought, our relationships, and our civilisations. Through language we transmit knowledge, from inviting someone for coffee, to promoting the latest scientific theory, to settling global political disputes. On our course you can study up to three languages choosing between French, German, Italian and Spanish from beginner or post-A level standard. Portuguese can be studied from a pre-A level standard. These languages can be studied alongside language expert modules which cover a range of cultural and professional skills. Each of these languages are widely used in the business world, and we take you to a level of near-fluency; so many of our graduates have gone on to develop successful global careers with international firms looking for language specialists. In addition to the language skills you develop on our course, you also explore a range of modules on global cultures, histories and politics so that you can really understand another country beyond just being able to communicate in the native language. Study topics include world cinema, translation, interpreting and subtitling, popular music, and visual history. If you want a global outlook, are interested in human communication, and want to study for a degree with real-world practical value in a world-class department, welcome to Essex. Companies and organisations in the UK and abroad are struggling to find university graduates who are fluent in at least one other language apart from English. Being an Essex modern languages graduate places you in a very advantageous position. You will be able to speak and write fluently, or to a very competent standard, in up to four languages. Language skills are in scarce supply and can be used in almost any job. Our graduates become teachers, translators, administrators and journalists, and their language skills have enabled them to work in fields including banking, entertainment, media, education and tourism, as well as for a host of UK and international companies. A degree in modern languages lends itself to careers in education, translation, interpretation, trade, public relations, communications, immigration or diplomacy. For example, one of our recent graduates is now a newspaper editor in Spain, while another teaches modern languages in Southampton.</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr">
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
         <is>
           <t>Studying languages not only unlocks global cultures but also transforms you into a versatile communicator, making you a valuable asset for many industries. When you choose languages, you’re opening a world of opportunities for career growth because knowing multiple languages makes you a valuable asset in our interconnected global landscape. Being multilingual puts you in high demand across various industries, from international business and diplomacy to translation, journalism, and tourism. Your ability to bridge communication gaps opens conversation for cross-cultural understanding, making you indispensable in an increasingly interconnected and multicultural world. Linguistics, translation and interpreting, written and oral grammar, science of language and communication, history of language, literature and culture, history and politics are areas you could study. Fluency in another language, ability to translate and interpret, understanding of different grammatical structures and knowledge of cultural traditions and customs are hard skills you'll develop. Cultural sensitivity, communication skills, curiosity and tolerance for ambiguity and uncertainty are soft skills you'll develop. Career options include translators, journalists, public relations professionals, hotel and accommodation managers and travel agency managers.</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>Essex: Language is fundamental to our thought, our relationships, and our civilisations. Through language we transmit knowledge, from inviting someone for coffee, to promoting the latest scientific theory, to settling global political disputes. On our course you can study up to three languages choosing between French, German, Italian and Spanish from beginner or post-A level standard. Portuguese can be studied from a pre-A level standard. These languages can be studied alongside language expert modules which cover a range of cultural and professional skills. Each of these languages are widely used in the business world, and we take you to a level of near-fluency; so many of our graduates have gone on to develop successful global careers with international firms looking for language specialists. In addition to the language skills you develop on our course, you also explore a range of modules on global cultures, histories and politics so that you can really understand another country beyond just being able to communicate in the native language. Study topics include world cinema, translation, interpreting and subtitling, popular music, and visual history. If you want a global outlook, are interested in human communication, and want to study for a degree with real-world practical value in a world-class department, welcome to Essex. Companies and organisations in the UK and abroad are struggling to find university graduates who are fluent in at least one other language apart from English. Being an Essex modern languages graduate places you in a very advantageous position. You will be able to speak and write fluently, or to a very competent standard, in up to four languages. Language skills are in scarce supply and can be used in almost any job. Our graduates become teachers, translators, administrators and journalists, and their language skills have enabled them to work in fields including banking, entertainment, media, education and tourism, as well as for a host of UK and international companies. A degree in modern languages lends itself to careers in education, translation, interpretation, trade, public relations, communications, immigration or diplomacy. For example, one of our recent graduates is now a newspaper editor in Spain, while another teaches modern languages in Southampton.
 UCAS: Studying languages not only unlocks global cultures but also transforms you into a versatile communicator, making you a valuable asset for many industries. When you choose languages, you’re opening a world of opportunities for career growth because knowing multiple languages makes you a valuable asset in our interconnected global landscape. Being multilingual puts you in high demand across various industries, from international business and diplomacy to translation, journalism, and tourism. Your ability to bridge communication gaps opens conversation for cross-cultural understanding, making you indispensable in an increasingly interconnected and multicultural world. Linguistics, translation and interpreting, written and oral grammar, science of language and communication, history of language, literature and culture, history and politics are areas you could study. Fluency in another language, ability to translate and interpret, understanding of different grammatical structures and knowledge of cultural traditions and customs are hard skills you'll develop. Cultural sensitivity, communication skills, curiosity and tolerance for ambiguity and uncertainty are soft skills you'll develop. Career options include translators, journalists, public relations professionals, hotel and accommodation managers and travel agency managers.</t>
@@ -1054,20 +1147,25 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
+          <t>Continental Philosophy; Law with Philosophy; Philosophy and Politics; Philosophy with Business Management; Philosophy, Politics and Economics</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
           <t>Our BA Philosophy will feed your intellectual curiosity and challenge your thinking. You'll acquire the skills required to dig deeper into ideas and question received wisdom. You'll rigorously examine the most fundamental questions about human life: Does God exist? Is material success all that counts in life? What do I owe to others? How free am I to decide my own future? At Essex, we take philosophy back to its roots in everyday existential, social, and political problems. We embrace the relevance of philosophy to other forms of enquiry – political, cultural, legal, medical and aesthetic – and bring this to bear on urgent issues in public life, such as the controversial issues raised by mental health legislation or public policy regarding end of life care. We cover a wide range of topics from the meaning of life to capitalism and its critics, from ancient philosophy to current trends in European thought, with particular strengths in ethics, political philosophy, philosophy of religion, and European philosophy including critical theory, phenomenology and existentialism. A degree in Philosophy at Essex provides you with the ability to analyse and solve difficult problems, the ability to think clearly, creatively and self-critically, and the ability to work in a team taking a collaborative approach to problems. Philosophy graduates are therefore well-suited to a wide range of occupations including law, PR, journalism and the media, the Civil Service, charity work, banking and the NHS.</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Studying BA Philosophy enables you to critically analyse answers to fundamental questions such as free will, ethics and the nature of reality. Students debate questions such as whether the world outside our minds exists, what makes something morally right, whether humans have free will, whether God exists and whether the human mind is purely physical. Students develop skills including presenting effective and rigorous arguments, developing criticisms of other people’s arguments and views, explaining complex material clearly and concisely, and analysing philosophical problems where reasonable people hold different views. Provide structured yet flexible study informed by current research. Provide a curriculum covering texts and questions central to the analytical tradition in philosophy and traditions outside it. Develop subject-specific knowledge, cognitive skills and transferable skills for employment or further academic study. Students may apply to study abroad for a year at partner universities. Students may apply for a paid Q-Step internship between Years 2 and 3. Students may undertake a Professional Experience Year, extending the degree to four years. Philosophy graduates pursue careers in journalism, media, charities, consultancy, civil service, finance, marketing, public relations, social work, teaching and law. Recent graduates have worked for organisations including Manchester City Council, Royal Bank of Scotland, Palgrave MacMillan, Lloyds TSB, the Foreign and Commonwealth Office, TeachFirst and Siemens. Many graduates undertake postgraduate study in philosophy, teaching, law, political theory, business or marketing.</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>Choose philosophy for a rigorous exploration into questioning, analysis, and the development of sharp, independent thinking skills that navigate the complexities of our world. Philosophy navigates human thought, offering an understanding of fundamental questions about existence, morality, and knowledge. Beyond fostering critical thinking and intellectual curiosity, a degree in philosophy cultivates skills highly sought after in lots of professions. Graduates often find themselves in careers such as law, journalism, education, business, and public policy. The ability to analyse complex issues, articulate compelling arguments, and engage in interesting discussions help philosophers to thrive in roles that demand clarity of thought and effective communication. The adaptability and broad perspective gained through philosophical studies set people up for success in a rapidly evolving job market, making philosophy not just a field of study, but a foundation for a choice of careers. Symbolic logic, reason, argument, and analysis, history of philosophy, Sartre and existentialism, metaphysics, social and political theory and engaging with the humanities are areas you could study. Analytical reasoning skills, accessing and evaluating academic sources, historical understanding and precision and attention to detail are hard skills you'll develop. Communication skills, both written and verbal, open mindedness, cultural awareness and flexibility in thinking are soft skills you'll develop. Career options include solicitors and lawyers, legal associate professionals, journalists, newspaper and periodical editors.</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>Essex: Our BA Philosophy will feed your intellectual curiosity and challenge your thinking. You'll acquire the skills required to dig deeper into ideas and question received wisdom. You'll rigorously examine the most fundamental questions about human life: Does God exist? Is material success all that counts in life? What do I owe to others? How free am I to decide my own future? At Essex, we take philosophy back to its roots in everyday existential, social, and political problems. We embrace the relevance of philosophy to other forms of enquiry – political, cultural, legal, medical and aesthetic – and bring this to bear on urgent issues in public life, such as the controversial issues raised by mental health legislation or public policy regarding end of life care. We cover a wide range of topics from the meaning of life to capitalism and its critics, from ancient philosophy to current trends in European thought, with particular strengths in ethics, political philosophy, philosophy of religion, and European philosophy including critical theory, phenomenology and existentialism. A degree in Philosophy at Essex provides you with the ability to analyse and solve difficult problems, the ability to think clearly, creatively and self-critically, and the ability to work in a team taking a collaborative approach to problems. Philosophy graduates are therefore well-suited to a wide range of occupations including law, PR, journalism and the media, the Civil Service, charity work, banking and the NHS.
 Manchester: Studying BA Philosophy enables you to critically analyse answers to fundamental questions such as free will, ethics and the nature of reality. Students debate questions such as whether the world outside our minds exists, what makes something morally right, whether humans have free will, whether God exists and whether the human mind is purely physical. Students develop skills including presenting effective and rigorous arguments, developing criticisms of other people’s arguments and views, explaining complex material clearly and concisely, and analysing philosophical problems where reasonable people hold different views. Provide structured yet flexible study informed by current research. Provide a curriculum covering texts and questions central to the analytical tradition in philosophy and traditions outside it. Develop subject-specific knowledge, cognitive skills and transferable skills for employment or further academic study. Students may apply to study abroad for a year at partner universities. Students may apply for a paid Q-Step internship between Years 2 and 3. Students may undertake a Professional Experience Year, extending the degree to four years. Philosophy graduates pursue careers in journalism, media, charities, consultancy, civil service, finance, marketing, public relations, social work, teaching and law. Recent graduates have worked for organisations including Manchester City Council, Royal Bank of Scotland, Palgrave MacMillan, Lloyds TSB, the Foreign and Commonwealth Office, TeachFirst and Siemens. Many graduates undertake postgraduate study in philosophy, teaching, law, political theory, business or marketing.
@@ -1086,16 +1184,21 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
+          <t>Economics and Politics; Global Politics; Journalism and Politics; Law with Politics; Modern History and Politics; Philosophy and Politics; Philosophy, Politics and Economics; Politics and International Relations; Politics with Business</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
           <t>What is the BA Politics? The BA Politics is a three-year degree. You’ll examine the structures, ideas, and decisions that shape societies, from political institutions and democratic processes to power, rights, and governance. Combining critical theory, case studies, and applied analysis, you’ll develop the insight and practical skills needed to interpret complex political issues, policy debates, and real-world political decision-making. The BA Politics degree trains you to go beyond opinion and ask the crucial question: how do you know? This makes the course particularly well suited to students who enjoy evidence, debate, and complexity rather than simple answers. You’ll tackle power, justice, democracy, and rights, while addressing real-world challenges like conflict, authoritarianism, and human rights. Learn from leading academics in a department whose research informs government policy, international organisations, and public debate. You’ll see first-hand how theory informs real-world decisions and develop practical skills in analysis, argumentation, and decision-making. Personalise your degree with a specialist module pathway, gaining expertise in a particular area of politics that strengthens your CV, postgraduate applications, and demonstrates your command of the field. This course will teach you how to analyse political systems, assess policy decisions, and apply theory to real-world governance challenges. You’ll develop the confidence and skills to think critically, argue persuasively, and make informed decisions, valuable skills for a wide range of early careers or further postgraduate study. The course covers areas including political systems and theory, examining how states, laws, wars, parties and institutions shape obligations, freedom, rights and equality; democracy and power, exploring why people engage or disengage with politics and how voting, participation and influence operate in practice; global politics, examining international relations, conflict and authoritarianism and how national and global forces intersect; applied analysis, connecting political science theory to real-world policy, governance and decision-making challenges; and research methods, developing rigorous quantitative and qualitative skills with the option to enhance expertise through advanced data analysis. Students can develop additional expertise through named specialisms such as Data Science (Q-Step Pathway), which provides advanced quantitative and data analysis skills alongside political study; Justice and Human Rights, focusing on justice, rights and accountability across domestic and international contexts; and Political Economy and Development, examining how political power, economic systems and inequality shape development at local, national and global levels. A BA Politics degree prepares graduates for careers in areas such as government and public service including policy advisors, civil servants, legislative assistants and political analysts; international organisations and diplomacy including the UN, EU, NATO, Commonwealth and development agencies; non-governmental and advocacy sectors such as human rights organisations and development charities; media and communications including political journalism and public affairs; consultancy and think tanks including political risk analysis and policy consultancy; and research or postgraduate study in politics, international relations or public policy. Graduates from this course have progressed to roles in organisations including the House of Commons, Essex Police Force, Essex County Council, London Borough of Lewisham and Sky News.</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr">
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
         <is>
           <t>Understand and address the key issues facing our country, and the wider world. Politics allows us to understand how governments, policies, and international relations work. Many important questions or global challenges, like human rights issues, poverty, equality, and welfare, can be addressed through an understanding of this topic. A degree in politics can lead to a career in many different sectors. If you become an MP, you could represent your constituents, and progress to party whip or leader, a committee chair, cabinet minister, or even prime minister. Or you could work in business, diplomacy, the civil service or human resources, among other things. Understanding politics, introduction to political theory, understanding international relations, global history, pathways to political research, political and economic data analysis and emerging powers in a changing world are areas you could study. Negotiation, effective debating and data analysis are hard skills you'll develop. Written and verbal communication, empathy, listening skills, leadership and logic and reasoning are soft skills you'll develop. Career options include politician, local government officer, public relations professional, journalist, human resources roles, finance roles and public services roles.</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>Essex: What is the BA Politics? The BA Politics is a three-year degree. You’ll examine the structures, ideas, and decisions that shape societies, from political institutions and democratic processes to power, rights, and governance. Combining critical theory, case studies, and applied analysis, you’ll develop the insight and practical skills needed to interpret complex political issues, policy debates, and real-world political decision-making. The BA Politics degree trains you to go beyond opinion and ask the crucial question: how do you know? This makes the course particularly well suited to students who enjoy evidence, debate, and complexity rather than simple answers. You’ll tackle power, justice, democracy, and rights, while addressing real-world challenges like conflict, authoritarianism, and human rights. Learn from leading academics in a department whose research informs government policy, international organisations, and public debate. You’ll see first-hand how theory informs real-world decisions and develop practical skills in analysis, argumentation, and decision-making. Personalise your degree with a specialist module pathway, gaining expertise in a particular area of politics that strengthens your CV, postgraduate applications, and demonstrates your command of the field. This course will teach you how to analyse political systems, assess policy decisions, and apply theory to real-world governance challenges. You’ll develop the confidence and skills to think critically, argue persuasively, and make informed decisions, valuable skills for a wide range of early careers or further postgraduate study. The course covers areas including political systems and theory, examining how states, laws, wars, parties and institutions shape obligations, freedom, rights and equality; democracy and power, exploring why people engage or disengage with politics and how voting, participation and influence operate in practice; global politics, examining international relations, conflict and authoritarianism and how national and global forces intersect; applied analysis, connecting political science theory to real-world policy, governance and decision-making challenges; and research methods, developing rigorous quantitative and qualitative skills with the option to enhance expertise through advanced data analysis. Students can develop additional expertise through named specialisms such as Data Science (Q-Step Pathway), which provides advanced quantitative and data analysis skills alongside political study; Justice and Human Rights, focusing on justice, rights and accountability across domestic and international contexts; and Political Economy and Development, examining how political power, economic systems and inequality shape development at local, national and global levels. A BA Politics degree prepares graduates for careers in areas such as government and public service including policy advisors, civil servants, legislative assistants and political analysts; international organisations and diplomacy including the UN, EU, NATO, Commonwealth and development agencies; non-governmental and advocacy sectors such as human rights organisations and development charities; media and communications including political journalism and public affairs; consultancy and think tanks including political risk analysis and policy consultancy; and research or postgraduate study in politics, international relations or public policy. Graduates from this course have progressed to roles in organisations including the House of Commons, Essex Police Force, Essex County Council, London Borough of Lewisham and Sky News.
 UCAS: Understand and address the key issues facing our country, and the wider world. Politics allows us to understand how governments, policies, and international relations work. Many important questions or global challenges, like human rights issues, poverty, equality, and welfare, can be addressed through an understanding of this topic. A degree in politics can lead to a career in many different sectors. If you become an MP, you could represent your constituents, and progress to party whip or leader, a committee chair, cabinet minister, or even prime minister. Or you could work in business, diplomacy, the civil service or human resources, among other things. Understanding politics, introduction to political theory, understanding international relations, global history, pathways to political research, political and economic data analysis and emerging powers in a changing world are areas you could study. Negotiation, effective debating and data analysis are hard skills you'll develop. Written and verbal communication, empathy, listening skills, leadership and logic and reasoning are soft skills you'll develop. Career options include politician, local government officer, public relations professional, journalist, human resources roles, finance roles and public services roles.</t>
@@ -1113,20 +1216,25 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
+          <t>Criminology with Social Psychology; Neural Engineering with Psychology; Psychology with Cognitive Neuroscience; Psychology with Economics; Psychology with Sport and Exercise; Sociology with Social Psychology</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
           <t>The BA (Hons) Psychology is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll gain a strong understanding of the theories and approaches in psychology today, preparing you to answer the world’s current challenges. The BA (Hons) Psychology gives you one of the most immersive and exciting experiences of studying human thoughts and behaviours in the UK. Your learning, like our research, focuses on innovative solutions to real societal challenges so you’ll develop the skills and knowledge to make a measurable difference in our world. Gain work experience alongside your studies by working one-on-one as a psychologist’s research assistant, undertaking an internship alongside health and wellbeing practitioners and supporting psychology outreach. You’ll graduate on the path to a psychologist or researcher career, with the foundations needed to specialise in areas such as clinical and educational psychology. The course explores different approaches to psychology including cognitive, developmental and social psychology, and allows you to tailor your degree through your choice of applied modules. A BA (Hons) Psychology degree prepares you for diverse careers including counselling and coaching, civil service roles such as policy development and social work, education including teaching and special education needs, business and finance roles such as market research and human resources, and psychology research. The course is accredited against the requirements for the Graduate Basis for Chartered Membership (GBC) of the British Psychological Society (BPS). This accreditation signifies that you have obtained a high standard of psychology education and is a crucial step for several career paths including becoming a chartered psychologist, ensuring the curriculum covers the knowledge and skills required for professional practice.</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>The BSc Psychology degree is accredited by the British Psychological Society. The course consists of compulsory and optional units within and outside psychology. In the first two years students study biological psychology, cognitive psychology, developmental psychology, individual differences, social psychology, research methods and conceptual and historical issues in psychology. Teaching includes lectures, tutorials, practical classes, laboratory sessions and seminars. Students complete semester-long laboratory units in Years 1 and 2 to develop skills in designing, conducting and analysing research. In the final year students undertake an independent research project. Students complete a 30-hour placement in Year 2 and may undertake a full-year placement between Years 2 and 3 or study abroad at partner universities. A BPS-accredited psychology degree provides the first step towards careers such as clinical psychology, counselling psychology, health psychology, forensic psychology, organisational psychology, educational psychology and sports psychology. Graduates also work in careers including marketing, advertising, journalism, human resources, management consulting, academic research, teaching, policing, mental health services, counselling and social work. The course confers eligibility for Graduate Membership of the British Psychological Society and the Graduate Basis for Registration.</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>Psychology is a fascinating journey into understanding and decoding the human mind, offering valuable insights into behaviour, emotions, and the science behind why we do what we do. Psychology delves into the complexities of the human mind, examining behaviour, cognition, and emotions. Studying psychology opens doors to many different career opportunities. From clinical psychologists providing therapeutic support, to industrial-organisational psychologists shaping workplace dynamics, this subject offers the chance for understanding and improving all kinds of aspects of human life. Psychology is also transferable to other exciting careers such as marketing, human resources, and healthcare, making it a versatile foundation for personal and professional growth. Whether you choose to pursue counselling, research, or organisational development, a background in psychology gives you valuable insights into human behaviour and the skills to make a positive impact on both individuals and communities. Applied psychology, child psychology, clinical psychology, educational psychology, forensic psychology, sport psychology and experimental psychology are areas you could study. Enhanced research skills, data and statistical analysis, application of therapeutic techniques and evaluation of cognitive functions are hard skills you'll develop. Attentive and active listening, empathising with others, ability to adapt to new information and critical thinking and problem-solving skills are soft skills you'll develop. Career options include clinical psychologists, other psychologists, health professionals, occupational therapists, therapy professionals, business and related research professionals, market research interviewers, human resources and industrial relations officers, and human resource managers and directors.</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>Essex: The BA (Hons) Psychology is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll gain a strong understanding of the theories and approaches in psychology today, preparing you to answer the world’s current challenges. The BA (Hons) Psychology gives you one of the most immersive and exciting experiences of studying human thoughts and behaviours in the UK. Your learning, like our research, focuses on innovative solutions to real societal challenges so you’ll develop the skills and knowledge to make a measurable difference in our world. Gain work experience alongside your studies by working one-on-one as a psychologist’s research assistant, undertaking an internship alongside health and wellbeing practitioners and supporting psychology outreach. You’ll graduate on the path to a psychologist or researcher career, with the foundations needed to specialise in areas such as clinical and educational psychology. The course explores different approaches to psychology including cognitive, developmental and social psychology, and allows you to tailor your degree through your choice of applied modules. A BA (Hons) Psychology degree prepares you for diverse careers including counselling and coaching, civil service roles such as policy development and social work, education including teaching and special education needs, business and finance roles such as market research and human resources, and psychology research. The course is accredited against the requirements for the Graduate Basis for Chartered Membership (GBC) of the British Psychological Society (BPS). This accreditation signifies that you have obtained a high standard of psychology education and is a crucial step for several career paths including becoming a chartered psychologist, ensuring the curriculum covers the knowledge and skills required for professional practice.
 Manchester: The BSc Psychology degree is accredited by the British Psychological Society. The course consists of compulsory and optional units within and outside psychology. In the first two years students study biological psychology, cognitive psychology, developmental psychology, individual differences, social psychology, research methods and conceptual and historical issues in psychology. Teaching includes lectures, tutorials, practical classes, laboratory sessions and seminars. Students complete semester-long laboratory units in Years 1 and 2 to develop skills in designing, conducting and analysing research. In the final year students undertake an independent research project. Students complete a 30-hour placement in Year 2 and may undertake a full-year placement between Years 2 and 3 or study abroad at partner universities. A BPS-accredited psychology degree provides the first step towards careers such as clinical psychology, counselling psychology, health psychology, forensic psychology, organisational psychology, educational psychology and sports psychology. Graduates also work in careers including marketing, advertising, journalism, human resources, management consulting, academic research, teaching, policing, mental health services, counselling and social work. The course confers eligibility for Graduate Membership of the British Psychological Society and the Graduate Basis for Registration.
@@ -1145,20 +1253,25 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
+          <t>History and Sociology; Sociology and Criminology; Sociology with Social Psychology</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
           <t>What holds societies together? Do people pull together because they have to or because they want to? What motivates so many people to migrate from their own societies to others? On our course you explore why individuals, groups, and cultures are the way they are, and examine why they might be different. At Essex we investigate what connects people with each other, as well as what divides them. You can study topics such as digital media and society, psychiatry and mental illness, sexualities, crime, childhood, and the art, film and personal testimony of war. We offer a range of specialisms including social divisions, inequality, the nature of work and commercial culture; culture, identity and subjectivity; public policy regarding health, the environment, crime and aging; citizenship, multiculturalism and human rights. You also receive training in sociological methods including how to design a survey, conduct an interview, and use quantitative analysis from basic statistics to big data in order to ask complex social questions. You also have the opportunity to complete a supervised dissertation on the topic that most inspires you, encouraging you to think differently, connect with contemporary social issues and debates, and prepare for your graduate career. Through our Q-Step Affiliate Status, you also have the opportunity to follow a specialised pathway that embeds quantitative methods in your degree, and successful completion of specified modules entitles you to receive the qualifier “Applied Quantitative Methods” on your degree transcript. Sociology graduates are in demand across a wide range of sectors including local and central government, NGOs, social work, market research, project management, fundraising, auditing, marketing, case-work, youth and community work, voluntary sector management and lobbying. Recent graduates have gone on to work for organisations including The Institute of Public Finance, Guardian Professional, United, and Synergy Healthcare Research.</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>The BSocSc Sociology course enables students to understand the social contexts and interconnected forces that shape communities and human behaviour while developing critical perspectives on how societies function, change and influence everyday life. Teaching and research focus on analysing social conditions and challenging assumptions about the social world. Students engage with a wide range of research areas including decolonial thought, sustainability and environment, personal life and relationships, media and technology, race and ethnicity, social inequality, social movements, social theory, globalisation and social change, cultural practices and consumption, migration, work and economy, urban life and ageing. Methodological training includes survey methods and qualitative research approaches, culminating in an independent social research project in the final year that allows students to refine their interests and critical perspective. The programme may also include opportunities to engage with quantitative social science training initiatives such as Q-Step internships. Graduates develop analytical, research and communication skills applicable across sectors including public policy, media, international organisations and business, with alumni working at organisations such as the Ministry of Justice, the NHS, the British Council, Fujitsu, the United Nations Refugee Agency and Unilever.</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>Studying sociology will decode the hidden patterns that govern human behaviour and give you the tools to drive positive change. Studying sociology opens doors to a fascinating exploration of the world we live in. You’ll learn the tools to understand how societies tick, unravelling the mysteries of human behaviour, and diving into the diverse world of cultures and communities. Sociology isn’t just about books and theories – it will also open up a world of possibilities for your future career. You could end up in roles where you can make a real impact; shaping policies, carrying out social research, contributing to community development, or even championing causes that matter to you are all realistic career paths. Sociology is a route to understanding people and making a positive mark on the world. So, if you're looking for a subject that combines curiosity, empathy, and the potential to make a difference, sociology is a great choice to a fulfilling career. Urban sociology, individuals and society, applied ethics, nature and society, media and crime, mobilisation, social movements, and protest are areas you could study. Statistical analysis, qualitative research techniques, data interpretation and interviewing techniques are hard skills you'll develop. Active listening, cultural competence, problem-solving and writing and presentation skills are soft skills you'll develop. Career options include actuaries, economists and statisticians, market research interviewers, and business and related research professionals.</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>Essex: What holds societies together? Do people pull together because they have to or because they want to? What motivates so many people to migrate from their own societies to others? On our course you explore why individuals, groups, and cultures are the way they are, and examine why they might be different. At Essex we investigate what connects people with each other, as well as what divides them. You can study topics such as digital media and society, psychiatry and mental illness, sexualities, crime, childhood, and the art, film and personal testimony of war. We offer a range of specialisms including social divisions, inequality, the nature of work and commercial culture; culture, identity and subjectivity; public policy regarding health, the environment, crime and aging; citizenship, multiculturalism and human rights. You also receive training in sociological methods including how to design a survey, conduct an interview, and use quantitative analysis from basic statistics to big data in order to ask complex social questions. You also have the opportunity to complete a supervised dissertation on the topic that most inspires you, encouraging you to think differently, connect with contemporary social issues and debates, and prepare for your graduate career. Through our Q-Step Affiliate Status, you also have the opportunity to follow a specialised pathway that embeds quantitative methods in your degree, and successful completion of specified modules entitles you to receive the qualifier “Applied Quantitative Methods” on your degree transcript. Sociology graduates are in demand across a wide range of sectors including local and central government, NGOs, social work, market research, project management, fundraising, auditing, marketing, case-work, youth and community work, voluntary sector management and lobbying. Recent graduates have gone on to work for organisations including The Institute of Public Finance, Guardian Professional, United, and Synergy Healthcare Research.
 Manchester: The BSocSc Sociology course enables students to understand the social contexts and interconnected forces that shape communities and human behaviour while developing critical perspectives on how societies function, change and influence everyday life. Teaching and research focus on analysing social conditions and challenging assumptions about the social world. Students engage with a wide range of research areas including decolonial thought, sustainability and environment, personal life and relationships, media and technology, race and ethnicity, social inequality, social movements, social theory, globalisation and social change, cultural practices and consumption, migration, work and economy, urban life and ageing. Methodological training includes survey methods and qualitative research approaches, culminating in an independent social research project in the final year that allows students to refine their interests and critical perspective. The programme may also include opportunities to engage with quantitative social science training initiatives such as Q-Step internships. Graduates develop analytical, research and communication skills applicable across sectors including public policy, media, international organisations and business, with alumni working at organisations such as the Ministry of Justice, the NHS, the British Council, Fujitsu, the United Nations Refugee Agency and Unilever.
@@ -1177,16 +1290,21 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
+          <t>Occupational Therapy; Psychology with Sport and Exercise; Speech and Language Therapy; Sports Performance and Coaching; Sports Therapy; Sports and Exercise Science</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
           <t>The BSc (Hons) Sports and Exercise Science is a three-year degree. You’ll gain a new and exciting perspective on the world of sport, exercise, health and physical fitness, ready to help athletes optimise their performance and improve the physical activity, health and wellbeing of individuals and communities. The BSc (Hons) Sports and Exercise Science provides you with a strong understanding of the role of physiology, psychology, biomechanics and nutrition in sports and exercise. By focusing on practical work in your first two years, you’ll consolidate your professional and scientific skills needed for your final-year research project. You can also gain more real-world experience at our renowned Human Performance Unit (HPU) where you can work with performance scholars, students, staff and members of the public. You’ll graduate on the path to a sports practitioner or sports scientist career, ready to further research on or implement changes to sport and exercise. The course is suitable for future sports practitioners, coaches or researchers, those looking to optimise athletes’ performance or the fitness and wellbeing of the public, students considering careers through a broad understanding of sport and exercise science, and practical learners eager to put new knowledge into practice. You will learn topics such as how and why different energy systems are deployed at different exercise intensities, the biomechanical principles behind acute and chronic sporting injuries and how these can be applied to prevent injuries, the role of ergogenic aids in improving athletic performance, how physical activity and nutrition can reduce the risk of cardio-metabolic disease, and the design and implementation of psychological skills training programmes. The degree also allows you to tailor your studies through a choice of optional modules. A BSc (Hons) Sports and Exercise Science degree prepares you for careers in areas such as sports teams and clubs including coaching, sports development, performance analysis and centre management; national bodies including health improvement, sports development and health and safety; education including physical education teaching; health professions such as sports therapy, nutrition, physiology and sport psychology; and the fitness industry including fitness training and personal training. Graduates from this course have progressed to roles in organisations such as Triathlon England Youth Forum and York St. John University. The CASES Undergraduate Endorsement Scheme awards endorsement to sport and exercise science degree courses that demonstrate the required mapping of knowledge and skills, providing graduates with the competencies needed to enter the profession.</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr">
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
         <is>
           <t>Whether you want to work with your sporting heroes, with children, or the general public, this subject area offers access to a range of rewarding, active, and hands-on jobs. With a qualification in sport and exercise science, you may want to work with athletes on sports performance, become a sports coach or teacher, or manage a gym or fitness centre. You might be employed by a professional sports team, a local authority, the NHS, or a private fitness company, among others. You could also work for yourself. Some roles, like coaching and teaching roles or sports psychology, may require further study. Alternatively, you may choose to go into business management or community engagement projects, depending on what inspires you; you could even become a sports broadcaster. On most courses – and certainly on an apprenticeship – you’ll spend time in industry, which will give you networking opportunities and a great insight into where this subject could take you. Anatomy and physiology, sport biomechanics and kinesiology, data description and analysis, biochemistry and cell biology, foundations of sport and exercise psychology and applied studies across sport performance and health are areas you could study. Physical education, child protection, risk analysis and lesson planning are hard skills you'll develop. Teaching, management and communication are soft skills you'll develop. Career options include sports player, physiotherapist, coach, fitness instructor, broadcasting and media administrator, public relations officer, sports journalist and sport and leisure management.</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>Essex: The BSc (Hons) Sports and Exercise Science is a three-year degree. You’ll gain a new and exciting perspective on the world of sport, exercise, health and physical fitness, ready to help athletes optimise their performance and improve the physical activity, health and wellbeing of individuals and communities. The BSc (Hons) Sports and Exercise Science provides you with a strong understanding of the role of physiology, psychology, biomechanics and nutrition in sports and exercise. By focusing on practical work in your first two years, you’ll consolidate your professional and scientific skills needed for your final-year research project. You can also gain more real-world experience at our renowned Human Performance Unit (HPU) where you can work with performance scholars, students, staff and members of the public. You’ll graduate on the path to a sports practitioner or sports scientist career, ready to further research on or implement changes to sport and exercise. The course is suitable for future sports practitioners, coaches or researchers, those looking to optimise athletes’ performance or the fitness and wellbeing of the public, students considering careers through a broad understanding of sport and exercise science, and practical learners eager to put new knowledge into practice. You will learn topics such as how and why different energy systems are deployed at different exercise intensities, the biomechanical principles behind acute and chronic sporting injuries and how these can be applied to prevent injuries, the role of ergogenic aids in improving athletic performance, how physical activity and nutrition can reduce the risk of cardio-metabolic disease, and the design and implementation of psychological skills training programmes. The degree also allows you to tailor your studies through a choice of optional modules. A BSc (Hons) Sports and Exercise Science degree prepares you for careers in areas such as sports teams and clubs including coaching, sports development, performance analysis and centre management; national bodies including health improvement, sports development and health and safety; education including physical education teaching; health professions such as sports therapy, nutrition, physiology and sport psychology; and the fitness industry including fitness training and personal training. Graduates from this course have progressed to roles in organisations such as Triathlon England Youth Forum and York St. John University. The CASES Undergraduate Endorsement Scheme awards endorsement to sport and exercise science degree courses that demonstrate the required mapping of knowledge and skills, providing graduates with the competencies needed to enter the profession.
 UCAS: Whether you want to work with your sporting heroes, with children, or the general public, this subject area offers access to a range of rewarding, active, and hands-on jobs. With a qualification in sport and exercise science, you may want to work with athletes on sports performance, become a sports coach or teacher, or manage a gym or fitness centre. You might be employed by a professional sports team, a local authority, the NHS, or a private fitness company, among others. You could also work for yourself. Some roles, like coaching and teaching roles or sports psychology, may require further study. Alternatively, you may choose to go into business management or community engagement projects, depending on what inspires you; you could even become a sports broadcaster. On most courses – and certainly on an apprenticeship – you’ll spend time in industry, which will give you networking opportunities and a great insight into where this subject could take you. Anatomy and physiology, sport biomechanics and kinesiology, data description and analysis, biochemistry and cell biology, foundations of sport and exercise psychology and applied studies across sport performance and health are areas you could study. Physical education, child protection, risk analysis and lesson planning are hard skills you'll develop. Teaching, management and communication are soft skills you'll develop. Career options include sports player, physiotherapist, coach, fitness instructor, broadcasting and media administrator, public relations officer, sports journalist and sport and leisure management.</t>
@@ -1204,20 +1322,25 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
+          <t>Applied Biomedical Science</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
           <t>The BSc (Hons) Biomedical Science is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll gain the practical skills and knowledge needed to work in labs and hospitals across the NHS and private sector. The BSc (Hons) Biomedical Science gives you key knowledge and modern strategies to diagnose and treat the human immune system, pathogenic and non-pathogenic bacteria, haematology and blood transfusion, cell pathology and mechanisms of neurological diseases. Previous students have placed with GlaxoSmithKline (GSK), Proctor &amp; Gamble (P&amp;G), AquaTerra, AstraZeneca, Genzyme, Reckitt Benckiser, Thermo Fisher and Isogenica – some of our 40 partner labs. In Year One, you’ll participate in Science Week at Public Health England (PHE) in Colindale. In Year Two, you can visit hospitals in the Eastern Region and beyond. In your Final Year, you’ll attend our Biomedical Employability Day and have the chance to contribute to the IBMS Congress. You’ll graduate on the path to a career as a biomedical scientist or medical researcher. The course is suited to future biomedical scientists, students wanting to work in the NHS, those aiming to advance medical research, and future students of postgraduate medicine. You will study the biology of disease including immunity and a range of diseases, explore microbiology, biochemistry, medical genetics, haematology and pharmacology, and specialise through applied modules in areas such as cancer, neurological disease and virology. A BSc (Hons) Biomedical Science degree prepares you for diverse careers in hospitals, clinics and healthcare companies including biomedical science roles in the NHS, andrology, clinical perfusion, microbiology, toxicology, biotechnology, forensic science and pharmaceuticals, as well as postgraduate medicine, postgraduate research programmes and science teaching. Graduates from this course have progressed to roles in NHS hospitals including Cambridge, Chelmsford, Colchester, Public Health England in Colindale, Basildon, London, Bury St Edmunds, Harlow, Hastings, Ipswich, Norwich, Peterborough, Kent, Bedford and Romford. The course is accredited by the Institute of Biomedical Science (IBMS).</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>The BSc Biomedical Sciences course provides grounding in medically related disciplines including physiology, pharmacology, neuroscience, cell biology, microbiology, anatomy and histology, genetics, biochemistry and immunology. Students learn to apply biological science for medical use in areas such as research, health monitoring and treatment, supported by a strong emphasis on practical laboratory experience. The curriculum allows flexibility through options to broaden study by taking units from interdisciplinary programmes or related subject areas. Teaching is supported by specialist laboratory facilities enabling training in techniques such as polymerase chain reaction, DNA sequencing, gel electrophoresis, spectrophotometry, dissection and histology, electromyography, electrocardiography and immunofluorescence microscopy. In the final year students undertake an independent research project in bioscience laboratories equipped with advanced research technology. Graduates pursue careers in university research, pharmaceutical and bioscience industries and clinical or technical laboratory roles including progression to the NHS Scientist Training Programme, while others enter fields such as medical writing, health communication or teaching.</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>Biomedical scientists endeavour to understand the inner workings of the human body so they can provide the right care for patients, and tackle some of the most serious diseases threatening mankind. Ever wondered who the scientists were behind the statistical data that informed governments’ decisions during the Covid-19 pandemic? As a biomedical scientist, you’ll research and understand how the human body works, both in health and disease. You’ll learn about genetics, genomics, pathology, cellular biology, and immunity, among other things. It could lead to a career as a biomedical scientist, medical laboratory assistant, research technician, or marketing assistant. You could progress to teaching, postgraduate study, or even into medicine or dentistry. It’s a relatively stable industry, with 3.31% job growth predicted over the next eight years. Biochemistry, molecular biology, laboratory science, genetics, microbiology, anatomy, physiology, cells of the nervous system and pharmacology are areas you could study. An IBMS accredited biomedical science degree is the key to becoming a registered biomedical scientist in the UK. To practise as a biomedical scientist in the UK, you must be registered with the Health &amp; Care Professions Council (HCPC), and an IBMS accredited degree is a crucial step in meeting their strict requirements. Getting your HCPC registration also involves hands-on training in an IBMS-approved training laboratory, and an accredited degree often streamlines this process, sometimes even incorporating a clinical placement to complete the IBMS Registration Training Portfolio into the program itself. These specialised degrees are designed to meet the requirements for a biomedical scientist role but also provide you with excellent transferable, technical, and practical skills that a variety of employers demand. Biology, biochemistry, project management, data analysis and microbiology are hard skills you'll develop. Research, communications, management, planning and innovation are soft skills you'll develop. Career options include environment professionals, conservation professionals, biochemists and biomedical scientists, biological scientists, chemical scientists, laboratory technicians, pharmacists, pharmaceutical technicians, specialist medical practitioners and nursing auxiliaries and assistants.</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>Essex: The BSc (Hons) Biomedical Science is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll gain the practical skills and knowledge needed to work in labs and hospitals across the NHS and private sector. The BSc (Hons) Biomedical Science gives you key knowledge and modern strategies to diagnose and treat the human immune system, pathogenic and non-pathogenic bacteria, haematology and blood transfusion, cell pathology and mechanisms of neurological diseases. Previous students have placed with GlaxoSmithKline (GSK), Proctor &amp; Gamble (P&amp;G), AquaTerra, AstraZeneca, Genzyme, Reckitt Benckiser, Thermo Fisher and Isogenica – some of our 40 partner labs. In Year One, you’ll participate in Science Week at Public Health England (PHE) in Colindale. In Year Two, you can visit hospitals in the Eastern Region and beyond. In your Final Year, you’ll attend our Biomedical Employability Day and have the chance to contribute to the IBMS Congress. You’ll graduate on the path to a career as a biomedical scientist or medical researcher. The course is suited to future biomedical scientists, students wanting to work in the NHS, those aiming to advance medical research, and future students of postgraduate medicine. You will study the biology of disease including immunity and a range of diseases, explore microbiology, biochemistry, medical genetics, haematology and pharmacology, and specialise through applied modules in areas such as cancer, neurological disease and virology. A BSc (Hons) Biomedical Science degree prepares you for diverse careers in hospitals, clinics and healthcare companies including biomedical science roles in the NHS, andrology, clinical perfusion, microbiology, toxicology, biotechnology, forensic science and pharmaceuticals, as well as postgraduate medicine, postgraduate research programmes and science teaching. Graduates from this course have progressed to roles in NHS hospitals including Cambridge, Chelmsford, Colchester, Public Health England in Colindale, Basildon, London, Bury St Edmunds, Harlow, Hastings, Ipswich, Norwich, Peterborough, Kent, Bedford and Romford. The course is accredited by the Institute of Biomedical Science (IBMS).
 Manchester: The BSc Biomedical Sciences course provides grounding in medically related disciplines including physiology, pharmacology, neuroscience, cell biology, microbiology, anatomy and histology, genetics, biochemistry and immunology. Students learn to apply biological science for medical use in areas such as research, health monitoring and treatment, supported by a strong emphasis on practical laboratory experience. The curriculum allows flexibility through options to broaden study by taking units from interdisciplinary programmes or related subject areas. Teaching is supported by specialist laboratory facilities enabling training in techniques such as polymerase chain reaction, DNA sequencing, gel electrophoresis, spectrophotometry, dissection and histology, electromyography, electrocardiography and immunofluorescence microscopy. In the final year students undertake an independent research project in bioscience laboratories equipped with advanced research technology. Graduates pursue careers in university research, pharmaceutical and bioscience industries and clinical or technical laboratory roles including progression to the NHS Scientist Training Programme, while others enter fields such as medical writing, health communication or teaching.
@@ -1234,18 +1357,19 @@
           <t>LIBERAL ARTS</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
         <is>
           <t>Knowledge is rooted in the experiences of people across the world. It is created from memory, culture, landscape and myth. This knowledge is often split into separate ‘disciplines' such as those in the sciences, maths, history, geography, literature and art. However, true knowledge does not recognise these boundaries; the world is complex, interconnected and networked. Our course is for you if you love studying a variety of subjects, and want to maintain this breadth of knowledge at university. With the opportunity to major in Psychology, History, Literature, Art History, Philosophy, Politics, Media Studies or Sociology, you broaden your horizons by exploring the ways in which the humanities and social sciences help us to think imaginatively and critically about the worlds we live in. You take modules which cover the historical foundations of the humanities, challenge dominant worldviews, and explore innovative and subversive essays and manifestos. The flexible structure of this course allows you to choose a range of optional modules across literature, film, philosophy, history of art, history, linguistics, politics, sociology and modern languages. The types of issues and problems you might explore include how commercial and independent films interpret human relationships, how to compose your own writing inspired by the great essayists, important philosophical questions about life, death and religion, great works of art and literature, and languages. Based within our School of Philosophical, Historical and Interdisciplinary Studies, the choice is yours: you choose your modules based on your own background and interests. You engage with unusual, controversial, and provocative ideas so that you can use the humanities and social sciences to become critically aware and possess the tools to change the world for the better. As a liberal arts graduate, you'll be provided with an all-round education that can lead to a more extensive range of knowledge, better communication skills and a more flexible and positive attitude to life. The best way to prepare for the future is to develop the abilities and skills which make you resilient; reasoning skills which mean that you do not accept easy answers so that you can always question. A Liberal Arts course can lead to a wide variety of careers in the media, journalism, publishing, local government, voluntary agencies, librarianship, finance, management and other fields. Many employers prefer to recruit students with a broad-based liberal arts education and provide them with vocational training during their first year at work rather than recruit students who have specialised in one discipline. Our recent graduates have gone on to work for a wide range of organisations including Euromoney, a financial publication company, a housing association, and an English language school in Japan.</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>Liberal Arts is highly flexible, allowing students to create their own unique course by combining different subject areas within and beyond the School of Arts, Languages and Cultures. With an emphasis on interdisciplinary learning, students can tailor the course to align with their interests while engaging with key issues that affect society. The programme enables students to develop a broad academic foundation across areas such as economics, globalisation, environmental science, anthropology, sociology and philosophy, supporting the ability to analyse complex real-world challenges from multiple perspectives. Teaching makes use of distinctive research and cultural resources including the internationally renowned John Rylands Library with its collections of rare books, manuscripts and archives, as well as engagement with institutions such as Manchester Museum, Whitworth Art Gallery, the Museum of Medicine and Health and the Museum of Science and Industry. Studying the degree helps develop transferable and specialist skills including independent working, time management and planning, collaboration, teamwork, leadership, communication across diverse audiences and the ability to conduct research that responds to real-world challenges through engagement with organisations and institutions. Graduates pursue careers across sectors including media, public policy, cultural organisations, business and research-oriented roles.</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr">
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
         <is>
           <t>Essex: Knowledge is rooted in the experiences of people across the world. It is created from memory, culture, landscape and myth. This knowledge is often split into separate ‘disciplines' such as those in the sciences, maths, history, geography, literature and art. However, true knowledge does not recognise these boundaries; the world is complex, interconnected and networked. Our course is for you if you love studying a variety of subjects, and want to maintain this breadth of knowledge at university. With the opportunity to major in Psychology, History, Literature, Art History, Philosophy, Politics, Media Studies or Sociology, you broaden your horizons by exploring the ways in which the humanities and social sciences help us to think imaginatively and critically about the worlds we live in. You take modules which cover the historical foundations of the humanities, challenge dominant worldviews, and explore innovative and subversive essays and manifestos. The flexible structure of this course allows you to choose a range of optional modules across literature, film, philosophy, history of art, history, linguistics, politics, sociology and modern languages. The types of issues and problems you might explore include how commercial and independent films interpret human relationships, how to compose your own writing inspired by the great essayists, important philosophical questions about life, death and religion, great works of art and literature, and languages. Based within our School of Philosophical, Historical and Interdisciplinary Studies, the choice is yours: you choose your modules based on your own background and interests. You engage with unusual, controversial, and provocative ideas so that you can use the humanities and social sciences to become critically aware and possess the tools to change the world for the better. As a liberal arts graduate, you'll be provided with an all-round education that can lead to a more extensive range of knowledge, better communication skills and a more flexible and positive attitude to life. The best way to prepare for the future is to develop the abilities and skills which make you resilient; reasoning skills which mean that you do not accept easy answers so that you can always question. A Liberal Arts course can lead to a wide variety of careers in the media, journalism, publishing, local government, voluntary agencies, librarianship, finance, management and other fields. Many employers prefer to recruit students with a broad-based liberal arts education and provide them with vocational training during their first year at work rather than recruit students who have specialised in one discipline. Our recent graduates have gone on to work for a wide range of organisations including Euromoney, a financial publication company, a housing association, and an English language school in Japan.
 Manchester: Liberal Arts is highly flexible, allowing students to create their own unique course by combining different subject areas within and beyond the School of Arts, Languages and Cultures. With an emphasis on interdisciplinary learning, students can tailor the course to align with their interests while engaging with key issues that affect society. The programme enables students to develop a broad academic foundation across areas such as economics, globalisation, environmental science, anthropology, sociology and philosophy, supporting the ability to analyse complex real-world challenges from multiple perspectives. Teaching makes use of distinctive research and cultural resources including the internationally renowned John Rylands Library with its collections of rare books, manuscripts and archives, as well as engagement with institutions such as Manchester Museum, Whitworth Art Gallery, the Museum of Medicine and Health and the Museum of Science and Industry. Studying the degree helps develop transferable and specialist skills including independent working, time management and planning, collaboration, teamwork, leadership, communication across diverse audiences and the ability to conduct research that responds to real-world challenges through engagement with organisations and institutions. Graduates pursue careers across sectors including media, public policy, cultural organisations, business and research-oriented roles.</t>
@@ -1263,16 +1387,21 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
+          <t>Electronic Engineering; Neural Engineering with Psychology</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
           <t>The BEng (Hons) Robotic Engineering is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll build a strong foundation in electrical engineering and computer science theory, as well as the skills and tools to develop and test your own robotic systems. The BEng (Hons) Robotic Engineering gives you the theory and practical knowledge to understand – and create – robotics that make a real impact on the world. Discover which areas you’re interested in exploring further such as assistive technologies, computer games, artificial intelligence, evolutionary computation, Big Data or robotics. You’ll also be able to undertake a project or product development specified by a member of academic staff or a partner company. You’ll graduate as a creative, experimental and focused robotics engineer ready to explore further how robots, animatronics and robotic equipment can impact the world around you. You will explore robotics and artificial intelligence, master the scientific and engineering foundations of electronics and digital systems, learn to programme and apply mathematical skills to engineering, and tailor your degree through your choice of optional modules. The course provides access to specialist robotics facilities including a robotics gaming laboratory and robot arena with one of the world’s largest powered lab floors, and specialist robotics equipment such as wheeled and flying robots, robotic fish, intelligent wheelchairs, robotic arms and robotic hands. A BEng (Hons) Robotic Engineering degree prepares you for diverse careers in engineering including design, development, research, diagnostics and manufacture; IT including software, hardware, systems integration, control systems and automation; healthcare technologies such as surgical instruments, diagnostic tools and assistive technologies; research fields including space and deep ocean exploration; and business roles such as marketing, management, consultancy and patent law. The course is accredited by BCS, the Chartered Institute for IT for the purposes of fully meeting the academic requirement for registration as a Chartered IT Professional, and by BCS and the Institution of Engineering and Technology (IET) on behalf of the Engineering Council for the purposes of fully meeting the academic requirement for registration as an Incorporated Engineer and partially meeting the academic requirement for registration as a Chartered Engineer.</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>Mechatronic Engineering combines mechanical engineering with electronics and intelligent control systems and is central to areas such as industrial automation and robotics. The programme develops understanding of how sensors detect position, orientation and signals, how electronic inputs are interpreted and how actuators perform controlled operations using feedback control systems. Students learn techniques required for the design and implementation of intelligent mechatronic and autonomous systems including robotics, embedded systems and control technologies. Practical application and project-based learning are strong themes throughout the course. The curriculum structure allows flexibility during the early stages of study, enabling students to transfer between Mechatronic Engineering and Electrical and Electronic Engineering pathways. Teaching is supported by access to specialist engineering research infrastructure and industry-standard equipment including facilities such as the High Voltage Laboratory, Photon Science Institute, National Graphene Institute and Rolls-Royce University Technology Centre. Graduates develop technical and problem-solving skills applicable across sectors including robotics development, automotive electronics, renewable energy systems, automation and control engineering and unmanned vehicle guidance systems, with alumni securing roles at organisations such as BP, Rolls-Royce, Jaguar Land Rover, ABB, BAE Systems, Siemens and Jacobs. The course is accredited by the Institution of Engineering and Technology and the Institute of Measurement and Control, supporting progression towards Incorporated or Chartered Engineer status.</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr">
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
         <is>
           <t>Essex: The BEng (Hons) Robotic Engineering is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll build a strong foundation in electrical engineering and computer science theory, as well as the skills and tools to develop and test your own robotic systems. The BEng (Hons) Robotic Engineering gives you the theory and practical knowledge to understand – and create – robotics that make a real impact on the world. Discover which areas you’re interested in exploring further such as assistive technologies, computer games, artificial intelligence, evolutionary computation, Big Data or robotics. You’ll also be able to undertake a project or product development specified by a member of academic staff or a partner company. You’ll graduate as a creative, experimental and focused robotics engineer ready to explore further how robots, animatronics and robotic equipment can impact the world around you. You will explore robotics and artificial intelligence, master the scientific and engineering foundations of electronics and digital systems, learn to programme and apply mathematical skills to engineering, and tailor your degree through your choice of optional modules. The course provides access to specialist robotics facilities including a robotics gaming laboratory and robot arena with one of the world’s largest powered lab floors, and specialist robotics equipment such as wheeled and flying robots, robotic fish, intelligent wheelchairs, robotic arms and robotic hands. A BEng (Hons) Robotic Engineering degree prepares you for diverse careers in engineering including design, development, research, diagnostics and manufacture; IT including software, hardware, systems integration, control systems and automation; healthcare technologies such as surgical instruments, diagnostic tools and assistive technologies; research fields including space and deep ocean exploration; and business roles such as marketing, management, consultancy and patent law. The course is accredited by BCS, the Chartered Institute for IT for the purposes of fully meeting the academic requirement for registration as a Chartered IT Professional, and by BCS and the Institution of Engineering and Technology (IET) on behalf of the Engineering Council for the purposes of fully meeting the academic requirement for registration as an Incorporated Engineer and partially meeting the academic requirement for registration as a Chartered Engineer.
 Manchester: Mechatronic Engineering combines mechanical engineering with electronics and intelligent control systems and is central to areas such as industrial automation and robotics. The programme develops understanding of how sensors detect position, orientation and signals, how electronic inputs are interpreted and how actuators perform controlled operations using feedback control systems. Students learn techniques required for the design and implementation of intelligent mechatronic and autonomous systems including robotics, embedded systems and control technologies. Practical application and project-based learning are strong themes throughout the course. The curriculum structure allows flexibility during the early stages of study, enabling students to transfer between Mechatronic Engineering and Electrical and Electronic Engineering pathways. Teaching is supported by access to specialist engineering research infrastructure and industry-standard equipment including facilities such as the High Voltage Laboratory, Photon Science Institute, National Graphene Institute and Rolls-Royce University Technology Centre. Graduates develop technical and problem-solving skills applicable across sectors including robotics development, automotive electronics, renewable energy systems, automation and control engineering and unmanned vehicle guidance systems, with alumni securing roles at organisations such as BP, Rolls-Royce, Jaguar Land Rover, ABB, BAE Systems, Siemens and Jacobs. The course is accredited by the Institution of Engineering and Technology and the Institute of Measurement and Control, supporting progression towards Incorporated or Chartered Engineer status.</t>

</xml_diff>

<commit_message>
(Semantic) Calculated chunk-level similarity
</commit_message>
<xml_diff>
--- a/data/reference/course_descriptions.xlsx
+++ b/data/reference/course_descriptions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,25 +429,20 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>related_terms</t>
+          <t>description_essex</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>description_essex</t>
+          <t>description_manchester</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>description_manchester</t>
+          <t>description_ucas</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
-        <is>
-          <t>description_ucas</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
         <is>
           <t>combined_description</t>
         </is>
@@ -464,25 +459,20 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Accounting; Accounting and Finance; Accounting and Management; Accounting with Economics; Banking and Finance; Finance and Management</t>
+          <t>How can finance professionals act responsibility, but still meet business objectives? How does accounting information inform business decisions? Our BSc Accounting and Finance degree provides access to our virtual trading floor, where you make use of real-world Bloomberg Market Data Feed (B-PIPE), information and analytics to practise trading stocks and securities in the type of environment found in City finance firms. You study a wide range of topics and develop your quantitative skills, giving you the flexibility to pursue a career in finance, accounting or business management after graduation. You'll explore areas such as the preparation of financial statements and budgets, accounting standards and corporate governance, financial theory, portfolio management, options and futures markets, and risk management. BSc Accounting and Finance includes an introductory first year to familiarise you with wider business topics, such as management and marketing. In your final year, you have the opportunity to put your knowledge into practice by completing an in-depth, independent research project or dissertation. This will give you the chance to further develop vital employment skills in areas of research, time management and critical thinking. The University of Essex is one of just three UK universities to have received Q-Step Affiliate status, including for our BSc Accounting and Finance course, to support the way we develop the quantitative skills of our graduates. This means we can provide work placement bursaries to develop your skills in evaluating numerical evidence, analysing data and designing research. We also offer the opportunity to follow a specialised degree path, where you graduate with enhanced quantitative skills. These are evidenced on your degree transcript, to help give you the competitive edge in the graduate job market. BSc Accounting and Finance is taught at Essex Business School. Our finance group is one of the largest and most respected in the country and our students and staff join us from all over the world. We not only teach you how financial information underpins leadership, strategy and planning, but how financial decisions can impact society and the economy. We develop your understanding of governance and ethics, so you can take actions for the good of organisations and the wider world. Essex Business School is an Investment Management Certificate (IMC) Advantage Partner and this course is aligned to the IMC syllabus, the industry's benchmark entry-level qualification. Accredited by the Association of Chartered Certified Accountants (ACCA) for the purpose of exemptions from some professional examinations. Accredited by the Chartered Institute of Management Accountants (CIMA) for the purpose of exemption from some professional examinations through the Accredited degree accelerated route. Accredited by the Institute of Chartered Accountants in England and Wales (ICAEW) for the purpose of exemption from some professional examinations. Experience of the dual disciplines of accounting and finance means that you will be well suited to sector specific roles in chartered accountancy and management accountancy as well as more generalist roles such as management consultancy or financial management. We embed a series of core and specific skills into our undergraduate curriculum for BSc Accounting and Finance to ensure that our graduates are suited to careers in finance, accounting and management roles. All of our taught modules embed elements of our skills map which emulate the skills which are required by employers of business, accounting and finance graduates, these generally include academic and cognitive skills, research skills, technology skills, communication skills, data analysis skills and soft skills. Our students have gone on to become financial analysts, accountants, hedge fund managers and insurance trainees, with recent graduate destinations including Private Client Tax Senior Associate at PwC, Treasury Analyst at Hiscox, Junior Tax Consultant at Deloitte, Global Finance &amp; Business Analyst at J.P. Morgan and Junior Consultant - Valuation &amp; Advisory at Cushman &amp; Wakefield. Our accounting and finance graduates enjoy successful careers in their fields.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>How can finance professionals act responsibility, but still meet business objectives? How does accounting information inform business decisions? Our BSc Accounting and Finance degree provides access to our virtual trading floor, where you make use of real-world Bloomberg Market Data Feed (B-PIPE), information and analytics to practise trading stocks and securities in the type of environment found in City finance firms. You study a wide range of topics and develop your quantitative skills, giving you the flexibility to pursue a career in finance, accounting or business management after graduation. You'll explore areas such as the preparation of financial statements and budgets, accounting standards and corporate governance, financial theory, portfolio management, options and futures markets, and risk management. BSc Accounting and Finance includes an introductory first year to familiarise you with wider business topics, such as management and marketing. In your final year, you have the opportunity to put your knowledge into practice by completing an in-depth, independent research project or dissertation. This will give you the chance to further develop vital employment skills in areas of research, time management and critical thinking. The University of Essex is one of just three UK universities to have received Q-Step Affiliate status, including for our BSc Accounting and Finance course, to support the way we develop the quantitative skills of our graduates. This means we can provide work placement bursaries to develop your skills in evaluating numerical evidence, analysing data and designing research. We also offer the opportunity to follow a specialised degree path, where you graduate with enhanced quantitative skills. These are evidenced on your degree transcript, to help give you the competitive edge in the graduate job market. BSc Accounting and Finance is taught at Essex Business School. Our finance group is one of the largest and most respected in the country and our students and staff join us from all over the world. We not only teach you how financial information underpins leadership, strategy and planning, but how financial decisions can impact society and the economy. We develop your understanding of governance and ethics, so you can take actions for the good of organisations and the wider world. Essex Business School is an Investment Management Certificate (IMC) Advantage Partner and this course is aligned to the IMC syllabus, the industry's benchmark entry-level qualification. Accredited by the Association of Chartered Certified Accountants (ACCA) for the purpose of exemptions from some professional examinations. Accredited by the Chartered Institute of Management Accountants (CIMA) for the purpose of exemption from some professional examinations through the Accredited degree accelerated route. Accredited by the Institute of Chartered Accountants in England and Wales (ICAEW) for the purpose of exemption from some professional examinations. Experience of the dual disciplines of accounting and finance means that you will be well suited to sector specific roles in chartered accountancy and management accountancy as well as more generalist roles such as management consultancy or financial management. We embed a series of core and specific skills into our undergraduate curriculum for BSc Accounting and Finance to ensure that our graduates are suited to careers in finance, accounting and management roles. All of our taught modules embed elements of our skills map which emulate the skills which are required by employers of business, accounting and finance graduates, these generally include academic and cognitive skills, research skills, technology skills, communication skills, data analysis skills and soft skills. Our students have gone on to become financial analysts, accountants, hedge fund managers and insurance trainees, with recent graduate destinations including Private Client Tax Senior Associate at PwC, Treasury Analyst at Hiscox, Junior Tax Consultant at Deloitte, Global Finance &amp; Business Analyst at J.P. Morgan and Junior Consultant - Valuation &amp; Advisory at Cushman &amp; Wakefield. Our accounting and finance graduates enjoy successful careers in their fields.</t>
+          <t>Our BA (Economic and Social Studies), known as the BA (Econ), is a flagship interdisciplinary degree designed for students who want to understand Accounting and Finance in their full social, political and technical context. The programme’s Accounting and Finance specialisation will provide you with a rigorous education in core accounting and finance theory and practice, and quantitative methods, while equipping you with the broader perspectives needed to address today’s most complex global challenges. The BA (Econ) is the parent programme to eight distinctive specialisations: Economics, Economics and Politics, Economics and Philosophy, Economics and Sociology, Economics and Finance, Data Science and Economics, Accounting and Finance, and Finance. This structure allows students to gain a strong shared foundation in economics while benefiting from the intellectual richness of other social science disciplines. The BA (Economic and Social Studies) with specialisation in Accounting and Finance is designed for students seeking a rigorous academic foundation for careers in professional accounting and related financial roles. This pathway integrates core economics with a strong sequence of accounting and finance units, enabling you to understand how organisations measure performance, manage financial information and comply with regulatory and governance requirements. A defining feature of the Accounting and Finance pathway is its close collaboration with Alliance Manchester Business School (AMBS). Accounting and finance units are taught by AMBS academics, ensuring your learning reflects current professional standards and industry practice. Throughout the degree, you will develop expertise in financial reporting and accounting regulation, management accounting and decision-making, auditing, accountability and corporate governance, investment and financial analysis, financial markets and institutions, and applying economic reasoning to organisational and financial decisions. Subject to your optional unit choices, the degree offers exemptions from professional examinations with ICAEW, CIMA and ACCA, making it an excellent route into chartered accountancy and related professions. This pathway places accounting firmly within its wider economic, institutional and regulatory environment. You will explore how accounting information is used by investors, managers, regulators and policymakers, and how financial reporting shapes organisational behaviour and market outcomes. You will also develop an understanding of professional ethics, accountability and governance, central to modern accounting practice. Year 1 provides a strong foundation in core economics, financial and management accounting, and quantitative methods, including introductory microeconomics and macroeconomics, financial reporting, management accounting and financial decision-making, mathematics and statistics for economists, and a core social sciences unit exploring power and value. In Year 2, students develop deeper accounting and finance expertise through units including Financial Reporting and Accountability, Intermediate Management Accounting, Foundations of Finance, Financial Statement Analysis, and Investment Analysis. In Year 3, students specialise further in accounting or finance while maintaining a strong professional and analytical focus. Students take a core unit such as Financial Analysis of Corporate Performance or Empirical Finance and may pursue an accounting route focusing on financial reporting and accounting regulation, auditing, accountability and corporate governance, and advanced management accounting and performance measurement, or a finance route including corporate finance, financial markets and institutions, investment analysis and valuation, and risk management and financial decision-making. Graduates develop strong skills in financial reporting, analysis and regulation and pursue careers in audit and assurance, chartered and management accounting, professional services and consultancy, corporate finance and financial management, and public-sector accounting and regulation. The BA (Economic and Social Studies) Accounting and Finance pathway is accredited with professional accountancy bodies including the Institute of Chartered Accountants, the Association of Chartered Certified Accountants and the Chartered Institute of Management Accountants, and students may be eligible for exemptions from professional accountancy examinations depending on the course units chosen. Recent graduates have gone on to careers with organisations including Ernst and Young, KPMG, Deloitte, PricewaterhouseCoopers, Grant Thornton, BDO, American Express, Bloomberg, Bank of America, Deutsche Bank, Merrill Lynch, Morgan Stanley, Royal Bank of Canada, Santander and UBS, as well as roles in government institutions such as HM Treasury, HMRC, the National Audit Office and the Ministry of Justice.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Our BA (Economic and Social Studies), known as the BA (Econ), is a flagship interdisciplinary degree designed for students who want to understand Accounting and Finance in their full social, political and technical context. The programme’s Accounting and Finance specialisation will provide you with a rigorous education in core accounting and finance theory and practice, and quantitative methods, while equipping you with the broader perspectives needed to address today’s most complex global challenges. The BA (Econ) is the parent programme to eight distinctive specialisations: Economics, Economics and Politics, Economics and Philosophy, Economics and Sociology, Economics and Finance, Data Science and Economics, Accounting and Finance, and Finance. This structure allows students to gain a strong shared foundation in economics while benefiting from the intellectual richness of other social science disciplines. The BA (Economic and Social Studies) with specialisation in Accounting and Finance is designed for students seeking a rigorous academic foundation for careers in professional accounting and related financial roles. This pathway integrates core economics with a strong sequence of accounting and finance units, enabling you to understand how organisations measure performance, manage financial information and comply with regulatory and governance requirements. A defining feature of the Accounting and Finance pathway is its close collaboration with Alliance Manchester Business School (AMBS). Accounting and finance units are taught by AMBS academics, ensuring your learning reflects current professional standards and industry practice. Throughout the degree, you will develop expertise in financial reporting and accounting regulation, management accounting and decision-making, auditing, accountability and corporate governance, investment and financial analysis, financial markets and institutions, and applying economic reasoning to organisational and financial decisions. Subject to your optional unit choices, the degree offers exemptions from professional examinations with ICAEW, CIMA and ACCA, making it an excellent route into chartered accountancy and related professions. This pathway places accounting firmly within its wider economic, institutional and regulatory environment. You will explore how accounting information is used by investors, managers, regulators and policymakers, and how financial reporting shapes organisational behaviour and market outcomes. You will also develop an understanding of professional ethics, accountability and governance, central to modern accounting practice. Year 1 provides a strong foundation in core economics, financial and management accounting, and quantitative methods, including introductory microeconomics and macroeconomics, financial reporting, management accounting and financial decision-making, mathematics and statistics for economists, and a core social sciences unit exploring power and value. In Year 2, students develop deeper accounting and finance expertise through units including Financial Reporting and Accountability, Intermediate Management Accounting, Foundations of Finance, Financial Statement Analysis, and Investment Analysis. In Year 3, students specialise further in accounting or finance while maintaining a strong professional and analytical focus. Students take a core unit such as Financial Analysis of Corporate Performance or Empirical Finance and may pursue an accounting route focusing on financial reporting and accounting regulation, auditing, accountability and corporate governance, and advanced management accounting and performance measurement, or a finance route including corporate finance, financial markets and institutions, investment analysis and valuation, and risk management and financial decision-making. Graduates develop strong skills in financial reporting, analysis and regulation and pursue careers in audit and assurance, chartered and management accounting, professional services and consultancy, corporate finance and financial management, and public-sector accounting and regulation. The BA (Economic and Social Studies) Accounting and Finance pathway is accredited with professional accountancy bodies including the Institute of Chartered Accountants, the Association of Chartered Certified Accountants and the Chartered Institute of Management Accountants, and students may be eligible for exemptions from professional accountancy examinations depending on the course units chosen. Recent graduates have gone on to careers with organisations including Ernst and Young, KPMG, Deloitte, PricewaterhouseCoopers, Grant Thornton, BDO, American Express, Bloomberg, Bank of America, Deutsche Bank, Merrill Lynch, Morgan Stanley, Royal Bank of Canada, Santander and UBS, as well as roles in government institutions such as HM Treasury, HMRC, the National Audit Office and the Ministry of Justice.</t>
+          <t>Where precision meets strategy, accounting and finance paves the way for a solid understanding of financial landscapes and decision-making in the business world. If you choose accounting and finance it opens doors to a strategic understanding of the financial architecture that underpins every business. You’ll gain proficiency in financial reporting, budgeting, and analysis, honing the skills needed to navigate the world of corporate finance. It can lead to many different career paths, from becoming a certified public accountant (CPA) or financial analyst, to going into roles such as financial management, investment banking, or corporate strategy. You could be at the heart of financial decision-making, contributing to the financial health of organisations and influencing business growth. Whether ensuring regulatory compliance, conducting financial audits, or crafting investment strategies, accounting and finance offers a great opportunity for those looking for a rewarding career in the financial sector. Financial markets, taxation, banking and investment, corporate finance, accounting, business policies, management accounting and business ethics are areas you could study. Ability to prepare accurate and compliant financial reports, develop expertise in identifying and managing financial risks, solid understanding of tax laws and regulations and hands-on experience with accounting software used in the industry are hard skills you’ll develop. Analytical thinking, attention to detail, time management and integrity and ethical decision-making are soft skills you’ll develop. Career options include chartered and certified accountants, finance and investment analysts and advisers, financial account managers, taxation experts, business and financial project management professionals, management consultants and business analysts, purchasing managers and directors.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
-        <is>
-          <t>Where precision meets strategy, accounting and finance paves the way for a solid understanding of financial landscapes and decision-making in the business world. If you choose accounting and finance it opens doors to a strategic understanding of the financial architecture that underpins every business. You’ll gain proficiency in financial reporting, budgeting, and analysis, honing the skills needed to navigate the world of corporate finance. It can lead to many different career paths, from becoming a certified public accountant (CPA) or financial analyst, to going into roles such as financial management, investment banking, or corporate strategy. You could be at the heart of financial decision-making, contributing to the financial health of organisations and influencing business growth. Whether ensuring regulatory compliance, conducting financial audits, or crafting investment strategies, accounting and finance offers a great opportunity for those looking for a rewarding career in the financial sector. Financial markets, taxation, banking and investment, corporate finance, accounting, business policies, management accounting and business ethics are areas you could study. Ability to prepare accurate and compliant financial reports, develop expertise in identifying and managing financial risks, solid understanding of tax laws and regulations and hands-on experience with accounting software used in the industry are hard skills you’ll develop. Analytical thinking, attention to detail, time management and integrity and ethical decision-making are soft skills you’ll develop. Career options include chartered and certified accountants, finance and investment analysts and advisers, financial account managers, taxation experts, business and financial project management professionals, management consultants and business analysts, purchasing managers and directors.</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
         <is>
           <t>Essex: How can finance professionals act responsibility, but still meet business objectives? How does accounting information inform business decisions? Our BSc Accounting and Finance degree provides access to our virtual trading floor, where you make use of real-world Bloomberg Market Data Feed (B-PIPE), information and analytics to practise trading stocks and securities in the type of environment found in City finance firms. You study a wide range of topics and develop your quantitative skills, giving you the flexibility to pursue a career in finance, accounting or business management after graduation. You'll explore areas such as the preparation of financial statements and budgets, accounting standards and corporate governance, financial theory, portfolio management, options and futures markets, and risk management. BSc Accounting and Finance includes an introductory first year to familiarise you with wider business topics, such as management and marketing. In your final year, you have the opportunity to put your knowledge into practice by completing an in-depth, independent research project or dissertation. This will give you the chance to further develop vital employment skills in areas of research, time management and critical thinking. The University of Essex is one of just three UK universities to have received Q-Step Affiliate status, including for our BSc Accounting and Finance course, to support the way we develop the quantitative skills of our graduates. This means we can provide work placement bursaries to develop your skills in evaluating numerical evidence, analysing data and designing research. We also offer the opportunity to follow a specialised degree path, where you graduate with enhanced quantitative skills. These are evidenced on your degree transcript, to help give you the competitive edge in the graduate job market. BSc Accounting and Finance is taught at Essex Business School. Our finance group is one of the largest and most respected in the country and our students and staff join us from all over the world. We not only teach you how financial information underpins leadership, strategy and planning, but how financial decisions can impact society and the economy. We develop your understanding of governance and ethics, so you can take actions for the good of organisations and the wider world. Essex Business School is an Investment Management Certificate (IMC) Advantage Partner and this course is aligned to the IMC syllabus, the industry's benchmark entry-level qualification. Accredited by the Association of Chartered Certified Accountants (ACCA) for the purpose of exemptions from some professional examinations. Accredited by the Chartered Institute of Management Accountants (CIMA) for the purpose of exemption from some professional examinations through the Accredited degree accelerated route. Accredited by the Institute of Chartered Accountants in England and Wales (ICAEW) for the purpose of exemption from some professional examinations. Experience of the dual disciplines of accounting and finance means that you will be well suited to sector specific roles in chartered accountancy and management accountancy as well as more generalist roles such as management consultancy or financial management. We embed a series of core and specific skills into our undergraduate curriculum for BSc Accounting and Finance to ensure that our graduates are suited to careers in finance, accounting and management roles. All of our taught modules embed elements of our skills map which emulate the skills which are required by employers of business, accounting and finance graduates, these generally include academic and cognitive skills, research skills, technology skills, communication skills, data analysis skills and soft skills. Our students have gone on to become financial analysts, accountants, hedge fund managers and insurance trainees, with recent graduate destinations including Private Client Tax Senior Associate at PwC, Treasury Analyst at Hiscox, Junior Tax Consultant at Deloitte, Global Finance &amp; Business Analyst at J.P. Morgan and Junior Consultant - Valuation &amp; Advisory at Cushman &amp; Wakefield. Our accounting and finance graduates enjoy successful careers in their fields.
 Manchester: Our BA (Economic and Social Studies), known as the BA (Econ), is a flagship interdisciplinary degree designed for students who want to understand Accounting and Finance in their full social, political and technical context. The programme’s Accounting and Finance specialisation will provide you with a rigorous education in core accounting and finance theory and practice, and quantitative methods, while equipping you with the broader perspectives needed to address today’s most complex global challenges. The BA (Econ) is the parent programme to eight distinctive specialisations: Economics, Economics and Politics, Economics and Philosophy, Economics and Sociology, Economics and Finance, Data Science and Economics, Accounting and Finance, and Finance. This structure allows students to gain a strong shared foundation in economics while benefiting from the intellectual richness of other social science disciplines. The BA (Economic and Social Studies) with specialisation in Accounting and Finance is designed for students seeking a rigorous academic foundation for careers in professional accounting and related financial roles. This pathway integrates core economics with a strong sequence of accounting and finance units, enabling you to understand how organisations measure performance, manage financial information and comply with regulatory and governance requirements. A defining feature of the Accounting and Finance pathway is its close collaboration with Alliance Manchester Business School (AMBS). Accounting and finance units are taught by AMBS academics, ensuring your learning reflects current professional standards and industry practice. Throughout the degree, you will develop expertise in financial reporting and accounting regulation, management accounting and decision-making, auditing, accountability and corporate governance, investment and financial analysis, financial markets and institutions, and applying economic reasoning to organisational and financial decisions. Subject to your optional unit choices, the degree offers exemptions from professional examinations with ICAEW, CIMA and ACCA, making it an excellent route into chartered accountancy and related professions. This pathway places accounting firmly within its wider economic, institutional and regulatory environment. You will explore how accounting information is used by investors, managers, regulators and policymakers, and how financial reporting shapes organisational behaviour and market outcomes. You will also develop an understanding of professional ethics, accountability and governance, central to modern accounting practice. Year 1 provides a strong foundation in core economics, financial and management accounting, and quantitative methods, including introductory microeconomics and macroeconomics, financial reporting, management accounting and financial decision-making, mathematics and statistics for economists, and a core social sciences unit exploring power and value. In Year 2, students develop deeper accounting and finance expertise through units including Financial Reporting and Accountability, Intermediate Management Accounting, Foundations of Finance, Financial Statement Analysis, and Investment Analysis. In Year 3, students specialise further in accounting or finance while maintaining a strong professional and analytical focus. Students take a core unit such as Financial Analysis of Corporate Performance or Empirical Finance and may pursue an accounting route focusing on financial reporting and accounting regulation, auditing, accountability and corporate governance, and advanced management accounting and performance measurement, or a finance route including corporate finance, financial markets and institutions, investment analysis and valuation, and risk management and financial decision-making. Graduates develop strong skills in financial reporting, analysis and regulation and pursue careers in audit and assurance, chartered and management accounting, professional services and consultancy, corporate finance and financial management, and public-sector accounting and regulation. The BA (Economic and Social Studies) Accounting and Finance pathway is accredited with professional accountancy bodies including the Institute of Chartered Accountants, the Association of Chartered Certified Accountants and the Chartered Institute of Management Accountants, and students may be eligible for exemptions from professional accountancy examinations depending on the course units chosen. Recent graduates have gone on to careers with organisations including Ernst and Young, KPMG, Deloitte, PricewaterhouseCoopers, Grant Thornton, BDO, American Express, Bloomberg, Bank of America, Deutsche Bank, Merrill Lynch, Morgan Stanley, Royal Bank of Canada, Santander and UBS, as well as roles in government institutions such as HM Treasury, HMRC, the National Audit Office and the Ministry of Justice.
@@ -499,19 +489,18 @@
           <t>ACTUARIAL SCIENCE</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Actuarial science teaches you the art of turning risks into opportunities. Actuaries provide assessments of financial security systems, with a focus on their complexity, their mathematics, and their mechanisms. You benefit from an excellent starting salary, with graduates earning upwards of £30,000 on average. Our BSc (Hons) Actuarial Science course covers the syllabus of many core subjects of the Institute and Faculty of Actuaries. Depending on your choice of optional modules, and upon sufficient attainment, this can lead to exemptions from the professional exams CS1, CS2, CM1, CM2, CB1 and CB2. More generally, our course features an attractive blend of solid mathematics, an understanding of real-world financial issues, optimisation, experimental design and computing skills which provide you with core skills for entering the world of actuaries and data scientists. You study topics including mathematical finance, financial reporting, contingencies, risk management and survival analysis, mathematical, statistical and probabilistic techniques, and programming and computation in languages such as MATLAB and R. Professional actuaries in the insurance industry, including influential businesses AXA and Buck Consultants, contribute to our employability module and also host students at their offices to show typical challenges that actuaries face. As part of our School of Mathematics, Statistics and Actuarial Science, you are a member of an inclusive and approachable research community which allows you to explore topics in pure, high-level mathematics and applied mathematics. Accredited by the Institute and Faculty of Actuaries for the purpose of exemption from some professional examinations. This programme will meet the educational requirements of the Chartered Mathematician designation, awarded by the Institute of Mathematics and its Applications, when it is followed by subsequent training and experience in employment to obtain equivalent competences to those specified by the Quality Assurance Agency (QAA) for taught masters degrees. We expect our graduates of BSc (Hons) Actuarial Science to become actuaries in a range of industries. It is predicted by the US Department of Labor that the employment of actuaries is expected to grow faster than any other occupation, making it a great prospect for a graduate job. Aside from a rewarding career as an actuary, clear thinkers are required in every profession, so the successful mathematician has an extensive choice of potential careers.</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Actuarial science teaches you the art of turning risks into opportunities. Actuaries provide assessments of financial security systems, with a focus on their complexity, their mathematics, and their mechanisms. You benefit from an excellent starting salary, with graduates earning upwards of £30,000 on average. Our BSc (Hons) Actuarial Science course covers the syllabus of many core subjects of the Institute and Faculty of Actuaries. Depending on your choice of optional modules, and upon sufficient attainment, this can lead to exemptions from the professional exams CS1, CS2, CM1, CM2, CB1 and CB2. More generally, our course features an attractive blend of solid mathematics, an understanding of real-world financial issues, optimisation, experimental design and computing skills which provide you with core skills for entering the world of actuaries and data scientists. You study topics including mathematical finance, financial reporting, contingencies, risk management and survival analysis, mathematical, statistical and probabilistic techniques, and programming and computation in languages such as MATLAB and R. Professional actuaries in the insurance industry, including influential businesses AXA and Buck Consultants, contribute to our employability module and also host students at their offices to show typical challenges that actuaries face. As part of our School of Mathematics, Statistics and Actuarial Science, you are a member of an inclusive and approachable research community which allows you to explore topics in pure, high-level mathematics and applied mathematics. Accredited by the Institute and Faculty of Actuaries for the purpose of exemption from some professional examinations. This programme will meet the educational requirements of the Chartered Mathematician designation, awarded by the Institute of Mathematics and its Applications, when it is followed by subsequent training and experience in employment to obtain equivalent competences to those specified by the Quality Assurance Agency (QAA) for taught masters degrees. We expect our graduates of BSc (Hons) Actuarial Science to become actuaries in a range of industries. It is predicted by the US Department of Labor that the employment of actuaries is expected to grow faster than any other occupation, making it a great prospect for a graduate job. Aside from a rewarding career as an actuary, clear thinkers are required in every profession, so the successful mathematician has an extensive choice of potential careers.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
           <t>Lay the foundations of a rewarding career with mathematics at its base by undertaking an undergraduate degree at the University of Manchester. The programme offers a highly flexible structure, ensuring you obtain a strong all-round mathematical knowledge while encouraging you to focus on the areas that appeal most. You will cover core topics in the first year, developing your capacity to learn and apply mathematical ideas. In the second year you choose two from three themes: Pure Mathematics, Applied Mathematics, and Probability and Statistics, along with optional units such as Programming with Python. You will understand the significance and power of mathematics and acquire a thorough knowledge and understanding of the mathematical topics that any employer would expect of a mathematics graduate. After the first two years you can choose the areas that interest you most and may also select options from other subject areas. In your final year you can undertake a staff-supervised mathematical project. Small group teaching is a significant part of the first year and a wide range of options is available in the third year. All undergraduate students have affiliate membership of the Institute of Mathematics and its Applications. The programme enables students to obtain up to five exemptions from the Institute and Faculty of Actuaries’ professional examinations (CS1, CS2, CM1, CB1 and CB2), subject to satisfactory performance and module options. By studying mathematics at Manchester you will develop analytical, logical and problem-solving skills valued across many professions. Graduates commonly enter areas including finance, industry, computing and operational research, management, administration, statistics, teaching and postgraduate study. Many graduates pursue careers in finance at firms such as KPMG, Goldman Sachs, PricewaterhouseCoopers, Deloitte, Barclays and Deutsche Bank. The course is accredited by the Institute and Faculty of Actuaries, and studying on this degree programme enables students to obtain up to five exemptions from the Institute and Faculty of Actuaries’ professional examinations (CS1, CS2, CM1, CB1 and CB2), subject to satisfactory performance and module options.</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
         <is>
           <t>Essex: Actuarial science teaches you the art of turning risks into opportunities. Actuaries provide assessments of financial security systems, with a focus on their complexity, their mathematics, and their mechanisms. You benefit from an excellent starting salary, with graduates earning upwards of £30,000 on average. Our BSc (Hons) Actuarial Science course covers the syllabus of many core subjects of the Institute and Faculty of Actuaries. Depending on your choice of optional modules, and upon sufficient attainment, this can lead to exemptions from the professional exams CS1, CS2, CM1, CM2, CB1 and CB2. More generally, our course features an attractive blend of solid mathematics, an understanding of real-world financial issues, optimisation, experimental design and computing skills which provide you with core skills for entering the world of actuaries and data scientists. You study topics including mathematical finance, financial reporting, contingencies, risk management and survival analysis, mathematical, statistical and probabilistic techniques, and programming and computation in languages such as MATLAB and R. Professional actuaries in the insurance industry, including influential businesses AXA and Buck Consultants, contribute to our employability module and also host students at their offices to show typical challenges that actuaries face. As part of our School of Mathematics, Statistics and Actuarial Science, you are a member of an inclusive and approachable research community which allows you to explore topics in pure, high-level mathematics and applied mathematics. Accredited by the Institute and Faculty of Actuaries for the purpose of exemption from some professional examinations. This programme will meet the educational requirements of the Chartered Mathematician designation, awarded by the Institute of Mathematics and its Applications, when it is followed by subsequent training and experience in employment to obtain equivalent competences to those specified by the Quality Assurance Agency (QAA) for taught masters degrees. We expect our graduates of BSc (Hons) Actuarial Science to become actuaries in a range of industries. It is predicted by the US Department of Labor that the employment of actuaries is expected to grow faster than any other occupation, making it a great prospect for a graduate job. Aside from a rewarding career as an actuary, clear thinkers are required in every profession, so the successful mathematician has an extensive choice of potential careers.
 Manchester: Lay the foundations of a rewarding career with mathematics at its base by undertaking an undergraduate degree at the University of Manchester. The programme offers a highly flexible structure, ensuring you obtain a strong all-round mathematical knowledge while encouraging you to focus on the areas that appeal most. You will cover core topics in the first year, developing your capacity to learn and apply mathematical ideas. In the second year you choose two from three themes: Pure Mathematics, Applied Mathematics, and Probability and Statistics, along with optional units such as Programming with Python. You will understand the significance and power of mathematics and acquire a thorough knowledge and understanding of the mathematical topics that any employer would expect of a mathematics graduate. After the first two years you can choose the areas that interest you most and may also select options from other subject areas. In your final year you can undertake a staff-supervised mathematical project. Small group teaching is a significant part of the first year and a wide range of options is available in the third year. All undergraduate students have affiliate membership of the Institute of Mathematics and its Applications. The programme enables students to obtain up to five exemptions from the Institute and Faculty of Actuaries’ professional examinations (CS1, CS2, CM1, CB1 and CB2), subject to satisfactory performance and module options. By studying mathematics at Manchester you will develop analytical, logical and problem-solving skills valued across many professions. Graduates commonly enter areas including finance, industry, computing and operational research, management, administration, statistics, teaching and postgraduate study. Many graduates pursue careers in finance at firms such as KPMG, Goldman Sachs, PricewaterhouseCoopers, Deloitte, Barclays and Deutsche Bank. The course is accredited by the Institute and Faculty of Actuaries, and studying on this degree programme enables students to obtain up to five exemptions from the Institute and Faculty of Actuaries’ professional examinations (CS1, CS2, CM1, CB1 and CB2), subject to satisfactory performance and module options.</t>
@@ -527,19 +516,14 @@
           <t>AMERICAN STUDIES</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Modern Languages with Latin American Studies</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
         <is>
           <t>Our three-year American Studies degree is very attractive to those wanting to develop a deep understanding of the US, both at home and around the world. The course enables you to think in interdisciplinary ways about the United States, including its extensive forms of ‘soft’ and ‘hard’ power. This course encourages you to integrate a variety of methods and approaches, allowing you to develop critical and contextual thinking. As you progress, you will have the choice to concentrate more on one approach: you might focus on historical topics – and we employ one of the largest groups of American historians in the UK, offering classes from the beginning of European colonization to the contemporary period – or you might decide to concentrate more on American literary and cultural studies. At Manchester, we train our students to be attentive to the counter currents of US history, society and literature, and many of our course units emphasise the themes of race, capitalism, sexuality, the cultures of labour, political protest, environmental crises and questions of governance. You will learn how to analyse a wide range of texts and materials, including historical documents, literary works, social media communication, films, manuscripts, political rhetoric, marketing campaigns and popular music. Having developed these interpretive skills, you will develop an advanced grasp of theories of change and continuity in a nation that continues to exert considerable influence over international politics, culture, and economics. A degree in American Studies from the University of Manchester provides you with the skills, knowledge and confidence to embark on a successful career in the global workplace. Graduates have entered fields including teaching, law, accountancy, journalism, publishing, surveying and roles within the creative industries in the UK and internationally.</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Manchester: Our three-year American Studies degree is very attractive to those wanting to develop a deep understanding of the US, both at home and around the world. The course enables you to think in interdisciplinary ways about the United States, including its extensive forms of ‘soft’ and ‘hard’ power. This course encourages you to integrate a variety of methods and approaches, allowing you to develop critical and contextual thinking. As you progress, you will have the choice to concentrate more on one approach: you might focus on historical topics – and we employ one of the largest groups of American historians in the UK, offering classes from the beginning of European colonization to the contemporary period – or you might decide to concentrate more on American literary and cultural studies. At Manchester, we train our students to be attentive to the counter currents of US history, society and literature, and many of our course units emphasise the themes of race, capitalism, sexuality, the cultures of labour, political protest, environmental crises and questions of governance. You will learn how to analyse a wide range of texts and materials, including historical documents, literary works, social media communication, films, manuscripts, political rhetoric, marketing campaigns and popular music. Having developed these interpretive skills, you will develop an advanced grasp of theories of change and continuity in a nation that continues to exert considerable influence over international politics, culture, and economics. A degree in American Studies from the University of Manchester provides you with the skills, knowledge and confidence to embark on a successful career in the global workplace. Graduates have entered fields including teaching, law, accountancy, journalism, publishing, surveying and roles within the creative industries in the UK and internationally.</t>
         </is>
@@ -556,25 +540,20 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Curating with History; History; History and Economics; History and Literature; History and Sociology; Modern History; Modern History and International Relations; Modern History and Politics</t>
+          <t>At Essex, you will acquire a broad foundation in the history of visual culture: both by learning about canonical forms of art and architecture and by discovering what has been overlooked or marginalised, such as medical photography, tattoos or objects from political protests. You will also develop the skills you need to make exciting new connections between the forms of visual culture you study, developments in other disciplines, and broader social and political forces. To study on our course, you don't need an Art History A-Level. In fact, we believe that the best art historians are those who bring fresh eyes and new perspectives to their objects of inquiry. You will develop the skills you need to transform your excitement about art, architecture and visual culture into the ability to uncover new insights about the material you study. You will also develop a solid grounding in the history of art and other forms of visual culture, including the ideas and forces that shaped their production, distribution and reception. For students with a particular interest in pursuing careers in curating and museumship, we provide modules that explore the histories, theories and practices of museums, exhibitions and galleries, as well as practical issues such as installing and marketing artwork. The visual arts and culture industries have become an increasingly significant part of the national and international economy, and our art history graduates leave Essex with the skills to take advantage of this growing opportunity. Some of the sectors with jobs well suited for our graduates include museums and galleries, auction houses, education in schools, universities and cultural institutions, marketing and advertising, and new media. Our degree also prepares students to run their own galleries, to work as specialist arts lawyers and PR agents, and for positions in charities, fashion and publishing. Our recent graduates have gone on to work for a wide range of high-profile organisations including the National Portrait Gallery, the Victoria and Albert Museum, Sotheby's New York, Momart Ltd and John Lewis.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>At Essex, you will acquire a broad foundation in the history of visual culture: both by learning about canonical forms of art and architecture and by discovering what has been overlooked or marginalised, such as medical photography, tattoos or objects from political protests. You will also develop the skills you need to make exciting new connections between the forms of visual culture you study, developments in other disciplines, and broader social and political forces. To study on our course, you don't need an Art History A-Level. In fact, we believe that the best art historians are those who bring fresh eyes and new perspectives to their objects of inquiry. You will develop the skills you need to transform your excitement about art, architecture and visual culture into the ability to uncover new insights about the material you study. You will also develop a solid grounding in the history of art and other forms of visual culture, including the ideas and forces that shaped their production, distribution and reception. For students with a particular interest in pursuing careers in curating and museumship, we provide modules that explore the histories, theories and practices of museums, exhibitions and galleries, as well as practical issues such as installing and marketing artwork. The visual arts and culture industries have become an increasingly significant part of the national and international economy, and our art history graduates leave Essex with the skills to take advantage of this growing opportunity. Some of the sectors with jobs well suited for our graduates include museums and galleries, auction houses, education in schools, universities and cultural institutions, marketing and advertising, and new media. Our degree also prepares students to run their own galleries, to work as specialist arts lawyers and PR agents, and for positions in charities, fashion and publishing. Our recent graduates have gone on to work for a wide range of high-profile organisations including the National Portrait Gallery, the Victoria and Albert Museum, Sotheby's New York, Momart Ltd and John Lewis.</t>
+          <t>BA History of Art is a wide-ranging degree which explores art history and visual culture from the Medieval era to the present. As you progress to Years 2 and 3, tailor your studies by selecting pathways of study that align with your interests. The range of staff expertise offers you the opportunity to study a varied and exciting curriculum. We provide a wide selection of subject areas, paired with in-depth research and study. Our expertise lies in Medieval, Renaissance, Post-Renaissance, Modern, Contemporary and Global art history. Additionally, we benefit from the expertise of faculty members within the Institute of Cultural Practice. Course units cover topics such as the study of museums as institutions, collecting, practical aspects of curating and exhibition-making, and art writing. The Manchester Museum and the Whitworth Art Gallery offer access to the environment of the working museum and art gallery as well as to important works of art, and the Whitworth’s collections of paintings, prints, textiles and wallpapers are used extensively in teaching. Students also benefit from the University Library and the Special Collections Department at the John Rylands Library, which holds significant collections of rare books, manuscripts and illustrated materials relevant to Art History. A degree in Art History equips students with intellectual and practical skills for analysing visual culture and interpreting images in contemporary society. Recent graduates have pursued careers across a range of sectors, with roles including Education Officer at the De Morgan Collection, Royal Collections Exhibitions Curator, Archivist at Tate Liverpool and Art Officer at English Heritage.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BA History of Art is a wide-ranging degree which explores art history and visual culture from the Medieval era to the present. As you progress to Years 2 and 3, tailor your studies by selecting pathways of study that align with your interests. The range of staff expertise offers you the opportunity to study a varied and exciting curriculum. We provide a wide selection of subject areas, paired with in-depth research and study. Our expertise lies in Medieval, Renaissance, Post-Renaissance, Modern, Contemporary and Global art history. Additionally, we benefit from the expertise of faculty members within the Institute of Cultural Practice. Course units cover topics such as the study of museums as institutions, collecting, practical aspects of curating and exhibition-making, and art writing. The Manchester Museum and the Whitworth Art Gallery offer access to the environment of the working museum and art gallery as well as to important works of art, and the Whitworth’s collections of paintings, prints, textiles and wallpapers are used extensively in teaching. Students also benefit from the University Library and the Special Collections Department at the John Rylands Library, which holds significant collections of rare books, manuscripts and illustrated materials relevant to Art History. A degree in Art History equips students with intellectual and practical skills for analysing visual culture and interpreting images in contemporary society. Recent graduates have pursued careers across a range of sectors, with roles including Education Officer at the De Morgan Collection, Royal Collections Exhibitions Curator, Archivist at Tate Liverpool and Art Officer at English Heritage.</t>
+          <t>Studying the history of art is like a journey through time, giving insights into human creativity, cultural evolution, and the timeless dialogue between artists and society. The study of the history of art unveils human creativity and expression. It also promotes critical analytical skills, an understanding of cultural contexts, and a deep appreciation for visual storytelling. Studying the history of art opens up many career opportunities like art curation, museum management, art conservation, education, art and cultural consultancy. The ability to interpret visual pieces is valuable in sectors where creativity, cultural understanding, and a discerning eye are essential. Museums and society, making and meaning in architecture, reading art history, making and meaning in western art, modern British art and art and the environment are areas you could study. Comparative art analysis, visual analysis, historical knowledge and museum and gallery practices are hard skills you’ll develop. Attention to detail, creativity, flexibility, curiosity and open-mindedness are soft skills you’ll develop. Career options include artists, arts officers, producers and directors, conservators and curators, and librarians.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
-        <is>
-          <t>Studying the history of art is like a journey through time, giving insights into human creativity, cultural evolution, and the timeless dialogue between artists and society. The study of the history of art unveils human creativity and expression. It also promotes critical analytical skills, an understanding of cultural contexts, and a deep appreciation for visual storytelling. Studying the history of art opens up many career opportunities like art curation, museum management, art conservation, education, art and cultural consultancy. The ability to interpret visual pieces is valuable in sectors where creativity, cultural understanding, and a discerning eye are essential. Museums and society, making and meaning in architecture, reading art history, making and meaning in western art, modern British art and art and the environment are areas you could study. Comparative art analysis, visual analysis, historical knowledge and museum and gallery practices are hard skills you’ll develop. Attention to detail, creativity, flexibility, curiosity and open-mindedness are soft skills you’ll develop. Career options include artists, arts officers, producers and directors, conservators and curators, and librarians.</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
         <is>
           <t>Essex: At Essex, you will acquire a broad foundation in the history of visual culture: both by learning about canonical forms of art and architecture and by discovering what has been overlooked or marginalised, such as medical photography, tattoos or objects from political protests. You will also develop the skills you need to make exciting new connections between the forms of visual culture you study, developments in other disciplines, and broader social and political forces. To study on our course, you don't need an Art History A-Level. In fact, we believe that the best art historians are those who bring fresh eyes and new perspectives to their objects of inquiry. You will develop the skills you need to transform your excitement about art, architecture and visual culture into the ability to uncover new insights about the material you study. You will also develop a solid grounding in the history of art and other forms of visual culture, including the ideas and forces that shaped their production, distribution and reception. For students with a particular interest in pursuing careers in curating and museumship, we provide modules that explore the histories, theories and practices of museums, exhibitions and galleries, as well as practical issues such as installing and marketing artwork. The visual arts and culture industries have become an increasingly significant part of the national and international economy, and our art history graduates leave Essex with the skills to take advantage of this growing opportunity. Some of the sectors with jobs well suited for our graduates include museums and galleries, auction houses, education in schools, universities and cultural institutions, marketing and advertising, and new media. Our degree also prepares students to run their own galleries, to work as specialist arts lawyers and PR agents, and for positions in charities, fashion and publishing. Our recent graduates have gone on to work for a wide range of high-profile organisations including the National Portrait Gallery, the Victoria and Albert Museum, Sotheby's New York, Momart Ltd and John Lewis.
 Manchester: BA History of Art is a wide-ranging degree which explores art history and visual culture from the Medieval era to the present. As you progress to Years 2 and 3, tailor your studies by selecting pathways of study that align with your interests. The range of staff expertise offers you the opportunity to study a varied and exciting curriculum. We provide a wide selection of subject areas, paired with in-depth research and study. Our expertise lies in Medieval, Renaissance, Post-Renaissance, Modern, Contemporary and Global art history. Additionally, we benefit from the expertise of faculty members within the Institute of Cultural Practice. Course units cover topics such as the study of museums as institutions, collecting, practical aspects of curating and exhibition-making, and art writing. The Manchester Museum and the Whitworth Art Gallery offer access to the environment of the working museum and art gallery as well as to important works of art, and the Whitworth’s collections of paintings, prints, textiles and wallpapers are used extensively in teaching. Students also benefit from the University Library and the Special Collections Department at the John Rylands Library, which holds significant collections of rare books, manuscripts and illustrated materials relevant to Art History. A degree in Art History equips students with intellectual and practical skills for analysing visual culture and interpreting images in contemporary society. Recent graduates have pursued careers across a range of sectors, with roles including Education Officer at the De Morgan Collection, Royal Collections Exhibitions Curator, Archivist at Tate Liverpool and Art Officer at English Heritage.
@@ -593,21 +572,16 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Applied Biomedical Science; Biochemistry; Biochemistry and Biotechnology; Biomedical Science</t>
+          <t>The BSc (Hons) Biochemistry is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll secure a strong understanding of biochemistry and biomolecules through computational approaches and bioinformatics. The BSc (Hons) Biochemistry lets you explore molecular enzymology, neurodegeneration, structural biology and bioenergetics, and you can expand your study into biomedical science, biotechnology and bioinformatics. Previous students have placed with organisations including GlaxoSmithKline (GSK), Proctor &amp; Gamble (P&amp;G), AquaTerra, AstraZeneca, Genzyme, Reckitt Benckiser, Thermo Fisher and Isogenica. You’ll graduate on the path to a career in biomedical science, biotechnology and other specialisms of biological sciences. This course is suitable for future biochemists and biochemistry researchers, those wanting to further our modern understanding of the complex cellular and molecular world, and practical learners wanting hands-on experience. In the first year you explore biochemistry, molecular cell biology, genetics and microbiology. You study areas such as enzymology, bioenergetics and macromolecular assemblies, and develop employability and transferable skills for the biosciences while tailoring your degree through a choice of applied modules. A BSc (Hons) Biochemistry degree prepares you for diverse careers including biotechnology and forensic science in biology, pharmacology and biomedical science in health, postgraduate medicine programmes, postgraduate research programmes, and primary and secondary science and biology teaching.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>The BSc (Hons) Biochemistry is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll secure a strong understanding of biochemistry and biomolecules through computational approaches and bioinformatics. The BSc (Hons) Biochemistry lets you explore molecular enzymology, neurodegeneration, structural biology and bioenergetics, and you can expand your study into biomedical science, biotechnology and bioinformatics. Previous students have placed with organisations including GlaxoSmithKline (GSK), Proctor &amp; Gamble (P&amp;G), AquaTerra, AstraZeneca, Genzyme, Reckitt Benckiser, Thermo Fisher and Isogenica. You’ll graduate on the path to a career in biomedical science, biotechnology and other specialisms of biological sciences. This course is suitable for future biochemists and biochemistry researchers, those wanting to further our modern understanding of the complex cellular and molecular world, and practical learners wanting hands-on experience. In the first year you explore biochemistry, molecular cell biology, genetics and microbiology. You study areas such as enzymology, bioenergetics and macromolecular assemblies, and develop employability and transferable skills for the biosciences while tailoring your degree through a choice of applied modules. A BSc (Hons) Biochemistry degree prepares you for diverse careers including biotechnology and forensic science in biology, pharmacology and biomedical science in health, postgraduate medicine programmes, postgraduate research programmes, and primary and secondary science and biology teaching.</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
           <t>Our BSc Biochemistry course will give you a grounding in a subject that forms the basis of virtually all of the biological sciences. Many exciting discoveries made in this area have contributed to our understanding of life, the solving of medical problems, and to the discovery and production of safe and effective drugs. You will learn about topics such as the structure of biomolecules and how they interact in essential processes and pathways in our cells. You will also study the actions of enzymes and how they can be inhibited by drugs, as well as genetic engineering and molecular biology. You will benefit from lectures, tutorials, practicals and research projects, including the final year project. A significant part of the final year is the project, which is assessed through a presentation and a written report. Our modern teaching laboratories are equipped for a range of biological and biomedical techniques including polymerase chain reaction (PCR), DNA sequencing, gel electrophoresis, spectrophotometry, electroencephalography (EEG), electrocardiography (ECG) and immunofluorescence microscopy. As a final year student, you have the opportunity to undertake a research project in the laboratories of bioscience researchers supported by extensive research facilities and advanced technology. Our graduates go into a wide range of sectors, with around one-third working in scientific research and development, often progressing to postgraduate study such as a PhD and careers as researchers at universities, pharmaceutical and bioscience companies and institutes. Other graduates pursue diverse careers including teaching, science communication, management, finance, marketing and the civil service.</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
         <is>
           <t>Essex: The BSc (Hons) Biochemistry is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll secure a strong understanding of biochemistry and biomolecules through computational approaches and bioinformatics. The BSc (Hons) Biochemistry lets you explore molecular enzymology, neurodegeneration, structural biology and bioenergetics, and you can expand your study into biomedical science, biotechnology and bioinformatics. Previous students have placed with organisations including GlaxoSmithKline (GSK), Proctor &amp; Gamble (P&amp;G), AquaTerra, AstraZeneca, Genzyme, Reckitt Benckiser, Thermo Fisher and Isogenica. You’ll graduate on the path to a career in biomedical science, biotechnology and other specialisms of biological sciences. This course is suitable for future biochemists and biochemistry researchers, those wanting to further our modern understanding of the complex cellular and molecular world, and practical learners wanting hands-on experience. In the first year you explore biochemistry, molecular cell biology, genetics and microbiology. You study areas such as enzymology, bioenergetics and macromolecular assemblies, and develop employability and transferable skills for the biosciences while tailoring your degree through a choice of applied modules. A BSc (Hons) Biochemistry degree prepares you for diverse careers including biotechnology and forensic science in biology, pharmacology and biomedical science in health, postgraduate medicine programmes, postgraduate research programmes, and primary and secondary science and biology teaching.
 Manchester: Our BSc Biochemistry course will give you a grounding in a subject that forms the basis of virtually all of the biological sciences. Many exciting discoveries made in this area have contributed to our understanding of life, the solving of medical problems, and to the discovery and production of safe and effective drugs. You will learn about topics such as the structure of biomolecules and how they interact in essential processes and pathways in our cells. You will also study the actions of enzymes and how they can be inhibited by drugs, as well as genetic engineering and molecular biology. You will benefit from lectures, tutorials, practicals and research projects, including the final year project. A significant part of the final year is the project, which is assessed through a presentation and a written report. Our modern teaching laboratories are equipped for a range of biological and biomedical techniques including polymerase chain reaction (PCR), DNA sequencing, gel electrophoresis, spectrophotometry, electroencephalography (EEG), electrocardiography (ECG) and immunofluorescence microscopy. As a final year student, you have the opportunity to undertake a research project in the laboratories of bioscience researchers supported by extensive research facilities and advanced technology. Our graduates go into a wide range of sectors, with around one-third working in scientific research and development, often progressing to postgraduate study such as a PhD and careers as researchers at universities, pharmaceutical and bioscience companies and institutes. Other graduates pursue diverse careers including teaching, science communication, management, finance, marketing and the civil service.</t>
@@ -623,23 +597,22 @@
           <t>BIOLOGICAL SCIENCES</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>What is the BSc (Hons) Biological Sciences? The BSc (Hons) Biological Sciences is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll secure a broad understanding of modern biology and a strong basis to specialise from, in your undergraduate degree or beyond. The BSc (Hons) Biological Sciences lets you explore the spectrum of biology and choose what to specialise in. Your first year offers broad insights into cell and molecular biology, genetics, ecology and evolution. For your second and final years, you can deepen your knowledge across disciplines or specialise in an area of your choosing, from molecular and cell biology to ecology and conservation biology. Previous students have placed with GlaxoSmithKline (GSK), Proctor &amp; Gamble (P&amp;G), AquaTerra, AstraZeneca, Genzyme, Reckitt Benckiser, Thermo Fisher and Isogenica, some of our 40 partner labs. You’ll graduate on the path to a biologist career in a range of specialisms, such as marine biology, conservation and molecular biology. In Year One you explore molecular cell biology, genetics, ecology and microbiology. You can choose employability skills for the biosciences or professional skills for ecology and marine scientists and tailor the last two years of your degree through your choice of applied modules. A BSc (Hons) Biological Sciences degree prepares you for diverse careers in areas such as biotechnology, microbiology, genetics and forensic science; ecology, marine biology, nature conservation, water quality and soil analysis; pharmacology, biomedical science and clinical science; postgraduate research programmes; and primary and secondary science and biology teaching. Graduates from this course have progressed to roles in organisations including GlaxoSmithKline (GSK), Sainsbury Laboratory (University of Cambridge), ALS Laboratories, the NHS, Essex Wildlife Trust, Natural England and Suffolk County Council.</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>What is the BSc (Hons) Biological Sciences? The BSc (Hons) Biological Sciences is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll secure a broad understanding of modern biology and a strong basis to specialise from, in your undergraduate degree or beyond. The BSc (Hons) Biological Sciences lets you explore the spectrum of biology and choose what to specialise in. Your first year offers broad insights into cell and molecular biology, genetics, ecology and evolution. For your second and final years, you can deepen your knowledge across disciplines or specialise in an area of your choosing, from molecular and cell biology to ecology and conservation biology. Previous students have placed with GlaxoSmithKline (GSK), Proctor &amp; Gamble (P&amp;G), AquaTerra, AstraZeneca, Genzyme, Reckitt Benckiser, Thermo Fisher and Isogenica, some of our 40 partner labs. You’ll graduate on the path to a biologist career in a range of specialisms, such as marine biology, conservation and molecular biology. In Year One you explore molecular cell biology, genetics, ecology and microbiology. You can choose employability skills for the biosciences or professional skills for ecology and marine scientists and tailor the last two years of your degree through your choice of applied modules. A BSc (Hons) Biological Sciences degree prepares you for diverse careers in areas such as biotechnology, microbiology, genetics and forensic science; ecology, marine biology, nature conservation, water quality and soil analysis; pharmacology, biomedical science and clinical science; postgraduate research programmes; and primary and secondary science and biology teaching. Graduates from this course have progressed to roles in organisations including GlaxoSmithKline (GSK), Sainsbury Laboratory (University of Cambridge), ALS Laboratories, the NHS, Essex Wildlife Trust, Natural England and Suffolk County Council.</t>
+          <t>Our BSc Biology course covers a diverse range of topics within the study of living organisms, allowing you to discover areas of interest early on in your degree and choose what you want to focus on. You can keep your options open and cover a wide variety of areas, or identify those that interest you and focus on particular biological topics. Interdisciplinarity is encouraged, and you have the opportunity to enrol on courses at the University College for Interdisciplinary Learning in the second and third year. Our modern teaching labs are equipped for a range of biological and biomedical techniques, including polymerase chain reaction (PCR), DNA sequencing, gel electrophoresis, spectrophotometry, dissection and histology, electroencephalography (EEG), electrocardiography (ECG) and immunofluorescence microscopy. As a final year student, you have the opportunity to undertake a project in the labs of our bioscience researchers. Our graduates go into a range of careers, with around one-third working in scientific research and development, which may require postgraduate study such as a PhD, while others pursue careers in teaching or communicating science, conservation and ecological consultancy, biotechnology and biomedical companies, as well as roles outside biological sciences including management, finance, marketing and the civil service.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Our BSc Biology course covers a diverse range of topics within the study of living organisms, allowing you to discover areas of interest early on in your degree and choose what you want to focus on. You can keep your options open and cover a wide variety of areas, or identify those that interest you and focus on particular biological topics. Interdisciplinarity is encouraged, and you have the opportunity to enrol on courses at the University College for Interdisciplinary Learning in the second and third year. Our modern teaching labs are equipped for a range of biological and biomedical techniques, including polymerase chain reaction (PCR), DNA sequencing, gel electrophoresis, spectrophotometry, dissection and histology, electroencephalography (EEG), electrocardiography (ECG) and immunofluorescence microscopy. As a final year student, you have the opportunity to undertake a project in the labs of our bioscience researchers. Our graduates go into a range of careers, with around one-third working in scientific research and development, which may require postgraduate study such as a PhD, while others pursue careers in teaching or communicating science, conservation and ecological consultancy, biotechnology and biomedical companies, as well as roles outside biological sciences including management, finance, marketing and the civil service.</t>
+          <t>Studying biology will unravel the complexities of life, from the tiniest cells to the grandest ecosystems, to discover the science that underlies the wonders of the natural world. Biology is the study of life in all its forms, from microscopic organisms to complex ecosystems. It covers a wide range of topics, including genetics, ecology, physiology and evolution, giving an overall understanding of the natural world. Biology opens doors to diverse career paths, including roles in research, healthcare, environmental conservation and education. You could explore careers such as research scientists, environmental consultants, healthcare professionals, educators or science communicators. Ecology, anatomy and physiology, biochemistry and biotechnology, genetics, molecular biology, immunology and plant physiology are areas you could study. Hands-on experience in laboratory techniques such as pipetting, microscopy and DNA extraction, data analysis and statistical interpretation, and skills in conducting observations, collecting samples and recording data in natural environments are hard skills you’ll develop. Critical thinking, attention to detail, patience and perseverance and ethical reasoning are soft skills you’ll develop. Career options include biological scientists, natural and social science professionals, laboratory technicians, conservation professionals and environment professionals.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
-        <is>
-          <t>Studying biology will unravel the complexities of life, from the tiniest cells to the grandest ecosystems, to discover the science that underlies the wonders of the natural world. Biology is the study of life in all its forms, from microscopic organisms to complex ecosystems. It covers a wide range of topics, including genetics, ecology, physiology and evolution, giving an overall understanding of the natural world. Biology opens doors to diverse career paths, including roles in research, healthcare, environmental conservation and education. You could explore careers such as research scientists, environmental consultants, healthcare professionals, educators or science communicators. Ecology, anatomy and physiology, biochemistry and biotechnology, genetics, molecular biology, immunology and plant physiology are areas you could study. Hands-on experience in laboratory techniques such as pipetting, microscopy and DNA extraction, data analysis and statistical interpretation, and skills in conducting observations, collecting samples and recording data in natural environments are hard skills you’ll develop. Critical thinking, attention to detail, patience and perseverance and ethical reasoning are soft skills you’ll develop. Career options include biological scientists, natural and social science professionals, laboratory technicians, conservation professionals and environment professionals.</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
         <is>
           <t>Essex: What is the BSc (Hons) Biological Sciences? The BSc (Hons) Biological Sciences is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll secure a broad understanding of modern biology and a strong basis to specialise from, in your undergraduate degree or beyond. The BSc (Hons) Biological Sciences lets you explore the spectrum of biology and choose what to specialise in. Your first year offers broad insights into cell and molecular biology, genetics, ecology and evolution. For your second and final years, you can deepen your knowledge across disciplines or specialise in an area of your choosing, from molecular and cell biology to ecology and conservation biology. Previous students have placed with GlaxoSmithKline (GSK), Proctor &amp; Gamble (P&amp;G), AquaTerra, AstraZeneca, Genzyme, Reckitt Benckiser, Thermo Fisher and Isogenica, some of our 40 partner labs. You’ll graduate on the path to a biologist career in a range of specialisms, such as marine biology, conservation and molecular biology. In Year One you explore molecular cell biology, genetics, ecology and microbiology. You can choose employability skills for the biosciences or professional skills for ecology and marine scientists and tailor the last two years of your degree through your choice of applied modules. A BSc (Hons) Biological Sciences degree prepares you for diverse careers in areas such as biotechnology, microbiology, genetics and forensic science; ecology, marine biology, nature conservation, water quality and soil analysis; pharmacology, biomedical science and clinical science; postgraduate research programmes; and primary and secondary science and biology teaching. Graduates from this course have progressed to roles in organisations including GlaxoSmithKline (GSK), Sainsbury Laboratory (University of Cambridge), ALS Laboratories, the NHS, Essex Wildlife Trust, Natural England and Suffolk County Council.
 Manchester: Our BSc Biology course covers a diverse range of topics within the study of living organisms, allowing you to discover areas of interest early on in your degree and choose what you want to focus on. You can keep your options open and cover a wide variety of areas, or identify those that interest you and focus on particular biological topics. Interdisciplinarity is encouraged, and you have the opportunity to enrol on courses at the University College for Interdisciplinary Learning in the second and third year. Our modern teaching labs are equipped for a range of biological and biomedical techniques, including polymerase chain reaction (PCR), DNA sequencing, gel electrophoresis, spectrophotometry, dissection and histology, electroencephalography (EEG), electrocardiography (ECG) and immunofluorescence microscopy. As a final year student, you have the opportunity to undertake a project in the labs of our bioscience researchers. Our graduates go into a range of careers, with around one-third working in scientific research and development, which may require postgraduate study such as a PhD, while others pursue careers in teaching or communicating science, conservation and ecological consultancy, biotechnology and biomedical companies, as well as roles outside biological sciences including management, finance, marketing and the civil service.
@@ -658,21 +631,16 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Accounting and Management; Business Administration; Business Administration and Supply Chain Management; Business Economics; Business Management; Business Management with a Modern Language; Events Management; Events Management with Hospitality; Finance and Management; Hospitality Management; Hotel Management; International Business and Entrepreneurship; Law with Business; Marketing Management; Philosophy with Business Management; Politics with Business</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
           <t>Businesses need effective managers now more than ever in a post Covid-19 world. But what makes an effective manager? And how can studying management theory create better managers for people and the planet? On this course, you learn what's involved in managing organisations in an increasingly complex world. We look at the enduring patterns in how people, groups, organisations, economies and societies function and interact. By understanding these behaviours, you can manage them effectively in times of significant change. With BSc Business Management, you gain a rich understanding of how organisations operate – what they do, how they develop strategies and why. Study areas include management, innovation and new technologies, the international business environment, organisational behaviour, operations and supply chain management, leadership, human resource management and ethical business management. The first year of your business management degree also introduces you to the core principles of accounting, finance and marketing to provide you with the essential business knowledge needed for a successful career. In your final year, you have the opportunity to put your knowledge into practice by completing an in-depth, independent research project or dissertation. This will give you the chance to further develop vital employability skills in areas of research, time management and critical thinking. This course is taught at Essex Business School. We champion responsible management and ethical business practices; you join a school not just committed to excellence in business education and social science research, but an intellectual community working to make business better. We don't just prepare you for a successful career; we'll help you shape the kind of world you want to live in. Business management skills are as highly valued as your degree by many graduate employers, therefore we embed a series of core and specific skills into our undergraduate curriculum for BSc Business Management to ensure that our graduates are suited to careers in business management and leadership roles. All of our taught modules embed elements of our skills map which emulate the skills required by employers of business graduates, including academic and cognitive skills, research skills, technology skills, communication skills, data analysis skills and soft skills. Our students have gone on to become business analysts, successful entrepreneurs, account managers and management trainees, with recent graduate destinations including CEO and Founders of WYSPR – a ‘Friendvertising' social media start-up, Business Development Manager at Footprint Digital – a digital marketing agency, Sales and Marketing Manager at Chrysodalia – a food manufacturing company, Digital Marketing Executive at Premier Labellers – a machinery manufacturer, Delivery Consultant at RED – The Global SAP Solutions Provider, and iX Business Consultant at IBM.</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Dive into the world of business and management, where every challenge is an opportunity, and every decision is another step forward to organisational success. Choosing business and management will give you a versatile skill set covering strategic planning, leadership and problem-solving, all essential for navigating the corporate world. This popular field opens doors into dynamic careers spanning corporate management, consulting, finance, marketing and entrepreneurship. Armed with a degree in business and management, individuals become catalysts for organisational growth, driving innovation, leading teams and shaping the strategic landscape of multiple sectors and industries on a global scale. Leadership, finance, marketing, entrepreneurship, management theory, human resources, strategy and market analysis are areas you could study. Strategic planning, market research and analysis, negotiation and conflict resolution, and entrepreneurship and innovation are hard skills you’ll develop. Communication, team collaboration, project management and networking are soft skills you’ll develop. Career options include chief executives and senior officials, financial managers and directors, purchasing managers and directors, human resource managers and directors, marketing and sales directors, advertising and public relations directors, business and related associate professionals, office managers, business and financial project management professionals and financial accounts managers.</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
-        <is>
-          <t>Dive into the world of business and management, where every challenge is an opportunity, and every decision is another step forward to organisational success. Choosing business and management will give you a versatile skill set covering strategic planning, leadership and problem-solving, all essential for navigating the corporate world. This popular field opens doors into dynamic careers spanning corporate management, consulting, finance, marketing and entrepreneurship. Armed with a degree in business and management, individuals become catalysts for organisational growth, driving innovation, leading teams and shaping the strategic landscape of multiple sectors and industries on a global scale. Leadership, finance, marketing, entrepreneurship, management theory, human resources, strategy and market analysis are areas you could study. Strategic planning, market research and analysis, negotiation and conflict resolution, and entrepreneurship and innovation are hard skills you’ll develop. Communication, team collaboration, project management and networking are soft skills you’ll develop. Career options include chief executives and senior officials, financial managers and directors, purchasing managers and directors, human resource managers and directors, marketing and sales directors, advertising and public relations directors, business and related associate professionals, office managers, business and financial project management professionals and financial accounts managers.</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
         <is>
           <t>Essex: Businesses need effective managers now more than ever in a post Covid-19 world. But what makes an effective manager? And how can studying management theory create better managers for people and the planet? On this course, you learn what's involved in managing organisations in an increasingly complex world. We look at the enduring patterns in how people, groups, organisations, economies and societies function and interact. By understanding these behaviours, you can manage them effectively in times of significant change. With BSc Business Management, you gain a rich understanding of how organisations operate – what they do, how they develop strategies and why. Study areas include management, innovation and new technologies, the international business environment, organisational behaviour, operations and supply chain management, leadership, human resource management and ethical business management. The first year of your business management degree also introduces you to the core principles of accounting, finance and marketing to provide you with the essential business knowledge needed for a successful career. In your final year, you have the opportunity to put your knowledge into practice by completing an in-depth, independent research project or dissertation. This will give you the chance to further develop vital employability skills in areas of research, time management and critical thinking. This course is taught at Essex Business School. We champion responsible management and ethical business practices; you join a school not just committed to excellence in business education and social science research, but an intellectual community working to make business better. We don't just prepare you for a successful career; we'll help you shape the kind of world you want to live in. Business management skills are as highly valued as your degree by many graduate employers, therefore we embed a series of core and specific skills into our undergraduate curriculum for BSc Business Management to ensure that our graduates are suited to careers in business management and leadership roles. All of our taught modules embed elements of our skills map which emulate the skills required by employers of business graduates, including academic and cognitive skills, research skills, technology skills, communication skills, data analysis skills and soft skills. Our students have gone on to become business analysts, successful entrepreneurs, account managers and management trainees, with recent graduate destinations including CEO and Founders of WYSPR – a ‘Friendvertising' social media start-up, Business Development Manager at Footprint Digital – a digital marketing agency, Sales and Marketing Manager at Chrysodalia – a food manufacturing company, Digital Marketing Executive at Premier Labellers – a machinery manufacturer, Delivery Consultant at RED – The Global SAP Solutions Provider, and iX Business Consultant at IBM.
 UCAS: Dive into the world of business and management, where every challenge is an opportunity, and every decision is another step forward to organisational success. Choosing business and management will give you a versatile skill set covering strategic planning, leadership and problem-solving, all essential for navigating the corporate world. This popular field opens doors into dynamic careers spanning corporate management, consulting, finance, marketing and entrepreneurship. Armed with a degree in business and management, individuals become catalysts for organisational growth, driving innovation, leading teams and shaping the strategic landscape of multiple sectors and industries on a global scale. Leadership, finance, marketing, entrepreneurship, management theory, human resources, strategy and market analysis are areas you could study. Strategic planning, market research and analysis, negotiation and conflict resolution, and entrepreneurship and innovation are hard skills you’ll develop. Communication, team collaboration, project management and networking are soft skills you’ll develop. Career options include chief executives and senior officials, financial managers and directors, purchasing managers and directors, human resource managers and directors, marketing and sales directors, advertising and public relations directors, business and related associate professionals, office managers, business and financial project management professionals and financial accounts managers.</t>
@@ -690,25 +658,20 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Computer Games</t>
+          <t>What is the BSc (Hons) Computer Science? The BSc (Hons) Computer Science is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll build a strong foundation in core computer science theory and explore its cutting-edge real-world applications, preparing you to create the technologies of tomorrow. Why this course The BSc (Hons) Computer Science gives you the theory and practical knowledge to understand – and create – computing technologies that make a real impact on the world. You’ll study a broad curriculum shaped by industry partners, gaining the most up-to-date understanding of computer science. Discover which areas you’re interested in exploring further, then specialise in assistive technologies, computer games, artificial intelligence, evolutionary computation, Big Data or robotics. By graduation, you’ll have the confidence and ability to dig deeper into how technology influences people’s lives. You’ll be ready for careers in software and systems analysis, engineering and programming. Who should apply Future software analysts and programmers, students eager to develop their own computer games, apps, online platforms and digital systems, those considering a career that benefits from a broad understanding of how computers and digital systems work, and computational thinkers with a great grasp of pattern recognition and algorithms. What you’ll learn Programming: learn to programme with multiple programming languages. Data: explore ways to work with data from data structures to Big Data. Web: understand the principles and technology behind web apps and websites. Digital systems: grasp the software and hardware underpinning digital computer systems. Your learning experience includes optional modules that allow you to tailor your degree and specialise in areas such as artificial intelligence, computer games and security. Careers and outcomes A BSc (Hons) Computer Science degree prepares you for diverse careers in IT including computer and information research, computer network architecture, database systems administration and security analysis; healthcare including health information technology, clinical data and systems administration; business and finance including financial analysis, data analysis, risk management and web development; energy including energy generation and distribution systems, data analysis and technological improvement; and computer games development and programming. Employers of graduates from this course include American Express, Red Bull Racing, JP Morgan, BT, Blizzard, Google, Formula One, IBM and Royal Bank of Scotland. Professional accreditation Accredited by BCS, the Chartered Institute for IT for the purposes of fully meeting the academic requirement for registration as a Chartered IT Professional. Accredited by BCS, the Chartered Institute for IT on behalf of the Engineering Council for the purposes of fully meeting the academic requirement for Incorporated Engineer and partially meeting the academic requirement for a Chartered Engineer. Accredited by the Institution of Engineering and Technology (IET) on behalf of the Engineering Council for the purposes of fully meeting the academic requirement for registration as an Incorporated Engineer and partially meeting the academic requirement for registration as a Chartered Engineer.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>What is the BSc (Hons) Computer Science? The BSc (Hons) Computer Science is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll build a strong foundation in core computer science theory and explore its cutting-edge real-world applications, preparing you to create the technologies of tomorrow. Why this course The BSc (Hons) Computer Science gives you the theory and practical knowledge to understand – and create – computing technologies that make a real impact on the world. You’ll study a broad curriculum shaped by industry partners, gaining the most up-to-date understanding of computer science. Discover which areas you’re interested in exploring further, then specialise in assistive technologies, computer games, artificial intelligence, evolutionary computation, Big Data or robotics. By graduation, you’ll have the confidence and ability to dig deeper into how technology influences people’s lives. You’ll be ready for careers in software and systems analysis, engineering and programming. Who should apply Future software analysts and programmers, students eager to develop their own computer games, apps, online platforms and digital systems, those considering a career that benefits from a broad understanding of how computers and digital systems work, and computational thinkers with a great grasp of pattern recognition and algorithms. What you’ll learn Programming: learn to programme with multiple programming languages. Data: explore ways to work with data from data structures to Big Data. Web: understand the principles and technology behind web apps and websites. Digital systems: grasp the software and hardware underpinning digital computer systems. Your learning experience includes optional modules that allow you to tailor your degree and specialise in areas such as artificial intelligence, computer games and security. Careers and outcomes A BSc (Hons) Computer Science degree prepares you for diverse careers in IT including computer and information research, computer network architecture, database systems administration and security analysis; healthcare including health information technology, clinical data and systems administration; business and finance including financial analysis, data analysis, risk management and web development; energy including energy generation and distribution systems, data analysis and technological improvement; and computer games development and programming. Employers of graduates from this course include American Express, Red Bull Racing, JP Morgan, BT, Blizzard, Google, Formula One, IBM and Royal Bank of Scotland. Professional accreditation Accredited by BCS, the Chartered Institute for IT for the purposes of fully meeting the academic requirement for registration as a Chartered IT Professional. Accredited by BCS, the Chartered Institute for IT on behalf of the Engineering Council for the purposes of fully meeting the academic requirement for Incorporated Engineer and partially meeting the academic requirement for a Chartered Engineer. Accredited by the Institution of Engineering and Technology (IET) on behalf of the Engineering Council for the purposes of fully meeting the academic requirement for registration as an Incorporated Engineer and partially meeting the academic requirement for registration as a Chartered Engineer.</t>
+          <t>Through the development of new applications in science, engineering, and business, Computer Science is radically changing the way in which we experience our world. This programme equips students with the skills needed to contribute to this exciting and rapidly evolving field. Computer Science is our most flexible programme, allowing you to choose course units to reflect your developing and changing interests, with a wide range of themes from across the discipline allowing you to specialise in the second and third years. You will gain not only knowledge and practical experience of the latest technologies, but also a grounding in the underlying principles of the subject. It is this combination of skills that enables graduates to keep pace with this fast-moving subject and secure rewarding careers that can be pursued almost anywhere in the world. The programme provides a broad and flexible structure that allows students to choose from a wide range of Computer Science topics while developing skills that are highly valued by industry. Graduates pursue careers in roles such as actuary, AI engineer, banker, cloud computing engineer, cyber security analyst, data analyst, games designer or developer, software engineer, and web designer or developer, working across sectors including finance, films and games, pharmaceuticals, healthcare, consumer products and public services. Employers that recruit graduates include organisations such as CERN, EA Games, IBM and Microsoft. This degree has been accredited by the British Computer Society (BCS), The Chartered Institute for IT, under licence from the Engineering Council. Accreditation confirms that the degree meets the standards set by the Engineering Council in the UK Standard for Professional Engineering Competence and provides the underpinning knowledge and skills required for registration as a Chartered IT Professional (CITP), Chartered Engineer (CEng) or Incorporated Engineer (IEng).</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Through the development of new applications in science, engineering, and business, Computer Science is radically changing the way in which we experience our world. This programme equips students with the skills needed to contribute to this exciting and rapidly evolving field. Computer Science is our most flexible programme, allowing you to choose course units to reflect your developing and changing interests, with a wide range of themes from across the discipline allowing you to specialise in the second and third years. You will gain not only knowledge and practical experience of the latest technologies, but also a grounding in the underlying principles of the subject. It is this combination of skills that enables graduates to keep pace with this fast-moving subject and secure rewarding careers that can be pursued almost anywhere in the world. The programme provides a broad and flexible structure that allows students to choose from a wide range of Computer Science topics while developing skills that are highly valued by industry. Graduates pursue careers in roles such as actuary, AI engineer, banker, cloud computing engineer, cyber security analyst, data analyst, games designer or developer, software engineer, and web designer or developer, working across sectors including finance, films and games, pharmaceuticals, healthcare, consumer products and public services. Employers that recruit graduates include organisations such as CERN, EA Games, IBM and Microsoft. This degree has been accredited by the British Computer Society (BCS), The Chartered Institute for IT, under licence from the Engineering Council. Accreditation confirms that the degree meets the standards set by the Engineering Council in the UK Standard for Professional Engineering Competence and provides the underpinning knowledge and skills required for registration as a Chartered IT Professional (CITP), Chartered Engineer (CEng) or Incorporated Engineer (IEng).</t>
+          <t>Whether it’s finance, health, the creative industries or sport, the study of computer science helps build the technology that fuels future innovation. In today's technology-driven world, the demand for skilled computer scientists continues to grow across various industries. Studying computer science equips you with technical skills, from programming languages to algorithm design, opening a range of career opportunities. It opens doors to high-growth sectors such as cybersecurity, data science and machine learning, and the skills you’ll learn make you well-suited for roles in finance, healthcare, entertainment and beyond. Algorithms and data structures, database systems, mathematical principles, programming languages and software development, web and mobile apps, cyber security and artificial intelligence are areas you might study. Understanding programming languages, working with data structures, knowledge of algorithms and understanding cybersecurity principles are hard skills you’ll develop. Critical thinking, problem-solving attitude, adaptability and attention to detail are soft skills you’ll develop. Career options include programmers and software developers, web designers, software testers, IT network testers, electrical and electronics technicians, cyber security analysts and systems analysts.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
-        <is>
-          <t>Whether it’s finance, health, the creative industries or sport, the study of computer science helps build the technology that fuels future innovation. In today's technology-driven world, the demand for skilled computer scientists continues to grow across various industries. Studying computer science equips you with technical skills, from programming languages to algorithm design, opening a range of career opportunities. It opens doors to high-growth sectors such as cybersecurity, data science and machine learning, and the skills you’ll learn make you well-suited for roles in finance, healthcare, entertainment and beyond. Algorithms and data structures, database systems, mathematical principles, programming languages and software development, web and mobile apps, cyber security and artificial intelligence are areas you might study. Understanding programming languages, working with data structures, knowledge of algorithms and understanding cybersecurity principles are hard skills you’ll develop. Critical thinking, problem-solving attitude, adaptability and attention to detail are soft skills you’ll develop. Career options include programmers and software developers, web designers, software testers, IT network testers, electrical and electronics technicians, cyber security analysts and systems analysts.</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
         <is>
           <t>Essex: What is the BSc (Hons) Computer Science? The BSc (Hons) Computer Science is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll build a strong foundation in core computer science theory and explore its cutting-edge real-world applications, preparing you to create the technologies of tomorrow. Why this course The BSc (Hons) Computer Science gives you the theory and practical knowledge to understand – and create – computing technologies that make a real impact on the world. You’ll study a broad curriculum shaped by industry partners, gaining the most up-to-date understanding of computer science. Discover which areas you’re interested in exploring further, then specialise in assistive technologies, computer games, artificial intelligence, evolutionary computation, Big Data or robotics. By graduation, you’ll have the confidence and ability to dig deeper into how technology influences people’s lives. You’ll be ready for careers in software and systems analysis, engineering and programming. Who should apply Future software analysts and programmers, students eager to develop their own computer games, apps, online platforms and digital systems, those considering a career that benefits from a broad understanding of how computers and digital systems work, and computational thinkers with a great grasp of pattern recognition and algorithms. What you’ll learn Programming: learn to programme with multiple programming languages. Data: explore ways to work with data from data structures to Big Data. Web: understand the principles and technology behind web apps and websites. Digital systems: grasp the software and hardware underpinning digital computer systems. Your learning experience includes optional modules that allow you to tailor your degree and specialise in areas such as artificial intelligence, computer games and security. Careers and outcomes A BSc (Hons) Computer Science degree prepares you for diverse careers in IT including computer and information research, computer network architecture, database systems administration and security analysis; healthcare including health information technology, clinical data and systems administration; business and finance including financial analysis, data analysis, risk management and web development; energy including energy generation and distribution systems, data analysis and technological improvement; and computer games development and programming. Employers of graduates from this course include American Express, Red Bull Racing, JP Morgan, BT, Blizzard, Google, Formula One, IBM and Royal Bank of Scotland. Professional accreditation Accredited by BCS, the Chartered Institute for IT for the purposes of fully meeting the academic requirement for registration as a Chartered IT Professional. Accredited by BCS, the Chartered Institute for IT on behalf of the Engineering Council for the purposes of fully meeting the academic requirement for Incorporated Engineer and partially meeting the academic requirement for a Chartered Engineer. Accredited by the Institution of Engineering and Technology (IET) on behalf of the Engineering Council for the purposes of fully meeting the academic requirement for registration as an Incorporated Engineer and partially meeting the academic requirement for registration as a Chartered Engineer.
 Manchester: Through the development of new applications in science, engineering, and business, Computer Science is radically changing the way in which we experience our world. This programme equips students with the skills needed to contribute to this exciting and rapidly evolving field. Computer Science is our most flexible programme, allowing you to choose course units to reflect your developing and changing interests, with a wide range of themes from across the discipline allowing you to specialise in the second and third years. You will gain not only knowledge and practical experience of the latest technologies, but also a grounding in the underlying principles of the subject. It is this combination of skills that enables graduates to keep pace with this fast-moving subject and secure rewarding careers that can be pursued almost anywhere in the world. The programme provides a broad and flexible structure that allows students to choose from a wide range of Computer Science topics while developing skills that are highly valued by industry. Graduates pursue careers in roles such as actuary, AI engineer, banker, cloud computing engineer, cyber security analyst, data analyst, games designer or developer, software engineer, and web designer or developer, working across sectors including finance, films and games, pharmaceuticals, healthcare, consumer products and public services. Employers that recruit graduates include organisations such as CERN, EA Games, IBM and Microsoft. This degree has been accredited by the British Computer Society (BCS), The Chartered Institute for IT, under licence from the Engineering Council. Accreditation confirms that the degree meets the standards set by the Engineering Council in the UK Standard for Professional Engineering Competence and provides the underpinning knowledge and skills required for registration as a Chartered IT Professional (CITP), Chartered Engineer (CEng) or Incorporated Engineer (IEng).
@@ -727,25 +690,20 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Drama and Creative Writing; Film and Drama</t>
+          <t>Theatre is a radical and influential art form. Its roots lie deep in the ancient world but its relevance to contemporary life is urgent and ongoing. Theatre enables different cultures and societies to confront the most important issues of our time; it provides a crucial space to laugh, to dream, and dare to project different worlds. Studying theatre and drama at Essex enables you to examine some of the most influential play-texts ever written, and to be ready to take part in shaping the essential performances of tomorrow. This degree is a chance to unlock and explore your creativity. You will be performing and producing work in a professional theatre context and will be developing a wide range of creative, critical and practical skills that will open the door to a future in the theatre, cultural industries or a wide range of other graduate careers. At Essex, we offer a rich combination of practical workshops, critical seminars and lectures delivered by an experienced team of playwrights, directors and actors, as well as leading academic theatre specialists. Areas of exploration in our modules include dramatic literature from Ancient Greek tragedy and Shakespeare to modern plays from around the world, contemporary playwriting and devising techniques, staging political ideas and social justice issues, gender, identity and sexual politics on stage, creating Applied Theatre in educational and community contexts, and emergent trends in interactive performance-making and audience participation. Through classroom teaching, practical experiment and professional experience, we help you craft the skillset that will be essential in your creative development. This approach reflects our core belief that engaging with both practice and theory produces a deeper understanding of how theatre works. Creativity, communication and versatility developed during the degree prepare graduates for a wide range of careers. Our students have gone on to become actors, directors and playwrights, as well as producers, live artists, dramaturgs, stage-managers and arts managers. Graduates have also pursued careers in related creative industries including journalism, television production, broadcasting, radio presenting, gaming, magazine editing, copywriting, press relations and marketing, as well as roles in business, commerce and law. Our graduates have gone on to work in roles such as Writer in Residence for the National Theatre, Artistic Director of Jermyn Street Theatre in London, Artistic Director of a touring company, Director for the Almeida Theatre in London, Manager at a regional theatre, Live Artist for Art Angel, BBC Journalist, Youth Theatre Leader and Workshop Facilitator, Outreach and Education Officer, Front of House Theatre Manager, Stage Manager and Secondary School Teacher.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Theatre is a radical and influential art form. Its roots lie deep in the ancient world but its relevance to contemporary life is urgent and ongoing. Theatre enables different cultures and societies to confront the most important issues of our time; it provides a crucial space to laugh, to dream, and dare to project different worlds. Studying theatre and drama at Essex enables you to examine some of the most influential play-texts ever written, and to be ready to take part in shaping the essential performances of tomorrow. This degree is a chance to unlock and explore your creativity. You will be performing and producing work in a professional theatre context and will be developing a wide range of creative, critical and practical skills that will open the door to a future in the theatre, cultural industries or a wide range of other graduate careers. At Essex, we offer a rich combination of practical workshops, critical seminars and lectures delivered by an experienced team of playwrights, directors and actors, as well as leading academic theatre specialists. Areas of exploration in our modules include dramatic literature from Ancient Greek tragedy and Shakespeare to modern plays from around the world, contemporary playwriting and devising techniques, staging political ideas and social justice issues, gender, identity and sexual politics on stage, creating Applied Theatre in educational and community contexts, and emergent trends in interactive performance-making and audience participation. Through classroom teaching, practical experiment and professional experience, we help you craft the skillset that will be essential in your creative development. This approach reflects our core belief that engaging with both practice and theory produces a deeper understanding of how theatre works. Creativity, communication and versatility developed during the degree prepare graduates for a wide range of careers. Our students have gone on to become actors, directors and playwrights, as well as producers, live artists, dramaturgs, stage-managers and arts managers. Graduates have also pursued careers in related creative industries including journalism, television production, broadcasting, radio presenting, gaming, magazine editing, copywriting, press relations and marketing, as well as roles in business, commerce and law. Our graduates have gone on to work in roles such as Writer in Residence for the National Theatre, Artistic Director of Jermyn Street Theatre in London, Artistic Director of a touring company, Director for the Almeida Theatre in London, Manager at a regional theatre, Live Artist for Art Angel, BBC Journalist, Youth Theatre Leader and Workshop Facilitator, Outreach and Education Officer, Front of House Theatre Manager, Stage Manager and Secondary School Teacher.</t>
+          <t>BA Drama embraces all forms of drama across stage, screen and performance contexts. Students explore areas such as literary adaptation, performance in public spaces, performance curation, audio design, playwriting, directing and experimental film cultures. Teaching is informed by recent innovations in theatre and performance alongside historical methods and practices. The programme is embedded within a strong creative ecosystem with links to arts organisations and opportunities to engage with professional practitioners during coursework. Specialist facilities include the purpose-built Martin Harris Centre and the John Thaw Studio, a fully staffed performance, rehearsal and workshop space supporting practical production work. Studying the degree develops transferable and specialist skills including theatre analysis, performance creation, presentation and communication, creative problem solving, teamwork and leadership. Graduates pursue careers across sectors including theatre, film, television, journalism, community arts, teaching, arts administration and business, with alumni working at organisations such as BBC, ITV, Sky TV, Contact Theatre and The Lowry Arts Centre.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BA Drama embraces all forms of drama across stage, screen and performance contexts. Students explore areas such as literary adaptation, performance in public spaces, performance curation, audio design, playwriting, directing and experimental film cultures. Teaching is informed by recent innovations in theatre and performance alongside historical methods and practices. The programme is embedded within a strong creative ecosystem with links to arts organisations and opportunities to engage with professional practitioners during coursework. Specialist facilities include the purpose-built Martin Harris Centre and the John Thaw Studio, a fully staffed performance, rehearsal and workshop space supporting practical production work. Studying the degree develops transferable and specialist skills including theatre analysis, performance creation, presentation and communication, creative problem solving, teamwork and leadership. Graduates pursue careers across sectors including theatre, film, television, journalism, community arts, teaching, arts administration and business, with alumni working at organisations such as BBC, ITV, Sky TV, Contact Theatre and The Lowry Arts Centre.</t>
+          <t>Drama, as an expressive subject, offers a perspective into the human experience through the art of performance. It enhances understanding of theatrical techniques, storytelling and the collaborative process of creating compelling narratives. Graduates can use creativity, adaptability and communication skills in fields such as film and television production, advertising, public relations and event management. Acting techniques, theatre history, play analysis, directing, design and technical theatre and performance studies are areas you could study. Master acting techniques including character development, emotional expression and physical embodiment, experience in technical aspects of theatre production and analysing scripts to understand dramatic structures are hard skills you’ll develop. Communication and teamwork, adaptability and creativity, empathy and emotional intelligence are soft skills you’ll develop. Career options include actors, entertainers and presenters, dancers and choreographers, public relations professionals, authors, writers and translators, advertising accounts managers and creative directors, and events managers and organisers.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
-        <is>
-          <t>Drama, as an expressive subject, offers a perspective into the human experience through the art of performance. It enhances understanding of theatrical techniques, storytelling and the collaborative process of creating compelling narratives. Graduates can use creativity, adaptability and communication skills in fields such as film and television production, advertising, public relations and event management. Acting techniques, theatre history, play analysis, directing, design and technical theatre and performance studies are areas you could study. Master acting techniques including character development, emotional expression and physical embodiment, experience in technical aspects of theatre production and analysing scripts to understand dramatic structures are hard skills you’ll develop. Communication and teamwork, adaptability and creativity, empathy and emotional intelligence are soft skills you’ll develop. Career options include actors, entertainers and presenters, dancers and choreographers, public relations professionals, authors, writers and translators, advertising accounts managers and creative directors, and events managers and organisers.</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
         <is>
           <t>Essex: Theatre is a radical and influential art form. Its roots lie deep in the ancient world but its relevance to contemporary life is urgent and ongoing. Theatre enables different cultures and societies to confront the most important issues of our time; it provides a crucial space to laugh, to dream, and dare to project different worlds. Studying theatre and drama at Essex enables you to examine some of the most influential play-texts ever written, and to be ready to take part in shaping the essential performances of tomorrow. This degree is a chance to unlock and explore your creativity. You will be performing and producing work in a professional theatre context and will be developing a wide range of creative, critical and practical skills that will open the door to a future in the theatre, cultural industries or a wide range of other graduate careers. At Essex, we offer a rich combination of practical workshops, critical seminars and lectures delivered by an experienced team of playwrights, directors and actors, as well as leading academic theatre specialists. Areas of exploration in our modules include dramatic literature from Ancient Greek tragedy and Shakespeare to modern plays from around the world, contemporary playwriting and devising techniques, staging political ideas and social justice issues, gender, identity and sexual politics on stage, creating Applied Theatre in educational and community contexts, and emergent trends in interactive performance-making and audience participation. Through classroom teaching, practical experiment and professional experience, we help you craft the skillset that will be essential in your creative development. This approach reflects our core belief that engaging with both practice and theory produces a deeper understanding of how theatre works. Creativity, communication and versatility developed during the degree prepare graduates for a wide range of careers. Our students have gone on to become actors, directors and playwrights, as well as producers, live artists, dramaturgs, stage-managers and arts managers. Graduates have also pursued careers in related creative industries including journalism, television production, broadcasting, radio presenting, gaming, magazine editing, copywriting, press relations and marketing, as well as roles in business, commerce and law. Our graduates have gone on to work in roles such as Writer in Residence for the National Theatre, Artistic Director of Jermyn Street Theatre in London, Artistic Director of a touring company, Director for the Almeida Theatre in London, Manager at a regional theatre, Live Artist for Art Angel, BBC Journalist, Youth Theatre Leader and Workshop Facilitator, Outreach and Education Officer, Front of House Theatre Manager, Stage Manager and Secondary School Teacher.
 Manchester: BA Drama embraces all forms of drama across stage, screen and performance contexts. Students explore areas such as literary adaptation, performance in public spaces, performance curation, audio design, playwriting, directing and experimental film cultures. Teaching is informed by recent innovations in theatre and performance alongside historical methods and practices. The programme is embedded within a strong creative ecosystem with links to arts organisations and opportunities to engage with professional practitioners during coursework. Specialist facilities include the purpose-built Martin Harris Centre and the John Thaw Studio, a fully staffed performance, rehearsal and workshop space supporting practical production work. Studying the degree develops transferable and specialist skills including theatre analysis, performance creation, presentation and communication, creative problem solving, teamwork and leadership. Graduates pursue careers across sectors including theatre, film, television, journalism, community arts, teaching, arts administration and business, with alumni working at organisations such as BBC, ITV, Sky TV, Contact Theatre and The Lowry Arts Centre.
@@ -764,25 +722,20 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Accounting with Economics; Business Economics; Economics and Mathematics; Economics and Politics; Economics with Data Science; Financial Economics; History and Economics; Philosophy, Politics and Economics; Psychology with Economics</t>
+          <t>What is the BSc Economics? The BSc Economics is a three-year degree. You’ll study how economies work, how people and institutions respond to incentives, and how economic evidence is used to explain real-world outcomes. With an emphasis on analysis, data, and economic reasoning, you’ll build the confidence to interpret evidence and apply quantitative insight to complex economic questions. The BSc Economics gives you the opportunity to analyse how people, markets, and governments behave and the quantitative tools to make sense of a world defined by uncertainty, incentives, and change. If you want a degree that explores not just what is happening in the economy but why and what to do about it, this programme gives you that foundation. You’ll explore how economic decisions shape wellbeing, inequality, opportunity, and how societies function. You’ll learn how policy choices affect real lives and how economists use data to create better outcomes. You’ll study micro and macroeconomics, econometrics, behavioural economics, development, labour markets, and public policy. You’ll be taught within a department whose research informs decision-making on labour markets, behavioural change, financial regulation, and development, illustrating how economic theory connects to real policy challenges. Throughout your degree, you’ll learn to think like an economist: breaking down problems, analysing evidence, interpreting data, predicting outcomes, and communicating insights clearly and confidently. By graduation, you’ll have the foundational skills to pursue early careers in government, business, finance and other sectors that value strong analytical ability, or progress to postgraduate study. Students develop skills in microeconomics and macroeconomics to understand how markets work, how incentives influence behaviour, and how economies respond to change; mathematical and quantitative economics to analyse economic problems using mathematical tools; econometrics and data analysis to study economic relationships using statistics and data; applied economics to analyse real-world economic issues and policy questions; and research skills and evidence-based analysis to interpret economic evidence and communicate insights clearly. A BSc Economics degree prepares graduates for careers in economic analysis and data careers such as economist, economic analyst, data analyst, or policy analyst roles using quantitative methods and econometrics; roles in government, regulation and central institutions such as HM Treasury, the Bank of England, government economic units and regulatory bodies; finance, risk and economic consultancy roles in banks and consultancies; research and applied economics roles in think tanks and research institutes; and postgraduate study in economics, econometrics, finance, data science or other quantitative social science disciplines. Graduates from this course have progressed to organisations such as Bank of England, JP Morgan &amp; Chase, Goldman Sachs, HM Treasury and the Financial Conduct Authority.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>What is the BSc Economics? The BSc Economics is a three-year degree. You’ll study how economies work, how people and institutions respond to incentives, and how economic evidence is used to explain real-world outcomes. With an emphasis on analysis, data, and economic reasoning, you’ll build the confidence to interpret evidence and apply quantitative insight to complex economic questions. The BSc Economics gives you the opportunity to analyse how people, markets, and governments behave and the quantitative tools to make sense of a world defined by uncertainty, incentives, and change. If you want a degree that explores not just what is happening in the economy but why and what to do about it, this programme gives you that foundation. You’ll explore how economic decisions shape wellbeing, inequality, opportunity, and how societies function. You’ll learn how policy choices affect real lives and how economists use data to create better outcomes. You’ll study micro and macroeconomics, econometrics, behavioural economics, development, labour markets, and public policy. You’ll be taught within a department whose research informs decision-making on labour markets, behavioural change, financial regulation, and development, illustrating how economic theory connects to real policy challenges. Throughout your degree, you’ll learn to think like an economist: breaking down problems, analysing evidence, interpreting data, predicting outcomes, and communicating insights clearly and confidently. By graduation, you’ll have the foundational skills to pursue early careers in government, business, finance and other sectors that value strong analytical ability, or progress to postgraduate study. Students develop skills in microeconomics and macroeconomics to understand how markets work, how incentives influence behaviour, and how economies respond to change; mathematical and quantitative economics to analyse economic problems using mathematical tools; econometrics and data analysis to study economic relationships using statistics and data; applied economics to analyse real-world economic issues and policy questions; and research skills and evidence-based analysis to interpret economic evidence and communicate insights clearly. A BSc Economics degree prepares graduates for careers in economic analysis and data careers such as economist, economic analyst, data analyst, or policy analyst roles using quantitative methods and econometrics; roles in government, regulation and central institutions such as HM Treasury, the Bank of England, government economic units and regulatory bodies; finance, risk and economic consultancy roles in banks and consultancies; research and applied economics roles in think tanks and research institutes; and postgraduate study in economics, econometrics, finance, data science or other quantitative social science disciplines. Graduates from this course have progressed to organisations such as Bank of England, JP Morgan &amp; Chase, Goldman Sachs, HM Treasury and the Financial Conduct Authority.</t>
+          <t>Today's turbulent economy demands high calibre, well-rounded graduates who not only specialise in economics but also understand the wider social issues and forces at play. Our BA (Economic and Social Studies), known as the BA (Econ), is a flagship interdisciplinary degree designed for students who want to understand economics in its full social, political and technical context. The programme’s Economics specialisation provides a rigorous education in core economic theory and quantitative methods while equipping students with broader perspectives to address complex global challenges. The BA (Econ) is the parent programme to eight distinctive specialisations including Economics, Economics and Politics, Economics and Philosophy, Economics and Sociology, Economics and Finance, Data Science and Economics, Accounting and Finance, and Finance, allowing students to gain a strong shared foundation in economics alongside insights from other social science disciplines. Students specialising in Economics develop technical skills expected of modern economists including economic modelling, statistical and data analysis, interpretation and policy evaluation, while also building critical thinking, ethical reasoning and real-world application skills. The programme enables students to analyse economic issues through mathematical and data-driven approaches as well as through understanding institutions, behaviour, history and social outcomes. It also examines how emerging technologies including generative AI are transforming economic decision-making, while emphasising the importance of human judgement, contextual understanding and interdisciplinary insight. Graduates are prepared to design effective policies, assess economic trade-offs critically and understand how economic decisions affect societies, communities and countries. The degree prepares students for careers in economics, public policy, finance, consultancy, data analysis and international development. Economics graduates from Manchester go on to careers across sectors including finance and banking, professional services, government and public policy, with recent graduates working at organisations such as Morgan Stanley, KPMG, the House of Lords and the Government Economic Service.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Today's turbulent economy demands high calibre, well-rounded graduates who not only specialise in economics but also understand the wider social issues and forces at play. Our BA (Economic and Social Studies), known as the BA (Econ), is a flagship interdisciplinary degree designed for students who want to understand economics in its full social, political and technical context. The programme’s Economics specialisation provides a rigorous education in core economic theory and quantitative methods while equipping students with broader perspectives to address complex global challenges. The BA (Econ) is the parent programme to eight distinctive specialisations including Economics, Economics and Politics, Economics and Philosophy, Economics and Sociology, Economics and Finance, Data Science and Economics, Accounting and Finance, and Finance, allowing students to gain a strong shared foundation in economics alongside insights from other social science disciplines. Students specialising in Economics develop technical skills expected of modern economists including economic modelling, statistical and data analysis, interpretation and policy evaluation, while also building critical thinking, ethical reasoning and real-world application skills. The programme enables students to analyse economic issues through mathematical and data-driven approaches as well as through understanding institutions, behaviour, history and social outcomes. It also examines how emerging technologies including generative AI are transforming economic decision-making, while emphasising the importance of human judgement, contextual understanding and interdisciplinary insight. Graduates are prepared to design effective policies, assess economic trade-offs critically and understand how economic decisions affect societies, communities and countries. The degree prepares students for careers in economics, public policy, finance, consultancy, data analysis and international development. Economics graduates from Manchester go on to careers across sectors including finance and banking, professional services, government and public policy, with recent graduates working at organisations such as Morgan Stanley, KPMG, the House of Lords and the Government Economic Service.</t>
+          <t>Economics is the study of how scarce resources are allocated within societies and how individuals, businesses and governments make decisions. The subject is typically divided into microeconomics, which examines the behaviour of households, firms and industries, and macroeconomics, which focuses on the performance of the economy as a whole. Key areas of study include macroeconomics, microeconomics, probability and statistics, mathematics for economists, econometrics and programming for economic analysis. Study develops quantitative and analytical skills such as statistical modelling, economic forecasting, financial and market analysis, data interpretation and research design. Graduates may pursue careers in sectors including finance, consulting, government, policy analysis, data analytics, business strategy and international organisations.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
-        <is>
-          <t>Economics is the study of how scarce resources are allocated within societies and how individuals, businesses and governments make decisions. The subject is typically divided into microeconomics, which examines the behaviour of households, firms and industries, and macroeconomics, which focuses on the performance of the economy as a whole. Key areas of study include macroeconomics, microeconomics, probability and statistics, mathematics for economists, econometrics and programming for economic analysis. Study develops quantitative and analytical skills such as statistical modelling, economic forecasting, financial and market analysis, data interpretation and research design. Graduates may pursue careers in sectors including finance, consulting, government, policy analysis, data analytics, business strategy and international organisations.</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
         <is>
           <t>Essex: What is the BSc Economics? The BSc Economics is a three-year degree. You’ll study how economies work, how people and institutions respond to incentives, and how economic evidence is used to explain real-world outcomes. With an emphasis on analysis, data, and economic reasoning, you’ll build the confidence to interpret evidence and apply quantitative insight to complex economic questions. The BSc Economics gives you the opportunity to analyse how people, markets, and governments behave and the quantitative tools to make sense of a world defined by uncertainty, incentives, and change. If you want a degree that explores not just what is happening in the economy but why and what to do about it, this programme gives you that foundation. You’ll explore how economic decisions shape wellbeing, inequality, opportunity, and how societies function. You’ll learn how policy choices affect real lives and how economists use data to create better outcomes. You’ll study micro and macroeconomics, econometrics, behavioural economics, development, labour markets, and public policy. You’ll be taught within a department whose research informs decision-making on labour markets, behavioural change, financial regulation, and development, illustrating how economic theory connects to real policy challenges. Throughout your degree, you’ll learn to think like an economist: breaking down problems, analysing evidence, interpreting data, predicting outcomes, and communicating insights clearly and confidently. By graduation, you’ll have the foundational skills to pursue early careers in government, business, finance and other sectors that value strong analytical ability, or progress to postgraduate study. Students develop skills in microeconomics and macroeconomics to understand how markets work, how incentives influence behaviour, and how economies respond to change; mathematical and quantitative economics to analyse economic problems using mathematical tools; econometrics and data analysis to study economic relationships using statistics and data; applied economics to analyse real-world economic issues and policy questions; and research skills and evidence-based analysis to interpret economic evidence and communicate insights clearly. A BSc Economics degree prepares graduates for careers in economic analysis and data careers such as economist, economic analyst, data analyst, or policy analyst roles using quantitative methods and econometrics; roles in government, regulation and central institutions such as HM Treasury, the Bank of England, government economic units and regulatory bodies; finance, risk and economic consultancy roles in banks and consultancies; research and applied economics roles in think tanks and research institutes; and postgraduate study in economics, econometrics, finance, data science or other quantitative social science disciplines. Graduates from this course have progressed to organisations such as Bank of England, JP Morgan &amp; Chase, Goldman Sachs, HM Treasury and the Financial Conduct Authority.
 Manchester: Today's turbulent economy demands high calibre, well-rounded graduates who not only specialise in economics but also understand the wider social issues and forces at play. Our BA (Economic and Social Studies), known as the BA (Econ), is a flagship interdisciplinary degree designed for students who want to understand economics in its full social, political and technical context. The programme’s Economics specialisation provides a rigorous education in core economic theory and quantitative methods while equipping students with broader perspectives to address complex global challenges. The BA (Econ) is the parent programme to eight distinctive specialisations including Economics, Economics and Politics, Economics and Philosophy, Economics and Sociology, Economics and Finance, Data Science and Economics, Accounting and Finance, and Finance, allowing students to gain a strong shared foundation in economics alongside insights from other social science disciplines. Students specialising in Economics develop technical skills expected of modern economists including economic modelling, statistical and data analysis, interpretation and policy evaluation, while also building critical thinking, ethical reasoning and real-world application skills. The programme enables students to analyse economic issues through mathematical and data-driven approaches as well as through understanding institutions, behaviour, history and social outcomes. It also examines how emerging technologies including generative AI are transforming economic decision-making, while emphasising the importance of human judgement, contextual understanding and interdisciplinary insight. Graduates are prepared to design effective policies, assess economic trade-offs critically and understand how economic decisions affect societies, communities and countries. The degree prepares students for careers in economics, public policy, finance, consultancy, data analysis and international development. Economics graduates from Manchester go on to careers across sectors including finance and banking, professional services, government and public policy, with recent graduates working at organisations such as Morgan Stanley, KPMG, the House of Lords and the Government Economic Service.
@@ -801,25 +754,20 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Business Management with a Modern Language; English Language and Literature; English Literature; Language Studies; Language Studies and Linguistics; Language Studies and Teaching English as a Foreign Language; Licence English and French Law; Linguistics; Linguistics with Data Science; Modern Languages and Linguistics; Speech and Language Therapy</t>
+          <t>What is the range of sounds found in human languages? Which of those sounds are used by English to construct words? How are words combined to form meaningful sentences in English, and are the same patterns of combination found in other languages? How does society and social pressure affect the way we speak? How do different varieties of English evolve? These are some of the questions you will address in the course. Language is central to all human activity, from important negotiations between nation states to doctor-patient interaction to spontaneous conversations in cafés. Through your study of language, you come to understand the nature of human social life. Foundational modules in the first and second year will teach you how to analyse linguistic sound systems, word structure, sentence structure, meaning and language use, and apply your knowledge to the analysis of English. You will then be able to make informed choices about areas of English or Linguistics you want to study in greater depth through study options such as Phonetics, English around the World, Language and the Mind, Conversation and Social Interaction, Institutional Talk, and English Language in the Media. We are 1st in UK for research impact in modern languages and linguistics (Grade Point Average, Research Excellence Framework 2021). You have an opportunity to study different kinds of linguistics from structural linguistics to applied and experimental linguistics. Studying language and linguistics allows you to develop your research and IT skills by collecting and analysing linguistic data using modern linguistic methods, and a combination of team-work and independent projects enhances your communication, problem-solving and management skills. Graduates of our department have gone on to have careers in a wide variety of fields including teaching (in the UK and abroad), journalism, branding, advertising, marketing, travel, communications, publishing, speech and occupational therapy, interpreting, translating and media. Other graduates have gone on to work for organisations including the British Council, English in Action, Royal Bank of Scotland, Macmillan Publishers, Cambridge University Press, Freshfields Bruckhaus Deringer and Decisive Media Ltd.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>What is the range of sounds found in human languages? Which of those sounds are used by English to construct words? How are words combined to form meaningful sentences in English, and are the same patterns of combination found in other languages? How does society and social pressure affect the way we speak? How do different varieties of English evolve? These are some of the questions you will address in the course. Language is central to all human activity, from important negotiations between nation states to doctor-patient interaction to spontaneous conversations in cafés. Through your study of language, you come to understand the nature of human social life. Foundational modules in the first and second year will teach you how to analyse linguistic sound systems, word structure, sentence structure, meaning and language use, and apply your knowledge to the analysis of English. You will then be able to make informed choices about areas of English or Linguistics you want to study in greater depth through study options such as Phonetics, English around the World, Language and the Mind, Conversation and Social Interaction, Institutional Talk, and English Language in the Media. We are 1st in UK for research impact in modern languages and linguistics (Grade Point Average, Research Excellence Framework 2021). You have an opportunity to study different kinds of linguistics from structural linguistics to applied and experimental linguistics. Studying language and linguistics allows you to develop your research and IT skills by collecting and analysing linguistic data using modern linguistic methods, and a combination of team-work and independent projects enhances your communication, problem-solving and management skills. Graduates of our department have gone on to have careers in a wide variety of fields including teaching (in the UK and abroad), journalism, branding, advertising, marketing, travel, communications, publishing, speech and occupational therapy, interpreting, translating and media. Other graduates have gone on to work for organisations including the British Council, English in Action, Royal Bank of Scotland, Macmillan Publishers, Cambridge University Press, Freshfields Bruckhaus Deringer and Decisive Media Ltd.</t>
+          <t>Our BA English Language and English Literature joint honours course will enable you to delve into the science of language while exploring a wide range of texts dating from a variety of periods. You will be taken on a broadly chronological journey of English Literature from the Anglo-Saxon period through to the present day. In addition, you will investigate the sounds, words and grammar of the English language, discovering where English comes from, how it developed over time, how it varies across the UK and further afield, and how it is used in different situations. You will acquire the skills required for analytical language study alongside the means to apply those skills to the study of historical and present-day English. You will practise key transferable skills such as essay writing and presentation. You can broaden the scope of your studies to investigate areas such as the interaction between psychology and language (psycholinguistics), child language development, and methodological approaches used in the study of English Language and English Literature. The course provides access to specialist resources including psycholinguistics and phonetics laboratories with facilities for signal analysis, speech synthesis, laryngography and electropalatography. Studying the degree helps you develop analytical and problem-solving skills as well as transferable skills that support careers across sectors including media, marketing, speech and language therapy, lexicography and teaching. Graduates have pursued careers at organisations such as The Guardian, L’Oreal, Universal Music Group and Vodafone.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Our BA English Language and English Literature joint honours course will enable you to delve into the science of language while exploring a wide range of texts dating from a variety of periods. You will be taken on a broadly chronological journey of English Literature from the Anglo-Saxon period through to the present day. In addition, you will investigate the sounds, words and grammar of the English language, discovering where English comes from, how it developed over time, how it varies across the UK and further afield, and how it is used in different situations. You will acquire the skills required for analytical language study alongside the means to apply those skills to the study of historical and present-day English. You will practise key transferable skills such as essay writing and presentation. You can broaden the scope of your studies to investigate areas such as the interaction between psychology and language (psycholinguistics), child language development, and methodological approaches used in the study of English Language and English Literature. The course provides access to specialist resources including psycholinguistics and phonetics laboratories with facilities for signal analysis, speech synthesis, laryngography and electropalatography. Studying the degree helps you develop analytical and problem-solving skills as well as transferable skills that support careers across sectors including media, marketing, speech and language therapy, lexicography and teaching. Graduates have pursued careers at organisations such as The Guardian, L’Oreal, Universal Music Group and Vodafone.</t>
+          <t>English Language is the study of the structure, history and use of English, including its sounds, grammar, vocabulary and variation across regions and social contexts. The subject covers areas such as linguistics, sociolinguistics, language and communication, sound and meaning, language change, digital communication, multilingualism and language revitalisation. Study develops analytical and research skills related to language description, discourse analysis, writing and communication. Graduates may pursue careers in sectors such as teaching, journalism, publishing, copywriting, public relations, digital content management, librarianship and administration, or continue to postgraduate study in linguistics or related fields.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
-        <is>
-          <t>English Language is the study of the structure, history and use of English, including its sounds, grammar, vocabulary and variation across regions and social contexts. The subject covers areas such as linguistics, sociolinguistics, language and communication, sound and meaning, language change, digital communication, multilingualism and language revitalisation. Study develops analytical and research skills related to language description, discourse analysis, writing and communication. Graduates may pursue careers in sectors such as teaching, journalism, publishing, copywriting, public relations, digital content management, librarianship and administration, or continue to postgraduate study in linguistics or related fields.</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
         <is>
           <t>Essex: What is the range of sounds found in human languages? Which of those sounds are used by English to construct words? How are words combined to form meaningful sentences in English, and are the same patterns of combination found in other languages? How does society and social pressure affect the way we speak? How do different varieties of English evolve? These are some of the questions you will address in the course. Language is central to all human activity, from important negotiations between nation states to doctor-patient interaction to spontaneous conversations in cafés. Through your study of language, you come to understand the nature of human social life. Foundational modules in the first and second year will teach you how to analyse linguistic sound systems, word structure, sentence structure, meaning and language use, and apply your knowledge to the analysis of English. You will then be able to make informed choices about areas of English or Linguistics you want to study in greater depth through study options such as Phonetics, English around the World, Language and the Mind, Conversation and Social Interaction, Institutional Talk, and English Language in the Media. We are 1st in UK for research impact in modern languages and linguistics (Grade Point Average, Research Excellence Framework 2021). You have an opportunity to study different kinds of linguistics from structural linguistics to applied and experimental linguistics. Studying language and linguistics allows you to develop your research and IT skills by collecting and analysing linguistic data using modern linguistic methods, and a combination of team-work and independent projects enhances your communication, problem-solving and management skills. Graduates of our department have gone on to have careers in a wide variety of fields including teaching (in the UK and abroad), journalism, branding, advertising, marketing, travel, communications, publishing, speech and occupational therapy, interpreting, translating and media. Other graduates have gone on to work for organisations including the British Council, English in Action, Royal Bank of Scotland, Macmillan Publishers, Cambridge University Press, Freshfields Bruckhaus Deringer and Decisive Media Ltd.
 Manchester: Our BA English Language and English Literature joint honours course will enable you to delve into the science of language while exploring a wide range of texts dating from a variety of periods. You will be taken on a broadly chronological journey of English Literature from the Anglo-Saxon period through to the present day. In addition, you will investigate the sounds, words and grammar of the English language, discovering where English comes from, how it developed over time, how it varies across the UK and further afield, and how it is used in different situations. You will acquire the skills required for analytical language study alongside the means to apply those skills to the study of historical and present-day English. You will practise key transferable skills such as essay writing and presentation. You can broaden the scope of your studies to investigate areas such as the interaction between psychology and language (psycholinguistics), child language development, and methodological approaches used in the study of English Language and English Literature. The course provides access to specialist resources including psycholinguistics and phonetics laboratories with facilities for signal analysis, speech synthesis, laryngography and electropalatography. Studying the degree helps you develop analytical and problem-solving skills as well as transferable skills that support careers across sectors including media, marketing, speech and language therapy, lexicography and teaching. Graduates have pursued careers at organisations such as The Guardian, L’Oreal, Universal Music Group and Vodafone.
@@ -838,21 +786,16 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Economics and Politics; Global Politics; Journalism and Politics; Law with Politics; Modern History and Politics; Philosophy and Politics; Philosophy, Politics and Economics; Politics; Politics and International Relations; Politics with Business</t>
+          <t>Switch on the news any day of the week, or pick up just about any national newspaper, and you will be sure to come across an item on Europe. It is clear that the future of Europe is a geo-political question of profound importance for the future of the world we live in. Yet, few of us truly understand the complex phenomenon that is modern Europe. You'll examine Europe's economic, legal, and sociological context, as well as its historical origins whilst acquiring an understanding of Europe's rich cultural traditions. The artists, writers, musicians, composers and film-makers of Europe have exerted a cultural influence that even now is not eclipsed by the dominance of America on the world's stage. Based within our School of Philosophical, Historical and Interdisciplinary Studies, European studies is a subject that approaches the complex idea of Europe via a wide range of disciplines in the humanities and social sciences. We have expertise in modern languages, literature, film, history of art, history, politics and sociology. Here at Essex, our teaching and research in European studies offers maximum flexibility for you to study areas that interest you, so you can pursue a wide range of topics including European identity and the development of the EU, representations of non-Europeans in art, Europe's colonial history, religion in Europe, and EU law. The study of Europe is vital for ongoing discussion of what Europe's future ought to be; a discussion that will profoundly affect every European citizen. Through a course in European studies, you can acquire the knowledge, skills and experience to make an active contribution to one of the most important political and cultural processes of the century. This course provides excellent preparation for areas which include import/export management, banking and financial sectors, academia, airlines, information technology, management, museums, teaching, non-governmental offices, and development agencies in the UK and abroad. Our graduates have gone on to work for a wide range of organisations including the Civil Service (especially the Foreign Office), embassies around the world, the European Council on Foreign Relations, the Europe Direct Contact Centre in Brussels, the Spanish Congress of Deputies, and LEAD Europe. Other recent graduates have also undertaken traineeships with the European Commission for the Directorate-General for Education and Culture, and various internships in journalism and with NGOs.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Switch on the news any day of the week, or pick up just about any national newspaper, and you will be sure to come across an item on Europe. It is clear that the future of Europe is a geo-political question of profound importance for the future of the world we live in. Yet, few of us truly understand the complex phenomenon that is modern Europe. You'll examine Europe's economic, legal, and sociological context, as well as its historical origins whilst acquiring an understanding of Europe's rich cultural traditions. The artists, writers, musicians, composers and film-makers of Europe have exerted a cultural influence that even now is not eclipsed by the dominance of America on the world's stage. Based within our School of Philosophical, Historical and Interdisciplinary Studies, European studies is a subject that approaches the complex idea of Europe via a wide range of disciplines in the humanities and social sciences. We have expertise in modern languages, literature, film, history of art, history, politics and sociology. Here at Essex, our teaching and research in European studies offers maximum flexibility for you to study areas that interest you, so you can pursue a wide range of topics including European identity and the development of the EU, representations of non-Europeans in art, Europe's colonial history, religion in Europe, and EU law. The study of Europe is vital for ongoing discussion of what Europe's future ought to be; a discussion that will profoundly affect every European citizen. Through a course in European studies, you can acquire the knowledge, skills and experience to make an active contribution to one of the most important political and cultural processes of the century. This course provides excellent preparation for areas which include import/export management, banking and financial sectors, academia, airlines, information technology, management, museums, teaching, non-governmental offices, and development agencies in the UK and abroad. Our graduates have gone on to work for a wide range of organisations including the Civil Service (especially the Foreign Office), embassies around the world, the European Council on Foreign Relations, the Europe Direct Contact Centre in Brussels, the Spanish Congress of Deputies, and LEAD Europe. Other recent graduates have also undertaken traineeships with the European Commission for the Directorate-General for Education and Culture, and various internships in journalism and with NGOs.</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
           <t>The BSocSc (Hons) in Politics and International Relations is a single honours course for politics specialists. Teaching and research are structured around three core themes including Comparative Politics, International Politics and Political Theory. In Years 1 and 2 students take course units from across the three core areas alongside options from disciplines such as Economics, Sociology, History, Philosophy or Languages. By the final year students develop an advanced understanding of politics that reflects the research expertise of staff. The programme supports internationally recognised research across a range of areas and offers a variety of course units that build directly on this research expertise. Students develop solid intellectual foundations within the discipline while gaining increasing choice and diversity of subjects and approaches as they progress. The course aims to provide the opportunity to study politics in depth and breadth through a single-honours specialisation, develop intellectual independence and autonomy, support the development of skills required to undertake independent research of a high standard, and build intellectual flexibility and adaptability. Research areas explored within the programme include topics such as security, migration, war, gender, ethics, resistance and international institutions. Graduates pursue careers across sectors including consultancy, public administration, diplomacy, policy and business, with alumni working at organisations such as Google, Thomson Reuters, Deloitte, HMRC, the Royal Danish Embassy, the Ministry of Justice, Greater Manchester Chamber of Commerce, Cicero Consultancy and Essex County Council.</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
         <is>
           <t>Essex: Switch on the news any day of the week, or pick up just about any national newspaper, and you will be sure to come across an item on Europe. It is clear that the future of Europe is a geo-political question of profound importance for the future of the world we live in. Yet, few of us truly understand the complex phenomenon that is modern Europe. You'll examine Europe's economic, legal, and sociological context, as well as its historical origins whilst acquiring an understanding of Europe's rich cultural traditions. The artists, writers, musicians, composers and film-makers of Europe have exerted a cultural influence that even now is not eclipsed by the dominance of America on the world's stage. Based within our School of Philosophical, Historical and Interdisciplinary Studies, European studies is a subject that approaches the complex idea of Europe via a wide range of disciplines in the humanities and social sciences. We have expertise in modern languages, literature, film, history of art, history, politics and sociology. Here at Essex, our teaching and research in European studies offers maximum flexibility for you to study areas that interest you, so you can pursue a wide range of topics including European identity and the development of the EU, representations of non-Europeans in art, Europe's colonial history, religion in Europe, and EU law. The study of Europe is vital for ongoing discussion of what Europe's future ought to be; a discussion that will profoundly affect every European citizen. Through a course in European studies, you can acquire the knowledge, skills and experience to make an active contribution to one of the most important political and cultural processes of the century. This course provides excellent preparation for areas which include import/export management, banking and financial sectors, academia, airlines, information technology, management, museums, teaching, non-governmental offices, and development agencies in the UK and abroad. Our graduates have gone on to work for a wide range of organisations including the Civil Service (especially the Foreign Office), embassies around the world, the European Council on Foreign Relations, the Europe Direct Contact Centre in Brussels, the Spanish Congress of Deputies, and LEAD Europe. Other recent graduates have also undertaken traineeships with the European Commission for the Directorate-General for Education and Culture, and various internships in journalism and with NGOs.
 Manchester: The BSocSc (Hons) in Politics and International Relations is a single honours course for politics specialists. Teaching and research are structured around three core themes including Comparative Politics, International Politics and Political Theory. In Years 1 and 2 students take course units from across the three core areas alongside options from disciplines such as Economics, Sociology, History, Philosophy or Languages. By the final year students develop an advanced understanding of politics that reflects the research expertise of staff. The programme supports internationally recognised research across a range of areas and offers a variety of course units that build directly on this research expertise. Students develop solid intellectual foundations within the discipline while gaining increasing choice and diversity of subjects and approaches as they progress. The course aims to provide the opportunity to study politics in depth and breadth through a single-honours specialisation, develop intellectual independence and autonomy, support the development of skills required to undertake independent research of a high standard, and build intellectual flexibility and adaptability. Research areas explored within the programme include topics such as security, migration, war, gender, ethics, resistance and international institutions. Graduates pursue careers across sectors including consultancy, public administration, diplomacy, policy and business, with alumni working at organisations such as Google, Thomson Reuters, Deloitte, HMRC, the Royal Danish Embassy, the Ministry of Justice, Greater Manchester Chamber of Commerce, Cicero Consultancy and Essex County Council.</t>
@@ -870,25 +813,20 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Film Studies and Literature; Film and Creative Writing; Film and Drama</t>
+          <t>How does cinema affect us as individuals and as groups, as communities or nations? Do the moving pictures reflect our beliefs or help to change how we see the world? How powerful are visual media in shaping our interpretations of modern life? These are some of the most pressing questions cinema asks us. Our ability to read and interpret the images and stories that films deliver is crucial to how we understand contemporary life. At Essex you combine studying the history and theory of cinema with practical film production, so you don't just critically examine cinema – you create it. Your production modules enable you to develop and apply your academic knowledge and understanding of film, refining and enriching your own practical work. We give you the opportunity to explore film across a broad range of genres, time periods, and regions, from Hollywood, world and independent cinema to documentaries and television. Simultaneously, you gain hands-on experience in film production and production management, essential for careers in the film and television industry. We nurture the creative talent for tomorrow, developing filmmakers, scholars and thinkers with a dynamic worldview. You gain hands-on experience of camera work, sound recording, editing, lighting and scriptwriting, explore the formal aesthetics of film composition and structure in relation to different contexts of production and reception, discover the history and social significance of film as a global medium, understand the links between critical analysis and creative practice, and produce both group films and personal projects. By graduation you will have built up a fully rounded portfolio of work, enabling you to showcase your experience, versatility and creative potential to future employers. We offer a varied, flexible and distinctive curriculum focused on developing your abilities in film while also enabling you to take options from other courses within our Department of Literature, Film and Theatre Studies including literature, creative writing, journalism and drama. You graduate from our course with key skills in writing close analysis, critical thinking, contextual research, time management and hands-on filmmaking. The short film you will make as part of your studies serves as a calling card, showcasing your individual creative potential as part of a portfolio of practical work developed during your course. Our students are well prepared to enter careers in film production, television, journalism, publishing and teaching. Recent graduates have gone on to roles including celebrity booking for Cactus TV, editor for BBC television, subtitle writer for Sky TV, and teachers of English and Media Studies.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>How does cinema affect us as individuals and as groups, as communities or nations? Do the moving pictures reflect our beliefs or help to change how we see the world? How powerful are visual media in shaping our interpretations of modern life? These are some of the most pressing questions cinema asks us. Our ability to read and interpret the images and stories that films deliver is crucial to how we understand contemporary life. At Essex you combine studying the history and theory of cinema with practical film production, so you don't just critically examine cinema – you create it. Your production modules enable you to develop and apply your academic knowledge and understanding of film, refining and enriching your own practical work. We give you the opportunity to explore film across a broad range of genres, time periods, and regions, from Hollywood, world and independent cinema to documentaries and television. Simultaneously, you gain hands-on experience in film production and production management, essential for careers in the film and television industry. We nurture the creative talent for tomorrow, developing filmmakers, scholars and thinkers with a dynamic worldview. You gain hands-on experience of camera work, sound recording, editing, lighting and scriptwriting, explore the formal aesthetics of film composition and structure in relation to different contexts of production and reception, discover the history and social significance of film as a global medium, understand the links between critical analysis and creative practice, and produce both group films and personal projects. By graduation you will have built up a fully rounded portfolio of work, enabling you to showcase your experience, versatility and creative potential to future employers. We offer a varied, flexible and distinctive curriculum focused on developing your abilities in film while also enabling you to take options from other courses within our Department of Literature, Film and Theatre Studies including literature, creative writing, journalism and drama. You graduate from our course with key skills in writing close analysis, critical thinking, contextual research, time management and hands-on filmmaking. The short film you will make as part of your studies serves as a calling card, showcasing your individual creative potential as part of a portfolio of practical work developed during your course. Our students are well prepared to enter careers in film production, television, journalism, publishing and teaching. Recent graduates have gone on to roles including celebrity booking for Cactus TV, editor for BBC television, subtitle writer for Sky TV, and teachers of English and Media Studies.</t>
+          <t>BA Drama and Film Studies enables students to benefit from teaching and research in Drama while engaging in the study of film and television. Students take courses in theatre and film history and theory alongside practical courses in theatre production and filmmaking, with opportunities to study video-making and engage with professional practitioners working in the cultural industries. Teaching reflects both contemporary innovations in theatre, performance and film studies and historical practices. The programme operates within a strong creative and cultural network with links to arts organisations and performance partners. Specialist facilities include the Martin Harris Centre and the John Thaw Studio as well as rehearsal rooms, screening rooms and sound and video-editing suites that support creative production work. Students develop skills including theatre and film analysis, creating original performance work, communication, creative problem solving, teamwork and leadership. Graduates pursue careers in theatre, film, television, journalism, arts administration and related sectors, with alumni working at organisations such as BBC, ITV, Sky TV, Tandem Theatre and The Lowry Arts Centre.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BA Drama and Film Studies enables students to benefit from teaching and research in Drama while engaging in the study of film and television. Students take courses in theatre and film history and theory alongside practical courses in theatre production and filmmaking, with opportunities to study video-making and engage with professional practitioners working in the cultural industries. Teaching reflects both contemporary innovations in theatre, performance and film studies and historical practices. The programme operates within a strong creative and cultural network with links to arts organisations and performance partners. Specialist facilities include the Martin Harris Centre and the John Thaw Studio as well as rehearsal rooms, screening rooms and sound and video-editing suites that support creative production work. Students develop skills including theatre and film analysis, creating original performance work, communication, creative problem solving, teamwork and leadership. Graduates pursue careers in theatre, film, television, journalism, arts administration and related sectors, with alumni working at organisations such as BBC, ITV, Sky TV, Tandem Theatre and The Lowry Arts Centre.</t>
+          <t>Film studies gives an understanding of visual storytelling, film history and cultural impact. Studying film studies opens doors to career paths such as film production, directing, screenwriting and digital content creation. Creative cinematography, storytelling for the screen, production skills, analogue and digital technology, the business of Hollywood, film and photography’s role in history, principles of creativity and society of the media are areas you could study. Film analysis, scriptwriting, story structure and project planning and coordination are hard skills you’ll develop. Critical thinking, communication skills, creative expression and presentation skills are soft skills you’ll develop. Career options include arts officers, producers and directors, photographers, audio-visual and broadcasting equipment operators, TV, video and audio servicers and repairers, authors, writers and translators.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
-        <is>
-          <t>Film studies gives an understanding of visual storytelling, film history and cultural impact. Studying film studies opens doors to career paths such as film production, directing, screenwriting and digital content creation. Creative cinematography, storytelling for the screen, production skills, analogue and digital technology, the business of Hollywood, film and photography’s role in history, principles of creativity and society of the media are areas you could study. Film analysis, scriptwriting, story structure and project planning and coordination are hard skills you’ll develop. Critical thinking, communication skills, creative expression and presentation skills are soft skills you’ll develop. Career options include arts officers, producers and directors, photographers, audio-visual and broadcasting equipment operators, TV, video and audio servicers and repairers, authors, writers and translators.</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
         <is>
           <t>Essex: How does cinema affect us as individuals and as groups, as communities or nations? Do the moving pictures reflect our beliefs or help to change how we see the world? How powerful are visual media in shaping our interpretations of modern life? These are some of the most pressing questions cinema asks us. Our ability to read and interpret the images and stories that films deliver is crucial to how we understand contemporary life. At Essex you combine studying the history and theory of cinema with practical film production, so you don't just critically examine cinema – you create it. Your production modules enable you to develop and apply your academic knowledge and understanding of film, refining and enriching your own practical work. We give you the opportunity to explore film across a broad range of genres, time periods, and regions, from Hollywood, world and independent cinema to documentaries and television. Simultaneously, you gain hands-on experience in film production and production management, essential for careers in the film and television industry. We nurture the creative talent for tomorrow, developing filmmakers, scholars and thinkers with a dynamic worldview. You gain hands-on experience of camera work, sound recording, editing, lighting and scriptwriting, explore the formal aesthetics of film composition and structure in relation to different contexts of production and reception, discover the history and social significance of film as a global medium, understand the links between critical analysis and creative practice, and produce both group films and personal projects. By graduation you will have built up a fully rounded portfolio of work, enabling you to showcase your experience, versatility and creative potential to future employers. We offer a varied, flexible and distinctive curriculum focused on developing your abilities in film while also enabling you to take options from other courses within our Department of Literature, Film and Theatre Studies including literature, creative writing, journalism and drama. You graduate from our course with key skills in writing close analysis, critical thinking, contextual research, time management and hands-on filmmaking. The short film you will make as part of your studies serves as a calling card, showcasing your individual creative potential as part of a portfolio of practical work developed during your course. Our students are well prepared to enter careers in film production, television, journalism, publishing and teaching. Recent graduates have gone on to roles including celebrity booking for Cactus TV, editor for BBC television, subtitle writer for Sky TV, and teachers of English and Media Studies.
 Manchester: BA Drama and Film Studies enables students to benefit from teaching and research in Drama while engaging in the study of film and television. Students take courses in theatre and film history and theory alongside practical courses in theatre production and filmmaking, with opportunities to study video-making and engage with professional practitioners working in the cultural industries. Teaching reflects both contemporary innovations in theatre, performance and film studies and historical practices. The programme operates within a strong creative and cultural network with links to arts organisations and performance partners. Specialist facilities include the Martin Harris Centre and the John Thaw Studio as well as rehearsal rooms, screening rooms and sound and video-editing suites that support creative production work. Students develop skills including theatre and film analysis, creating original performance work, communication, creative problem solving, teamwork and leadership. Graduates pursue careers in theatre, film, television, journalism, arts administration and related sectors, with alumni working at organisations such as BBC, ITV, Sky TV, Tandem Theatre and The Lowry Arts Centre.
@@ -907,25 +845,20 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Art History; Curating with History; History and Economics; History and Literature; History and Sociology; Modern History; Modern History and International Relations; Modern History and Politics</t>
+          <t>At the University of Essex we're about social conscience, wondering why, and understanding the bigger picture. We teach you to find your own critical voice and view history through the eyes of different people, telling hidden histories that might otherwise be forgotten. Our BA History allows you to explore challenging questions about the impact of political, social and cultural change on individuals, social groups and regions. From African-American slavery to Stalin's Russia—from households in Essex to witchcraft in Germany—from the history of disease to revolutions in China, we urge you to explore the past in order to better understand the present. You have the flexibility to choose from a wide range of optional modules about subjects close to home and further afield. We also provide you with opportunities to explore local history and have close ties with the Essex Record Office, one of the best county record offices in the UK. Assessed coursework generally consists of essays, concept studies, critical commentaries, research proposals and a 15,000-word dissertation. Students usually attend a two-hour seminar for each module each week, with seminar groups or workshops usually having about 15 students. In addition to the opportunity to learn about the past and come to a better understanding of the present, a course in history also provides you with important skills that will be of value after leaving university. You learn to absorb, analyse and assess a wide variety of information and viewpoints, to express your arguments in oral and written form, and to think and work both independently and in co-operation with others. You therefore graduate prepared for a wide range of careers including teaching, librarianship, museum and archive services, the Civil Service, local government, law enforcement and charity administration. Others have proceeded to work in banking, industrial and retail management, media research, electronic publishing, marketing, IT, health service administration, counselling and social work, while others have chosen to enhance their career opportunities by studying at postgraduate level. Some of our recent graduates have found employment as a warden for the Royal Collection at Windsor Castle, a planning support officer for a local council, a senior underwriting assistant at CNA Insurance Company Limited, a researcher at the House of Commons, a graduate trainee for the Royal Botanic Gardens at Kew and a library assistant for the University of Cambridge.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>At the University of Essex we're about social conscience, wondering why, and understanding the bigger picture. We teach you to find your own critical voice and view history through the eyes of different people, telling hidden histories that might otherwise be forgotten. Our BA History allows you to explore challenging questions about the impact of political, social and cultural change on individuals, social groups and regions. From African-American slavery to Stalin's Russia—from households in Essex to witchcraft in Germany—from the history of disease to revolutions in China, we urge you to explore the past in order to better understand the present. You have the flexibility to choose from a wide range of optional modules about subjects close to home and further afield. We also provide you with opportunities to explore local history and have close ties with the Essex Record Office, one of the best county record offices in the UK. Assessed coursework generally consists of essays, concept studies, critical commentaries, research proposals and a 15,000-word dissertation. Students usually attend a two-hour seminar for each module each week, with seminar groups or workshops usually having about 15 students. In addition to the opportunity to learn about the past and come to a better understanding of the present, a course in history also provides you with important skills that will be of value after leaving university. You learn to absorb, analyse and assess a wide variety of information and viewpoints, to express your arguments in oral and written form, and to think and work both independently and in co-operation with others. You therefore graduate prepared for a wide range of careers including teaching, librarianship, museum and archive services, the Civil Service, local government, law enforcement and charity administration. Others have proceeded to work in banking, industrial and retail management, media research, electronic publishing, marketing, IT, health service administration, counselling and social work, while others have chosen to enhance their career opportunities by studying at postgraduate level. Some of our recent graduates have found employment as a warden for the Royal Collection at Windsor Castle, a planning support officer for a local council, a senior underwriting assistant at CNA Insurance Company Limited, a researcher at the House of Commons, a graduate trainee for the Royal Botanic Gardens at Kew and a library assistant for the University of Cambridge.</t>
+          <t>Our BA History course will give you the opportunity to tailor your degree to suit your own interests while learning from one of the largest concentrations of historians in Britain. Students can choose course units covering a wide range of periods and topics including ancient, medieval, modern, economic and social history, as well as the history of science, technology and medicine. In Years 1 and 2 students may also take course units in other disciplines including languages, the humanities and the social sciences. Students have the option to specialise in a particular area of interest or continue to study a broad range of topics in their final year, choosing units covering British, European, American, African and Asian history across different periods and culminating in a dissertation. The programme provides expert training in analysis and critical reasoning while developing transferable skills in communication and presentation, argument and debate, teamwork, research and time management. Graduates pursue careers across sectors including teaching and academia, heritage and museums, the Civil Service, policy and thinktanks, creative industries, media and journalism, marketing and public relations, law and accountancy, finance and NGOs, with alumni working at organisations such as the BBC, KPMG, Deloitte, Marks and Spencer, Aviva, Accenture and Barclays.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Our BA History course will give you the opportunity to tailor your degree to suit your own interests while learning from one of the largest concentrations of historians in Britain. Students can choose course units covering a wide range of periods and topics including ancient, medieval, modern, economic and social history, as well as the history of science, technology and medicine. In Years 1 and 2 students may also take course units in other disciplines including languages, the humanities and the social sciences. Students have the option to specialise in a particular area of interest or continue to study a broad range of topics in their final year, choosing units covering British, European, American, African and Asian history across different periods and culminating in a dissertation. The programme provides expert training in analysis and critical reasoning while developing transferable skills in communication and presentation, argument and debate, teamwork, research and time management. Graduates pursue careers across sectors including teaching and academia, heritage and museums, the Civil Service, policy and thinktanks, creative industries, media and journalism, marketing and public relations, law and accountancy, finance and NGOs, with alumni working at organisations such as the BBC, KPMG, Deloitte, Marks and Spencer, Aviva, Accenture and Barclays.</t>
+          <t>Gain an understanding of the economies, societies, faiths, and cultures that have shaped our world over time. Studying history will allow you to read and analyse texts and evidence, and gain an in-depth understanding of the forces that have shaped our modern world. You could combine history with other subjects like English, languages, or economics, and focus on particular periods of history you’re fascinated by. The research and critical thinking skills you gain will equip you for roles in a variety of industries such as local and central government, journalism, education, heritage, publishing, and academia. You could also go on to further study. Political communities in world history, societies and economies in world history, 19th and 20th century Britain, Europe in the making, disease and society, theory and practice of oral history, arguments and analysis, evidence and methods, Latin America: themes and problems, history and politics of the modern Middle East, contemporary US race relations and corruption in Britain and its empire are areas you could study. Exhibitions, archives, curation, marketing and cataloguing are hard skills you'll develop. Communication, management, research, customer service and planning are soft skills you'll develop. Career options include archaeologist, art gallery manager, museum curator, arts administrator, antiques dealer, heritage manager, higher education lecturer or researcher, secondary school teacher, social researcher, journalist, writer, public relations roles, publishing assistant, academic librarian and archivist.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
-        <is>
-          <t>Gain an understanding of the economies, societies, faiths, and cultures that have shaped our world over time. Studying history will allow you to read and analyse texts and evidence, and gain an in-depth understanding of the forces that have shaped our modern world. You could combine history with other subjects like English, languages, or economics, and focus on particular periods of history you’re fascinated by. The research and critical thinking skills you gain will equip you for roles in a variety of industries such as local and central government, journalism, education, heritage, publishing, and academia. You could also go on to further study. Political communities in world history, societies and economies in world history, 19th and 20th century Britain, Europe in the making, disease and society, theory and practice of oral history, arguments and analysis, evidence and methods, Latin America: themes and problems, history and politics of the modern Middle East, contemporary US race relations and corruption in Britain and its empire are areas you could study. Exhibitions, archives, curation, marketing and cataloguing are hard skills you'll develop. Communication, management, research, customer service and planning are soft skills you'll develop. Career options include archaeologist, art gallery manager, museum curator, arts administrator, antiques dealer, heritage manager, higher education lecturer or researcher, secondary school teacher, social researcher, journalist, writer, public relations roles, publishing assistant, academic librarian and archivist.</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
         <is>
           <t>Essex: At the University of Essex we're about social conscience, wondering why, and understanding the bigger picture. We teach you to find your own critical voice and view history through the eyes of different people, telling hidden histories that might otherwise be forgotten. Our BA History allows you to explore challenging questions about the impact of political, social and cultural change on individuals, social groups and regions. From African-American slavery to Stalin's Russia—from households in Essex to witchcraft in Germany—from the history of disease to revolutions in China, we urge you to explore the past in order to better understand the present. You have the flexibility to choose from a wide range of optional modules about subjects close to home and further afield. We also provide you with opportunities to explore local history and have close ties with the Essex Record Office, one of the best county record offices in the UK. Assessed coursework generally consists of essays, concept studies, critical commentaries, research proposals and a 15,000-word dissertation. Students usually attend a two-hour seminar for each module each week, with seminar groups or workshops usually having about 15 students. In addition to the opportunity to learn about the past and come to a better understanding of the present, a course in history also provides you with important skills that will be of value after leaving university. You learn to absorb, analyse and assess a wide variety of information and viewpoints, to express your arguments in oral and written form, and to think and work both independently and in co-operation with others. You therefore graduate prepared for a wide range of careers including teaching, librarianship, museum and archive services, the Civil Service, local government, law enforcement and charity administration. Others have proceeded to work in banking, industrial and retail management, media research, electronic publishing, marketing, IT, health service administration, counselling and social work, while others have chosen to enhance their career opportunities by studying at postgraduate level. Some of our recent graduates have found employment as a warden for the Royal Collection at Windsor Castle, a planning support officer for a local council, a senior underwriting assistant at CNA Insurance Company Limited, a researcher at the House of Commons, a graduate trainee for the Royal Botanic Gardens at Kew and a library assistant for the University of Cambridge.
 Manchester: Our BA History course will give you the opportunity to tailor your degree to suit your own interests while learning from one of the largest concentrations of historians in Britain. Students can choose course units covering a wide range of periods and topics including ancient, medieval, modern, economic and social history, as well as the history of science, technology and medicine. In Years 1 and 2 students may also take course units in other disciplines including languages, the humanities and the social sciences. Students have the option to specialise in a particular area of interest or continue to study a broad range of topics in their final year, choosing units covering British, European, American, African and Asian history across different periods and culminating in a dissertation. The programme provides expert training in analysis and critical reasoning while developing transferable skills in communication and presentation, argument and debate, teamwork, research and time management. Graduates pursue careers across sectors including teaching and academia, heritage and museums, the Civil Service, policy and thinktanks, creative industries, media and journalism, marketing and public relations, law and accountancy, finance and NGOs, with alumni working at organisations such as the BBC, KPMG, Deloitte, Marks and Spencer, Aviva, Accenture and Barclays.
@@ -944,21 +877,16 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Modern Languages with Latin American Studies</t>
+          <t>BA Global Studies and Latin American Studies will equip you with a broad range of skills to become an active participant in a crucial time of change. You'll study some of today's most pressing issues from the migrant crisis to climate change, and you'll acquire a global perspective to face contemporary challenges. This interdisciplinary degree combines the breadth of Global Studies with deep engagement in Latin American history and culture. Latin America is one of the most fascinating and complex areas of the world, home to a rich diversity of indigenous people, as well as some of the world's fastest growing economies, greatest environmental challenges, and richest cultural traditions. Latin America is an area of study that will surprise you, challenge you and broaden your horizons. A core part of the course are modules from history and politics which explore international relations and global history, alongside Latin American Studies modules. You will study a range of topics including economic and political history of Latin America, indigenous issues in Latin America, global technologies, migration, and art and architecture in social context. Language is fundamental to our thought, our relationships and our civilisations. As part of this degree you will add a language to your portfolio through either learning Spanish from scratch or developing existing skills in Spanish and/or Brazilian Portuguese to a high level, and spending your third year at a university in a Latin American country. This course differs from BA Global Studies with Latin American Studies in that it includes a compulsory year abroad in a Latin American country and has a compulsory language component. Our graduates are well-placed to address the complex issues which confront the modern world. Our course provides you with an excellent basis for going onto a career in media, education, politics, the Civil Service, international organisations such as the UN and NATO or non-governmental organisations, and many other fields. Our Centre's recent graduates have gone on to work in a wide range of roles including an events co-ordinator for Age UK, a business provision manager for BT, an accountant in London, and an account executive for Bluesky PR.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>BA Global Studies and Latin American Studies will equip you with a broad range of skills to become an active participant in a crucial time of change. You'll study some of today's most pressing issues from the migrant crisis to climate change, and you'll acquire a global perspective to face contemporary challenges. This interdisciplinary degree combines the breadth of Global Studies with deep engagement in Latin American history and culture. Latin America is one of the most fascinating and complex areas of the world, home to a rich diversity of indigenous people, as well as some of the world's fastest growing economies, greatest environmental challenges, and richest cultural traditions. Latin America is an area of study that will surprise you, challenge you and broaden your horizons. A core part of the course are modules from history and politics which explore international relations and global history, alongside Latin American Studies modules. You will study a range of topics including economic and political history of Latin America, indigenous issues in Latin America, global technologies, migration, and art and architecture in social context. Language is fundamental to our thought, our relationships and our civilisations. As part of this degree you will add a language to your portfolio through either learning Spanish from scratch or developing existing skills in Spanish and/or Brazilian Portuguese to a high level, and spending your third year at a university in a Latin American country. This course differs from BA Global Studies with Latin American Studies in that it includes a compulsory year abroad in a Latin American country and has a compulsory language component. Our graduates are well-placed to address the complex issues which confront the modern world. Our course provides you with an excellent basis for going onto a career in media, education, politics, the Civil Service, international organisations such as the UN and NATO or non-governmental organisations, and many other fields. Our Centre's recent graduates have gone on to work in a wide range of roles including an events co-ordinator for Age UK, a business provision manager for BT, an accountant in London, and an account executive for Bluesky PR.</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
           <t>Our single honours BA Spanish, Portuguese and Latin American Studies course will give you a strong grounding in writing, speaking and understanding the Spanish and Portuguese languages, as well as the opportunity to learn Catalan. After Year 1, Portuguese language is not compulsory and students can choose to concentrate more on Spanish, maintain a balance between the languages or focus more on Portuguese by the final year, with the option to study Catalan. Language study enables students to explore diverse aspects of the culture, society, history, politics and literature of countries where Spanish and Portuguese are spoken while developing intercultural awareness and communication skills. A compulsory third year residence abroad allows students to live, study or work in Spanish- and Portuguese-speaking countries in Europe and Latin America, providing significant personal, linguistic and professional development. Language units are compulsory at all levels of the degree. The programme benefits from collaborations with cultural institutions such as Instituto Cervantes and links with Portuguese cultural organisations. Specialist facilities include extensive collections relating to Lusophone Africa, access to films and texts on Latin America, Portugal and Spain, and resources at the University Language Centre including interpreting suites, recording rooms and multilingual learning technologies. Graduates pursue careers across sectors including media, journalism, public relations, business services, marketing, banking and communications, with alumni working at organisations such as ASOS, Ernst &amp; Young, Procter &amp; Gamble, JD Sports, Oxfam, Greenpeace and Virgin.</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr">
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
         <is>
           <t>Essex: BA Global Studies and Latin American Studies will equip you with a broad range of skills to become an active participant in a crucial time of change. You'll study some of today's most pressing issues from the migrant crisis to climate change, and you'll acquire a global perspective to face contemporary challenges. This interdisciplinary degree combines the breadth of Global Studies with deep engagement in Latin American history and culture. Latin America is one of the most fascinating and complex areas of the world, home to a rich diversity of indigenous people, as well as some of the world's fastest growing economies, greatest environmental challenges, and richest cultural traditions. Latin America is an area of study that will surprise you, challenge you and broaden your horizons. A core part of the course are modules from history and politics which explore international relations and global history, alongside Latin American Studies modules. You will study a range of topics including economic and political history of Latin America, indigenous issues in Latin America, global technologies, migration, and art and architecture in social context. Language is fundamental to our thought, our relationships and our civilisations. As part of this degree you will add a language to your portfolio through either learning Spanish from scratch or developing existing skills in Spanish and/or Brazilian Portuguese to a high level, and spending your third year at a university in a Latin American country. This course differs from BA Global Studies with Latin American Studies in that it includes a compulsory year abroad in a Latin American country and has a compulsory language component. Our graduates are well-placed to address the complex issues which confront the modern world. Our course provides you with an excellent basis for going onto a career in media, education, politics, the Civil Service, international organisations such as the UN and NATO or non-governmental organisations, and many other fields. Our Centre's recent graduates have gone on to work in a wide range of roles including an events co-ordinator for Age UK, a business provision manager for BT, an accountant in London, and an account executive for Bluesky PR.
 Manchester: Our single honours BA Spanish, Portuguese and Latin American Studies course will give you a strong grounding in writing, speaking and understanding the Spanish and Portuguese languages, as well as the opportunity to learn Catalan. After Year 1, Portuguese language is not compulsory and students can choose to concentrate more on Spanish, maintain a balance between the languages or focus more on Portuguese by the final year, with the option to study Catalan. Language study enables students to explore diverse aspects of the culture, society, history, politics and literature of countries where Spanish and Portuguese are spoken while developing intercultural awareness and communication skills. A compulsory third year residence abroad allows students to live, study or work in Spanish- and Portuguese-speaking countries in Europe and Latin America, providing significant personal, linguistic and professional development. Language units are compulsory at all levels of the degree. The programme benefits from collaborations with cultural institutions such as Instituto Cervantes and links with Portuguese cultural organisations. Specialist facilities include extensive collections relating to Lusophone Africa, access to films and texts on Latin America, Portugal and Spain, and resources at the University Language Centre including interpreting suites, recording rooms and multilingual learning technologies. Graduates pursue careers across sectors including media, journalism, public relations, business services, marketing, banking and communications, with alumni working at organisations such as ASOS, Ernst &amp; Young, Procter &amp; Gamble, JD Sports, Oxfam, Greenpeace and Virgin.</t>
@@ -976,25 +904,20 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Criminology with Criminal Law; Law; Law with Business; Law with Criminology; Law with Human Rights; Law with Philosophy; Law with Politics; Licence English and French Law</t>
+          <t>What is LLB Law with Human Rights? The LLB Law with Human Rights is a three-year undergraduate qualifying law degree. It combines a full legal education with a dedicated focus on human rights at domestic, European, and international levels. You’ll study the core foundations of English law alongside specialist human rights modules, graduating with in-depth knowledge of how rights are protected and applied across different legal systems. The LLB Law with Human Rights combines a qualifying law degree with specialist training in UK, European, and international human rights law. It is ideal for students who want to study law through the lens of justice, rights, and social impact. The course is shaped by internationally recognised expertise in human rights. You’ll develop strong legal reasoning, research, and analytical skills while applying law to real-world human rights issues. Your studies explore how law operates as a practical tool for protecting individuals and contributing to fairer societies. Students study core legal foundations including legal method, contract, criminal law, public law, tort, land law, and equity, while also exploring UK and European human rights law and international human rights law as dedicated areas of study. The course examines how domestic law interacts with European and international legal frameworks and develops skills in case analysis, rights-based argumentation, and legal research. Students critically evaluate law within social, political, and ethical settings. An LLB Law with Human Rights prepares graduates for careers in law and policy including roles such as solicitor, barrister, paralegal or legal adviser, as well as careers within human rights organisations, charities and advocacy groups, government and public bodies, international organisations, policy research institutes and social justice organisations, and roles in compliance, governance and corporate responsibility.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>What is LLB Law with Human Rights? The LLB Law with Human Rights is a three-year undergraduate qualifying law degree. It combines a full legal education with a dedicated focus on human rights at domestic, European, and international levels. You’ll study the core foundations of English law alongside specialist human rights modules, graduating with in-depth knowledge of how rights are protected and applied across different legal systems. The LLB Law with Human Rights combines a qualifying law degree with specialist training in UK, European, and international human rights law. It is ideal for students who want to study law through the lens of justice, rights, and social impact. The course is shaped by internationally recognised expertise in human rights. You’ll develop strong legal reasoning, research, and analytical skills while applying law to real-world human rights issues. Your studies explore how law operates as a practical tool for protecting individuals and contributing to fairer societies. Students study core legal foundations including legal method, contract, criminal law, public law, tort, land law, and equity, while also exploring UK and European human rights law and international human rights law as dedicated areas of study. The course examines how domestic law interacts with European and international legal frameworks and develops skills in case analysis, rights-based argumentation, and legal research. Students critically evaluate law within social, political, and ethical settings. An LLB Law with Human Rights prepares graduates for careers in law and policy including roles such as solicitor, barrister, paralegal or legal adviser, as well as careers within human rights organisations, charities and advocacy groups, government and public bodies, international organisations, policy research institutes and social justice organisations, and roles in compliance, governance and corporate responsibility.</t>
+          <t>Law is at the heart of our society, informing and governing our everyday actions. The LLB Law course offers a distinctive approach to legal education that combines research-informed study with practice-led approaches. Students study the foundations of English and Welsh law and have the freedom to follow their own interests through a broad range of optional units while being challenged to analyse and critique the law and understand the social, economic, ethical and political contexts in which it operates. Career-focused learning is embedded throughout the course, including opportunities to apply legal theory in practice through clinical legal education at the Justice Hub, which offers free legal advice to members of the public and supports partnerships with the public, charitable and private sectors. Students develop a global perspective on law alongside essential skills, knowledge and experience for careers both within and beyond the legal profession. The programme includes engagement with areas such as family law, business law and criminal law, and introduces students to emerging fields such as LegalTech. Facilities supporting study include a moot court for simulated legal practice and access to specialist law library resources. The course provides preparation relevant to professional pathways including the Solicitors Qualifying Exam and academic requirements associated with training for the Bar. Graduates pursue careers across legal, business and public sector fields.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Law is at the heart of our society, informing and governing our everyday actions. The LLB Law course offers a distinctive approach to legal education that combines research-informed study with practice-led approaches. Students study the foundations of English and Welsh law and have the freedom to follow their own interests through a broad range of optional units while being challenged to analyse and critique the law and understand the social, economic, ethical and political contexts in which it operates. Career-focused learning is embedded throughout the course, including opportunities to apply legal theory in practice through clinical legal education at the Justice Hub, which offers free legal advice to members of the public and supports partnerships with the public, charitable and private sectors. Students develop a global perspective on law alongside essential skills, knowledge and experience for careers both within and beyond the legal profession. The programme includes engagement with areas such as family law, business law and criminal law, and introduces students to emerging fields such as LegalTech. Facilities supporting study include a moot court for simulated legal practice and access to specialist law library resources. The course provides preparation relevant to professional pathways including the Solicitors Qualifying Exam and academic requirements associated with training for the Bar. Graduates pursue careers across legal, business and public sector fields.</t>
+          <t>Whether you want to argue for human rights in the international courts, or help families closer to home, studying law means you can make a difference to people’s lives. If you choose a law degree, you’ll acquire a broad set of transferable skills and a greater understanding of the world we live in. Studying law helps you better understand how we interact as humans, and how we create the frameworks of a civilised society. You’ll learn to analyse and problem solve, articulate yourself in the written and spoken word, use your initiative, bond with other people, and likely become a passionate advocate on issues you care about. You could become an advice worker, trading standards officer or even a coroner. Roles as barristers and solicitors are expected to grow by around 3.5% over the next eight years, so there are plenty of places your law career could take you. Criminal law, law of contract, public and European law, foundations of law and social justice, law of tort and land use and regulation are areas you could study. Lawsuits, business development, conveyancing, finance, concise writing and legal research skills and commercial awareness are hard skills you'll develop. Communications, listening skills and empathy, sales, critical thinking and attention to detail are soft skills you'll develop.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
-        <is>
-          <t>Whether you want to argue for human rights in the international courts, or help families closer to home, studying law means you can make a difference to people’s lives. If you choose a law degree, you’ll acquire a broad set of transferable skills and a greater understanding of the world we live in. Studying law helps you better understand how we interact as humans, and how we create the frameworks of a civilised society. You’ll learn to analyse and problem solve, articulate yourself in the written and spoken word, use your initiative, bond with other people, and likely become a passionate advocate on issues you care about. You could become an advice worker, trading standards officer or even a coroner. Roles as barristers and solicitors are expected to grow by around 3.5% over the next eight years, so there are plenty of places your law career could take you. Criminal law, law of contract, public and European law, foundations of law and social justice, law of tort and land use and regulation are areas you could study. Lawsuits, business development, conveyancing, finance, concise writing and legal research skills and commercial awareness are hard skills you'll develop. Communications, listening skills and empathy, sales, critical thinking and attention to detail are soft skills you'll develop.</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
         <is>
           <t>Essex: What is LLB Law with Human Rights? The LLB Law with Human Rights is a three-year undergraduate qualifying law degree. It combines a full legal education with a dedicated focus on human rights at domestic, European, and international levels. You’ll study the core foundations of English law alongside specialist human rights modules, graduating with in-depth knowledge of how rights are protected and applied across different legal systems. The LLB Law with Human Rights combines a qualifying law degree with specialist training in UK, European, and international human rights law. It is ideal for students who want to study law through the lens of justice, rights, and social impact. The course is shaped by internationally recognised expertise in human rights. You’ll develop strong legal reasoning, research, and analytical skills while applying law to real-world human rights issues. Your studies explore how law operates as a practical tool for protecting individuals and contributing to fairer societies. Students study core legal foundations including legal method, contract, criminal law, public law, tort, land law, and equity, while also exploring UK and European human rights law and international human rights law as dedicated areas of study. The course examines how domestic law interacts with European and international legal frameworks and develops skills in case analysis, rights-based argumentation, and legal research. Students critically evaluate law within social, political, and ethical settings. An LLB Law with Human Rights prepares graduates for careers in law and policy including roles such as solicitor, barrister, paralegal or legal adviser, as well as careers within human rights organisations, charities and advocacy groups, government and public bodies, international organisations, policy research institutes and social justice organisations, and roles in compliance, governance and corporate responsibility.
 Manchester: Law is at the heart of our society, informing and governing our everyday actions. The LLB Law course offers a distinctive approach to legal education that combines research-informed study with practice-led approaches. Students study the foundations of English and Welsh law and have the freedom to follow their own interests through a broad range of optional units while being challenged to analyse and critique the law and understand the social, economic, ethical and political contexts in which it operates. Career-focused learning is embedded throughout the course, including opportunities to apply legal theory in practice through clinical legal education at the Justice Hub, which offers free legal advice to members of the public and supports partnerships with the public, charitable and private sectors. Students develop a global perspective on law alongside essential skills, knowledge and experience for careers both within and beyond the legal profession. The programme includes engagement with areas such as family law, business law and criminal law, and introduces students to emerging fields such as LegalTech. Facilities supporting study include a moot court for simulated legal practice and access to specialist law library resources. The course provides preparation relevant to professional pathways including the Solicitors Qualifying Exam and academic requirements associated with training for the Bar. Graduates pursue careers across legal, business and public sector fields.
@@ -1011,19 +934,18 @@
           <t>LIBERAL ARTS</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Knowledge is rooted in the experiences of people across the world. It is created from memory, culture, landscape and myth. This knowledge is often split into separate ‘disciplines' such as those in the sciences, maths, history, geography, literature and art. However, true knowledge does not recognise these boundaries; the world is complex, interconnected and networked. Our course is for you if you love studying a variety of subjects, and want to maintain this breadth of knowledge at university. With the opportunity to major in Psychology, History, Literature, Art History, Philosophy, Politics, Media Studies or Sociology, you broaden your horizons by exploring the ways in which the humanities and social sciences help us to think imaginatively and critically about the worlds we live in. You take modules which cover the historical foundations of the humanities, challenge dominant worldviews, and explore innovative and subversive essays and manifestos. The flexible structure of this course allows you to choose a range of optional modules across literature, film, philosophy, history of art, history, linguistics, politics, sociology and modern languages. The types of issues and problems you might explore include how commercial and independent films interpret human relationships, how to compose your own writing inspired by the great essayists, important philosophical questions about life, death and religion, great works of art and literature, and languages. Based within our School of Philosophical, Historical and Interdisciplinary Studies, the choice is yours: you choose your modules based on your own background and interests. You engage with unusual, controversial and provocative ideas so that you can use the humanities and social sciences to become critically aware and possess the tools to change the world for the better. As a liberal arts graduate, you'll be provided with an all-round education that can lead to a broad range of knowledge, strong communication skills and the ability to think critically. A Liberal Arts course can lead to a wide variety of careers in fields such as media, journalism, publishing, local government, voluntary agencies, librarianship, finance and management. Our recent graduates have gone on to work for organisations including Euromoney, a financial publication company, a housing association and an English language school in Japan.</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Knowledge is rooted in the experiences of people across the world. It is created from memory, culture, landscape and myth. This knowledge is often split into separate ‘disciplines' such as those in the sciences, maths, history, geography, literature and art. However, true knowledge does not recognise these boundaries; the world is complex, interconnected and networked. Our course is for you if you love studying a variety of subjects, and want to maintain this breadth of knowledge at university. With the opportunity to major in Psychology, History, Literature, Art History, Philosophy, Politics, Media Studies or Sociology, you broaden your horizons by exploring the ways in which the humanities and social sciences help us to think imaginatively and critically about the worlds we live in. You take modules which cover the historical foundations of the humanities, challenge dominant worldviews, and explore innovative and subversive essays and manifestos. The flexible structure of this course allows you to choose a range of optional modules across literature, film, philosophy, history of art, history, linguistics, politics, sociology and modern languages. The types of issues and problems you might explore include how commercial and independent films interpret human relationships, how to compose your own writing inspired by the great essayists, important philosophical questions about life, death and religion, great works of art and literature, and languages. Based within our School of Philosophical, Historical and Interdisciplinary Studies, the choice is yours: you choose your modules based on your own background and interests. You engage with unusual, controversial and provocative ideas so that you can use the humanities and social sciences to become critically aware and possess the tools to change the world for the better. As a liberal arts graduate, you'll be provided with an all-round education that can lead to a broad range of knowledge, strong communication skills and the ability to think critically. A Liberal Arts course can lead to a wide variety of careers in fields such as media, journalism, publishing, local government, voluntary agencies, librarianship, finance and management. Our recent graduates have gone on to work for organisations including Euromoney, a financial publication company, a housing association and an English language school in Japan.</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
           <t>Liberal Arts is highly flexible, allowing students to create their own unique course, combining different subject areas within and beyond the School of Arts, Languages and Cultures. With an emphasis on interdisciplinary learning, students can tailor the course, aligning it to their interests and passions, whilst responding to key issues that affect the flourishing of free citizens. This course is ideal for individuals who have a wide range of interests and a passion for making a difference in the world. Our most distinctive research resource is internationally renowned The John Rylands Library, which holds one of the finest collections of rare books, manuscripts, and archives in the world. Manchester Museum, Whitworth Art Gallery, and Museum of Medicine and Health all feature throughout the course, and we also have strong links with the Museum of Science and Industry (MOSI). Studying with us helps you develop versatile, transferable and specialist skills, including independent working, time management and planning skills, collaboration, teamwork, leadership, communications skills to relate to a range of audiences, and an ability to develop research that responds to real-world challenges by engaging with organisations and institutions. Gain professional experience through a work placement year. Our undergraduate degrees are designed to make it easy to progress into postgraduate study if you choose. We offer a wide range of specialist master’s courses, with fast-tracked enrolment available for high-achieving undergraduate students. You can also take part in our Stellify programme, developing leadership and professional skills while contributing to your community through volunteering.</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
         <is>
           <t>Essex: Knowledge is rooted in the experiences of people across the world. It is created from memory, culture, landscape and myth. This knowledge is often split into separate ‘disciplines' such as those in the sciences, maths, history, geography, literature and art. However, true knowledge does not recognise these boundaries; the world is complex, interconnected and networked. Our course is for you if you love studying a variety of subjects, and want to maintain this breadth of knowledge at university. With the opportunity to major in Psychology, History, Literature, Art History, Philosophy, Politics, Media Studies or Sociology, you broaden your horizons by exploring the ways in which the humanities and social sciences help us to think imaginatively and critically about the worlds we live in. You take modules which cover the historical foundations of the humanities, challenge dominant worldviews, and explore innovative and subversive essays and manifestos. The flexible structure of this course allows you to choose a range of optional modules across literature, film, philosophy, history of art, history, linguistics, politics, sociology and modern languages. The types of issues and problems you might explore include how commercial and independent films interpret human relationships, how to compose your own writing inspired by the great essayists, important philosophical questions about life, death and religion, great works of art and literature, and languages. Based within our School of Philosophical, Historical and Interdisciplinary Studies, the choice is yours: you choose your modules based on your own background and interests. You engage with unusual, controversial and provocative ideas so that you can use the humanities and social sciences to become critically aware and possess the tools to change the world for the better. As a liberal arts graduate, you'll be provided with an all-round education that can lead to a broad range of knowledge, strong communication skills and the ability to think critically. A Liberal Arts course can lead to a wide variety of careers in fields such as media, journalism, publishing, local government, voluntary agencies, librarianship, finance and management. Our recent graduates have gone on to work for organisations including Euromoney, a financial publication company, a housing association and an English language school in Japan.
 Manchester: Liberal Arts is highly flexible, allowing students to create their own unique course, combining different subject areas within and beyond the School of Arts, Languages and Cultures. With an emphasis on interdisciplinary learning, students can tailor the course, aligning it to their interests and passions, whilst responding to key issues that affect the flourishing of free citizens. This course is ideal for individuals who have a wide range of interests and a passion for making a difference in the world. Our most distinctive research resource is internationally renowned The John Rylands Library, which holds one of the finest collections of rare books, manuscripts, and archives in the world. Manchester Museum, Whitworth Art Gallery, and Museum of Medicine and Health all feature throughout the course, and we also have strong links with the Museum of Science and Industry (MOSI). Studying with us helps you develop versatile, transferable and specialist skills, including independent working, time management and planning skills, collaboration, teamwork, leadership, communications skills to relate to a range of audiences, and an ability to develop research that responds to real-world challenges by engaging with organisations and institutions. Gain professional experience through a work placement year. Our undergraduate degrees are designed to make it easy to progress into postgraduate study if you choose. We offer a wide range of specialist master’s courses, with fast-tracked enrolment available for high-achieving undergraduate students. You can also take part in our Stellify programme, developing leadership and professional skills while contributing to your community through volunteering.</t>
@@ -1041,25 +963,20 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Creative Producing; Creative Writing; Drama and Creative Writing; English Language and Literature; English Literature; Film Studies and Literature; Film and Creative Writing; History and Literature; Journalism and Literature</t>
+          <t>All writers are first of all readers and all readers are writers, for without the active participation of readers a book is never fully realised. Our BA Literature and Creative Writing offers a unique approach to the practice of reading and writing, combining more familiar British and American perspectives and readings with other influential schools of writing, from the study of tradition and myth to the innovative practice of the Workshop of Potential Literature or Oulipo in France. You deepen your knowledge of literary tradition across a variety of genres in order to develop your practical skills of understanding, expression and invention. Pursue your love of reading and explore some of the most important novels, poems, and plays from the United States, the Caribbean and Europe while developing your own writing through a variety of planned readings and writing exercises. We'll teach you to be your own editor; critically judging your own and others' work is invaluable in transforming your work from something good to something great. At the beginning of your course, you receive a highly focused introduction to the study of literature alongside intensive modules in creative writing, covering myth, innovation and tradition, prose, and poetry. A module on writing for radio allows you to go into a studio and record a radio play. You then progress to look at a range of specialist topics such as experimental writing and surrealism, myth and fairytale, translating novels for the screen, American literature, Shakespeare, and science fiction. Our course develops your abilities as a reader and writer while allowing you to take options from the other courses within our Department of Literature, Film, and Theatre Studies including filmmaking, journalism and drama. Essex has nurtured a long tradition of distinguished writers whose work has shaped literature as we know it today, from past giants such as the American poets Robert Lowell and Ted Berrigan, to contemporary writers such as mythographer and novelist Dame Marina Warner, and Booker Prize-winner Ben Okri. Many of our creative writing students have gone on to successfully publish their work, notable recent alumni including Ida Løkås, who won a major literary prize in Norway for The Beauty That Flows Past securing a book deal; Alexia Casale, whose novel Bone Dragon was published by Faber &amp; Faber and featured on The Financial Times Young Adult Books of the Year list and The Independent's Books of the Year list; Elaine Ewert, who placed second in the New Welsh Writing Awards; Patricia Borlenghi, founder of Patrician Press which has published works by a number of our alumni; and Petra Mcqueen, who has written for The Guardian and runs creative writing courses. Our graduates are also ideally prepared for careers in the media, education, publishing, advertising, and the film and theatre industries, with particular success in publishing and theatre.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>All writers are first of all readers and all readers are writers, for without the active participation of readers a book is never fully realised. Our BA Literature and Creative Writing offers a unique approach to the practice of reading and writing, combining more familiar British and American perspectives and readings with other influential schools of writing, from the study of tradition and myth to the innovative practice of the Workshop of Potential Literature or Oulipo in France. You deepen your knowledge of literary tradition across a variety of genres in order to develop your practical skills of understanding, expression and invention. Pursue your love of reading and explore some of the most important novels, poems, and plays from the United States, the Caribbean and Europe while developing your own writing through a variety of planned readings and writing exercises. We'll teach you to be your own editor; critically judging your own and others' work is invaluable in transforming your work from something good to something great. At the beginning of your course, you receive a highly focused introduction to the study of literature alongside intensive modules in creative writing, covering myth, innovation and tradition, prose, and poetry. A module on writing for radio allows you to go into a studio and record a radio play. You then progress to look at a range of specialist topics such as experimental writing and surrealism, myth and fairytale, translating novels for the screen, American literature, Shakespeare, and science fiction. Our course develops your abilities as a reader and writer while allowing you to take options from the other courses within our Department of Literature, Film, and Theatre Studies including filmmaking, journalism and drama. Essex has nurtured a long tradition of distinguished writers whose work has shaped literature as we know it today, from past giants such as the American poets Robert Lowell and Ted Berrigan, to contemporary writers such as mythographer and novelist Dame Marina Warner, and Booker Prize-winner Ben Okri. Many of our creative writing students have gone on to successfully publish their work, notable recent alumni including Ida Løkås, who won a major literary prize in Norway for The Beauty That Flows Past securing a book deal; Alexia Casale, whose novel Bone Dragon was published by Faber &amp; Faber and featured on The Financial Times Young Adult Books of the Year list and The Independent's Books of the Year list; Elaine Ewert, who placed second in the New Welsh Writing Awards; Patricia Borlenghi, founder of Patrician Press which has published works by a number of our alumni; and Petra Mcqueen, who has written for The Guardian and runs creative writing courses. Our graduates are also ideally prepared for careers in the media, education, publishing, advertising, and the film and theatre industries, with particular success in publishing and theatre.</t>
+          <t>BA English Literature with Creative Writing is a small, specialised creative writing pathway within an English Literature degree, in which you will take 33% of your credits in creative writing in your second and third years. The course covers the full range of English literature from Old English to the present day. The creative writing component of the course focuses on fiction and poetry writing. The course will introduce you to techniques of fiction and poetry writing, and develop your understanding of the craft of writing, the nature and necessity of revision, and the importance of being able to give and receive constructive feedback. The creative writing component of the degree will be taught in small group workshops. You will write your own poems and stories regularly, read relevant work from established writers, and respond to examples of contemporary poetry and fiction. There will be in-class writing exercises and an introduction to workshopping. You will become part of a thriving community of students, lecturers, and writers at The University of Manchester, based in the heart of a UNESCO City of Literature that has produced some of the world's greatest writers and has a thriving literature and arts scene, including major events like Manchester Literature Festival. Apply your subject-specific knowledge in a real-world context through a placement year in your third year of study. You can apply to spend one semester studying abroad during the second year of your degree. Exchange partners are offered in Europe, USA, Canada, Australia, New Zealand, Hong Kong, and Singapore. Manchester Literature Festival holds literary events across Manchester throughout the year, many in partnership with the University. The Centre for New Writing also hosts a regular public event series, Literature Live, which brings contemporary novelists and poets to the University to read and engage in conversation. The John Rylands Library is home to one of the world's richest and most unique collections of manuscripts, maps, works of art, and objects. The University is home to the Centre for New Writing, a major hub for new writing excellence and award-winning teaching staff. The University of Manchester Library is one of only five National Research Libraries and provides access to internationally renowned archival collections. Students also have access to cultural assets including the Whitworth Art Gallery and Manchester Museum. All courses are designed to equip students with strong critical analysis skills, the ability to articulate knowledge of concepts and theories, and the ability to work and think independently, critically and creatively. Students have access to dedicated, subject-specific careers support throughout their studies and for up to two years after graduation. Undergraduate courses are designed to provide an easy transition into postgraduate study. Students can take part in the Stellify programme alongside their degrees, developing professional and leadership skills while contributing to their communities through volunteering. Graduates have gone on to work in a variety of industries including positions with the BBC, KPMG, Deloitte, Marks and Spencer, Aviva, Accenture and Barclays.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BA English Literature with Creative Writing is a small, specialised creative writing pathway within an English Literature degree, in which you will take 33% of your credits in creative writing in your second and third years. The course covers the full range of English literature from Old English to the present day. The creative writing component of the course focuses on fiction and poetry writing. The course will introduce you to techniques of fiction and poetry writing, and develop your understanding of the craft of writing, the nature and necessity of revision, and the importance of being able to give and receive constructive feedback. The creative writing component of the degree will be taught in small group workshops. You will write your own poems and stories regularly, read relevant work from established writers, and respond to examples of contemporary poetry and fiction. There will be in-class writing exercises and an introduction to workshopping. You will become part of a thriving community of students, lecturers, and writers at The University of Manchester, based in the heart of a UNESCO City of Literature that has produced some of the world's greatest writers and has a thriving literature and arts scene, including major events like Manchester Literature Festival. Apply your subject-specific knowledge in a real-world context through a placement year in your third year of study. You can apply to spend one semester studying abroad during the second year of your degree. Exchange partners are offered in Europe, USA, Canada, Australia, New Zealand, Hong Kong, and Singapore. Manchester Literature Festival holds literary events across Manchester throughout the year, many in partnership with the University. The Centre for New Writing also hosts a regular public event series, Literature Live, which brings contemporary novelists and poets to the University to read and engage in conversation. The John Rylands Library is home to one of the world's richest and most unique collections of manuscripts, maps, works of art, and objects. The University is home to the Centre for New Writing, a major hub for new writing excellence and award-winning teaching staff. The University of Manchester Library is one of only five National Research Libraries and provides access to internationally renowned archival collections. Students also have access to cultural assets including the Whitworth Art Gallery and Manchester Museum. All courses are designed to equip students with strong critical analysis skills, the ability to articulate knowledge of concepts and theories, and the ability to work and think independently, critically and creatively. Students have access to dedicated, subject-specific careers support throughout their studies and for up to two years after graduation. Undergraduate courses are designed to provide an easy transition into postgraduate study. Students can take part in the Stellify programme alongside their degrees, developing professional and leadership skills while contributing to their communities through volunteering. Graduates have gone on to work in a variety of industries including positions with the BBC, KPMG, Deloitte, Marks and Spencer, Aviva, Accenture and Barclays.</t>
+          <t>We’re all natural storytellers, and studying English literature and creative writing offers a way into the human imagination and the key to creative expression. Studying English literature and creative writing engrosses you in literary masterpieces and builds essential skills that are sought after in the professional world. It encourages critical thinking, analytical skills, and effective communication, creating storytellers and perceptive interpreters of cultural differences. The comprehensive understanding of language, narrative structures, and different genres equips graduates for a variety of career paths. Whether looking at roles in publishing, journalism, content creation, marketing, or education, graduates will have the ability to craft compelling narratives and adapt to different communication styles. Beyond traditional careers, the creative and analytical skills gained prepare you for roles in digital media, advertising, and even entrepreneurship, where the power of persuasive storytelling is essential. Literature in theory, modern world literatures, creative thinking, Shakespeare, American poetry, modes of reading and contemporary fiction are areas you could study. Ability to critically analyse and interpret literary texts, close reading skills, development of characters, plot structures and dialogue, and analyse arguments and evaluate evidence are hard skills you'll develop. Creativity, critical thinking, written communication and storytelling are soft skills you'll develop. Career options include journalist, newspaper and periodical editors, authors, writers and translators, web content professionals, advertising account managers, public relations professionals, customer service managers and supervisors, human resources and industrial relations officers, business and related research professionals, and research and development managers.</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
-        <is>
-          <t>We’re all natural storytellers, and studying English literature and creative writing offers a way into the human imagination and the key to creative expression. Studying English literature and creative writing engrosses you in literary masterpieces and builds essential skills that are sought after in the professional world. It encourages critical thinking, analytical skills, and effective communication, creating storytellers and perceptive interpreters of cultural differences. The comprehensive understanding of language, narrative structures, and different genres equips graduates for a variety of career paths. Whether looking at roles in publishing, journalism, content creation, marketing, or education, graduates will have the ability to craft compelling narratives and adapt to different communication styles. Beyond traditional careers, the creative and analytical skills gained prepare you for roles in digital media, advertising, and even entrepreneurship, where the power of persuasive storytelling is essential. Literature in theory, modern world literatures, creative thinking, Shakespeare, American poetry, modes of reading and contemporary fiction are areas you could study. Ability to critically analyse and interpret literary texts, close reading skills, development of characters, plot structures and dialogue, and analyse arguments and evaluate evidence are hard skills you'll develop. Creativity, critical thinking, written communication and storytelling are soft skills you'll develop. Career options include journalist, newspaper and periodical editors, authors, writers and translators, web content professionals, advertising account managers, public relations professionals, customer service managers and supervisors, human resources and industrial relations officers, business and related research professionals, and research and development managers.</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
         <is>
           <t>Essex: All writers are first of all readers and all readers are writers, for without the active participation of readers a book is never fully realised. Our BA Literature and Creative Writing offers a unique approach to the practice of reading and writing, combining more familiar British and American perspectives and readings with other influential schools of writing, from the study of tradition and myth to the innovative practice of the Workshop of Potential Literature or Oulipo in France. You deepen your knowledge of literary tradition across a variety of genres in order to develop your practical skills of understanding, expression and invention. Pursue your love of reading and explore some of the most important novels, poems, and plays from the United States, the Caribbean and Europe while developing your own writing through a variety of planned readings and writing exercises. We'll teach you to be your own editor; critically judging your own and others' work is invaluable in transforming your work from something good to something great. At the beginning of your course, you receive a highly focused introduction to the study of literature alongside intensive modules in creative writing, covering myth, innovation and tradition, prose, and poetry. A module on writing for radio allows you to go into a studio and record a radio play. You then progress to look at a range of specialist topics such as experimental writing and surrealism, myth and fairytale, translating novels for the screen, American literature, Shakespeare, and science fiction. Our course develops your abilities as a reader and writer while allowing you to take options from the other courses within our Department of Literature, Film, and Theatre Studies including filmmaking, journalism and drama. Essex has nurtured a long tradition of distinguished writers whose work has shaped literature as we know it today, from past giants such as the American poets Robert Lowell and Ted Berrigan, to contemporary writers such as mythographer and novelist Dame Marina Warner, and Booker Prize-winner Ben Okri. Many of our creative writing students have gone on to successfully publish their work, notable recent alumni including Ida Løkås, who won a major literary prize in Norway for The Beauty That Flows Past securing a book deal; Alexia Casale, whose novel Bone Dragon was published by Faber &amp; Faber and featured on The Financial Times Young Adult Books of the Year list and The Independent's Books of the Year list; Elaine Ewert, who placed second in the New Welsh Writing Awards; Patricia Borlenghi, founder of Patrician Press which has published works by a number of our alumni; and Petra Mcqueen, who has written for The Guardian and runs creative writing courses. Our graduates are also ideally prepared for careers in the media, education, publishing, advertising, and the film and theatre industries, with particular success in publishing and theatre.
 Manchester: BA English Literature with Creative Writing is a small, specialised creative writing pathway within an English Literature degree, in which you will take 33% of your credits in creative writing in your second and third years. The course covers the full range of English literature from Old English to the present day. The creative writing component of the course focuses on fiction and poetry writing. The course will introduce you to techniques of fiction and poetry writing, and develop your understanding of the craft of writing, the nature and necessity of revision, and the importance of being able to give and receive constructive feedback. The creative writing component of the degree will be taught in small group workshops. You will write your own poems and stories regularly, read relevant work from established writers, and respond to examples of contemporary poetry and fiction. There will be in-class writing exercises and an introduction to workshopping. You will become part of a thriving community of students, lecturers, and writers at The University of Manchester, based in the heart of a UNESCO City of Literature that has produced some of the world's greatest writers and has a thriving literature and arts scene, including major events like Manchester Literature Festival. Apply your subject-specific knowledge in a real-world context through a placement year in your third year of study. You can apply to spend one semester studying abroad during the second year of your degree. Exchange partners are offered in Europe, USA, Canada, Australia, New Zealand, Hong Kong, and Singapore. Manchester Literature Festival holds literary events across Manchester throughout the year, many in partnership with the University. The Centre for New Writing also hosts a regular public event series, Literature Live, which brings contemporary novelists and poets to the University to read and engage in conversation. The John Rylands Library is home to one of the world's richest and most unique collections of manuscripts, maps, works of art, and objects. The University is home to the Centre for New Writing, a major hub for new writing excellence and award-winning teaching staff. The University of Manchester Library is one of only five National Research Libraries and provides access to internationally renowned archival collections. Students also have access to cultural assets including the Whitworth Art Gallery and Manchester Museum. All courses are designed to equip students with strong critical analysis skills, the ability to articulate knowledge of concepts and theories, and the ability to work and think independently, critically and creatively. Students have access to dedicated, subject-specific careers support throughout their studies and for up to two years after graduation. Undergraduate courses are designed to provide an easy transition into postgraduate study. Students can take part in the Stellify programme alongside their degrees, developing professional and leadership skills while contributing to their communities through volunteering. Graduates have gone on to work in a variety of industries including positions with the BBC, KPMG, Deloitte, Marks and Spencer, Aviva, Accenture and Barclays.
@@ -1078,25 +995,20 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Economics and Mathematics; Mathematics and Data Science; Mathematics with Computing; Mathematics with Physics</t>
+          <t>Mathematics provides the logical foundations on which all of science, engineering and technology are built. Our BSc (Hons) Mathematics course gives you the chance to study both fundamental topics and their modern applications, including pure mathematics such as geometry, algebra, analysis and number theory, applied topics such as mathematical physics, cryptography, mathematical modelling, differential equations and dynamical systems, and statistical, financial and analytical methods such as optimisation and the study of risk. As well as these mathematical topics, your degree will develop your programming skills in languages such as Python and SQL, and you will learn to solve sophisticated problems using computational toolkits such as MATLAB, Maple and R. Our School of Mathematics, Statistics and Actuarial Science recognises the stand-alone and interdisciplinary aspects of mathematics, and this degree provides an exceptional range of in-demand transferrable skills for mathematically oriented careers from business, finance and commerce to industry, research, government and education. All our mathematical sciences degrees feature an employability component in every year of study, explicitly training sought-after skills and incorporating careers day events and seminars from speakers in industry. This programme will meet the educational requirements of the Chartered Mathematician designation, awarded by the Institute of Mathematics and its Applications, when it is followed by subsequent training and experience in employment to obtain equivalent competences to those specified by the Quality Assurance Agency (QAA) for taught masters degrees. Clear thinkers are required in every profession, so the successful mathematician has an extensive choice of potential careers. Mathematics students are in demand from a wide range of employers in a host of occupations, including financial analysis, management, public administration and accountancy. Our recent graduates have gone on to work for a wide range of high-profile companies, including KPMG, British Arab Commercial Bank and Johal and Company.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Mathematics provides the logical foundations on which all of science, engineering and technology are built. Our BSc (Hons) Mathematics course gives you the chance to study both fundamental topics and their modern applications, including pure mathematics such as geometry, algebra, analysis and number theory, applied topics such as mathematical physics, cryptography, mathematical modelling, differential equations and dynamical systems, and statistical, financial and analytical methods such as optimisation and the study of risk. As well as these mathematical topics, your degree will develop your programming skills in languages such as Python and SQL, and you will learn to solve sophisticated problems using computational toolkits such as MATLAB, Maple and R. Our School of Mathematics, Statistics and Actuarial Science recognises the stand-alone and interdisciplinary aspects of mathematics, and this degree provides an exceptional range of in-demand transferrable skills for mathematically oriented careers from business, finance and commerce to industry, research, government and education. All our mathematical sciences degrees feature an employability component in every year of study, explicitly training sought-after skills and incorporating careers day events and seminars from speakers in industry. This programme will meet the educational requirements of the Chartered Mathematician designation, awarded by the Institute of Mathematics and its Applications, when it is followed by subsequent training and experience in employment to obtain equivalent competences to those specified by the Quality Assurance Agency (QAA) for taught masters degrees. Clear thinkers are required in every profession, so the successful mathematician has an extensive choice of potential careers. Mathematics students are in demand from a wide range of employers in a host of occupations, including financial analysis, management, public administration and accountancy. Our recent graduates have gone on to work for a wide range of high-profile companies, including KPMG, British Arab Commercial Bank and Johal and Company.</t>
+          <t>Lay the foundations of a rewarding career with mathematics at its base by undertaking an undergraduate degree at Manchester. We offer a highly flexible degree programme, ensuring you obtain a strong all-round mathematical knowledge while encouraging you to focus on the areas that appeal most. You will cover core topics in the first year, developing your capacity to learn and apply mathematical ideas. In the second year you choose two from three themes: Pure Mathematics, Applied Mathematics, and Probability and Statistics, along with optional units such as Programming with Python. After the first two years you can choose the areas that interest you most and select options from other subject areas. In your final year you can undertake a staff-supervised mathematical project. You will develop a firm all-round mathematical knowledge and experience specialised results, methods and ideas. You can pursue whichever areas of mathematics interest you most and choose lecture courses from a widening range of options. Our flexible degree programme allows students to choose courses from other disciplines and a wide range of mathematics options. Small-group teaching in the first year supports student learning. Students may undertake a year on a work-based placement to gain professional experience. The Department of Mathematics is based in the Alan Turing Building. Facilities include computer clusters with mathematical and statistical software including Matlab and Mathematica. Studying mathematics develops skills and knowledge valued across professions including finance, industry, computing, management, statistics and teaching. Graduates have pursued careers in finance in firms such as KPMG, Goldman Sachs, PricewaterhouseCoopers, Deloitte, Barclays and Deutsche Bank. Many graduates undertake further programmes of study such as MSc degrees in Mathematics, Applied Mathematics, Finance, Business, Management and Computer Science.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Lay the foundations of a rewarding career with mathematics at its base by undertaking an undergraduate degree at Manchester. We offer a highly flexible degree programme, ensuring you obtain a strong all-round mathematical knowledge while encouraging you to focus on the areas that appeal most. You will cover core topics in the first year, developing your capacity to learn and apply mathematical ideas. In the second year you choose two from three themes: Pure Mathematics, Applied Mathematics, and Probability and Statistics, along with optional units such as Programming with Python. After the first two years you can choose the areas that interest you most and select options from other subject areas. In your final year you can undertake a staff-supervised mathematical project. You will develop a firm all-round mathematical knowledge and experience specialised results, methods and ideas. You can pursue whichever areas of mathematics interest you most and choose lecture courses from a widening range of options. Our flexible degree programme allows students to choose courses from other disciplines and a wide range of mathematics options. Small-group teaching in the first year supports student learning. Students may undertake a year on a work-based placement to gain professional experience. The Department of Mathematics is based in the Alan Turing Building. Facilities include computer clusters with mathematical and statistical software including Matlab and Mathematica. Studying mathematics develops skills and knowledge valued across professions including finance, industry, computing, management, statistics and teaching. Graduates have pursued careers in finance in firms such as KPMG, Goldman Sachs, PricewaterhouseCoopers, Deloitte, Barclays and Deutsche Bank. Many graduates undertake further programmes of study such as MSc degrees in Mathematics, Applied Mathematics, Finance, Business, Management and Computer Science.</t>
+          <t>Use logic and reason to analyse data and provide solutions in a wide range of employment sectors. As a mathematician or statistician you’ll use your problem-solving, analytical, and technical skills to help businesses in a range of sectors, from finance to government. Your interpretations could be used in anything from clinical trials, to climate predictions, to financial forecasting. You could end up in a management role, leading a team, or become self-employed as a consultant or financial adviser. You could also go on to further study, teaching or academic research, or work as a data scientist. Pure mathematics, applied mathematics, real analysis, statistics, mathematical modelling, probability and data science, differential equations, dynamics and motion, Bayesian statistics, medical statistics, stochastic modelling, scientistic computing and machine learning are areas you could study. Economics and finance, programming languages, project management, data analysis and statistics are hard skills you'll develop. Communication, management, research, planning and innovation are soft skills you'll develop. Career options include chartered accountant, bank clerk, investment analyst, insurance underwriter, actuary, financial manager, IT manager, software developers and programmers, quantity surveyor, research manager and teacher in further or higher education.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
-        <is>
-          <t>Use logic and reason to analyse data and provide solutions in a wide range of employment sectors. As a mathematician or statistician you’ll use your problem-solving, analytical, and technical skills to help businesses in a range of sectors, from finance to government. Your interpretations could be used in anything from clinical trials, to climate predictions, to financial forecasting. You could end up in a management role, leading a team, or become self-employed as a consultant or financial adviser. You could also go on to further study, teaching or academic research, or work as a data scientist. Pure mathematics, applied mathematics, real analysis, statistics, mathematical modelling, probability and data science, differential equations, dynamics and motion, Bayesian statistics, medical statistics, stochastic modelling, scientistic computing and machine learning are areas you could study. Economics and finance, programming languages, project management, data analysis and statistics are hard skills you'll develop. Communication, management, research, planning and innovation are soft skills you'll develop. Career options include chartered accountant, bank clerk, investment analyst, insurance underwriter, actuary, financial manager, IT manager, software developers and programmers, quantity surveyor, research manager and teacher in further or higher education.</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
         <is>
           <t>Essex: Mathematics provides the logical foundations on which all of science, engineering and technology are built. Our BSc (Hons) Mathematics course gives you the chance to study both fundamental topics and their modern applications, including pure mathematics such as geometry, algebra, analysis and number theory, applied topics such as mathematical physics, cryptography, mathematical modelling, differential equations and dynamical systems, and statistical, financial and analytical methods such as optimisation and the study of risk. As well as these mathematical topics, your degree will develop your programming skills in languages such as Python and SQL, and you will learn to solve sophisticated problems using computational toolkits such as MATLAB, Maple and R. Our School of Mathematics, Statistics and Actuarial Science recognises the stand-alone and interdisciplinary aspects of mathematics, and this degree provides an exceptional range of in-demand transferrable skills for mathematically oriented careers from business, finance and commerce to industry, research, government and education. All our mathematical sciences degrees feature an employability component in every year of study, explicitly training sought-after skills and incorporating careers day events and seminars from speakers in industry. This programme will meet the educational requirements of the Chartered Mathematician designation, awarded by the Institute of Mathematics and its Applications, when it is followed by subsequent training and experience in employment to obtain equivalent competences to those specified by the Quality Assurance Agency (QAA) for taught masters degrees. Clear thinkers are required in every profession, so the successful mathematician has an extensive choice of potential careers. Mathematics students are in demand from a wide range of employers in a host of occupations, including financial analysis, management, public administration and accountancy. Our recent graduates have gone on to work for a wide range of high-profile companies, including KPMG, British Arab Commercial Bank and Johal and Company.
 Manchester: Lay the foundations of a rewarding career with mathematics at its base by undertaking an undergraduate degree at Manchester. We offer a highly flexible degree programme, ensuring you obtain a strong all-round mathematical knowledge while encouraging you to focus on the areas that appeal most. You will cover core topics in the first year, developing your capacity to learn and apply mathematical ideas. In the second year you choose two from three themes: Pure Mathematics, Applied Mathematics, and Probability and Statistics, along with optional units such as Programming with Python. After the first two years you can choose the areas that interest you most and select options from other subject areas. In your final year you can undertake a staff-supervised mathematical project. You will develop a firm all-round mathematical knowledge and experience specialised results, methods and ideas. You can pursue whichever areas of mathematics interest you most and choose lecture courses from a widening range of options. Our flexible degree programme allows students to choose courses from other disciplines and a wide range of mathematics options. Small-group teaching in the first year supports student learning. Students may undertake a year on a work-based placement to gain professional experience. The Department of Mathematics is based in the Alan Turing Building. Facilities include computer clusters with mathematical and statistical software including Matlab and Mathematica. Studying mathematics develops skills and knowledge valued across professions including finance, industry, computing, management, statistics and teaching. Graduates have pursued careers in finance in firms such as KPMG, Goldman Sachs, PricewaterhouseCoopers, Deloitte, Barclays and Deutsche Bank. Many graduates undertake further programmes of study such as MSc degrees in Mathematics, Applied Mathematics, Finance, Business, Management and Computer Science.
@@ -1115,21 +1027,16 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Business Management with a Modern Language; Global Studies and Modern Languages; Journalism and Modern Languages; Modern History; Modern History and International Relations; Modern History and Politics; Modern Languages and Linguistics; Modern Languages with Latin American Studies; Spanish Studies and Modern Languages</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
           <t>Language is fundamental to our thought, our relationships, and our civilisations. Through language we transmit knowledge, from inviting someone for coffee, to promoting the latest scientific theory, to settling global political disputes. On our course you can study up to three languages choosing between French, German, Italian and Spanish from beginner or post-A level standard. Portuguese can be studied from a pre-A level standard. These languages can be studied alongside language expert modules which cover a range of cultural and professional skills. Each of these languages are widely used in the business world, and we take you to a level of near-fluency; so many of our graduates have gone on to develop successful global careers with international firms looking for language specialists. In addition to the language skills you develop on our course, you also explore a range of modules on global cultures, histories and politics so that you can really understand another country beyond just being able to communicate in the native language. Study topics include world cinema, translation, interpreting and subtitling, popular music, and visual history. If you want a global outlook, are interested in human communication, and want to study for a degree with real-world practical value in a world-class department, welcome to Essex. Companies and organisations in the UK and abroad are struggling to find university graduates who are fluent in at least one other language apart from English. Being an Essex modern languages graduate places you in a very advantageous position. You will be able to speak and write fluently, or to a very competent standard, in up to four languages. Language skills are in scarce supply and can be used in almost any job. Our graduates become teachers, translators, administrators and journalists, and their language skills have enabled them to work in fields including banking, entertainment, media, education and tourism, as well as for a host of UK and international companies. A degree in modern languages lends itself to careers in education, translation, interpretation, trade, public relations, communications, immigration or diplomacy. For example, one of our recent graduates is now a newspaper editor in Spain, while another teaches modern languages in Southampton.</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Studying languages not only unlocks global cultures but also transforms you into a versatile communicator, making you a valuable asset for many industries. When you choose languages, you’re opening a world of opportunities for career growth because knowing multiple languages makes you a valuable asset in our interconnected global landscape. Being multilingual puts you in high demand across various industries, from international business and diplomacy to translation, journalism, and tourism. Your ability to bridge communication gaps opens conversation for cross-cultural understanding, making you indispensable in an increasingly interconnected and multicultural world. Linguistics, translation and interpreting, written and oral grammar, science of language and communication, history of language, literature and culture, history and politics are areas you could study. Fluency in another language, ability to translate and interpret, understanding of different grammatical structures and knowledge of cultural traditions and customs are hard skills you'll develop. Cultural sensitivity, communication skills, curiosity and tolerance for ambiguity and uncertainty are soft skills you'll develop. Career options include translators, journalists, public relations professionals, hotel and accommodation managers and travel agency managers.</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr">
-        <is>
-          <t>Studying languages not only unlocks global cultures but also transforms you into a versatile communicator, making you a valuable asset for many industries. When you choose languages, you’re opening a world of opportunities for career growth because knowing multiple languages makes you a valuable asset in our interconnected global landscape. Being multilingual puts you in high demand across various industries, from international business and diplomacy to translation, journalism, and tourism. Your ability to bridge communication gaps opens conversation for cross-cultural understanding, making you indispensable in an increasingly interconnected and multicultural world. Linguistics, translation and interpreting, written and oral grammar, science of language and communication, history of language, literature and culture, history and politics are areas you could study. Fluency in another language, ability to translate and interpret, understanding of different grammatical structures and knowledge of cultural traditions and customs are hard skills you'll develop. Cultural sensitivity, communication skills, curiosity and tolerance for ambiguity and uncertainty are soft skills you'll develop. Career options include translators, journalists, public relations professionals, hotel and accommodation managers and travel agency managers.</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
         <is>
           <t>Essex: Language is fundamental to our thought, our relationships, and our civilisations. Through language we transmit knowledge, from inviting someone for coffee, to promoting the latest scientific theory, to settling global political disputes. On our course you can study up to three languages choosing between French, German, Italian and Spanish from beginner or post-A level standard. Portuguese can be studied from a pre-A level standard. These languages can be studied alongside language expert modules which cover a range of cultural and professional skills. Each of these languages are widely used in the business world, and we take you to a level of near-fluency; so many of our graduates have gone on to develop successful global careers with international firms looking for language specialists. In addition to the language skills you develop on our course, you also explore a range of modules on global cultures, histories and politics so that you can really understand another country beyond just being able to communicate in the native language. Study topics include world cinema, translation, interpreting and subtitling, popular music, and visual history. If you want a global outlook, are interested in human communication, and want to study for a degree with real-world practical value in a world-class department, welcome to Essex. Companies and organisations in the UK and abroad are struggling to find university graduates who are fluent in at least one other language apart from English. Being an Essex modern languages graduate places you in a very advantageous position. You will be able to speak and write fluently, or to a very competent standard, in up to four languages. Language skills are in scarce supply and can be used in almost any job. Our graduates become teachers, translators, administrators and journalists, and their language skills have enabled them to work in fields including banking, entertainment, media, education and tourism, as well as for a host of UK and international companies. A degree in modern languages lends itself to careers in education, translation, interpretation, trade, public relations, communications, immigration or diplomacy. For example, one of our recent graduates is now a newspaper editor in Spain, while another teaches modern languages in Southampton.
 UCAS: Studying languages not only unlocks global cultures but also transforms you into a versatile communicator, making you a valuable asset for many industries. When you choose languages, you’re opening a world of opportunities for career growth because knowing multiple languages makes you a valuable asset in our interconnected global landscape. Being multilingual puts you in high demand across various industries, from international business and diplomacy to translation, journalism, and tourism. Your ability to bridge communication gaps opens conversation for cross-cultural understanding, making you indispensable in an increasingly interconnected and multicultural world. Linguistics, translation and interpreting, written and oral grammar, science of language and communication, history of language, literature and culture, history and politics are areas you could study. Fluency in another language, ability to translate and interpret, understanding of different grammatical structures and knowledge of cultural traditions and customs are hard skills you'll develop. Cultural sensitivity, communication skills, curiosity and tolerance for ambiguity and uncertainty are soft skills you'll develop. Career options include translators, journalists, public relations professionals, hotel and accommodation managers and travel agency managers.</t>
@@ -1147,25 +1054,20 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Continental Philosophy; Law with Philosophy; Philosophy and Politics; Philosophy with Business Management; Philosophy, Politics and Economics</t>
+          <t>Our BA Philosophy will feed your intellectual curiosity and challenge your thinking. You'll acquire the skills required to dig deeper into ideas and question received wisdom. You'll rigorously examine the most fundamental questions about human life: Does God exist? Is material success all that counts in life? What do I owe to others? How free am I to decide my own future? At Essex, we take philosophy back to its roots in everyday existential, social, and political problems. We embrace the relevance of philosophy to other forms of enquiry – political, cultural, legal, medical and aesthetic – and bring this to bear on urgent issues in public life, such as the controversial issues raised by mental health legislation or public policy regarding end of life care. We cover a wide range of topics from the meaning of life to capitalism and its critics, from ancient philosophy to current trends in European thought, with particular strengths in ethics, political philosophy, philosophy of religion, and European philosophy including critical theory, phenomenology and existentialism. A degree in Philosophy at Essex provides you with the ability to analyse and solve difficult problems, the ability to think clearly, creatively and self-critically, and the ability to work in a team taking a collaborative approach to problems. Philosophy graduates are therefore well-suited to a wide range of occupations including law, PR, journalism and the media, the Civil Service, charity work, banking and the NHS.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Our BA Philosophy will feed your intellectual curiosity and challenge your thinking. You'll acquire the skills required to dig deeper into ideas and question received wisdom. You'll rigorously examine the most fundamental questions about human life: Does God exist? Is material success all that counts in life? What do I owe to others? How free am I to decide my own future? At Essex, we take philosophy back to its roots in everyday existential, social, and political problems. We embrace the relevance of philosophy to other forms of enquiry – political, cultural, legal, medical and aesthetic – and bring this to bear on urgent issues in public life, such as the controversial issues raised by mental health legislation or public policy regarding end of life care. We cover a wide range of topics from the meaning of life to capitalism and its critics, from ancient philosophy to current trends in European thought, with particular strengths in ethics, political philosophy, philosophy of religion, and European philosophy including critical theory, phenomenology and existentialism. A degree in Philosophy at Essex provides you with the ability to analyse and solve difficult problems, the ability to think clearly, creatively and self-critically, and the ability to work in a team taking a collaborative approach to problems. Philosophy graduates are therefore well-suited to a wide range of occupations including law, PR, journalism and the media, the Civil Service, charity work, banking and the NHS.</t>
+          <t>Studying BA Philosophy enables you to critically analyse answers to fundamental questions such as free will, ethics and the nature of reality. Students debate questions such as whether the world outside our minds exists, what makes something morally right, whether humans have free will, whether God exists and whether the human mind is purely physical. Students develop skills including presenting effective and rigorous arguments, developing criticisms of other people’s arguments and views, explaining complex material clearly and concisely, and analysing philosophical problems where reasonable people hold different views. Provide structured yet flexible study informed by current research. Provide a curriculum covering texts and questions central to the analytical tradition in philosophy and traditions outside it. Develop subject-specific knowledge, cognitive skills and transferable skills for employment or further academic study. Students may apply to study abroad for a year at partner universities. Students may apply for a paid Q-Step internship between Years 2 and 3. Students may undertake a Professional Experience Year, extending the degree to four years. Philosophy graduates pursue careers in journalism, media, charities, consultancy, civil service, finance, marketing, public relations, social work, teaching and law. Recent graduates have worked for organisations including Manchester City Council, Royal Bank of Scotland, Palgrave MacMillan, Lloyds TSB, the Foreign and Commonwealth Office, TeachFirst and Siemens. Many graduates undertake postgraduate study in philosophy, teaching, law, political theory, business or marketing.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Studying BA Philosophy enables you to critically analyse answers to fundamental questions such as free will, ethics and the nature of reality. Students debate questions such as whether the world outside our minds exists, what makes something morally right, whether humans have free will, whether God exists and whether the human mind is purely physical. Students develop skills including presenting effective and rigorous arguments, developing criticisms of other people’s arguments and views, explaining complex material clearly and concisely, and analysing philosophical problems where reasonable people hold different views. Provide structured yet flexible study informed by current research. Provide a curriculum covering texts and questions central to the analytical tradition in philosophy and traditions outside it. Develop subject-specific knowledge, cognitive skills and transferable skills for employment or further academic study. Students may apply to study abroad for a year at partner universities. Students may apply for a paid Q-Step internship between Years 2 and 3. Students may undertake a Professional Experience Year, extending the degree to four years. Philosophy graduates pursue careers in journalism, media, charities, consultancy, civil service, finance, marketing, public relations, social work, teaching and law. Recent graduates have worked for organisations including Manchester City Council, Royal Bank of Scotland, Palgrave MacMillan, Lloyds TSB, the Foreign and Commonwealth Office, TeachFirst and Siemens. Many graduates undertake postgraduate study in philosophy, teaching, law, political theory, business or marketing.</t>
+          <t>Choose philosophy for a rigorous exploration into questioning, analysis, and the development of sharp, independent thinking skills that navigate the complexities of our world. Philosophy navigates human thought, offering an understanding of fundamental questions about existence, morality, and knowledge. Beyond fostering critical thinking and intellectual curiosity, a degree in philosophy cultivates skills highly sought after in lots of professions. Graduates often find themselves in careers such as law, journalism, education, business, and public policy. The ability to analyse complex issues, articulate compelling arguments, and engage in interesting discussions help philosophers to thrive in roles that demand clarity of thought and effective communication. The adaptability and broad perspective gained through philosophical studies set people up for success in a rapidly evolving job market, making philosophy not just a field of study, but a foundation for a choice of careers. Symbolic logic, reason, argument, and analysis, history of philosophy, Sartre and existentialism, metaphysics, social and political theory and engaging with the humanities are areas you could study. Analytical reasoning skills, accessing and evaluating academic sources, historical understanding and precision and attention to detail are hard skills you'll develop. Communication skills, both written and verbal, open mindedness, cultural awareness and flexibility in thinking are soft skills you'll develop. Career options include solicitors and lawyers, legal associate professionals, journalists, newspaper and periodical editors.</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
-        <is>
-          <t>Choose philosophy for a rigorous exploration into questioning, analysis, and the development of sharp, independent thinking skills that navigate the complexities of our world. Philosophy navigates human thought, offering an understanding of fundamental questions about existence, morality, and knowledge. Beyond fostering critical thinking and intellectual curiosity, a degree in philosophy cultivates skills highly sought after in lots of professions. Graduates often find themselves in careers such as law, journalism, education, business, and public policy. The ability to analyse complex issues, articulate compelling arguments, and engage in interesting discussions help philosophers to thrive in roles that demand clarity of thought and effective communication. The adaptability and broad perspective gained through philosophical studies set people up for success in a rapidly evolving job market, making philosophy not just a field of study, but a foundation for a choice of careers. Symbolic logic, reason, argument, and analysis, history of philosophy, Sartre and existentialism, metaphysics, social and political theory and engaging with the humanities are areas you could study. Analytical reasoning skills, accessing and evaluating academic sources, historical understanding and precision and attention to detail are hard skills you'll develop. Communication skills, both written and verbal, open mindedness, cultural awareness and flexibility in thinking are soft skills you'll develop. Career options include solicitors and lawyers, legal associate professionals, journalists, newspaper and periodical editors.</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
         <is>
           <t>Essex: Our BA Philosophy will feed your intellectual curiosity and challenge your thinking. You'll acquire the skills required to dig deeper into ideas and question received wisdom. You'll rigorously examine the most fundamental questions about human life: Does God exist? Is material success all that counts in life? What do I owe to others? How free am I to decide my own future? At Essex, we take philosophy back to its roots in everyday existential, social, and political problems. We embrace the relevance of philosophy to other forms of enquiry – political, cultural, legal, medical and aesthetic – and bring this to bear on urgent issues in public life, such as the controversial issues raised by mental health legislation or public policy regarding end of life care. We cover a wide range of topics from the meaning of life to capitalism and its critics, from ancient philosophy to current trends in European thought, with particular strengths in ethics, political philosophy, philosophy of religion, and European philosophy including critical theory, phenomenology and existentialism. A degree in Philosophy at Essex provides you with the ability to analyse and solve difficult problems, the ability to think clearly, creatively and self-critically, and the ability to work in a team taking a collaborative approach to problems. Philosophy graduates are therefore well-suited to a wide range of occupations including law, PR, journalism and the media, the Civil Service, charity work, banking and the NHS.
 Manchester: Studying BA Philosophy enables you to critically analyse answers to fundamental questions such as free will, ethics and the nature of reality. Students debate questions such as whether the world outside our minds exists, what makes something morally right, whether humans have free will, whether God exists and whether the human mind is purely physical. Students develop skills including presenting effective and rigorous arguments, developing criticisms of other people’s arguments and views, explaining complex material clearly and concisely, and analysing philosophical problems where reasonable people hold different views. Provide structured yet flexible study informed by current research. Provide a curriculum covering texts and questions central to the analytical tradition in philosophy and traditions outside it. Develop subject-specific knowledge, cognitive skills and transferable skills for employment or further academic study. Students may apply to study abroad for a year at partner universities. Students may apply for a paid Q-Step internship between Years 2 and 3. Students may undertake a Professional Experience Year, extending the degree to four years. Philosophy graduates pursue careers in journalism, media, charities, consultancy, civil service, finance, marketing, public relations, social work, teaching and law. Recent graduates have worked for organisations including Manchester City Council, Royal Bank of Scotland, Palgrave MacMillan, Lloyds TSB, the Foreign and Commonwealth Office, TeachFirst and Siemens. Many graduates undertake postgraduate study in philosophy, teaching, law, political theory, business or marketing.
@@ -1184,21 +1086,16 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Economics and Politics; Global Politics; Journalism and Politics; Law with Politics; Modern History and Politics; Philosophy and Politics; Philosophy, Politics and Economics; Politics and International Relations; Politics with Business</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
           <t>What is the BA Politics? The BA Politics is a three-year degree. You’ll examine the structures, ideas, and decisions that shape societies, from political institutions and democratic processes to power, rights, and governance. Combining critical theory, case studies, and applied analysis, you’ll develop the insight and practical skills needed to interpret complex political issues, policy debates, and real-world political decision-making. The BA Politics degree trains you to go beyond opinion and ask the crucial question: how do you know? This makes the course particularly well suited to students who enjoy evidence, debate, and complexity rather than simple answers. You’ll tackle power, justice, democracy, and rights, while addressing real-world challenges like conflict, authoritarianism, and human rights. Learn from leading academics in a department whose research informs government policy, international organisations, and public debate. You’ll see first-hand how theory informs real-world decisions and develop practical skills in analysis, argumentation, and decision-making. Personalise your degree with a specialist module pathway, gaining expertise in a particular area of politics that strengthens your CV, postgraduate applications, and demonstrates your command of the field. This course will teach you how to analyse political systems, assess policy decisions, and apply theory to real-world governance challenges. You’ll develop the confidence and skills to think critically, argue persuasively, and make informed decisions, valuable skills for a wide range of early careers or further postgraduate study. The course covers areas including political systems and theory, examining how states, laws, wars, parties and institutions shape obligations, freedom, rights and equality; democracy and power, exploring why people engage or disengage with politics and how voting, participation and influence operate in practice; global politics, examining international relations, conflict and authoritarianism and how national and global forces intersect; applied analysis, connecting political science theory to real-world policy, governance and decision-making challenges; and research methods, developing rigorous quantitative and qualitative skills with the option to enhance expertise through advanced data analysis. Students can develop additional expertise through named specialisms such as Data Science (Q-Step Pathway), which provides advanced quantitative and data analysis skills alongside political study; Justice and Human Rights, focusing on justice, rights and accountability across domestic and international contexts; and Political Economy and Development, examining how political power, economic systems and inequality shape development at local, national and global levels. A BA Politics degree prepares graduates for careers in areas such as government and public service including policy advisors, civil servants, legislative assistants and political analysts; international organisations and diplomacy including the UN, EU, NATO, Commonwealth and development agencies; non-governmental and advocacy sectors such as human rights organisations and development charities; media and communications including political journalism and public affairs; consultancy and think tanks including political risk analysis and policy consultancy; and research or postgraduate study in politics, international relations or public policy. Graduates from this course have progressed to roles in organisations including the House of Commons, Essex Police Force, Essex County Council, London Borough of Lewisham and Sky News.</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Understand and address the key issues facing our country, and the wider world. Politics allows us to understand how governments, policies, and international relations work. Many important questions or global challenges, like human rights issues, poverty, equality, and welfare, can be addressed through an understanding of this topic. A degree in politics can lead to a career in many different sectors. If you become an MP, you could represent your constituents, and progress to party whip or leader, a committee chair, cabinet minister, or even prime minister. Or you could work in business, diplomacy, the civil service or human resources, among other things. Understanding politics, introduction to political theory, understanding international relations, global history, pathways to political research, political and economic data analysis and emerging powers in a changing world are areas you could study. Negotiation, effective debating and data analysis are hard skills you'll develop. Written and verbal communication, empathy, listening skills, leadership and logic and reasoning are soft skills you'll develop. Career options include politician, local government officer, public relations professional, journalist, human resources roles, finance roles and public services roles.</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr">
-        <is>
-          <t>Understand and address the key issues facing our country, and the wider world. Politics allows us to understand how governments, policies, and international relations work. Many important questions or global challenges, like human rights issues, poverty, equality, and welfare, can be addressed through an understanding of this topic. A degree in politics can lead to a career in many different sectors. If you become an MP, you could represent your constituents, and progress to party whip or leader, a committee chair, cabinet minister, or even prime minister. Or you could work in business, diplomacy, the civil service or human resources, among other things. Understanding politics, introduction to political theory, understanding international relations, global history, pathways to political research, political and economic data analysis and emerging powers in a changing world are areas you could study. Negotiation, effective debating and data analysis are hard skills you'll develop. Written and verbal communication, empathy, listening skills, leadership and logic and reasoning are soft skills you'll develop. Career options include politician, local government officer, public relations professional, journalist, human resources roles, finance roles and public services roles.</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
         <is>
           <t>Essex: What is the BA Politics? The BA Politics is a three-year degree. You’ll examine the structures, ideas, and decisions that shape societies, from political institutions and democratic processes to power, rights, and governance. Combining critical theory, case studies, and applied analysis, you’ll develop the insight and practical skills needed to interpret complex political issues, policy debates, and real-world political decision-making. The BA Politics degree trains you to go beyond opinion and ask the crucial question: how do you know? This makes the course particularly well suited to students who enjoy evidence, debate, and complexity rather than simple answers. You’ll tackle power, justice, democracy, and rights, while addressing real-world challenges like conflict, authoritarianism, and human rights. Learn from leading academics in a department whose research informs government policy, international organisations, and public debate. You’ll see first-hand how theory informs real-world decisions and develop practical skills in analysis, argumentation, and decision-making. Personalise your degree with a specialist module pathway, gaining expertise in a particular area of politics that strengthens your CV, postgraduate applications, and demonstrates your command of the field. This course will teach you how to analyse political systems, assess policy decisions, and apply theory to real-world governance challenges. You’ll develop the confidence and skills to think critically, argue persuasively, and make informed decisions, valuable skills for a wide range of early careers or further postgraduate study. The course covers areas including political systems and theory, examining how states, laws, wars, parties and institutions shape obligations, freedom, rights and equality; democracy and power, exploring why people engage or disengage with politics and how voting, participation and influence operate in practice; global politics, examining international relations, conflict and authoritarianism and how national and global forces intersect; applied analysis, connecting political science theory to real-world policy, governance and decision-making challenges; and research methods, developing rigorous quantitative and qualitative skills with the option to enhance expertise through advanced data analysis. Students can develop additional expertise through named specialisms such as Data Science (Q-Step Pathway), which provides advanced quantitative and data analysis skills alongside political study; Justice and Human Rights, focusing on justice, rights and accountability across domestic and international contexts; and Political Economy and Development, examining how political power, economic systems and inequality shape development at local, national and global levels. A BA Politics degree prepares graduates for careers in areas such as government and public service including policy advisors, civil servants, legislative assistants and political analysts; international organisations and diplomacy including the UN, EU, NATO, Commonwealth and development agencies; non-governmental and advocacy sectors such as human rights organisations and development charities; media and communications including political journalism and public affairs; consultancy and think tanks including political risk analysis and policy consultancy; and research or postgraduate study in politics, international relations or public policy. Graduates from this course have progressed to roles in organisations including the House of Commons, Essex Police Force, Essex County Council, London Borough of Lewisham and Sky News.
 UCAS: Understand and address the key issues facing our country, and the wider world. Politics allows us to understand how governments, policies, and international relations work. Many important questions or global challenges, like human rights issues, poverty, equality, and welfare, can be addressed through an understanding of this topic. A degree in politics can lead to a career in many different sectors. If you become an MP, you could represent your constituents, and progress to party whip or leader, a committee chair, cabinet minister, or even prime minister. Or you could work in business, diplomacy, the civil service or human resources, among other things. Understanding politics, introduction to political theory, understanding international relations, global history, pathways to political research, political and economic data analysis and emerging powers in a changing world are areas you could study. Negotiation, effective debating and data analysis are hard skills you'll develop. Written and verbal communication, empathy, listening skills, leadership and logic and reasoning are soft skills you'll develop. Career options include politician, local government officer, public relations professional, journalist, human resources roles, finance roles and public services roles.</t>
@@ -1216,25 +1113,20 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Criminology with Social Psychology; Neural Engineering with Psychology; Psychology with Cognitive Neuroscience; Psychology with Economics; Psychology with Sport and Exercise; Sociology with Social Psychology</t>
+          <t>The BA (Hons) Psychology is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll gain a strong understanding of the theories and approaches in psychology today, preparing you to answer the world’s current challenges. The BA (Hons) Psychology gives you one of the most immersive and exciting experiences of studying human thoughts and behaviours in the UK. Your learning, like our research, focuses on innovative solutions to real societal challenges so you’ll develop the skills and knowledge to make a measurable difference in our world. Gain work experience alongside your studies by working one-on-one as a psychologist’s research assistant, undertaking an internship alongside health and wellbeing practitioners and supporting psychology outreach. You’ll graduate on the path to a psychologist or researcher career, with the foundations needed to specialise in areas such as clinical and educational psychology. The course explores different approaches to psychology including cognitive, developmental and social psychology, and allows you to tailor your degree through your choice of applied modules. A BA (Hons) Psychology degree prepares you for diverse careers including counselling and coaching, civil service roles such as policy development and social work, education including teaching and special education needs, business and finance roles such as market research and human resources, and psychology research. The course is accredited against the requirements for the Graduate Basis for Chartered Membership (GBC) of the British Psychological Society (BPS). This accreditation signifies that you have obtained a high standard of psychology education and is a crucial step for several career paths including becoming a chartered psychologist, ensuring the curriculum covers the knowledge and skills required for professional practice.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>The BA (Hons) Psychology is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll gain a strong understanding of the theories and approaches in psychology today, preparing you to answer the world’s current challenges. The BA (Hons) Psychology gives you one of the most immersive and exciting experiences of studying human thoughts and behaviours in the UK. Your learning, like our research, focuses on innovative solutions to real societal challenges so you’ll develop the skills and knowledge to make a measurable difference in our world. Gain work experience alongside your studies by working one-on-one as a psychologist’s research assistant, undertaking an internship alongside health and wellbeing practitioners and supporting psychology outreach. You’ll graduate on the path to a psychologist or researcher career, with the foundations needed to specialise in areas such as clinical and educational psychology. The course explores different approaches to psychology including cognitive, developmental and social psychology, and allows you to tailor your degree through your choice of applied modules. A BA (Hons) Psychology degree prepares you for diverse careers including counselling and coaching, civil service roles such as policy development and social work, education including teaching and special education needs, business and finance roles such as market research and human resources, and psychology research. The course is accredited against the requirements for the Graduate Basis for Chartered Membership (GBC) of the British Psychological Society (BPS). This accreditation signifies that you have obtained a high standard of psychology education and is a crucial step for several career paths including becoming a chartered psychologist, ensuring the curriculum covers the knowledge and skills required for professional practice.</t>
+          <t>The BSc Psychology degree is accredited by the British Psychological Society. The course consists of compulsory and optional units within and outside psychology. In the first two years students study biological psychology, cognitive psychology, developmental psychology, individual differences, social psychology, research methods and conceptual and historical issues in psychology. Teaching includes lectures, tutorials, practical classes, laboratory sessions and seminars. Students complete semester-long laboratory units in Years 1 and 2 to develop skills in designing, conducting and analysing research. In the final year students undertake an independent research project. Students complete a 30-hour placement in Year 2 and may undertake a full-year placement between Years 2 and 3 or study abroad at partner universities. A BPS-accredited psychology degree provides the first step towards careers such as clinical psychology, counselling psychology, health psychology, forensic psychology, organisational psychology, educational psychology and sports psychology. Graduates also work in careers including marketing, advertising, journalism, human resources, management consulting, academic research, teaching, policing, mental health services, counselling and social work. The course confers eligibility for Graduate Membership of the British Psychological Society and the Graduate Basis for Registration.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>The BSc Psychology degree is accredited by the British Psychological Society. The course consists of compulsory and optional units within and outside psychology. In the first two years students study biological psychology, cognitive psychology, developmental psychology, individual differences, social psychology, research methods and conceptual and historical issues in psychology. Teaching includes lectures, tutorials, practical classes, laboratory sessions and seminars. Students complete semester-long laboratory units in Years 1 and 2 to develop skills in designing, conducting and analysing research. In the final year students undertake an independent research project. Students complete a 30-hour placement in Year 2 and may undertake a full-year placement between Years 2 and 3 or study abroad at partner universities. A BPS-accredited psychology degree provides the first step towards careers such as clinical psychology, counselling psychology, health psychology, forensic psychology, organisational psychology, educational psychology and sports psychology. Graduates also work in careers including marketing, advertising, journalism, human resources, management consulting, academic research, teaching, policing, mental health services, counselling and social work. The course confers eligibility for Graduate Membership of the British Psychological Society and the Graduate Basis for Registration.</t>
+          <t>Psychology is a fascinating journey into understanding and decoding the human mind, offering valuable insights into behaviour, emotions, and the science behind why we do what we do. Psychology delves into the complexities of the human mind, examining behaviour, cognition, and emotions. Studying psychology opens doors to many different career opportunities. From clinical psychologists providing therapeutic support, to industrial-organisational psychologists shaping workplace dynamics, this subject offers the chance for understanding and improving all kinds of aspects of human life. Psychology is also transferable to other exciting careers such as marketing, human resources, and healthcare, making it a versatile foundation for personal and professional growth. Whether you choose to pursue counselling, research, or organisational development, a background in psychology gives you valuable insights into human behaviour and the skills to make a positive impact on both individuals and communities. Applied psychology, child psychology, clinical psychology, educational psychology, forensic psychology, sport psychology and experimental psychology are areas you could study. Enhanced research skills, data and statistical analysis, application of therapeutic techniques and evaluation of cognitive functions are hard skills you'll develop. Attentive and active listening, empathising with others, ability to adapt to new information and critical thinking and problem-solving skills are soft skills you'll develop. Career options include clinical psychologists, other psychologists, health professionals, occupational therapists, therapy professionals, business and related research professionals, market research interviewers, human resources and industrial relations officers, and human resource managers and directors.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
-        <is>
-          <t>Psychology is a fascinating journey into understanding and decoding the human mind, offering valuable insights into behaviour, emotions, and the science behind why we do what we do. Psychology delves into the complexities of the human mind, examining behaviour, cognition, and emotions. Studying psychology opens doors to many different career opportunities. From clinical psychologists providing therapeutic support, to industrial-organisational psychologists shaping workplace dynamics, this subject offers the chance for understanding and improving all kinds of aspects of human life. Psychology is also transferable to other exciting careers such as marketing, human resources, and healthcare, making it a versatile foundation for personal and professional growth. Whether you choose to pursue counselling, research, or organisational development, a background in psychology gives you valuable insights into human behaviour and the skills to make a positive impact on both individuals and communities. Applied psychology, child psychology, clinical psychology, educational psychology, forensic psychology, sport psychology and experimental psychology are areas you could study. Enhanced research skills, data and statistical analysis, application of therapeutic techniques and evaluation of cognitive functions are hard skills you'll develop. Attentive and active listening, empathising with others, ability to adapt to new information and critical thinking and problem-solving skills are soft skills you'll develop. Career options include clinical psychologists, other psychologists, health professionals, occupational therapists, therapy professionals, business and related research professionals, market research interviewers, human resources and industrial relations officers, and human resource managers and directors.</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
         <is>
           <t>Essex: The BA (Hons) Psychology is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll gain a strong understanding of the theories and approaches in psychology today, preparing you to answer the world’s current challenges. The BA (Hons) Psychology gives you one of the most immersive and exciting experiences of studying human thoughts and behaviours in the UK. Your learning, like our research, focuses on innovative solutions to real societal challenges so you’ll develop the skills and knowledge to make a measurable difference in our world. Gain work experience alongside your studies by working one-on-one as a psychologist’s research assistant, undertaking an internship alongside health and wellbeing practitioners and supporting psychology outreach. You’ll graduate on the path to a psychologist or researcher career, with the foundations needed to specialise in areas such as clinical and educational psychology. The course explores different approaches to psychology including cognitive, developmental and social psychology, and allows you to tailor your degree through your choice of applied modules. A BA (Hons) Psychology degree prepares you for diverse careers including counselling and coaching, civil service roles such as policy development and social work, education including teaching and special education needs, business and finance roles such as market research and human resources, and psychology research. The course is accredited against the requirements for the Graduate Basis for Chartered Membership (GBC) of the British Psychological Society (BPS). This accreditation signifies that you have obtained a high standard of psychology education and is a crucial step for several career paths including becoming a chartered psychologist, ensuring the curriculum covers the knowledge and skills required for professional practice.
 Manchester: The BSc Psychology degree is accredited by the British Psychological Society. The course consists of compulsory and optional units within and outside psychology. In the first two years students study biological psychology, cognitive psychology, developmental psychology, individual differences, social psychology, research methods and conceptual and historical issues in psychology. Teaching includes lectures, tutorials, practical classes, laboratory sessions and seminars. Students complete semester-long laboratory units in Years 1 and 2 to develop skills in designing, conducting and analysing research. In the final year students undertake an independent research project. Students complete a 30-hour placement in Year 2 and may undertake a full-year placement between Years 2 and 3 or study abroad at partner universities. A BPS-accredited psychology degree provides the first step towards careers such as clinical psychology, counselling psychology, health psychology, forensic psychology, organisational psychology, educational psychology and sports psychology. Graduates also work in careers including marketing, advertising, journalism, human resources, management consulting, academic research, teaching, policing, mental health services, counselling and social work. The course confers eligibility for Graduate Membership of the British Psychological Society and the Graduate Basis for Registration.
@@ -1253,25 +1145,20 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>History and Sociology; Sociology and Criminology; Sociology with Social Psychology</t>
+          <t>What holds societies together? Do people pull together because they have to or because they want to? What motivates so many people to migrate from their own societies to others? On our course you explore why individuals, groups, and cultures are the way they are, and examine why they might be different. At Essex we investigate what connects people with each other, as well as what divides them. You can study topics such as digital media and society, psychiatry and mental illness, sexualities, crime, childhood, and the art, film and personal testimony of war. We offer a range of specialisms including social divisions, inequality, the nature of work and commercial culture; culture, identity and subjectivity; public policy regarding health, the environment, crime and aging; citizenship, multiculturalism and human rights. You also receive training in sociological methods including how to design a survey, conduct an interview, and use quantitative analysis from basic statistics to big data in order to ask complex social questions. You also have the opportunity to complete a supervised dissertation on the topic that most inspires you, encouraging you to think differently, connect with contemporary social issues and debates, and prepare for your graduate career. Through our Q-Step Affiliate Status, you also have the opportunity to follow a specialised pathway that embeds quantitative methods in your degree, and successful completion of specified modules entitles you to receive the qualifier “Applied Quantitative Methods” on your degree transcript. Sociology graduates are in demand across a wide range of sectors including local and central government, NGOs, social work, market research, project management, fundraising, auditing, marketing, case-work, youth and community work, voluntary sector management and lobbying. Recent graduates have gone on to work for organisations including The Institute of Public Finance, Guardian Professional, United, and Synergy Healthcare Research.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>What holds societies together? Do people pull together because they have to or because they want to? What motivates so many people to migrate from their own societies to others? On our course you explore why individuals, groups, and cultures are the way they are, and examine why they might be different. At Essex we investigate what connects people with each other, as well as what divides them. You can study topics such as digital media and society, psychiatry and mental illness, sexualities, crime, childhood, and the art, film and personal testimony of war. We offer a range of specialisms including social divisions, inequality, the nature of work and commercial culture; culture, identity and subjectivity; public policy regarding health, the environment, crime and aging; citizenship, multiculturalism and human rights. You also receive training in sociological methods including how to design a survey, conduct an interview, and use quantitative analysis from basic statistics to big data in order to ask complex social questions. You also have the opportunity to complete a supervised dissertation on the topic that most inspires you, encouraging you to think differently, connect with contemporary social issues and debates, and prepare for your graduate career. Through our Q-Step Affiliate Status, you also have the opportunity to follow a specialised pathway that embeds quantitative methods in your degree, and successful completion of specified modules entitles you to receive the qualifier “Applied Quantitative Methods” on your degree transcript. Sociology graduates are in demand across a wide range of sectors including local and central government, NGOs, social work, market research, project management, fundraising, auditing, marketing, case-work, youth and community work, voluntary sector management and lobbying. Recent graduates have gone on to work for organisations including The Institute of Public Finance, Guardian Professional, United, and Synergy Healthcare Research.</t>
+          <t>The BSocSc Sociology course enables students to understand the social contexts and interconnected forces that shape communities and human behaviour while developing critical perspectives on how societies function, change and influence everyday life. Teaching and research focus on analysing social conditions and challenging assumptions about the social world. Students engage with a wide range of research areas including decolonial thought, sustainability and environment, personal life and relationships, media and technology, race and ethnicity, social inequality, social movements, social theory, globalisation and social change, cultural practices and consumption, migration, work and economy, urban life and ageing. Methodological training includes survey methods and qualitative research approaches, culminating in an independent social research project in the final year that allows students to refine their interests and critical perspective. The programme may also include opportunities to engage with quantitative social science training initiatives such as Q-Step internships. Graduates develop analytical, research and communication skills applicable across sectors including public policy, media, international organisations and business, with alumni working at organisations such as the Ministry of Justice, the NHS, the British Council, Fujitsu, the United Nations Refugee Agency and Unilever.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>The BSocSc Sociology course enables students to understand the social contexts and interconnected forces that shape communities and human behaviour while developing critical perspectives on how societies function, change and influence everyday life. Teaching and research focus on analysing social conditions and challenging assumptions about the social world. Students engage with a wide range of research areas including decolonial thought, sustainability and environment, personal life and relationships, media and technology, race and ethnicity, social inequality, social movements, social theory, globalisation and social change, cultural practices and consumption, migration, work and economy, urban life and ageing. Methodological training includes survey methods and qualitative research approaches, culminating in an independent social research project in the final year that allows students to refine their interests and critical perspective. The programme may also include opportunities to engage with quantitative social science training initiatives such as Q-Step internships. Graduates develop analytical, research and communication skills applicable across sectors including public policy, media, international organisations and business, with alumni working at organisations such as the Ministry of Justice, the NHS, the British Council, Fujitsu, the United Nations Refugee Agency and Unilever.</t>
+          <t>Studying sociology will decode the hidden patterns that govern human behaviour and give you the tools to drive positive change. Studying sociology opens doors to a fascinating exploration of the world we live in. You’ll learn the tools to understand how societies tick, unravelling the mysteries of human behaviour, and diving into the diverse world of cultures and communities. Sociology isn’t just about books and theories – it will also open up a world of possibilities for your future career. You could end up in roles where you can make a real impact; shaping policies, carrying out social research, contributing to community development, or even championing causes that matter to you are all realistic career paths. Sociology is a route to understanding people and making a positive mark on the world. So, if you're looking for a subject that combines curiosity, empathy, and the potential to make a difference, sociology is a great choice to a fulfilling career. Urban sociology, individuals and society, applied ethics, nature and society, media and crime, mobilisation, social movements, and protest are areas you could study. Statistical analysis, qualitative research techniques, data interpretation and interviewing techniques are hard skills you'll develop. Active listening, cultural competence, problem-solving and writing and presentation skills are soft skills you'll develop. Career options include actuaries, economists and statisticians, market research interviewers, and business and related research professionals.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
-        <is>
-          <t>Studying sociology will decode the hidden patterns that govern human behaviour and give you the tools to drive positive change. Studying sociology opens doors to a fascinating exploration of the world we live in. You’ll learn the tools to understand how societies tick, unravelling the mysteries of human behaviour, and diving into the diverse world of cultures and communities. Sociology isn’t just about books and theories – it will also open up a world of possibilities for your future career. You could end up in roles where you can make a real impact; shaping policies, carrying out social research, contributing to community development, or even championing causes that matter to you are all realistic career paths. Sociology is a route to understanding people and making a positive mark on the world. So, if you're looking for a subject that combines curiosity, empathy, and the potential to make a difference, sociology is a great choice to a fulfilling career. Urban sociology, individuals and society, applied ethics, nature and society, media and crime, mobilisation, social movements, and protest are areas you could study. Statistical analysis, qualitative research techniques, data interpretation and interviewing techniques are hard skills you'll develop. Active listening, cultural competence, problem-solving and writing and presentation skills are soft skills you'll develop. Career options include actuaries, economists and statisticians, market research interviewers, and business and related research professionals.</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
         <is>
           <t>Essex: What holds societies together? Do people pull together because they have to or because they want to? What motivates so many people to migrate from their own societies to others? On our course you explore why individuals, groups, and cultures are the way they are, and examine why they might be different. At Essex we investigate what connects people with each other, as well as what divides them. You can study topics such as digital media and society, psychiatry and mental illness, sexualities, crime, childhood, and the art, film and personal testimony of war. We offer a range of specialisms including social divisions, inequality, the nature of work and commercial culture; culture, identity and subjectivity; public policy regarding health, the environment, crime and aging; citizenship, multiculturalism and human rights. You also receive training in sociological methods including how to design a survey, conduct an interview, and use quantitative analysis from basic statistics to big data in order to ask complex social questions. You also have the opportunity to complete a supervised dissertation on the topic that most inspires you, encouraging you to think differently, connect with contemporary social issues and debates, and prepare for your graduate career. Through our Q-Step Affiliate Status, you also have the opportunity to follow a specialised pathway that embeds quantitative methods in your degree, and successful completion of specified modules entitles you to receive the qualifier “Applied Quantitative Methods” on your degree transcript. Sociology graduates are in demand across a wide range of sectors including local and central government, NGOs, social work, market research, project management, fundraising, auditing, marketing, case-work, youth and community work, voluntary sector management and lobbying. Recent graduates have gone on to work for organisations including The Institute of Public Finance, Guardian Professional, United, and Synergy Healthcare Research.
 Manchester: The BSocSc Sociology course enables students to understand the social contexts and interconnected forces that shape communities and human behaviour while developing critical perspectives on how societies function, change and influence everyday life. Teaching and research focus on analysing social conditions and challenging assumptions about the social world. Students engage with a wide range of research areas including decolonial thought, sustainability and environment, personal life and relationships, media and technology, race and ethnicity, social inequality, social movements, social theory, globalisation and social change, cultural practices and consumption, migration, work and economy, urban life and ageing. Methodological training includes survey methods and qualitative research approaches, culminating in an independent social research project in the final year that allows students to refine their interests and critical perspective. The programme may also include opportunities to engage with quantitative social science training initiatives such as Q-Step internships. Graduates develop analytical, research and communication skills applicable across sectors including public policy, media, international organisations and business, with alumni working at organisations such as the Ministry of Justice, the NHS, the British Council, Fujitsu, the United Nations Refugee Agency and Unilever.
@@ -1290,21 +1177,16 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Occupational Therapy; Psychology with Sport and Exercise; Speech and Language Therapy; Sports Performance and Coaching; Sports Therapy; Sports and Exercise Science</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
           <t>The BSc (Hons) Sports and Exercise Science is a three-year degree. You’ll gain a new and exciting perspective on the world of sport, exercise, health and physical fitness, ready to help athletes optimise their performance and improve the physical activity, health and wellbeing of individuals and communities. The BSc (Hons) Sports and Exercise Science provides you with a strong understanding of the role of physiology, psychology, biomechanics and nutrition in sports and exercise. By focusing on practical work in your first two years, you’ll consolidate your professional and scientific skills needed for your final-year research project. You can also gain more real-world experience at our renowned Human Performance Unit (HPU) where you can work with performance scholars, students, staff and members of the public. You’ll graduate on the path to a sports practitioner or sports scientist career, ready to further research on or implement changes to sport and exercise. The course is suitable for future sports practitioners, coaches or researchers, those looking to optimise athletes’ performance or the fitness and wellbeing of the public, students considering careers through a broad understanding of sport and exercise science, and practical learners eager to put new knowledge into practice. You will learn topics such as how and why different energy systems are deployed at different exercise intensities, the biomechanical principles behind acute and chronic sporting injuries and how these can be applied to prevent injuries, the role of ergogenic aids in improving athletic performance, how physical activity and nutrition can reduce the risk of cardio-metabolic disease, and the design and implementation of psychological skills training programmes. The degree also allows you to tailor your studies through a choice of optional modules. A BSc (Hons) Sports and Exercise Science degree prepares you for careers in areas such as sports teams and clubs including coaching, sports development, performance analysis and centre management; national bodies including health improvement, sports development and health and safety; education including physical education teaching; health professions such as sports therapy, nutrition, physiology and sport psychology; and the fitness industry including fitness training and personal training. Graduates from this course have progressed to roles in organisations such as Triathlon England Youth Forum and York St. John University. The CASES Undergraduate Endorsement Scheme awards endorsement to sport and exercise science degree courses that demonstrate the required mapping of knowledge and skills, providing graduates with the competencies needed to enter the profession.</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Whether you want to work with your sporting heroes, with children, or the general public, this subject area offers access to a range of rewarding, active, and hands-on jobs. With a qualification in sport and exercise science, you may want to work with athletes on sports performance, become a sports coach or teacher, or manage a gym or fitness centre. You might be employed by a professional sports team, a local authority, the NHS, or a private fitness company, among others. You could also work for yourself. Some roles, like coaching and teaching roles or sports psychology, may require further study. Alternatively, you may choose to go into business management or community engagement projects, depending on what inspires you; you could even become a sports broadcaster. On most courses – and certainly on an apprenticeship – you’ll spend time in industry, which will give you networking opportunities and a great insight into where this subject could take you. Anatomy and physiology, sport biomechanics and kinesiology, data description and analysis, biochemistry and cell biology, foundations of sport and exercise psychology and applied studies across sport performance and health are areas you could study. Physical education, child protection, risk analysis and lesson planning are hard skills you'll develop. Teaching, management and communication are soft skills you'll develop. Career options include sports player, physiotherapist, coach, fitness instructor, broadcasting and media administrator, public relations officer, sports journalist and sport and leisure management.</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
-        <is>
-          <t>Whether you want to work with your sporting heroes, with children, or the general public, this subject area offers access to a range of rewarding, active, and hands-on jobs. With a qualification in sport and exercise science, you may want to work with athletes on sports performance, become a sports coach or teacher, or manage a gym or fitness centre. You might be employed by a professional sports team, a local authority, the NHS, or a private fitness company, among others. You could also work for yourself. Some roles, like coaching and teaching roles or sports psychology, may require further study. Alternatively, you may choose to go into business management or community engagement projects, depending on what inspires you; you could even become a sports broadcaster. On most courses – and certainly on an apprenticeship – you’ll spend time in industry, which will give you networking opportunities and a great insight into where this subject could take you. Anatomy and physiology, sport biomechanics and kinesiology, data description and analysis, biochemistry and cell biology, foundations of sport and exercise psychology and applied studies across sport performance and health are areas you could study. Physical education, child protection, risk analysis and lesson planning are hard skills you'll develop. Teaching, management and communication are soft skills you'll develop. Career options include sports player, physiotherapist, coach, fitness instructor, broadcasting and media administrator, public relations officer, sports journalist and sport and leisure management.</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
         <is>
           <t>Essex: The BSc (Hons) Sports and Exercise Science is a three-year degree. You’ll gain a new and exciting perspective on the world of sport, exercise, health and physical fitness, ready to help athletes optimise their performance and improve the physical activity, health and wellbeing of individuals and communities. The BSc (Hons) Sports and Exercise Science provides you with a strong understanding of the role of physiology, psychology, biomechanics and nutrition in sports and exercise. By focusing on practical work in your first two years, you’ll consolidate your professional and scientific skills needed for your final-year research project. You can also gain more real-world experience at our renowned Human Performance Unit (HPU) where you can work with performance scholars, students, staff and members of the public. You’ll graduate on the path to a sports practitioner or sports scientist career, ready to further research on or implement changes to sport and exercise. The course is suitable for future sports practitioners, coaches or researchers, those looking to optimise athletes’ performance or the fitness and wellbeing of the public, students considering careers through a broad understanding of sport and exercise science, and practical learners eager to put new knowledge into practice. You will learn topics such as how and why different energy systems are deployed at different exercise intensities, the biomechanical principles behind acute and chronic sporting injuries and how these can be applied to prevent injuries, the role of ergogenic aids in improving athletic performance, how physical activity and nutrition can reduce the risk of cardio-metabolic disease, and the design and implementation of psychological skills training programmes. The degree also allows you to tailor your studies through a choice of optional modules. A BSc (Hons) Sports and Exercise Science degree prepares you for careers in areas such as sports teams and clubs including coaching, sports development, performance analysis and centre management; national bodies including health improvement, sports development and health and safety; education including physical education teaching; health professions such as sports therapy, nutrition, physiology and sport psychology; and the fitness industry including fitness training and personal training. Graduates from this course have progressed to roles in organisations such as Triathlon England Youth Forum and York St. John University. The CASES Undergraduate Endorsement Scheme awards endorsement to sport and exercise science degree courses that demonstrate the required mapping of knowledge and skills, providing graduates with the competencies needed to enter the profession.
 UCAS: Whether you want to work with your sporting heroes, with children, or the general public, this subject area offers access to a range of rewarding, active, and hands-on jobs. With a qualification in sport and exercise science, you may want to work with athletes on sports performance, become a sports coach or teacher, or manage a gym or fitness centre. You might be employed by a professional sports team, a local authority, the NHS, or a private fitness company, among others. You could also work for yourself. Some roles, like coaching and teaching roles or sports psychology, may require further study. Alternatively, you may choose to go into business management or community engagement projects, depending on what inspires you; you could even become a sports broadcaster. On most courses – and certainly on an apprenticeship – you’ll spend time in industry, which will give you networking opportunities and a great insight into where this subject could take you. Anatomy and physiology, sport biomechanics and kinesiology, data description and analysis, biochemistry and cell biology, foundations of sport and exercise psychology and applied studies across sport performance and health are areas you could study. Physical education, child protection, risk analysis and lesson planning are hard skills you'll develop. Teaching, management and communication are soft skills you'll develop. Career options include sports player, physiotherapist, coach, fitness instructor, broadcasting and media administrator, public relations officer, sports journalist and sport and leisure management.</t>
@@ -1322,25 +1204,20 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Applied Biomedical Science</t>
+          <t>The BSc (Hons) Biomedical Science is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll gain the practical skills and knowledge needed to work in labs and hospitals across the NHS and private sector. The BSc (Hons) Biomedical Science gives you key knowledge and modern strategies to diagnose and treat the human immune system, pathogenic and non-pathogenic bacteria, haematology and blood transfusion, cell pathology and mechanisms of neurological diseases. Previous students have placed with GlaxoSmithKline (GSK), Proctor &amp; Gamble (P&amp;G), AquaTerra, AstraZeneca, Genzyme, Reckitt Benckiser, Thermo Fisher and Isogenica – some of our 40 partner labs. In Year One, you’ll participate in Science Week at Public Health England (PHE) in Colindale. In Year Two, you can visit hospitals in the Eastern Region and beyond. In your Final Year, you’ll attend our Biomedical Employability Day and have the chance to contribute to the IBMS Congress. You’ll graduate on the path to a career as a biomedical scientist or medical researcher. The course is suited to future biomedical scientists, students wanting to work in the NHS, those aiming to advance medical research, and future students of postgraduate medicine. You will study the biology of disease including immunity and a range of diseases, explore microbiology, biochemistry, medical genetics, haematology and pharmacology, and specialise through applied modules in areas such as cancer, neurological disease and virology. A BSc (Hons) Biomedical Science degree prepares you for diverse careers in hospitals, clinics and healthcare companies including biomedical science roles in the NHS, andrology, clinical perfusion, microbiology, toxicology, biotechnology, forensic science and pharmaceuticals, as well as postgraduate medicine, postgraduate research programmes and science teaching. Graduates from this course have progressed to roles in NHS hospitals including Cambridge, Chelmsford, Colchester, Public Health England in Colindale, Basildon, London, Bury St Edmunds, Harlow, Hastings, Ipswich, Norwich, Peterborough, Kent, Bedford and Romford. The course is accredited by the Institute of Biomedical Science (IBMS).</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>The BSc (Hons) Biomedical Science is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll gain the practical skills and knowledge needed to work in labs and hospitals across the NHS and private sector. The BSc (Hons) Biomedical Science gives you key knowledge and modern strategies to diagnose and treat the human immune system, pathogenic and non-pathogenic bacteria, haematology and blood transfusion, cell pathology and mechanisms of neurological diseases. Previous students have placed with GlaxoSmithKline (GSK), Proctor &amp; Gamble (P&amp;G), AquaTerra, AstraZeneca, Genzyme, Reckitt Benckiser, Thermo Fisher and Isogenica – some of our 40 partner labs. In Year One, you’ll participate in Science Week at Public Health England (PHE) in Colindale. In Year Two, you can visit hospitals in the Eastern Region and beyond. In your Final Year, you’ll attend our Biomedical Employability Day and have the chance to contribute to the IBMS Congress. You’ll graduate on the path to a career as a biomedical scientist or medical researcher. The course is suited to future biomedical scientists, students wanting to work in the NHS, those aiming to advance medical research, and future students of postgraduate medicine. You will study the biology of disease including immunity and a range of diseases, explore microbiology, biochemistry, medical genetics, haematology and pharmacology, and specialise through applied modules in areas such as cancer, neurological disease and virology. A BSc (Hons) Biomedical Science degree prepares you for diverse careers in hospitals, clinics and healthcare companies including biomedical science roles in the NHS, andrology, clinical perfusion, microbiology, toxicology, biotechnology, forensic science and pharmaceuticals, as well as postgraduate medicine, postgraduate research programmes and science teaching. Graduates from this course have progressed to roles in NHS hospitals including Cambridge, Chelmsford, Colchester, Public Health England in Colindale, Basildon, London, Bury St Edmunds, Harlow, Hastings, Ipswich, Norwich, Peterborough, Kent, Bedford and Romford. The course is accredited by the Institute of Biomedical Science (IBMS).</t>
+          <t>The BSc Biomedical Sciences course provides grounding in medically related disciplines including physiology, pharmacology, neuroscience, cell biology, microbiology, anatomy and histology, genetics, biochemistry and immunology. Students learn to apply biological science for medical use in areas such as research, health monitoring and treatment, supported by a strong emphasis on practical laboratory experience. The curriculum allows flexibility through options to broaden study by taking units from interdisciplinary programmes or related subject areas. Teaching is supported by specialist laboratory facilities enabling training in techniques such as polymerase chain reaction, DNA sequencing, gel electrophoresis, spectrophotometry, dissection and histology, electromyography, electrocardiography and immunofluorescence microscopy. In the final year students undertake an independent research project in bioscience laboratories equipped with advanced research technology. Graduates pursue careers in university research, pharmaceutical and bioscience industries and clinical or technical laboratory roles including progression to the NHS Scientist Training Programme, while others enter fields such as medical writing, health communication or teaching.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>The BSc Biomedical Sciences course provides grounding in medically related disciplines including physiology, pharmacology, neuroscience, cell biology, microbiology, anatomy and histology, genetics, biochemistry and immunology. Students learn to apply biological science for medical use in areas such as research, health monitoring and treatment, supported by a strong emphasis on practical laboratory experience. The curriculum allows flexibility through options to broaden study by taking units from interdisciplinary programmes or related subject areas. Teaching is supported by specialist laboratory facilities enabling training in techniques such as polymerase chain reaction, DNA sequencing, gel electrophoresis, spectrophotometry, dissection and histology, electromyography, electrocardiography and immunofluorescence microscopy. In the final year students undertake an independent research project in bioscience laboratories equipped with advanced research technology. Graduates pursue careers in university research, pharmaceutical and bioscience industries and clinical or technical laboratory roles including progression to the NHS Scientist Training Programme, while others enter fields such as medical writing, health communication or teaching.</t>
+          <t>Biomedical scientists endeavour to understand the inner workings of the human body so they can provide the right care for patients, and tackle some of the most serious diseases threatening mankind. Ever wondered who the scientists were behind the statistical data that informed governments’ decisions during the Covid-19 pandemic? As a biomedical scientist, you’ll research and understand how the human body works, both in health and disease. You’ll learn about genetics, genomics, pathology, cellular biology, and immunity, among other things. It could lead to a career as a biomedical scientist, medical laboratory assistant, research technician, or marketing assistant. You could progress to teaching, postgraduate study, or even into medicine or dentistry. It’s a relatively stable industry, with 3.31% job growth predicted over the next eight years. Biochemistry, molecular biology, laboratory science, genetics, microbiology, anatomy, physiology, cells of the nervous system and pharmacology are areas you could study. An IBMS accredited biomedical science degree is the key to becoming a registered biomedical scientist in the UK. To practise as a biomedical scientist in the UK, you must be registered with the Health &amp; Care Professions Council (HCPC), and an IBMS accredited degree is a crucial step in meeting their strict requirements. Getting your HCPC registration also involves hands-on training in an IBMS-approved training laboratory, and an accredited degree often streamlines this process, sometimes even incorporating a clinical placement to complete the IBMS Registration Training Portfolio into the program itself. These specialised degrees are designed to meet the requirements for a biomedical scientist role but also provide you with excellent transferable, technical, and practical skills that a variety of employers demand. Biology, biochemistry, project management, data analysis and microbiology are hard skills you'll develop. Research, communications, management, planning and innovation are soft skills you'll develop. Career options include environment professionals, conservation professionals, biochemists and biomedical scientists, biological scientists, chemical scientists, laboratory technicians, pharmacists, pharmaceutical technicians, specialist medical practitioners and nursing auxiliaries and assistants.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
-        <is>
-          <t>Biomedical scientists endeavour to understand the inner workings of the human body so they can provide the right care for patients, and tackle some of the most serious diseases threatening mankind. Ever wondered who the scientists were behind the statistical data that informed governments’ decisions during the Covid-19 pandemic? As a biomedical scientist, you’ll research and understand how the human body works, both in health and disease. You’ll learn about genetics, genomics, pathology, cellular biology, and immunity, among other things. It could lead to a career as a biomedical scientist, medical laboratory assistant, research technician, or marketing assistant. You could progress to teaching, postgraduate study, or even into medicine or dentistry. It’s a relatively stable industry, with 3.31% job growth predicted over the next eight years. Biochemistry, molecular biology, laboratory science, genetics, microbiology, anatomy, physiology, cells of the nervous system and pharmacology are areas you could study. An IBMS accredited biomedical science degree is the key to becoming a registered biomedical scientist in the UK. To practise as a biomedical scientist in the UK, you must be registered with the Health &amp; Care Professions Council (HCPC), and an IBMS accredited degree is a crucial step in meeting their strict requirements. Getting your HCPC registration also involves hands-on training in an IBMS-approved training laboratory, and an accredited degree often streamlines this process, sometimes even incorporating a clinical placement to complete the IBMS Registration Training Portfolio into the program itself. These specialised degrees are designed to meet the requirements for a biomedical scientist role but also provide you with excellent transferable, technical, and practical skills that a variety of employers demand. Biology, biochemistry, project management, data analysis and microbiology are hard skills you'll develop. Research, communications, management, planning and innovation are soft skills you'll develop. Career options include environment professionals, conservation professionals, biochemists and biomedical scientists, biological scientists, chemical scientists, laboratory technicians, pharmacists, pharmaceutical technicians, specialist medical practitioners and nursing auxiliaries and assistants.</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
         <is>
           <t>Essex: The BSc (Hons) Biomedical Science is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll gain the practical skills and knowledge needed to work in labs and hospitals across the NHS and private sector. The BSc (Hons) Biomedical Science gives you key knowledge and modern strategies to diagnose and treat the human immune system, pathogenic and non-pathogenic bacteria, haematology and blood transfusion, cell pathology and mechanisms of neurological diseases. Previous students have placed with GlaxoSmithKline (GSK), Proctor &amp; Gamble (P&amp;G), AquaTerra, AstraZeneca, Genzyme, Reckitt Benckiser, Thermo Fisher and Isogenica – some of our 40 partner labs. In Year One, you’ll participate in Science Week at Public Health England (PHE) in Colindale. In Year Two, you can visit hospitals in the Eastern Region and beyond. In your Final Year, you’ll attend our Biomedical Employability Day and have the chance to contribute to the IBMS Congress. You’ll graduate on the path to a career as a biomedical scientist or medical researcher. The course is suited to future biomedical scientists, students wanting to work in the NHS, those aiming to advance medical research, and future students of postgraduate medicine. You will study the biology of disease including immunity and a range of diseases, explore microbiology, biochemistry, medical genetics, haematology and pharmacology, and specialise through applied modules in areas such as cancer, neurological disease and virology. A BSc (Hons) Biomedical Science degree prepares you for diverse careers in hospitals, clinics and healthcare companies including biomedical science roles in the NHS, andrology, clinical perfusion, microbiology, toxicology, biotechnology, forensic science and pharmaceuticals, as well as postgraduate medicine, postgraduate research programmes and science teaching. Graduates from this course have progressed to roles in NHS hospitals including Cambridge, Chelmsford, Colchester, Public Health England in Colindale, Basildon, London, Bury St Edmunds, Harlow, Hastings, Ipswich, Norwich, Peterborough, Kent, Bedford and Romford. The course is accredited by the Institute of Biomedical Science (IBMS).
 Manchester: The BSc Biomedical Sciences course provides grounding in medically related disciplines including physiology, pharmacology, neuroscience, cell biology, microbiology, anatomy and histology, genetics, biochemistry and immunology. Students learn to apply biological science for medical use in areas such as research, health monitoring and treatment, supported by a strong emphasis on practical laboratory experience. The curriculum allows flexibility through options to broaden study by taking units from interdisciplinary programmes or related subject areas. Teaching is supported by specialist laboratory facilities enabling training in techniques such as polymerase chain reaction, DNA sequencing, gel electrophoresis, spectrophotometry, dissection and histology, electromyography, electrocardiography and immunofluorescence microscopy. In the final year students undertake an independent research project in bioscience laboratories equipped with advanced research technology. Graduates pursue careers in university research, pharmaceutical and bioscience industries and clinical or technical laboratory roles including progression to the NHS Scientist Training Programme, while others enter fields such as medical writing, health communication or teaching.
@@ -1357,19 +1234,18 @@
           <t>LIBERAL ARTS</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Knowledge is rooted in the experiences of people across the world. It is created from memory, culture, landscape and myth. This knowledge is often split into separate ‘disciplines' such as those in the sciences, maths, history, geography, literature and art. However, true knowledge does not recognise these boundaries; the world is complex, interconnected and networked. Our course is for you if you love studying a variety of subjects, and want to maintain this breadth of knowledge at university. With the opportunity to major in Psychology, History, Literature, Art History, Philosophy, Politics, Media Studies or Sociology, you broaden your horizons by exploring the ways in which the humanities and social sciences help us to think imaginatively and critically about the worlds we live in. You take modules which cover the historical foundations of the humanities, challenge dominant worldviews, and explore innovative and subversive essays and manifestos. The flexible structure of this course allows you to choose a range of optional modules across literature, film, philosophy, history of art, history, linguistics, politics, sociology and modern languages. The types of issues and problems you might explore include how commercial and independent films interpret human relationships, how to compose your own writing inspired by the great essayists, important philosophical questions about life, death and religion, great works of art and literature, and languages. Based within our School of Philosophical, Historical and Interdisciplinary Studies, the choice is yours: you choose your modules based on your own background and interests. You engage with unusual, controversial, and provocative ideas so that you can use the humanities and social sciences to become critically aware and possess the tools to change the world for the better. As a liberal arts graduate, you'll be provided with an all-round education that can lead to a more extensive range of knowledge, better communication skills and a more flexible and positive attitude to life. The best way to prepare for the future is to develop the abilities and skills which make you resilient; reasoning skills which mean that you do not accept easy answers so that you can always question. A Liberal Arts course can lead to a wide variety of careers in the media, journalism, publishing, local government, voluntary agencies, librarianship, finance, management and other fields. Many employers prefer to recruit students with a broad-based liberal arts education and provide them with vocational training during their first year at work rather than recruit students who have specialised in one discipline. Our recent graduates have gone on to work for a wide range of organisations including Euromoney, a financial publication company, a housing association, and an English language school in Japan.</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Knowledge is rooted in the experiences of people across the world. It is created from memory, culture, landscape and myth. This knowledge is often split into separate ‘disciplines' such as those in the sciences, maths, history, geography, literature and art. However, true knowledge does not recognise these boundaries; the world is complex, interconnected and networked. Our course is for you if you love studying a variety of subjects, and want to maintain this breadth of knowledge at university. With the opportunity to major in Psychology, History, Literature, Art History, Philosophy, Politics, Media Studies or Sociology, you broaden your horizons by exploring the ways in which the humanities and social sciences help us to think imaginatively and critically about the worlds we live in. You take modules which cover the historical foundations of the humanities, challenge dominant worldviews, and explore innovative and subversive essays and manifestos. The flexible structure of this course allows you to choose a range of optional modules across literature, film, philosophy, history of art, history, linguistics, politics, sociology and modern languages. The types of issues and problems you might explore include how commercial and independent films interpret human relationships, how to compose your own writing inspired by the great essayists, important philosophical questions about life, death and religion, great works of art and literature, and languages. Based within our School of Philosophical, Historical and Interdisciplinary Studies, the choice is yours: you choose your modules based on your own background and interests. You engage with unusual, controversial, and provocative ideas so that you can use the humanities and social sciences to become critically aware and possess the tools to change the world for the better. As a liberal arts graduate, you'll be provided with an all-round education that can lead to a more extensive range of knowledge, better communication skills and a more flexible and positive attitude to life. The best way to prepare for the future is to develop the abilities and skills which make you resilient; reasoning skills which mean that you do not accept easy answers so that you can always question. A Liberal Arts course can lead to a wide variety of careers in the media, journalism, publishing, local government, voluntary agencies, librarianship, finance, management and other fields. Many employers prefer to recruit students with a broad-based liberal arts education and provide them with vocational training during their first year at work rather than recruit students who have specialised in one discipline. Our recent graduates have gone on to work for a wide range of organisations including Euromoney, a financial publication company, a housing association, and an English language school in Japan.</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
           <t>Liberal Arts is highly flexible, allowing students to create their own unique course by combining different subject areas within and beyond the School of Arts, Languages and Cultures. With an emphasis on interdisciplinary learning, students can tailor the course to align with their interests while engaging with key issues that affect society. The programme enables students to develop a broad academic foundation across areas such as economics, globalisation, environmental science, anthropology, sociology and philosophy, supporting the ability to analyse complex real-world challenges from multiple perspectives. Teaching makes use of distinctive research and cultural resources including the internationally renowned John Rylands Library with its collections of rare books, manuscripts and archives, as well as engagement with institutions such as Manchester Museum, Whitworth Art Gallery, the Museum of Medicine and Health and the Museum of Science and Industry. Studying the degree helps develop transferable and specialist skills including independent working, time management and planning, collaboration, teamwork, leadership, communication across diverse audiences and the ability to conduct research that responds to real-world challenges through engagement with organisations and institutions. Graduates pursue careers across sectors including media, public policy, cultural organisations, business and research-oriented roles.</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr">
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
         <is>
           <t>Essex: Knowledge is rooted in the experiences of people across the world. It is created from memory, culture, landscape and myth. This knowledge is often split into separate ‘disciplines' such as those in the sciences, maths, history, geography, literature and art. However, true knowledge does not recognise these boundaries; the world is complex, interconnected and networked. Our course is for you if you love studying a variety of subjects, and want to maintain this breadth of knowledge at university. With the opportunity to major in Psychology, History, Literature, Art History, Philosophy, Politics, Media Studies or Sociology, you broaden your horizons by exploring the ways in which the humanities and social sciences help us to think imaginatively and critically about the worlds we live in. You take modules which cover the historical foundations of the humanities, challenge dominant worldviews, and explore innovative and subversive essays and manifestos. The flexible structure of this course allows you to choose a range of optional modules across literature, film, philosophy, history of art, history, linguistics, politics, sociology and modern languages. The types of issues and problems you might explore include how commercial and independent films interpret human relationships, how to compose your own writing inspired by the great essayists, important philosophical questions about life, death and religion, great works of art and literature, and languages. Based within our School of Philosophical, Historical and Interdisciplinary Studies, the choice is yours: you choose your modules based on your own background and interests. You engage with unusual, controversial, and provocative ideas so that you can use the humanities and social sciences to become critically aware and possess the tools to change the world for the better. As a liberal arts graduate, you'll be provided with an all-round education that can lead to a more extensive range of knowledge, better communication skills and a more flexible and positive attitude to life. The best way to prepare for the future is to develop the abilities and skills which make you resilient; reasoning skills which mean that you do not accept easy answers so that you can always question. A Liberal Arts course can lead to a wide variety of careers in the media, journalism, publishing, local government, voluntary agencies, librarianship, finance, management and other fields. Many employers prefer to recruit students with a broad-based liberal arts education and provide them with vocational training during their first year at work rather than recruit students who have specialised in one discipline. Our recent graduates have gone on to work for a wide range of organisations including Euromoney, a financial publication company, a housing association, and an English language school in Japan.
 Manchester: Liberal Arts is highly flexible, allowing students to create their own unique course by combining different subject areas within and beyond the School of Arts, Languages and Cultures. With an emphasis on interdisciplinary learning, students can tailor the course to align with their interests while engaging with key issues that affect society. The programme enables students to develop a broad academic foundation across areas such as economics, globalisation, environmental science, anthropology, sociology and philosophy, supporting the ability to analyse complex real-world challenges from multiple perspectives. Teaching makes use of distinctive research and cultural resources including the internationally renowned John Rylands Library with its collections of rare books, manuscripts and archives, as well as engagement with institutions such as Manchester Museum, Whitworth Art Gallery, the Museum of Medicine and Health and the Museum of Science and Industry. Studying the degree helps develop transferable and specialist skills including independent working, time management and planning, collaboration, teamwork, leadership, communication across diverse audiences and the ability to conduct research that responds to real-world challenges through engagement with organisations and institutions. Graduates pursue careers across sectors including media, public policy, cultural organisations, business and research-oriented roles.</t>
@@ -1387,21 +1263,16 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Electronic Engineering; Neural Engineering with Psychology</t>
+          <t>The BEng (Hons) Robotic Engineering is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll build a strong foundation in electrical engineering and computer science theory, as well as the skills and tools to develop and test your own robotic systems. The BEng (Hons) Robotic Engineering gives you the theory and practical knowledge to understand – and create – robotics that make a real impact on the world. Discover which areas you’re interested in exploring further such as assistive technologies, computer games, artificial intelligence, evolutionary computation, Big Data or robotics. You’ll also be able to undertake a project or product development specified by a member of academic staff or a partner company. You’ll graduate as a creative, experimental and focused robotics engineer ready to explore further how robots, animatronics and robotic equipment can impact the world around you. You will explore robotics and artificial intelligence, master the scientific and engineering foundations of electronics and digital systems, learn to programme and apply mathematical skills to engineering, and tailor your degree through your choice of optional modules. The course provides access to specialist robotics facilities including a robotics gaming laboratory and robot arena with one of the world’s largest powered lab floors, and specialist robotics equipment such as wheeled and flying robots, robotic fish, intelligent wheelchairs, robotic arms and robotic hands. A BEng (Hons) Robotic Engineering degree prepares you for diverse careers in engineering including design, development, research, diagnostics and manufacture; IT including software, hardware, systems integration, control systems and automation; healthcare technologies such as surgical instruments, diagnostic tools and assistive technologies; research fields including space and deep ocean exploration; and business roles such as marketing, management, consultancy and patent law. The course is accredited by BCS, the Chartered Institute for IT for the purposes of fully meeting the academic requirement for registration as a Chartered IT Professional, and by BCS and the Institution of Engineering and Technology (IET) on behalf of the Engineering Council for the purposes of fully meeting the academic requirement for registration as an Incorporated Engineer and partially meeting the academic requirement for registration as a Chartered Engineer.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>The BEng (Hons) Robotic Engineering is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll build a strong foundation in electrical engineering and computer science theory, as well as the skills and tools to develop and test your own robotic systems. The BEng (Hons) Robotic Engineering gives you the theory and practical knowledge to understand – and create – robotics that make a real impact on the world. Discover which areas you’re interested in exploring further such as assistive technologies, computer games, artificial intelligence, evolutionary computation, Big Data or robotics. You’ll also be able to undertake a project or product development specified by a member of academic staff or a partner company. You’ll graduate as a creative, experimental and focused robotics engineer ready to explore further how robots, animatronics and robotic equipment can impact the world around you. You will explore robotics and artificial intelligence, master the scientific and engineering foundations of electronics and digital systems, learn to programme and apply mathematical skills to engineering, and tailor your degree through your choice of optional modules. The course provides access to specialist robotics facilities including a robotics gaming laboratory and robot arena with one of the world’s largest powered lab floors, and specialist robotics equipment such as wheeled and flying robots, robotic fish, intelligent wheelchairs, robotic arms and robotic hands. A BEng (Hons) Robotic Engineering degree prepares you for diverse careers in engineering including design, development, research, diagnostics and manufacture; IT including software, hardware, systems integration, control systems and automation; healthcare technologies such as surgical instruments, diagnostic tools and assistive technologies; research fields including space and deep ocean exploration; and business roles such as marketing, management, consultancy and patent law. The course is accredited by BCS, the Chartered Institute for IT for the purposes of fully meeting the academic requirement for registration as a Chartered IT Professional, and by BCS and the Institution of Engineering and Technology (IET) on behalf of the Engineering Council for the purposes of fully meeting the academic requirement for registration as an Incorporated Engineer and partially meeting the academic requirement for registration as a Chartered Engineer.</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
           <t>Mechatronic Engineering combines mechanical engineering with electronics and intelligent control systems and is central to areas such as industrial automation and robotics. The programme develops understanding of how sensors detect position, orientation and signals, how electronic inputs are interpreted and how actuators perform controlled operations using feedback control systems. Students learn techniques required for the design and implementation of intelligent mechatronic and autonomous systems including robotics, embedded systems and control technologies. Practical application and project-based learning are strong themes throughout the course. The curriculum structure allows flexibility during the early stages of study, enabling students to transfer between Mechatronic Engineering and Electrical and Electronic Engineering pathways. Teaching is supported by access to specialist engineering research infrastructure and industry-standard equipment including facilities such as the High Voltage Laboratory, Photon Science Institute, National Graphene Institute and Rolls-Royce University Technology Centre. Graduates develop technical and problem-solving skills applicable across sectors including robotics development, automotive electronics, renewable energy systems, automation and control engineering and unmanned vehicle guidance systems, with alumni securing roles at organisations such as BP, Rolls-Royce, Jaguar Land Rover, ABB, BAE Systems, Siemens and Jacobs. The course is accredited by the Institution of Engineering and Technology and the Institute of Measurement and Control, supporting progression towards Incorporated or Chartered Engineer status.</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr">
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
         <is>
           <t>Essex: The BEng (Hons) Robotic Engineering is a three-year degree, extendable to four with an optional year in placement or abroad. You’ll build a strong foundation in electrical engineering and computer science theory, as well as the skills and tools to develop and test your own robotic systems. The BEng (Hons) Robotic Engineering gives you the theory and practical knowledge to understand – and create – robotics that make a real impact on the world. Discover which areas you’re interested in exploring further such as assistive technologies, computer games, artificial intelligence, evolutionary computation, Big Data or robotics. You’ll also be able to undertake a project or product development specified by a member of academic staff or a partner company. You’ll graduate as a creative, experimental and focused robotics engineer ready to explore further how robots, animatronics and robotic equipment can impact the world around you. You will explore robotics and artificial intelligence, master the scientific and engineering foundations of electronics and digital systems, learn to programme and apply mathematical skills to engineering, and tailor your degree through your choice of optional modules. The course provides access to specialist robotics facilities including a robotics gaming laboratory and robot arena with one of the world’s largest powered lab floors, and specialist robotics equipment such as wheeled and flying robots, robotic fish, intelligent wheelchairs, robotic arms and robotic hands. A BEng (Hons) Robotic Engineering degree prepares you for diverse careers in engineering including design, development, research, diagnostics and manufacture; IT including software, hardware, systems integration, control systems and automation; healthcare technologies such as surgical instruments, diagnostic tools and assistive technologies; research fields including space and deep ocean exploration; and business roles such as marketing, management, consultancy and patent law. The course is accredited by BCS, the Chartered Institute for IT for the purposes of fully meeting the academic requirement for registration as a Chartered IT Professional, and by BCS and the Institution of Engineering and Technology (IET) on behalf of the Engineering Council for the purposes of fully meeting the academic requirement for registration as an Incorporated Engineer and partially meeting the academic requirement for registration as a Chartered Engineer.
 Manchester: Mechatronic Engineering combines mechanical engineering with electronics and intelligent control systems and is central to areas such as industrial automation and robotics. The programme develops understanding of how sensors detect position, orientation and signals, how electronic inputs are interpreted and how actuators perform controlled operations using feedback control systems. Students learn techniques required for the design and implementation of intelligent mechatronic and autonomous systems including robotics, embedded systems and control technologies. Practical application and project-based learning are strong themes throughout the course. The curriculum structure allows flexibility during the early stages of study, enabling students to transfer between Mechatronic Engineering and Electrical and Electronic Engineering pathways. Teaching is supported by access to specialist engineering research infrastructure and industry-standard equipment including facilities such as the High Voltage Laboratory, Photon Science Institute, National Graphene Institute and Rolls-Royce University Technology Centre. Graduates develop technical and problem-solving skills applicable across sectors including robotics development, automotive electronics, renewable energy systems, automation and control engineering and unmanned vehicle guidance systems, with alumni securing roles at organisations such as BP, Rolls-Royce, Jaguar Land Rover, ABB, BAE Systems, Siemens and Jacobs. The course is accredited by the Institution of Engineering and Technology and the Institute of Measurement and Control, supporting progression towards Incorporated or Chartered Engineer status.</t>

</xml_diff>